<commit_message>
Agrega columnas VENTAS SII / DIFERENCIA en cuadre de saldo
</commit_message>
<xml_diff>
--- a/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
+++ b/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1733" uniqueCount="499">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1739" uniqueCount="502">
   <si>
     <t xml:space="preserve">PRESUPUESTO Y FLUJO DE CAJA — AGOSTO 2026 (3 equipos)</t>
   </si>
@@ -1067,6 +1067,12 @@
     <t xml:space="preserve">D) CUADRE DE SALDO (control matemático de la cartola)</t>
   </si>
   <si>
+    <t xml:space="preserve">VENTAS SII</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIFERENCIA</t>
+  </si>
+  <si>
     <t xml:space="preserve">Saldo Inicial</t>
   </si>
   <si>
@@ -1083,6 +1089,9 @@
   </si>
   <si>
     <t xml:space="preserve">Diferencia (debe ser $0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nota columnas VENTAS SII / DIFERENCIA: comparación agregada (no factura por factura, esa está en la sección A) entre el total de Abonos reales de la cartola y el total facturado en Ventas RCV del mismo mes. La diferencia refleja: costo de factoring descontado, ingresos no facturados (ej. GETNET), facturas aún no cobradas, y/o pagos recibidos en la cuenta antigua (Santa Berenice) — pendiente de confirmar esto último.</t>
   </si>
   <si>
     <t xml:space="preserve">CONCILIACIÓN BANCARIA — JULIO 2026 (Global Solutions SPA, cartola PROVISORIA al 25-07-2026)</t>
@@ -1778,7 +1787,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="37">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1889,6 +1898,18 @@
     </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="7" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -3324,7 +3345,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I219"/>
+  <dimension ref="A1:I221"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -7615,10 +7636,16 @@
       <c r="B213" s="22" t="s">
         <v>3</v>
       </c>
+      <c r="C213" s="28" t="s">
+        <v>347</v>
+      </c>
+      <c r="D213" s="28" t="s">
+        <v>348</v>
+      </c>
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A214" s="23" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B214" s="24" t="n">
         <v>191906</v>
@@ -7626,15 +7653,23 @@
     </row>
     <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A215" s="23" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B215" s="24" t="n">
         <v>17630696</v>
       </c>
+      <c r="C215" s="29" t="n">
+        <f aca="false">F20</f>
+        <v>16410814</v>
+      </c>
+      <c r="D215" s="29" t="n">
+        <f aca="false">B215-C215</f>
+        <v>1219882</v>
+      </c>
     </row>
     <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A216" s="23" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B216" s="24" t="n">
         <v>-17555396</v>
@@ -7642,7 +7677,7 @@
     </row>
     <row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A217" s="25" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B217" s="26" t="n">
         <f aca="false">SUM(B214:B216)</f>
@@ -7651,7 +7686,7 @@
     </row>
     <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A218" s="25" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B218" s="26" t="n">
         <v>267206</v>
@@ -7659,21 +7694,34 @@
     </row>
     <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A219" s="25" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B219" s="26" t="n">
         <f aca="false">B217-B218</f>
         <v>0</v>
       </c>
     </row>
+    <row r="221" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A221" s="30" t="s">
+        <v>355</v>
+      </c>
+      <c r="B221" s="30"/>
+      <c r="C221" s="30"/>
+      <c r="D221" s="30"/>
+      <c r="E221" s="30"/>
+      <c r="F221" s="30"/>
+      <c r="G221" s="30"/>
+      <c r="H221" s="30"/>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A4:I4"/>
     <mergeCell ref="A22:I22"/>
     <mergeCell ref="A96:I96"/>
     <mergeCell ref="A212:I212"/>
+    <mergeCell ref="A221:H221"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -7690,7 +7738,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I160"/>
+  <dimension ref="A1:I162"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -7702,7 +7750,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -7715,7 +7763,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="20" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="B2" s="20"/>
       <c r="C2" s="20"/>
@@ -7767,13 +7815,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="D6" s="24" t="n">
         <v>370000</v>
@@ -7788,7 +7836,7 @@
         <v>156</v>
       </c>
       <c r="H6" s="23" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7796,10 +7844,10 @@
         <v>117</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="D7" s="24" t="n">
         <v>1818400</v>
@@ -7822,10 +7870,10 @@
         <v>117</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="D8" s="24" t="n">
         <v>2006400</v>
@@ -7845,13 +7893,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="23" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="D9" s="24" t="n">
         <v>580000</v>
@@ -7877,7 +7925,7 @@
         <v>123</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="D10" s="24" t="n">
         <v>370000</v>
@@ -7903,7 +7951,7 @@
         <v>6122312</v>
       </c>
       <c r="G11" s="27" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7947,13 +7995,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="23" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="D15" s="24" t="n">
         <v>17017</v>
@@ -7973,13 +8021,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="23" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="D16" s="24" t="n">
         <v>10168</v>
@@ -8002,10 +8050,10 @@
         <v>153</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="D17" s="24" t="n">
         <v>892481</v>
@@ -8020,18 +8068,18 @@
         <v>156</v>
       </c>
       <c r="H17" s="23" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="23" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="D18" s="24" t="n">
         <v>25210</v>
@@ -8046,7 +8094,7 @@
         <v>156</v>
       </c>
       <c r="H18" s="23" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8054,10 +8102,10 @@
         <v>158</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="D19" s="24" t="n">
         <v>19061</v>
@@ -8080,10 +8128,10 @@
         <v>235</v>
       </c>
       <c r="B20" s="23" t="s">
+        <v>380</v>
+      </c>
+      <c r="C20" s="23" t="s">
         <v>377</v>
-      </c>
-      <c r="C20" s="23" t="s">
-        <v>374</v>
       </c>
       <c r="D20" s="24" t="n">
         <v>251770</v>
@@ -8098,7 +8146,7 @@
         <v>156</v>
       </c>
       <c r="H20" s="23" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8106,10 +8154,10 @@
         <v>235</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="C21" s="23" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="D21" s="24" t="n">
         <v>18674</v>
@@ -8132,10 +8180,10 @@
         <v>191</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="D22" s="24" t="n">
         <v>77600</v>
@@ -8150,7 +8198,7 @@
         <v>156</v>
       </c>
       <c r="H22" s="23" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8158,10 +8206,10 @@
         <v>193</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="C23" s="23" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="D23" s="24" t="n">
         <v>15109</v>
@@ -8176,18 +8224,18 @@
         <v>156</v>
       </c>
       <c r="H23" s="23" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="23" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="B24" s="23" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="C24" s="23" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="D24" s="24" t="n">
         <v>66387</v>
@@ -8210,10 +8258,10 @@
         <v>182</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="C25" s="23" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="D25" s="24" t="n">
         <v>8403</v>
@@ -8236,10 +8284,10 @@
         <v>182</v>
       </c>
       <c r="B26" s="23" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="C26" s="23" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="D26" s="24" t="n">
         <v>29418</v>
@@ -8262,10 +8310,10 @@
         <v>182</v>
       </c>
       <c r="B27" s="23" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="C27" s="23" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="D27" s="24" t="n">
         <v>33298</v>
@@ -8280,7 +8328,7 @@
         <v>156</v>
       </c>
       <c r="H27" s="23" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8288,10 +8336,10 @@
         <v>182</v>
       </c>
       <c r="B28" s="23" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="D28" s="24" t="n">
         <v>8403</v>
@@ -8314,10 +8362,10 @@
         <v>158</v>
       </c>
       <c r="B29" s="23" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="C29" s="23" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="D29" s="24" t="n">
         <v>17771</v>
@@ -8340,10 +8388,10 @@
         <v>219</v>
       </c>
       <c r="B30" s="23" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="C30" s="23" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="D30" s="24" t="n">
         <v>30470</v>
@@ -8358,7 +8406,7 @@
         <v>156</v>
       </c>
       <c r="H30" s="23" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8366,10 +8414,10 @@
         <v>235</v>
       </c>
       <c r="B31" s="23" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="C31" s="23" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="D31" s="24" t="n">
         <v>40516</v>
@@ -8392,10 +8440,10 @@
         <v>235</v>
       </c>
       <c r="B32" s="23" t="s">
+        <v>402</v>
+      </c>
+      <c r="C32" s="23" t="s">
         <v>399</v>
-      </c>
-      <c r="C32" s="23" t="s">
-        <v>396</v>
       </c>
       <c r="D32" s="24" t="n">
         <v>12480</v>
@@ -8418,10 +8466,10 @@
         <v>182</v>
       </c>
       <c r="B33" s="23" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="C33" s="23" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="D33" s="24" t="n">
         <v>33097</v>
@@ -8436,18 +8484,18 @@
         <v>156</v>
       </c>
       <c r="H33" s="23" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="23" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="B34" s="23" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="C34" s="23" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="D34" s="24" t="n">
         <v>74011</v>
@@ -8462,7 +8510,7 @@
         <v>156</v>
       </c>
       <c r="H34" s="23" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8470,10 +8518,10 @@
         <v>193</v>
       </c>
       <c r="B35" s="23" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="C35" s="23" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="D35" s="24" t="n">
         <v>65538</v>
@@ -8488,7 +8536,7 @@
         <v>156</v>
       </c>
       <c r="H35" s="23" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8496,10 +8544,10 @@
         <v>158</v>
       </c>
       <c r="B36" s="23" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="C36" s="23" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="D36" s="24" t="n">
         <v>11904</v>
@@ -8522,10 +8570,10 @@
         <v>182</v>
       </c>
       <c r="B37" s="23" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="C37" s="23" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="D37" s="24" t="n">
         <v>37951</v>
@@ -8540,7 +8588,7 @@
         <v>156</v>
       </c>
       <c r="H37" s="23" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8548,10 +8596,10 @@
         <v>158</v>
       </c>
       <c r="B38" s="23" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="C38" s="23" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="D38" s="24" t="n">
         <v>189112</v>
@@ -8574,10 +8622,10 @@
         <v>262</v>
       </c>
       <c r="B39" s="23" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="C39" s="23" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="D39" s="24" t="n">
         <v>22771</v>
@@ -8592,7 +8640,7 @@
         <v>156</v>
       </c>
       <c r="H39" s="23" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8600,10 +8648,10 @@
         <v>153</v>
       </c>
       <c r="B40" s="23" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="C40" s="23" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="D40" s="24" t="n">
         <v>759419</v>
@@ -8618,7 +8666,7 @@
         <v>156</v>
       </c>
       <c r="H40" s="23" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8626,10 +8674,10 @@
         <v>169</v>
       </c>
       <c r="B41" s="23" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="C41" s="23" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="D41" s="24" t="n">
         <v>536255</v>
@@ -8652,10 +8700,10 @@
         <v>182</v>
       </c>
       <c r="B42" s="23" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="C42" s="23" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="D42" s="24" t="n">
         <v>8403</v>
@@ -8675,13 +8723,13 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="23" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="B43" s="23" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="C43" s="23" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="D43" s="24" t="n">
         <v>70000</v>
@@ -8696,7 +8744,7 @@
         <v>156</v>
       </c>
       <c r="H43" s="23" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8704,10 +8752,10 @@
         <v>182</v>
       </c>
       <c r="B44" s="23" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="C44" s="23" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="D44" s="24" t="n">
         <v>75752</v>
@@ -8722,7 +8770,7 @@
         <v>156</v>
       </c>
       <c r="H44" s="23" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8730,10 +8778,10 @@
         <v>262</v>
       </c>
       <c r="B45" s="23" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="C45" s="23" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="D45" s="24" t="n">
         <v>16347</v>
@@ -8748,7 +8796,7 @@
         <v>156</v>
       </c>
       <c r="H45" s="23" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8756,10 +8804,10 @@
         <v>162</v>
       </c>
       <c r="B46" s="23" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="C46" s="23" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="D46" s="24" t="n">
         <v>37807</v>
@@ -8782,10 +8830,10 @@
         <v>162</v>
       </c>
       <c r="B47" s="23" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="C47" s="23" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="D47" s="24" t="n">
         <v>18977</v>
@@ -8808,10 +8856,10 @@
         <v>153</v>
       </c>
       <c r="B48" s="23" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="C48" s="23" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="D48" s="24" t="n">
         <v>811375</v>
@@ -8826,18 +8874,18 @@
         <v>156</v>
       </c>
       <c r="H48" s="23" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="23" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="B49" s="23" t="s">
+        <v>441</v>
+      </c>
+      <c r="C49" s="23" t="s">
         <v>438</v>
-      </c>
-      <c r="C49" s="23" t="s">
-        <v>435</v>
       </c>
       <c r="D49" s="24" t="n">
         <v>983773</v>
@@ -8857,13 +8905,13 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="23" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="B50" s="23" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="C50" s="23" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="D50" s="24" t="n">
         <v>21008</v>
@@ -8878,7 +8926,7 @@
         <v>156</v>
       </c>
       <c r="H50" s="23" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8886,10 +8934,10 @@
         <v>182</v>
       </c>
       <c r="B51" s="23" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="C51" s="23" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="D51" s="24" t="n">
         <v>12605</v>
@@ -8904,7 +8952,7 @@
         <v>156</v>
       </c>
       <c r="H51" s="23" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8912,10 +8960,10 @@
         <v>153</v>
       </c>
       <c r="B52" s="23" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="C52" s="23" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="D52" s="24" t="n">
         <v>121706</v>
@@ -8930,7 +8978,7 @@
         <v>156</v>
       </c>
       <c r="H52" s="23" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8938,10 +8986,10 @@
         <v>153</v>
       </c>
       <c r="B53" s="23" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="C53" s="23" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="D53" s="24" t="n">
         <v>129820</v>
@@ -8956,7 +9004,7 @@
         <v>156</v>
       </c>
       <c r="H53" s="23" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8964,10 +9012,10 @@
         <v>153</v>
       </c>
       <c r="B54" s="23" t="s">
+        <v>451</v>
+      </c>
+      <c r="C54" s="23" t="s">
         <v>448</v>
-      </c>
-      <c r="C54" s="23" t="s">
-        <v>445</v>
       </c>
       <c r="D54" s="24" t="n">
         <v>811375</v>
@@ -8982,7 +9030,7 @@
         <v>156</v>
       </c>
       <c r="H54" s="23" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8990,10 +9038,10 @@
         <v>182</v>
       </c>
       <c r="B55" s="23" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="C55" s="23" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="D55" s="24" t="n">
         <v>44769</v>
@@ -9008,7 +9056,7 @@
         <v>156</v>
       </c>
       <c r="H55" s="23" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9016,10 +9064,10 @@
         <v>235</v>
       </c>
       <c r="B56" s="23" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="C56" s="23" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="D56" s="24" t="n">
         <v>16806</v>
@@ -9034,7 +9082,7 @@
         <v>156</v>
       </c>
       <c r="H56" s="23" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9042,10 +9090,10 @@
         <v>235</v>
       </c>
       <c r="B57" s="23" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="C57" s="23" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="D57" s="24" t="n">
         <v>16623</v>
@@ -9060,7 +9108,7 @@
         <v>156</v>
       </c>
       <c r="H57" s="23" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9068,10 +9116,10 @@
         <v>182</v>
       </c>
       <c r="B58" s="23" t="s">
+        <v>460</v>
+      </c>
+      <c r="C58" s="23" t="s">
         <v>457</v>
-      </c>
-      <c r="C58" s="23" t="s">
-        <v>454</v>
       </c>
       <c r="D58" s="24" t="n">
         <v>53759</v>
@@ -9086,7 +9134,7 @@
         <v>156</v>
       </c>
       <c r="H58" s="23" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9094,10 +9142,10 @@
         <v>169</v>
       </c>
       <c r="B59" s="23" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="C59" s="23" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="D59" s="24" t="n">
         <v>248771</v>
@@ -9112,7 +9160,7 @@
         <v>156</v>
       </c>
       <c r="H59" s="23" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9120,10 +9168,10 @@
         <v>182</v>
       </c>
       <c r="B60" s="23" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="C60" s="23" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="D60" s="24" t="n">
         <v>71678</v>
@@ -9138,18 +9186,18 @@
         <v>156</v>
       </c>
       <c r="H60" s="23" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="23" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="B61" s="23" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="C61" s="23" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="D61" s="24" t="n">
         <v>2479</v>
@@ -9172,10 +9220,10 @@
         <v>235</v>
       </c>
       <c r="B62" s="23" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="C62" s="23" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="D62" s="24" t="n">
         <v>18674</v>
@@ -9201,7 +9249,7 @@
         <v>189</v>
       </c>
       <c r="C63" s="23" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="D63" s="24" t="n">
         <v>20124</v>
@@ -9227,7 +9275,7 @@
         <v>8677299</v>
       </c>
       <c r="G64" s="27" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9262,7 +9310,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="23" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="B68" s="23" t="s">
         <v>311</v>
@@ -9279,7 +9327,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="23" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="B69" s="23" t="s">
         <v>315</v>
@@ -9296,7 +9344,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="23" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="B70" s="23" t="s">
         <v>311</v>
@@ -9313,7 +9361,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="23" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="B71" s="23" t="s">
         <v>306</v>
@@ -9330,10 +9378,10 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="23" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="B72" s="23" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="C72" s="24" t="n">
         <v>-190000</v>
@@ -9347,10 +9395,10 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="23" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="B73" s="23" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="C73" s="24" t="n">
         <v>-54000</v>
@@ -9364,7 +9412,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="23" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="B74" s="23" t="s">
         <v>331</v>
@@ -9381,10 +9429,10 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="23" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="B75" s="23" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="C75" s="24" t="n">
         <v>-2700</v>
@@ -9398,7 +9446,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="23" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="B76" s="23" t="s">
         <v>335</v>
@@ -9415,7 +9463,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="23" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="B77" s="23" t="s">
         <v>318</v>
@@ -9432,10 +9480,10 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="23" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="B78" s="23" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="C78" s="24" t="n">
         <v>-280000</v>
@@ -9449,7 +9497,7 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="23" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="B79" s="23" t="s">
         <v>311</v>
@@ -9466,7 +9514,7 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="23" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="B80" s="23" t="s">
         <v>345</v>
@@ -9483,7 +9531,7 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="23" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="B81" s="23" t="s">
         <v>333</v>
@@ -9500,7 +9548,7 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="23" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B82" s="23" t="s">
         <v>318</v>
@@ -9517,7 +9565,7 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="23" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B83" s="23" t="s">
         <v>318</v>
@@ -9534,7 +9582,7 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="23" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B84" s="23" t="s">
         <v>315</v>
@@ -9551,7 +9599,7 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="23" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B85" s="23" t="s">
         <v>314</v>
@@ -9568,7 +9616,7 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="23" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B86" s="23" t="s">
         <v>331</v>
@@ -9585,7 +9633,7 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="23" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B87" s="23" t="s">
         <v>311</v>
@@ -9602,7 +9650,7 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="23" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B88" s="23" t="s">
         <v>332</v>
@@ -9619,10 +9667,10 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="23" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B89" s="23" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="C89" s="24" t="n">
         <v>320000</v>
@@ -9636,7 +9684,7 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="23" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B90" s="23" t="s">
         <v>318</v>
@@ -9653,7 +9701,7 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="23" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B91" s="23" t="s">
         <v>318</v>
@@ -9670,7 +9718,7 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="23" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="B92" s="23" t="s">
         <v>319</v>
@@ -9687,7 +9735,7 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="23" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="B93" s="23" t="s">
         <v>318</v>
@@ -9704,10 +9752,10 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="23" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="B94" s="23" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="C94" s="24" t="n">
         <v>-4700</v>
@@ -9721,7 +9769,7 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="23" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="B95" s="23" t="s">
         <v>318</v>
@@ -9738,10 +9786,10 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="23" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="B96" s="23" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="C96" s="24" t="n">
         <v>-14880</v>
@@ -9755,7 +9803,7 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="23" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="B97" s="23" t="s">
         <v>318</v>
@@ -9772,10 +9820,10 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="23" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="B98" s="23" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="C98" s="24" t="n">
         <v>-31955</v>
@@ -9789,10 +9837,10 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="23" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="B99" s="23" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="C99" s="24" t="n">
         <v>-63065</v>
@@ -9806,7 +9854,7 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="23" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="B100" s="23" t="s">
         <v>318</v>
@@ -9823,7 +9871,7 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="23" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="B101" s="23" t="s">
         <v>311</v>
@@ -9840,10 +9888,10 @@
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="23" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="B102" s="23" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="C102" s="24" t="n">
         <v>-21470</v>
@@ -9857,7 +9905,7 @@
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="23" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="B103" s="23" t="s">
         <v>335</v>
@@ -9874,7 +9922,7 @@
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="23" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="B104" s="23" t="s">
         <v>306</v>
@@ -9891,7 +9939,7 @@
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="23" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="B105" s="23" t="s">
         <v>318</v>
@@ -9908,7 +9956,7 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="23" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="B106" s="23" t="s">
         <v>318</v>
@@ -9925,7 +9973,7 @@
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="23" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="B107" s="23" t="s">
         <v>331</v>
@@ -9942,7 +9990,7 @@
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="23" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="B108" s="23" t="s">
         <v>314</v>
@@ -9959,7 +10007,7 @@
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="23" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="B109" s="23" t="s">
         <v>318</v>
@@ -9976,7 +10024,7 @@
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="23" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="B110" s="23" t="s">
         <v>314</v>
@@ -9993,7 +10041,7 @@
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="23" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="B111" s="23" t="s">
         <v>318</v>
@@ -10010,7 +10058,7 @@
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="23" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="B112" s="23" t="s">
         <v>314</v>
@@ -10027,7 +10075,7 @@
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="23" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="B113" s="23" t="s">
         <v>318</v>
@@ -10044,7 +10092,7 @@
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="23" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="B114" s="23" t="s">
         <v>314</v>
@@ -10061,10 +10109,10 @@
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="23" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="B115" s="23" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="C115" s="24" t="n">
         <v>2813595</v>
@@ -10078,7 +10126,7 @@
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="23" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="B116" s="23" t="s">
         <v>331</v>
@@ -10095,10 +10143,10 @@
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="23" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="B117" s="23" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="C117" s="24" t="n">
         <v>-1000000</v>
@@ -10112,7 +10160,7 @@
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="23" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="B118" s="23" t="s">
         <v>332</v>
@@ -10129,7 +10177,7 @@
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="23" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="B119" s="23" t="s">
         <v>315</v>
@@ -10146,7 +10194,7 @@
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="23" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="B120" s="23" t="s">
         <v>314</v>
@@ -10163,7 +10211,7 @@
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="23" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="B121" s="23" t="s">
         <v>318</v>
@@ -10180,7 +10228,7 @@
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="23" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="B122" s="23" t="s">
         <v>343</v>
@@ -10197,7 +10245,7 @@
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="23" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="B123" s="23" t="s">
         <v>311</v>
@@ -10214,7 +10262,7 @@
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="23" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="B124" s="23" t="s">
         <v>319</v>
@@ -10231,7 +10279,7 @@
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="23" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="B125" s="23" t="s">
         <v>314</v>
@@ -10248,7 +10296,7 @@
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="23" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="B126" s="23" t="s">
         <v>319</v>
@@ -10265,10 +10313,10 @@
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="23" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="B127" s="23" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="C127" s="24" t="n">
         <v>-9471</v>
@@ -10282,10 +10330,10 @@
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="23" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="B128" s="23" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="C128" s="24" t="n">
         <v>2234722</v>
@@ -10299,7 +10347,7 @@
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="23" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="B129" s="23" t="s">
         <v>318</v>
@@ -10316,7 +10364,7 @@
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="23" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="B130" s="23" t="s">
         <v>314</v>
@@ -10333,10 +10381,10 @@
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="23" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="B131" s="23" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
       <c r="C131" s="24" t="n">
         <v>-31319</v>
@@ -10350,7 +10398,7 @@
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="23" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="B132" s="23" t="s">
         <v>306</v>
@@ -10367,7 +10415,7 @@
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="23" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="B133" s="23" t="s">
         <v>319</v>
@@ -10384,10 +10432,10 @@
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="23" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="B134" s="23" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="C134" s="24" t="n">
         <v>-405600</v>
@@ -10401,7 +10449,7 @@
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="23" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="B135" s="23" t="s">
         <v>314</v>
@@ -10418,10 +10466,10 @@
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="23" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="B136" s="23" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="C136" s="24" t="n">
         <v>-5770</v>
@@ -10435,7 +10483,7 @@
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="23" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="B137" s="23" t="s">
         <v>318</v>
@@ -10452,7 +10500,7 @@
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="23" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="B138" s="23" t="s">
         <v>331</v>
@@ -10469,7 +10517,7 @@
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="23" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="B139" s="23" t="s">
         <v>315</v>
@@ -10486,7 +10534,7 @@
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="23" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="B140" s="23" t="s">
         <v>319</v>
@@ -10503,10 +10551,10 @@
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="23" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="B141" s="23" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="C141" s="24" t="n">
         <v>357000</v>
@@ -10520,7 +10568,7 @@
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="23" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="B142" s="23" t="s">
         <v>314</v>
@@ -10537,7 +10585,7 @@
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="23" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="B143" s="23" t="s">
         <v>318</v>
@@ -10554,10 +10602,10 @@
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="23" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="B144" s="23" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="C144" s="24" t="n">
         <v>-38000</v>
@@ -10571,7 +10619,7 @@
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="23" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="B145" s="23" t="s">
         <v>315</v>
@@ -10588,7 +10636,7 @@
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="23" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="B146" s="23" t="s">
         <v>331</v>
@@ -10605,7 +10653,7 @@
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="23" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="B147" s="23" t="s">
         <v>314</v>
@@ -10622,7 +10670,7 @@
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="23" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="B148" s="23" t="s">
         <v>314</v>
@@ -10639,7 +10687,7 @@
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="23" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="B149" s="23" t="s">
         <v>318</v>
@@ -10656,7 +10704,7 @@
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="23" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="B150" s="23" t="s">
         <v>335</v>
@@ -10673,10 +10721,10 @@
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="23" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="B151" s="23" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="C151" s="24" t="n">
         <v>200000</v>
@@ -10708,10 +10756,16 @@
       <c r="B154" s="22" t="s">
         <v>3</v>
       </c>
+      <c r="C154" s="28" t="s">
+        <v>347</v>
+      </c>
+      <c r="D154" s="28" t="s">
+        <v>348</v>
+      </c>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="23" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B155" s="24" t="n">
         <v>267206</v>
@@ -10719,15 +10773,23 @@
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="23" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B156" s="24" t="n">
         <v>14053438</v>
       </c>
+      <c r="C156" s="29" t="n">
+        <f aca="false">F11</f>
+        <v>6122312</v>
+      </c>
+      <c r="D156" s="29" t="n">
+        <f aca="false">B156-C156</f>
+        <v>7931126</v>
+      </c>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="23" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B157" s="24" t="n">
         <v>-13156244</v>
@@ -10735,7 +10797,7 @@
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="25" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B158" s="26" t="n">
         <f aca="false">SUM(B155:B157)</f>
@@ -10744,7 +10806,7 @@
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="25" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B159" s="26" t="n">
         <v>1164400</v>
@@ -10752,21 +10814,34 @@
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="25" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B160" s="26" t="n">
         <f aca="false">B158-B159</f>
         <v>0</v>
       </c>
     </row>
+    <row r="162" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A162" s="30" t="s">
+        <v>355</v>
+      </c>
+      <c r="B162" s="30"/>
+      <c r="C162" s="30"/>
+      <c r="D162" s="30"/>
+      <c r="E162" s="30"/>
+      <c r="F162" s="30"/>
+      <c r="G162" s="30"/>
+      <c r="H162" s="30"/>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A4:I4"/>
     <mergeCell ref="A13:I13"/>
     <mergeCell ref="A66:I66"/>
     <mergeCell ref="A153:I153"/>
+    <mergeCell ref="A162:H162"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -10793,7 +10868,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -10807,23 +10882,23 @@
       <c r="K1" s="19"/>
     </row>
     <row r="2" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="28" t="s">
-        <v>486</v>
-      </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
-      <c r="J2" s="28"/>
-      <c r="K2" s="28"/>
+      <c r="A2" s="31" t="s">
+        <v>489</v>
+      </c>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="21" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="B5" s="21"/>
       <c r="C5" s="21"/>
@@ -10841,60 +10916,60 @@
         <v>15</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="C6" s="22" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
       <c r="D6" s="22" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="E6" s="22" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="F6" s="22" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="G6" s="22" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="H6" s="22" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="I6" s="22" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="J6" s="22" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="K6" s="22" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="29" t="str">
+      <c r="A7" s="32" t="str">
         <f aca="false">Agosto!A20</f>
         <v>S0 (01-02 ago)</v>
       </c>
-      <c r="B7" s="30" t="n">
+      <c r="B7" s="33" t="n">
         <f aca="false">Agosto!B20</f>
         <v>0</v>
       </c>
-      <c r="C7" s="31"/>
+      <c r="C7" s="34"/>
       <c r="D7" s="24" t="str">
         <f aca="false">IF(C7="","",C7-B7)</f>
         <v/>
       </c>
-      <c r="E7" s="30" t="n">
+      <c r="E7" s="33" t="n">
         <f aca="false">Agosto!C20</f>
         <v>3949000</v>
       </c>
-      <c r="F7" s="31"/>
+      <c r="F7" s="34"/>
       <c r="G7" s="24" t="str">
         <f aca="false">IF(F7="","",F7-E7)</f>
         <v/>
       </c>
-      <c r="H7" s="30" t="n">
+      <c r="H7" s="33" t="n">
         <f aca="false">Agosto!D20</f>
         <v>-3949000</v>
       </c>
@@ -10902,36 +10977,36 @@
         <f aca="false">IF(OR(C7="",F7=""),"",C7-F7)</f>
         <v/>
       </c>
-      <c r="J7" s="32" t="str">
+      <c r="J7" s="35" t="str">
         <f aca="false">IF(I7="","Pendiente",IF(I7&gt;=H7,"Sí","No"))</f>
         <v>Pendiente</v>
       </c>
-      <c r="K7" s="33"/>
+      <c r="K7" s="36"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="29" t="str">
+      <c r="A8" s="32" t="str">
         <f aca="false">Agosto!A21</f>
         <v>S1 (03-09 ago)</v>
       </c>
-      <c r="B8" s="30" t="n">
+      <c r="B8" s="33" t="n">
         <f aca="false">Agosto!B21</f>
         <v>7390238</v>
       </c>
-      <c r="C8" s="31"/>
+      <c r="C8" s="34"/>
       <c r="D8" s="24" t="str">
         <f aca="false">IF(C8="","",C8-B8)</f>
         <v/>
       </c>
-      <c r="E8" s="30" t="n">
+      <c r="E8" s="33" t="n">
         <f aca="false">Agosto!C21</f>
         <v>6466656</v>
       </c>
-      <c r="F8" s="31"/>
+      <c r="F8" s="34"/>
       <c r="G8" s="24" t="str">
         <f aca="false">IF(F8="","",F8-E8)</f>
         <v/>
       </c>
-      <c r="H8" s="30" t="n">
+      <c r="H8" s="33" t="n">
         <f aca="false">Agosto!D21</f>
         <v>923582</v>
       </c>
@@ -10939,36 +11014,36 @@
         <f aca="false">IF(OR(C8="",F8=""),"",C8-F8)</f>
         <v/>
       </c>
-      <c r="J8" s="32" t="str">
+      <c r="J8" s="35" t="str">
         <f aca="false">IF(I8="","Pendiente",IF(I8&gt;=H8,"Sí","No"))</f>
         <v>Pendiente</v>
       </c>
-      <c r="K8" s="33"/>
+      <c r="K8" s="36"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="29" t="str">
+      <c r="A9" s="32" t="str">
         <f aca="false">Agosto!A22</f>
         <v>S2 (10-16 ago)</v>
       </c>
-      <c r="B9" s="30" t="n">
+      <c r="B9" s="33" t="n">
         <f aca="false">Agosto!B22</f>
         <v>7390238</v>
       </c>
-      <c r="C9" s="31"/>
+      <c r="C9" s="34"/>
       <c r="D9" s="24" t="str">
         <f aca="false">IF(C9="","",C9-B9)</f>
         <v/>
       </c>
-      <c r="E9" s="30" t="n">
+      <c r="E9" s="33" t="n">
         <f aca="false">Agosto!C22</f>
         <v>5053147</v>
       </c>
-      <c r="F9" s="31"/>
+      <c r="F9" s="34"/>
       <c r="G9" s="24" t="str">
         <f aca="false">IF(F9="","",F9-E9)</f>
         <v/>
       </c>
-      <c r="H9" s="30" t="n">
+      <c r="H9" s="33" t="n">
         <f aca="false">Agosto!D22</f>
         <v>2337091</v>
       </c>
@@ -10976,36 +11051,36 @@
         <f aca="false">IF(OR(C9="",F9=""),"",C9-F9)</f>
         <v/>
       </c>
-      <c r="J9" s="32" t="str">
+      <c r="J9" s="35" t="str">
         <f aca="false">IF(I9="","Pendiente",IF(I9&gt;=H9,"Sí","No"))</f>
         <v>Pendiente</v>
       </c>
-      <c r="K9" s="33"/>
+      <c r="K9" s="36"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="29" t="str">
+      <c r="A10" s="32" t="str">
         <f aca="false">Agosto!A23</f>
         <v>S3 (17-23 ago)</v>
       </c>
-      <c r="B10" s="30" t="n">
+      <c r="B10" s="33" t="n">
         <f aca="false">Agosto!B23</f>
         <v>7390238</v>
       </c>
-      <c r="C10" s="31"/>
+      <c r="C10" s="34"/>
       <c r="D10" s="24" t="str">
         <f aca="false">IF(C10="","",C10-B10)</f>
         <v/>
       </c>
-      <c r="E10" s="30" t="n">
+      <c r="E10" s="33" t="n">
         <f aca="false">Agosto!C23</f>
         <v>3390000</v>
       </c>
-      <c r="F10" s="31"/>
+      <c r="F10" s="34"/>
       <c r="G10" s="24" t="str">
         <f aca="false">IF(F10="","",F10-E10)</f>
         <v/>
       </c>
-      <c r="H10" s="30" t="n">
+      <c r="H10" s="33" t="n">
         <f aca="false">Agosto!D23</f>
         <v>4000238</v>
       </c>
@@ -11013,36 +11088,36 @@
         <f aca="false">IF(OR(C10="",F10=""),"",C10-F10)</f>
         <v/>
       </c>
-      <c r="J10" s="32" t="str">
+      <c r="J10" s="35" t="str">
         <f aca="false">IF(I10="","Pendiente",IF(I10&gt;=H10,"Sí","No"))</f>
         <v>Pendiente</v>
       </c>
-      <c r="K10" s="33"/>
+      <c r="K10" s="36"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="29" t="str">
+      <c r="A11" s="32" t="str">
         <f aca="false">Agosto!A24</f>
         <v>S4 (24-30 ago)</v>
       </c>
-      <c r="B11" s="30" t="n">
+      <c r="B11" s="33" t="n">
         <f aca="false">Agosto!B24</f>
         <v>7390238</v>
       </c>
-      <c r="C11" s="31"/>
+      <c r="C11" s="34"/>
       <c r="D11" s="24" t="str">
         <f aca="false">IF(C11="","",C11-B11)</f>
         <v/>
       </c>
-      <c r="E11" s="30" t="n">
+      <c r="E11" s="33" t="n">
         <f aca="false">Agosto!C24</f>
         <v>2887500</v>
       </c>
-      <c r="F11" s="31"/>
+      <c r="F11" s="34"/>
       <c r="G11" s="24" t="str">
         <f aca="false">IF(F11="","",F11-E11)</f>
         <v/>
       </c>
-      <c r="H11" s="30" t="n">
+      <c r="H11" s="33" t="n">
         <f aca="false">Agosto!D24</f>
         <v>4502738</v>
       </c>
@@ -11050,36 +11125,36 @@
         <f aca="false">IF(OR(C11="",F11=""),"",C11-F11)</f>
         <v/>
       </c>
-      <c r="J11" s="32" t="str">
+      <c r="J11" s="35" t="str">
         <f aca="false">IF(I11="","Pendiente",IF(I11&gt;=H11,"Sí","No"))</f>
         <v>Pendiente</v>
       </c>
-      <c r="K11" s="33"/>
+      <c r="K11" s="36"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="29" t="str">
+      <c r="A12" s="32" t="str">
         <f aca="false">Agosto!A25</f>
         <v>S5 (31 ago)</v>
       </c>
-      <c r="B12" s="30" t="n">
+      <c r="B12" s="33" t="n">
         <f aca="false">Agosto!B25</f>
         <v>1478048</v>
       </c>
-      <c r="C12" s="31"/>
+      <c r="C12" s="34"/>
       <c r="D12" s="24" t="str">
         <f aca="false">IF(C12="","",C12-B12)</f>
         <v/>
       </c>
-      <c r="E12" s="30" t="n">
+      <c r="E12" s="33" t="n">
         <f aca="false">Agosto!C25</f>
         <v>3540000</v>
       </c>
-      <c r="F12" s="31"/>
+      <c r="F12" s="34"/>
       <c r="G12" s="24" t="str">
         <f aca="false">IF(F12="","",F12-E12)</f>
         <v/>
       </c>
-      <c r="H12" s="30" t="n">
+      <c r="H12" s="33" t="n">
         <f aca="false">Agosto!D25</f>
         <v>-2061952</v>
       </c>
@@ -11087,15 +11162,15 @@
         <f aca="false">IF(OR(C12="",F12=""),"",C12-F12)</f>
         <v/>
       </c>
-      <c r="J12" s="32" t="str">
+      <c r="J12" s="35" t="str">
         <f aca="false">IF(I12="","Pendiente",IF(I12&gt;=H12,"Sí","No"))</f>
         <v>Pendiente</v>
       </c>
-      <c r="K12" s="33"/>
+      <c r="K12" s="36"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="21" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="B14" s="21"/>
       <c r="C14" s="21"/>
@@ -11113,60 +11188,60 @@
         <v>15</v>
       </c>
       <c r="B15" s="22" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="C15" s="22" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
       <c r="D15" s="22" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="E15" s="22" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="F15" s="22" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="G15" s="22" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="H15" s="22" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="I15" s="22" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="J15" s="22" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="K15" s="22" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="29" t="str">
+      <c r="A16" s="32" t="str">
         <f aca="false">Septiembre!A20</f>
         <v>S0 (01-06 sep)</v>
       </c>
-      <c r="B16" s="30" t="n">
+      <c r="B16" s="33" t="n">
         <f aca="false">Septiembre!B20</f>
         <v>7524608</v>
       </c>
-      <c r="C16" s="31"/>
+      <c r="C16" s="34"/>
       <c r="D16" s="24" t="str">
         <f aca="false">IF(C16="","",C16-B16)</f>
         <v/>
       </c>
-      <c r="E16" s="30" t="n">
+      <c r="E16" s="33" t="n">
         <f aca="false">Septiembre!C20</f>
         <v>11814844</v>
       </c>
-      <c r="F16" s="31"/>
+      <c r="F16" s="34"/>
       <c r="G16" s="24" t="str">
         <f aca="false">IF(F16="","",F16-E16)</f>
         <v/>
       </c>
-      <c r="H16" s="30" t="n">
+      <c r="H16" s="33" t="n">
         <f aca="false">Septiembre!D20</f>
         <v>-4290236</v>
       </c>
@@ -11174,36 +11249,36 @@
         <f aca="false">IF(OR(C16="",F16=""),"",C16-F16)</f>
         <v/>
       </c>
-      <c r="J16" s="32" t="str">
+      <c r="J16" s="35" t="str">
         <f aca="false">IF(I16="","Pendiente",IF(I16&gt;=H16,"Sí","No"))</f>
         <v>Pendiente</v>
       </c>
-      <c r="K16" s="33"/>
+      <c r="K16" s="36"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="29" t="str">
+      <c r="A17" s="32" t="str">
         <f aca="false">Septiembre!A21</f>
         <v>S1 (07-13 sep)</v>
       </c>
-      <c r="B17" s="30" t="n">
+      <c r="B17" s="33" t="n">
         <f aca="false">Septiembre!B21</f>
         <v>9405760</v>
       </c>
-      <c r="C17" s="31"/>
+      <c r="C17" s="34"/>
       <c r="D17" s="24" t="str">
         <f aca="false">IF(C17="","",C17-B17)</f>
         <v/>
       </c>
-      <c r="E17" s="30" t="n">
+      <c r="E17" s="33" t="n">
         <f aca="false">Septiembre!C21</f>
         <v>6207692</v>
       </c>
-      <c r="F17" s="31"/>
+      <c r="F17" s="34"/>
       <c r="G17" s="24" t="str">
         <f aca="false">IF(F17="","",F17-E17)</f>
         <v/>
       </c>
-      <c r="H17" s="30" t="n">
+      <c r="H17" s="33" t="n">
         <f aca="false">Septiembre!D21</f>
         <v>3198068</v>
       </c>
@@ -11211,36 +11286,36 @@
         <f aca="false">IF(OR(C17="",F17=""),"",C17-F17)</f>
         <v/>
       </c>
-      <c r="J17" s="32" t="str">
+      <c r="J17" s="35" t="str">
         <f aca="false">IF(I17="","Pendiente",IF(I17&gt;=H17,"Sí","No"))</f>
         <v>Pendiente</v>
       </c>
-      <c r="K17" s="33"/>
+      <c r="K17" s="36"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="29" t="str">
+      <c r="A18" s="32" t="str">
         <f aca="false">Septiembre!A22</f>
         <v>S2 (14-20 sep)</v>
       </c>
-      <c r="B18" s="30" t="n">
+      <c r="B18" s="33" t="n">
         <f aca="false">Septiembre!B22</f>
         <v>9405760</v>
       </c>
-      <c r="C18" s="31"/>
+      <c r="C18" s="34"/>
       <c r="D18" s="24" t="str">
         <f aca="false">IF(C18="","",C18-B18)</f>
         <v/>
       </c>
-      <c r="E18" s="30" t="n">
+      <c r="E18" s="33" t="n">
         <f aca="false">Septiembre!C22</f>
         <v>4374545</v>
       </c>
-      <c r="F18" s="31"/>
+      <c r="F18" s="34"/>
       <c r="G18" s="24" t="str">
         <f aca="false">IF(F18="","",F18-E18)</f>
         <v/>
       </c>
-      <c r="H18" s="30" t="n">
+      <c r="H18" s="33" t="n">
         <f aca="false">Septiembre!D22</f>
         <v>5031215</v>
       </c>
@@ -11248,36 +11323,36 @@
         <f aca="false">IF(OR(C18="",F18=""),"",C18-F18)</f>
         <v/>
       </c>
-      <c r="J18" s="32" t="str">
+      <c r="J18" s="35" t="str">
         <f aca="false">IF(I18="","Pendiente",IF(I18&gt;=H18,"Sí","No"))</f>
         <v>Pendiente</v>
       </c>
-      <c r="K18" s="33"/>
+      <c r="K18" s="36"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="29" t="str">
+      <c r="A19" s="32" t="str">
         <f aca="false">Septiembre!A23</f>
         <v>S3 (21-27 sep)</v>
       </c>
-      <c r="B19" s="30" t="n">
+      <c r="B19" s="33" t="n">
         <f aca="false">Septiembre!B23</f>
         <v>9405760</v>
       </c>
-      <c r="C19" s="31"/>
+      <c r="C19" s="34"/>
       <c r="D19" s="24" t="str">
         <f aca="false">IF(C19="","",C19-B19)</f>
         <v/>
       </c>
-      <c r="E19" s="30" t="n">
+      <c r="E19" s="33" t="n">
         <f aca="false">Septiembre!C23</f>
         <v>3704545</v>
       </c>
-      <c r="F19" s="31"/>
+      <c r="F19" s="34"/>
       <c r="G19" s="24" t="str">
         <f aca="false">IF(F19="","",F19-E19)</f>
         <v/>
       </c>
-      <c r="H19" s="30" t="n">
+      <c r="H19" s="33" t="n">
         <f aca="false">Septiembre!D23</f>
         <v>5701215</v>
       </c>
@@ -11285,36 +11360,36 @@
         <f aca="false">IF(OR(C19="",F19=""),"",C19-F19)</f>
         <v/>
       </c>
-      <c r="J19" s="32" t="str">
+      <c r="J19" s="35" t="str">
         <f aca="false">IF(I19="","Pendiente",IF(I19&gt;=H19,"Sí","No"))</f>
         <v>Pendiente</v>
       </c>
-      <c r="K19" s="33"/>
+      <c r="K19" s="36"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="29" t="str">
+      <c r="A20" s="32" t="str">
         <f aca="false">Septiembre!A24</f>
         <v>S4 (28-30 sep)</v>
       </c>
-      <c r="B20" s="30" t="n">
+      <c r="B20" s="33" t="n">
         <f aca="false">Septiembre!B24</f>
         <v>5643456</v>
       </c>
-      <c r="C20" s="31"/>
+      <c r="C20" s="34"/>
       <c r="D20" s="24" t="str">
         <f aca="false">IF(C20="","",C20-B20)</f>
         <v/>
       </c>
-      <c r="E20" s="30" t="n">
+      <c r="E20" s="33" t="n">
         <f aca="false">Septiembre!C24</f>
         <v>5912727</v>
       </c>
-      <c r="F20" s="31"/>
+      <c r="F20" s="34"/>
       <c r="G20" s="24" t="str">
         <f aca="false">IF(F20="","",F20-E20)</f>
         <v/>
       </c>
-      <c r="H20" s="30" t="n">
+      <c r="H20" s="33" t="n">
         <f aca="false">Septiembre!D24</f>
         <v>-269271</v>
       </c>
@@ -11322,11 +11397,11 @@
         <f aca="false">IF(OR(C20="",F20=""),"",C20-F20)</f>
         <v/>
       </c>
-      <c r="J20" s="32" t="str">
+      <c r="J20" s="35" t="str">
         <f aca="false">IF(I20="","Pendiente",IF(I20&gt;=H20,"Sí","No"))</f>
         <v>Pendiente</v>
       </c>
-      <c r="K20" s="33"/>
+      <c r="K20" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
Agrega hoja Resumen_Ejecutivo (foto financiera plan vs real vs reproyeccion)
</commit_message>
<xml_diff>
--- a/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
+++ b/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Conciliación_Junio" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Conciliación_Julio" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Real_vs_Presupuesto" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Resumen_Ejecutivo" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1739" uniqueCount="502">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1763" uniqueCount="513">
   <si>
     <t xml:space="preserve">PRESUPUESTO Y FLUJO DE CAJA — AGOSTO 2026 (3 equipos)</t>
   </si>
@@ -1538,16 +1539,56 @@
   </si>
   <si>
     <t xml:space="preserve">CONTROL SEMANAL — SEPTIEMBRE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RESUMEN EJECUTIVO — CUMPLIMIENTO DE PRESUPUESTO Y FLUJO DE CAJA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La "foto financiera" completa: lo planeado (Presupuesto) vs. lo que va ocurriendo semana a semana (Real, tomado de la hoja Real_vs_Presupuesto, que a su vez sale del cruce SII+Cartola de la Conciliación) vs. la Reproyección de fin de mes = Real acumulado a la fecha + Presupuesto de las semanas que aún no tienen dato real (supuesto: lo que falta del mes se cumple según lo planeado, hasta que se reemplace con datos reales semana a semana). Se actualiza solo a medida que se llena la columna "Real" en Real_vs_Presupuesto — no hay que tocar nada acá.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AGOSTO 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Presupuesto
+Mensual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real
+Acumulado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Semanas
+con dato real</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Presupuesto
+de lo que falta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reproyección
+Fin de Mes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% Cumplimiento
+(Reproyección/Presup.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saldo (Ingreso − Egreso)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SEPTIEMBRE 2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -1787,7 +1828,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="39">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1934,6 +1975,14 @@
     </xf>
     <xf numFmtId="164" fontId="12" fillId="7" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -11418,4 +11467,285 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="17"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="19" t="s">
+        <v>502</v>
+      </c>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+    </row>
+    <row r="2" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="31" t="s">
+        <v>503</v>
+      </c>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="21" t="s">
+        <v>504</v>
+      </c>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
+    </row>
+    <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="22" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>505</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>506</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>507</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>508</v>
+      </c>
+      <c r="F5" s="22" t="s">
+        <v>509</v>
+      </c>
+      <c r="G5" s="22" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="33" t="n">
+        <f aca="false">Agosto!B26</f>
+        <v>31039000</v>
+      </c>
+      <c r="C6" s="24" t="n">
+        <f aca="false">SUM(Real_vs_Presupuesto!C7:C12)</f>
+        <v>0</v>
+      </c>
+      <c r="D6" s="35" t="str">
+        <f aca="false">COUNT(Real_vs_Presupuesto!C7:C12)&amp;" de 6"</f>
+        <v>0 de 6</v>
+      </c>
+      <c r="E6" s="24" t="n">
+        <f aca="false">SUMIF(Real_vs_Presupuesto!C7:C12,"",Real_vs_Presupuesto!B7:B12)</f>
+        <v>31039000</v>
+      </c>
+      <c r="F6" s="26" t="n">
+        <f aca="false">C6+E6</f>
+        <v>31039000</v>
+      </c>
+      <c r="G6" s="37" t="n">
+        <f aca="false">F6/B6</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="33" t="n">
+        <f aca="false">Agosto!C26</f>
+        <v>25286303</v>
+      </c>
+      <c r="C7" s="24" t="n">
+        <f aca="false">SUM(Real_vs_Presupuesto!F7:F12)</f>
+        <v>0</v>
+      </c>
+      <c r="D7" s="35" t="str">
+        <f aca="false">COUNT(Real_vs_Presupuesto!F7:F12)&amp;" de 6"</f>
+        <v>0 de 6</v>
+      </c>
+      <c r="E7" s="24" t="n">
+        <f aca="false">SUMIF(Real_vs_Presupuesto!F7:F12,"",Real_vs_Presupuesto!E7:E12)</f>
+        <v>25286303</v>
+      </c>
+      <c r="F7" s="26" t="n">
+        <f aca="false">C7+E7</f>
+        <v>25286303</v>
+      </c>
+      <c r="G7" s="37" t="n">
+        <f aca="false">F7/B7</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="25" t="s">
+        <v>511</v>
+      </c>
+      <c r="B8" s="26" t="n">
+        <f aca="false">B6-B7</f>
+        <v>5752697</v>
+      </c>
+      <c r="C8" s="26" t="n">
+        <f aca="false">C6-C7</f>
+        <v>0</v>
+      </c>
+      <c r="D8" s="38"/>
+      <c r="E8" s="26" t="n">
+        <f aca="false">E6-E7</f>
+        <v>5752697</v>
+      </c>
+      <c r="F8" s="26" t="n">
+        <f aca="false">F6-F7</f>
+        <v>5752697</v>
+      </c>
+      <c r="G8" s="38"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="21" t="s">
+        <v>512</v>
+      </c>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="21"/>
+    </row>
+    <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="22" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" s="22" t="s">
+        <v>505</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>506</v>
+      </c>
+      <c r="D11" s="22" t="s">
+        <v>507</v>
+      </c>
+      <c r="E11" s="22" t="s">
+        <v>508</v>
+      </c>
+      <c r="F11" s="22" t="s">
+        <v>509</v>
+      </c>
+      <c r="G11" s="22" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="33" t="n">
+        <f aca="false">Septiembre!B25</f>
+        <v>41385344</v>
+      </c>
+      <c r="C12" s="24" t="n">
+        <f aca="false">SUM(Real_vs_Presupuesto!C16:C20)</f>
+        <v>0</v>
+      </c>
+      <c r="D12" s="35" t="str">
+        <f aca="false">COUNT(Real_vs_Presupuesto!C16:C20)&amp;" de 5"</f>
+        <v>0 de 5</v>
+      </c>
+      <c r="E12" s="24" t="n">
+        <f aca="false">SUMIF(Real_vs_Presupuesto!C16:C20,"",Real_vs_Presupuesto!B16:B20)</f>
+        <v>41385344</v>
+      </c>
+      <c r="F12" s="26" t="n">
+        <f aca="false">C12+E12</f>
+        <v>41385344</v>
+      </c>
+      <c r="G12" s="37" t="n">
+        <f aca="false">F12/B12</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" s="33" t="n">
+        <f aca="false">Septiembre!C25</f>
+        <v>32014353</v>
+      </c>
+      <c r="C13" s="24" t="n">
+        <f aca="false">SUM(Real_vs_Presupuesto!F16:F20)</f>
+        <v>0</v>
+      </c>
+      <c r="D13" s="35" t="str">
+        <f aca="false">COUNT(Real_vs_Presupuesto!F16:F20)&amp;" de 5"</f>
+        <v>0 de 5</v>
+      </c>
+      <c r="E13" s="24" t="n">
+        <f aca="false">SUMIF(Real_vs_Presupuesto!F16:F20,"",Real_vs_Presupuesto!E16:E20)</f>
+        <v>32014353</v>
+      </c>
+      <c r="F13" s="26" t="n">
+        <f aca="false">C13+E13</f>
+        <v>32014353</v>
+      </c>
+      <c r="G13" s="37" t="n">
+        <f aca="false">F13/B13</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="25" t="s">
+        <v>511</v>
+      </c>
+      <c r="B14" s="26" t="n">
+        <f aca="false">B12-B13</f>
+        <v>9370991</v>
+      </c>
+      <c r="C14" s="26" t="n">
+        <f aca="false">C12-C13</f>
+        <v>0</v>
+      </c>
+      <c r="D14" s="38"/>
+      <c r="E14" s="26" t="n">
+        <f aca="false">E12-E13</f>
+        <v>9370991</v>
+      </c>
+      <c r="F14" s="26" t="n">
+        <f aca="false">F12-F13</f>
+        <v>9370991</v>
+      </c>
+      <c r="G14" s="38"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A10:G10"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Actualiza Conciliacion_Julio con cartola de movimientos completa al 29-07-2026
</commit_message>
<xml_diff>
--- a/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
+++ b/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1852" uniqueCount="596">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1924" uniqueCount="614">
   <si>
     <t xml:space="preserve">SUPUESTOS DEL PRESUPUESTO — SOLLEM + TRAST</t>
   </si>
@@ -1323,10 +1323,10 @@
     <t xml:space="preserve">Nota: comparación agregada entre Abonos reales de la cartola y total facturado en Ventas RCV del mismo mes.</t>
   </si>
   <si>
-    <t xml:space="preserve">CONCILIACIÓN BANCARIA — JULIO 2026 (Global Solutions SPA, cartola PROVISORIA al 25-07-2026)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuente: Cartola provisoria N°3 (30/06 al 25/07/2026) + RCV Compra/Venta SII período 202607. Mes en curso, repetir con la cartola definitiva.</t>
+    <t xml:space="preserve">CONCILIACIÓN BANCARIA — JULIO 2026 (Global Solutions SPA, cartola completa al 29-07-2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuente: Cartola de movimientos completa (01/07 al 29/07/2026, 131 movimientos) + RCV Compra/Venta SII período 202607. Mes en curso (faltan 2 días hábiles), repetir con la cartola de cierre de mes.</t>
   </si>
   <si>
     <t xml:space="preserve">LOGÍSTICA Y TRANSPORTES ALFA JAM SPA</t>
@@ -1338,7 +1338,7 @@
     <t xml:space="preserve">01-07-2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Abono cartola 09-07-2026 — 0780993812 Transf. LOGISTICA Y TRA</t>
+    <t xml:space="preserve">Abono cartola 09-07-2026 — 0780993812 Transf. LOGISTICA Y TRANSPORTES A </t>
   </si>
   <si>
     <t xml:space="preserve">20</t>
@@ -1389,7 +1389,7 @@
     <t xml:space="preserve">02-07-2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Cargo cartola 02-07-2026 — 076630639K Transf a Servicios inte</t>
+    <t xml:space="preserve">Cargo cartola 02-07-2026 — 076630639K Transf a Servicios integrales FYR </t>
   </si>
   <si>
     <t xml:space="preserve">2666</t>
@@ -1434,7 +1434,7 @@
     <t xml:space="preserve">32124410</t>
   </si>
   <si>
-    <t xml:space="preserve">Cargo cartola 06-07-2026 — 0153706123 Transf a Francisco Manc</t>
+    <t xml:space="preserve">Cargo cartola 06-07-2026 — 0153706123 Transf a Francisco Mancilla</t>
   </si>
   <si>
     <t xml:space="preserve">32133874</t>
@@ -1467,7 +1467,7 @@
     <t xml:space="preserve">32142210</t>
   </si>
   <si>
-    <t xml:space="preserve">Cargo cartola 13-07-2026 — 0142013436 Transf a Felipe Madaria</t>
+    <t xml:space="preserve">Cargo cartola 13-07-2026 — 0153706123 Transf a Francisco Mancilla</t>
   </si>
   <si>
     <t xml:space="preserve">96815130-4</t>
@@ -1497,7 +1497,7 @@
     <t xml:space="preserve">11-07-2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Cargo cartola 13-07-2026 — 0153706123 Transf a Francisco Manc</t>
+    <t xml:space="preserve">Cargo cartola 13-07-2026 — 0142013436 Transf a Felipe Madariaga Parra</t>
   </si>
   <si>
     <t xml:space="preserve">2706</t>
@@ -1545,7 +1545,7 @@
     <t xml:space="preserve">32166690</t>
   </si>
   <si>
-    <t xml:space="preserve">Cargo cartola 09-07-2026 — 0153706123 Transf a Francisco Manc</t>
+    <t xml:space="preserve">Cargo cartola 09-07-2026 — 0153706123 Transf a Francisco Mancilla</t>
   </si>
   <si>
     <t xml:space="preserve">36566</t>
@@ -1572,7 +1572,7 @@
     <t xml:space="preserve">20-07-2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Cargo cartola 20-07-2026 — 0967985503 Transf a Multiaceros SA</t>
+    <t xml:space="preserve">Cargo cartola 20-07-2026 — PAGO EN LINEA ESMAX</t>
   </si>
   <si>
     <t xml:space="preserve">96798550-3</t>
@@ -1593,7 +1593,7 @@
     <t xml:space="preserve">32186742</t>
   </si>
   <si>
-    <t xml:space="preserve">Cargo cartola 21-07-2026 — 0142013436 Transf a Felipe Madaria</t>
+    <t xml:space="preserve">Cargo cartola 21-07-2026 — 0142013436 Transf a Felipe Madariaga Parra</t>
   </si>
   <si>
     <t xml:space="preserve">2754792</t>
@@ -1620,7 +1620,7 @@
     <t xml:space="preserve">23-07-2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Cargo cartola 23-07-2026 — 0783031345 Transf a Global Solutio</t>
+    <t xml:space="preserve">Cargo cartola 23-07-2026 — 0783031345 Transf a Global Solutions</t>
   </si>
   <si>
     <t xml:space="preserve">301679</t>
@@ -1638,7 +1638,7 @@
     <t xml:space="preserve">32203513</t>
   </si>
   <si>
-    <t xml:space="preserve">Cargo cartola 27-07-2026 — 0783031345 Transf a Global Solutio</t>
+    <t xml:space="preserve">Cargo cartola 27-07-2026 — 0783031345 Transf a Global Solutions</t>
   </si>
   <si>
     <t xml:space="preserve">22908735</t>
@@ -1662,19 +1662,43 @@
     <t xml:space="preserve">Identificado: 28 de 49 ($6,200,514)</t>
   </si>
   <si>
-    <t xml:space="preserve">0175020268 Transf a Nicolás Carval</t>
+    <t xml:space="preserve">0783031345 Transf. GLOBAL SOLUTIONS SPA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0159957802 Transf a RIQUELME OLEA PABLO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TUU*COMERCIAL ESCORPIO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0175020268 Transf a Nicolás Carvallo</t>
   </si>
   <si>
     <t xml:space="preserve">0119944848 Transf a José Acevedo</t>
   </si>
   <si>
-    <t xml:space="preserve">TUU*COMERCIAL ESCORPIO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0197068833 Transf a Felipe Tapia D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">019591141K Transf. Nicolas Matias</t>
+    <t xml:space="preserve">0168844255 Transf a Sebastián Zúñiga</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0772906366 Transf. SERVICIOS EL ENANO SPA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0776497649 Transf. COMERCIALIZADORA Y PR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0197068833 Transf a Felipe Tapia Diez</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0142013436 Transf a Felipe Madariaga Parra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0159957802 Transf de PABLO SEBASTIAN RIQ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0153706123 Transf a Francisco Mancilla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">019591141K Transf. Nicolas Matias Vega</t>
   </si>
   <si>
     <t xml:space="preserve">TUU*comercialEscorpion</t>
@@ -1683,40 +1707,70 @@
     <t xml:space="preserve">40574-SBX ROSARIO 100</t>
   </si>
   <si>
+    <t xml:space="preserve">COMERCIAL RIHE LTDA</t>
+  </si>
+  <si>
     <t xml:space="preserve">EL PALACIO DEL POROTO</t>
   </si>
   <si>
-    <t xml:space="preserve">COMERCIAL RIHE LTDA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0761971018 Transf. Financia Capita</t>
+    <t xml:space="preserve">0761971018 Transf. Financia Capital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0186584856 Transf. Andoni Luciano Sandova</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0967985503 Transf a Multiaceros SA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PAGO EN LINEA S.I.I.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RedGloba*PCY LTDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compra Nacional MD PROSERCOM SPA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compra Nacional MD VULKO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0771337724 PAGO PROVEEDOR Agricola Ge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27-07-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MERCADOPAGO *ELECTROS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compra Nacional MD FEDICAR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compra Nacional MD APRO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0140569097 Transf. ANDREA CLEMENTINA ALARCON LARA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GUILLERMO TOBIAS MOLIN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compra Nacional MD SOLMET SPA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28-07-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0070082349 Transf a VALDES CORNEJO NIBA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0783031345 Transf a Global Solutions</t>
   </si>
   <si>
     <t xml:space="preserve">PAGO EN LINEA ESMAX</t>
   </si>
   <si>
-    <t xml:space="preserve">PAGO EN LINEA S.I.I.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RedGloba*PCY LTDA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Compra Nacional MD VULKO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Compra Nacional MD PROSERCOM SPA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0771337724 PAGO PROVEEDOR Agricol</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27-07-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Compra Nacional MD SOLMET SPA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0140569097 Transf. ANDREA CLEMENTI</t>
+    <t xml:space="preserve">29-07-2026</t>
   </si>
   <si>
     <t xml:space="preserve">CONTROL DE CUMPLIMIENTO — REAL vs. PRESUPUESTO Y FLUJO DE CAJA</t>
@@ -9818,7 +9872,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I162"/>
+  <dimension ref="A1:I180"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -11410,16 +11464,16 @@
         <v>434</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>389</v>
+        <v>543</v>
       </c>
       <c r="C69" s="12" t="n">
-        <v>-70000</v>
+        <v>2326472</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11427,10 +11481,10 @@
         <v>434</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>385</v>
+        <v>544</v>
       </c>
       <c r="C70" s="12" t="n">
-        <v>-6000</v>
+        <v>-70000</v>
       </c>
       <c r="D70" s="3" t="s">
         <v>386</v>
@@ -11444,16 +11498,16 @@
         <v>434</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="C71" s="12" t="n">
-        <v>2326472</v>
+        <v>-6000</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11461,16 +11515,16 @@
         <v>451</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="C72" s="12" t="n">
-        <v>-190000</v>
+        <v>-2700</v>
       </c>
       <c r="D72" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>387</v>
+        <v>408</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11478,10 +11532,10 @@
         <v>451</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="C73" s="12" t="n">
-        <v>-54000</v>
+        <v>-190000</v>
       </c>
       <c r="D73" s="3" t="s">
         <v>386</v>
@@ -11495,10 +11549,10 @@
         <v>451</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>405</v>
+        <v>547</v>
       </c>
       <c r="C74" s="12" t="n">
-        <v>-225000</v>
+        <v>-54000</v>
       </c>
       <c r="D74" s="3" t="s">
         <v>386</v>
@@ -11512,16 +11566,16 @@
         <v>451</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="C75" s="12" t="n">
-        <v>-2700</v>
+        <v>-225000</v>
       </c>
       <c r="D75" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E75" s="3" t="s">
-        <v>408</v>
+        <v>387</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11529,13 +11583,13 @@
         <v>465</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>409</v>
+        <v>385</v>
       </c>
       <c r="C76" s="12" t="n">
-        <v>1200000</v>
+        <v>-17000</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="E76" s="3" t="s">
         <v>387</v>
@@ -11546,16 +11600,16 @@
         <v>465</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>392</v>
+        <v>549</v>
       </c>
       <c r="C77" s="12" t="n">
-        <v>-15000</v>
+        <v>83100</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="E77" s="3" t="s">
-        <v>387</v>
+        <v>408</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11563,16 +11617,16 @@
         <v>465</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>546</v>
+        <v>550</v>
       </c>
       <c r="C78" s="12" t="n">
-        <v>-280000</v>
+        <v>270000</v>
       </c>
       <c r="D78" s="3" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="E78" s="3" t="s">
-        <v>387</v>
+        <v>408</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11580,10 +11634,10 @@
         <v>465</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>385</v>
+        <v>551</v>
       </c>
       <c r="C79" s="12" t="n">
-        <v>-17000</v>
+        <v>-280000</v>
       </c>
       <c r="D79" s="3" t="s">
         <v>386</v>
@@ -11597,16 +11651,16 @@
         <v>465</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>419</v>
+        <v>552</v>
       </c>
       <c r="C80" s="12" t="n">
-        <v>83100</v>
+        <v>-15000</v>
       </c>
       <c r="D80" s="3" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="E80" s="3" t="s">
-        <v>408</v>
+        <v>387</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11614,16 +11668,16 @@
         <v>465</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>407</v>
+        <v>553</v>
       </c>
       <c r="C81" s="12" t="n">
-        <v>270000</v>
+        <v>1200000</v>
       </c>
       <c r="D81" s="3" t="s">
         <v>381</v>
       </c>
       <c r="E81" s="3" t="s">
-        <v>408</v>
+        <v>387</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11631,10 +11685,10 @@
         <v>469</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>392</v>
+        <v>544</v>
       </c>
       <c r="C82" s="12" t="n">
-        <v>-150000</v>
+        <v>-270000</v>
       </c>
       <c r="D82" s="3" t="s">
         <v>386</v>
@@ -11648,10 +11702,10 @@
         <v>469</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>392</v>
+        <v>548</v>
       </c>
       <c r="C83" s="12" t="n">
-        <v>-12000</v>
+        <v>-225000</v>
       </c>
       <c r="D83" s="3" t="s">
         <v>386</v>
@@ -11665,10 +11719,10 @@
         <v>469</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>389</v>
+        <v>552</v>
       </c>
       <c r="C84" s="12" t="n">
-        <v>-270000</v>
+        <v>-150000</v>
       </c>
       <c r="D84" s="3" t="s">
         <v>386</v>
@@ -11682,7 +11736,7 @@
         <v>469</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>388</v>
+        <v>554</v>
       </c>
       <c r="C85" s="12" t="n">
         <v>-180000</v>
@@ -11699,16 +11753,16 @@
         <v>469</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>405</v>
+        <v>555</v>
       </c>
       <c r="C86" s="12" t="n">
-        <v>-225000</v>
+        <v>320000</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="E86" s="3" t="s">
-        <v>387</v>
+        <v>408</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11750,16 +11804,16 @@
         <v>469</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>547</v>
+        <v>552</v>
       </c>
       <c r="C89" s="12" t="n">
-        <v>320000</v>
+        <v>-12000</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="E89" s="3" t="s">
-        <v>408</v>
+        <v>387</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11767,10 +11821,10 @@
         <v>469</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>392</v>
+        <v>552</v>
       </c>
       <c r="C90" s="12" t="n">
-        <v>-100000</v>
+        <v>-120000</v>
       </c>
       <c r="D90" s="3" t="s">
         <v>386</v>
@@ -11784,10 +11838,10 @@
         <v>469</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>392</v>
+        <v>552</v>
       </c>
       <c r="C91" s="12" t="n">
-        <v>-120000</v>
+        <v>-100000</v>
       </c>
       <c r="D91" s="3" t="s">
         <v>386</v>
@@ -11801,16 +11855,16 @@
         <v>471</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>393</v>
+        <v>556</v>
       </c>
       <c r="C92" s="12" t="n">
-        <v>-17000</v>
+        <v>-4700</v>
       </c>
       <c r="D92" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E92" s="3" t="s">
-        <v>387</v>
+        <v>408</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11818,10 +11872,10 @@
         <v>471</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C93" s="12" t="n">
-        <v>-12000</v>
+        <v>-17000</v>
       </c>
       <c r="D93" s="3" t="s">
         <v>386</v>
@@ -11835,16 +11889,16 @@
         <v>471</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>548</v>
+        <v>552</v>
       </c>
       <c r="C94" s="12" t="n">
-        <v>-4700</v>
+        <v>-12000</v>
       </c>
       <c r="D94" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E94" s="3" t="s">
-        <v>408</v>
+        <v>387</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11852,7 +11906,7 @@
         <v>473</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>392</v>
+        <v>552</v>
       </c>
       <c r="C95" s="12" t="n">
         <v>-8000</v>
@@ -11869,7 +11923,7 @@
         <v>473</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>549</v>
+        <v>557</v>
       </c>
       <c r="C96" s="12" t="n">
         <v>-14880</v>
@@ -11886,7 +11940,7 @@
         <v>473</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>392</v>
+        <v>552</v>
       </c>
       <c r="C97" s="12" t="n">
         <v>-32000</v>
@@ -11903,10 +11957,10 @@
         <v>483</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>550</v>
+        <v>558</v>
       </c>
       <c r="C98" s="12" t="n">
-        <v>-31955</v>
+        <v>-63065</v>
       </c>
       <c r="D98" s="3" t="s">
         <v>386</v>
@@ -11920,10 +11974,10 @@
         <v>483</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>551</v>
+        <v>559</v>
       </c>
       <c r="C99" s="12" t="n">
-        <v>-63065</v>
+        <v>-31955</v>
       </c>
       <c r="D99" s="3" t="s">
         <v>386</v>
@@ -11937,7 +11991,7 @@
         <v>490</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>392</v>
+        <v>552</v>
       </c>
       <c r="C100" s="12" t="n">
         <v>-17000</v>
@@ -11988,7 +12042,7 @@
         <v>497</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>409</v>
+        <v>553</v>
       </c>
       <c r="C103" s="12" t="n">
         <v>200000</v>
@@ -12005,7 +12059,7 @@
         <v>497</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>380</v>
+        <v>543</v>
       </c>
       <c r="C104" s="12" t="n">
         <v>1650249</v>
@@ -12022,7 +12076,7 @@
         <v>497</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>392</v>
+        <v>552</v>
       </c>
       <c r="C105" s="12" t="n">
         <v>-12000</v>
@@ -12039,10 +12093,10 @@
         <v>501</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>392</v>
+        <v>554</v>
       </c>
       <c r="C106" s="12" t="n">
-        <v>-16000</v>
+        <v>-15000</v>
       </c>
       <c r="D106" s="3" t="s">
         <v>386</v>
@@ -12056,10 +12110,10 @@
         <v>501</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>405</v>
+        <v>552</v>
       </c>
       <c r="C107" s="12" t="n">
-        <v>-225000</v>
+        <v>-16000</v>
       </c>
       <c r="D107" s="3" t="s">
         <v>386</v>
@@ -12073,10 +12127,10 @@
         <v>501</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>388</v>
+        <v>548</v>
       </c>
       <c r="C108" s="12" t="n">
-        <v>-15000</v>
+        <v>-225000</v>
       </c>
       <c r="D108" s="3" t="s">
         <v>386</v>
@@ -12090,10 +12144,10 @@
         <v>437</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>392</v>
+        <v>552</v>
       </c>
       <c r="C109" s="12" t="n">
-        <v>-50000</v>
+        <v>-6800</v>
       </c>
       <c r="D109" s="3" t="s">
         <v>386</v>
@@ -12107,10 +12161,10 @@
         <v>437</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>388</v>
+        <v>554</v>
       </c>
       <c r="C110" s="12" t="n">
-        <v>-15000</v>
+        <v>-30000</v>
       </c>
       <c r="D110" s="3" t="s">
         <v>386</v>
@@ -12124,10 +12178,10 @@
         <v>437</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>392</v>
+        <v>552</v>
       </c>
       <c r="C111" s="12" t="n">
-        <v>-6800</v>
+        <v>-6000</v>
       </c>
       <c r="D111" s="3" t="s">
         <v>386</v>
@@ -12141,10 +12195,10 @@
         <v>437</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>388</v>
+        <v>554</v>
       </c>
       <c r="C112" s="12" t="n">
-        <v>-30000</v>
+        <v>-15000</v>
       </c>
       <c r="D112" s="3" t="s">
         <v>386</v>
@@ -12158,10 +12212,10 @@
         <v>437</v>
       </c>
       <c r="B113" s="3" t="s">
-        <v>392</v>
+        <v>552</v>
       </c>
       <c r="C113" s="12" t="n">
-        <v>-6000</v>
+        <v>-50000</v>
       </c>
       <c r="D113" s="3" t="s">
         <v>386</v>
@@ -12175,7 +12229,7 @@
         <v>506</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>388</v>
+        <v>554</v>
       </c>
       <c r="C114" s="12" t="n">
         <v>-50000</v>
@@ -12192,7 +12246,7 @@
         <v>506</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>552</v>
+        <v>560</v>
       </c>
       <c r="C115" s="12" t="n">
         <v>2813595</v>
@@ -12209,10 +12263,10 @@
         <v>512</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>405</v>
+        <v>385</v>
       </c>
       <c r="C116" s="12" t="n">
-        <v>-55000</v>
+        <v>-400000</v>
       </c>
       <c r="D116" s="3" t="s">
         <v>386</v>
@@ -12226,16 +12280,16 @@
         <v>512</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>553</v>
+        <v>561</v>
       </c>
       <c r="C117" s="12" t="n">
-        <v>-1000000</v>
+        <v>760000</v>
       </c>
       <c r="D117" s="3" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="E117" s="3" t="s">
-        <v>77</v>
+        <v>408</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12243,10 +12297,10 @@
         <v>512</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>406</v>
+        <v>552</v>
       </c>
       <c r="C118" s="12" t="n">
-        <v>-150000</v>
+        <v>-250000</v>
       </c>
       <c r="D118" s="3" t="s">
         <v>386</v>
@@ -12260,7 +12314,7 @@
         <v>512</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="C119" s="12" t="n">
         <v>-300000</v>
@@ -12277,10 +12331,10 @@
         <v>512</v>
       </c>
       <c r="B120" s="3" t="s">
-        <v>388</v>
+        <v>544</v>
       </c>
       <c r="C120" s="12" t="n">
-        <v>-70000</v>
+        <v>-300000</v>
       </c>
       <c r="D120" s="3" t="s">
         <v>386</v>
@@ -12294,10 +12348,10 @@
         <v>512</v>
       </c>
       <c r="B121" s="3" t="s">
-        <v>392</v>
+        <v>406</v>
       </c>
       <c r="C121" s="12" t="n">
-        <v>-250000</v>
+        <v>-150000</v>
       </c>
       <c r="D121" s="3" t="s">
         <v>386</v>
@@ -12311,16 +12365,16 @@
         <v>512</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>417</v>
+        <v>562</v>
       </c>
       <c r="C122" s="12" t="n">
-        <v>760000</v>
+        <v>-1000000</v>
       </c>
       <c r="D122" s="3" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="E122" s="3" t="s">
-        <v>408</v>
+        <v>387</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12328,10 +12382,10 @@
         <v>512</v>
       </c>
       <c r="B123" s="3" t="s">
-        <v>385</v>
+        <v>548</v>
       </c>
       <c r="C123" s="12" t="n">
-        <v>-400000</v>
+        <v>-55000</v>
       </c>
       <c r="D123" s="3" t="s">
         <v>386</v>
@@ -12345,10 +12399,10 @@
         <v>512</v>
       </c>
       <c r="B124" s="3" t="s">
-        <v>393</v>
+        <v>554</v>
       </c>
       <c r="C124" s="12" t="n">
-        <v>-300000</v>
+        <v>-70000</v>
       </c>
       <c r="D124" s="3" t="s">
         <v>386</v>
@@ -12362,7 +12416,7 @@
         <v>439</v>
       </c>
       <c r="B125" s="3" t="s">
-        <v>388</v>
+        <v>554</v>
       </c>
       <c r="C125" s="12" t="n">
         <v>-17000</v>
@@ -12396,7 +12450,7 @@
         <v>439</v>
       </c>
       <c r="B127" s="3" t="s">
-        <v>554</v>
+        <v>563</v>
       </c>
       <c r="C127" s="12" t="n">
         <v>-9471</v>
@@ -12413,16 +12467,16 @@
         <v>522</v>
       </c>
       <c r="B128" s="3" t="s">
-        <v>552</v>
+        <v>564</v>
       </c>
       <c r="C128" s="12" t="n">
-        <v>2234722</v>
+        <v>-31319</v>
       </c>
       <c r="D128" s="3" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="E128" s="3" t="s">
-        <v>391</v>
+        <v>408</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12430,16 +12484,16 @@
         <v>522</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>392</v>
+        <v>543</v>
       </c>
       <c r="C129" s="12" t="n">
-        <v>-12000</v>
+        <v>198000</v>
       </c>
       <c r="D129" s="3" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="E129" s="3" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12447,7 +12501,7 @@
         <v>522</v>
       </c>
       <c r="B130" s="3" t="s">
-        <v>388</v>
+        <v>552</v>
       </c>
       <c r="C130" s="12" t="n">
         <v>-12000</v>
@@ -12464,16 +12518,16 @@
         <v>522</v>
       </c>
       <c r="B131" s="3" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="C131" s="12" t="n">
-        <v>-31319</v>
+        <v>-12000</v>
       </c>
       <c r="D131" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E131" s="3" t="s">
-        <v>408</v>
+        <v>387</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12481,16 +12535,16 @@
         <v>522</v>
       </c>
       <c r="B132" s="3" t="s">
-        <v>380</v>
+        <v>560</v>
       </c>
       <c r="C132" s="12" t="n">
-        <v>198000</v>
+        <v>2234722</v>
       </c>
       <c r="D132" s="3" t="s">
         <v>381</v>
       </c>
       <c r="E132" s="3" t="s">
-        <v>382</v>
+        <v>391</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12498,10 +12552,10 @@
         <v>528</v>
       </c>
       <c r="B133" s="3" t="s">
-        <v>393</v>
+        <v>548</v>
       </c>
       <c r="C133" s="12" t="n">
-        <v>-15000</v>
+        <v>-350000</v>
       </c>
       <c r="D133" s="3" t="s">
         <v>386</v>
@@ -12515,16 +12569,16 @@
         <v>528</v>
       </c>
       <c r="B134" s="3" t="s">
-        <v>556</v>
+        <v>552</v>
       </c>
       <c r="C134" s="12" t="n">
-        <v>-405600</v>
+        <v>-16000</v>
       </c>
       <c r="D134" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E134" s="3" t="s">
-        <v>395</v>
+        <v>387</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12532,16 +12586,16 @@
         <v>528</v>
       </c>
       <c r="B135" s="3" t="s">
-        <v>388</v>
+        <v>565</v>
       </c>
       <c r="C135" s="12" t="n">
-        <v>-20000</v>
+        <v>-5770</v>
       </c>
       <c r="D135" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E135" s="3" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12549,16 +12603,16 @@
         <v>528</v>
       </c>
       <c r="B136" s="3" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="C136" s="12" t="n">
-        <v>-5770</v>
+        <v>-20000</v>
       </c>
       <c r="D136" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E136" s="3" t="s">
-        <v>395</v>
+        <v>387</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12566,16 +12620,16 @@
         <v>528</v>
       </c>
       <c r="B137" s="3" t="s">
-        <v>392</v>
+        <v>566</v>
       </c>
       <c r="C137" s="12" t="n">
-        <v>-16000</v>
+        <v>-405600</v>
       </c>
       <c r="D137" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E137" s="3" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12583,10 +12637,10 @@
         <v>528</v>
       </c>
       <c r="B138" s="3" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
       <c r="C138" s="12" t="n">
-        <v>-350000</v>
+        <v>-15000</v>
       </c>
       <c r="D138" s="3" t="s">
         <v>386</v>
@@ -12600,7 +12654,7 @@
         <v>531</v>
       </c>
       <c r="B139" s="3" t="s">
-        <v>389</v>
+        <v>554</v>
       </c>
       <c r="C139" s="12" t="n">
         <v>-20000</v>
@@ -12617,10 +12671,10 @@
         <v>531</v>
       </c>
       <c r="B140" s="3" t="s">
-        <v>393</v>
+        <v>552</v>
       </c>
       <c r="C140" s="12" t="n">
-        <v>-29000</v>
+        <v>-20000</v>
       </c>
       <c r="D140" s="3" t="s">
         <v>386</v>
@@ -12634,7 +12688,7 @@
         <v>531</v>
       </c>
       <c r="B141" s="3" t="s">
-        <v>558</v>
+        <v>567</v>
       </c>
       <c r="C141" s="12" t="n">
         <v>357000</v>
@@ -12651,10 +12705,10 @@
         <v>531</v>
       </c>
       <c r="B142" s="3" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="C142" s="12" t="n">
-        <v>-20000</v>
+        <v>-29000</v>
       </c>
       <c r="D142" s="3" t="s">
         <v>386</v>
@@ -12668,7 +12722,7 @@
         <v>531</v>
       </c>
       <c r="B143" s="3" t="s">
-        <v>392</v>
+        <v>544</v>
       </c>
       <c r="C143" s="12" t="n">
         <v>-20000</v>
@@ -12682,64 +12736,64 @@
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="3" t="s">
-        <v>559</v>
+        <v>568</v>
       </c>
       <c r="B144" s="3" t="s">
-        <v>560</v>
+        <v>554</v>
       </c>
       <c r="C144" s="12" t="n">
-        <v>-38000</v>
+        <v>-12000</v>
       </c>
       <c r="D144" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E144" s="3" t="s">
-        <v>395</v>
+        <v>387</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="3" t="s">
-        <v>559</v>
+        <v>568</v>
       </c>
       <c r="B145" s="3" t="s">
-        <v>389</v>
+        <v>569</v>
       </c>
       <c r="C145" s="12" t="n">
-        <v>-25000</v>
+        <v>-58001</v>
       </c>
       <c r="D145" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E145" s="3" t="s">
-        <v>387</v>
+        <v>408</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="3" t="s">
-        <v>559</v>
+        <v>568</v>
       </c>
       <c r="B146" s="3" t="s">
-        <v>405</v>
+        <v>570</v>
       </c>
       <c r="C146" s="12" t="n">
-        <v>-18000</v>
+        <v>-6950</v>
       </c>
       <c r="D146" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E146" s="3" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="3" t="s">
-        <v>559</v>
+        <v>568</v>
       </c>
       <c r="B147" s="3" t="s">
-        <v>388</v>
+        <v>552</v>
       </c>
       <c r="C147" s="12" t="n">
-        <v>-3000</v>
+        <v>-15000</v>
       </c>
       <c r="D147" s="3" t="s">
         <v>386</v>
@@ -12750,168 +12804,474 @@
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="3" t="s">
-        <v>559</v>
+        <v>568</v>
       </c>
       <c r="B148" s="3" t="s">
-        <v>388</v>
+        <v>571</v>
       </c>
       <c r="C148" s="12" t="n">
-        <v>-120000</v>
+        <v>-66878</v>
       </c>
       <c r="D148" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E148" s="3" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="3" t="s">
-        <v>559</v>
+        <v>568</v>
       </c>
       <c r="B149" s="3" t="s">
-        <v>392</v>
+        <v>572</v>
       </c>
       <c r="C149" s="12" t="n">
-        <v>-70000</v>
+        <v>490200</v>
       </c>
       <c r="D149" s="3" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="E149" s="3" t="s">
-        <v>387</v>
+        <v>408</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="3" t="s">
-        <v>559</v>
+        <v>568</v>
       </c>
       <c r="B150" s="3" t="s">
-        <v>409</v>
+        <v>573</v>
       </c>
       <c r="C150" s="12" t="n">
-        <v>1000000</v>
+        <v>-4200</v>
       </c>
       <c r="D150" s="3" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="E150" s="3" t="s">
-        <v>387</v>
+        <v>408</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="3" t="s">
-        <v>559</v>
+        <v>568</v>
       </c>
       <c r="B151" s="3" t="s">
-        <v>561</v>
+        <v>573</v>
       </c>
       <c r="C151" s="12" t="n">
-        <v>200000</v>
+        <v>-6700</v>
       </c>
       <c r="D151" s="3" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="E151" s="3" t="s">
         <v>408</v>
       </c>
     </row>
+    <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A152" s="3" t="s">
+        <v>568</v>
+      </c>
+      <c r="B152" s="3" t="s">
+        <v>548</v>
+      </c>
+      <c r="C152" s="12" t="n">
+        <v>-18000</v>
+      </c>
+      <c r="D152" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="E152" s="3" t="s">
+        <v>387</v>
+      </c>
+    </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A153" s="2" t="s">
-        <v>420</v>
-      </c>
-      <c r="B153" s="2"/>
-      <c r="C153" s="2"/>
-      <c r="D153" s="2"/>
-      <c r="E153" s="2"/>
-      <c r="F153" s="2"/>
-      <c r="G153" s="2"/>
-      <c r="H153" s="2"/>
-      <c r="I153" s="2"/>
+      <c r="A153" s="3" t="s">
+        <v>568</v>
+      </c>
+      <c r="B153" s="3" t="s">
+        <v>572</v>
+      </c>
+      <c r="C153" s="12" t="n">
+        <v>200000</v>
+      </c>
+      <c r="D153" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="E153" s="3" t="s">
+        <v>408</v>
+      </c>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A154" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="B154" s="9" t="s">
-        <v>377</v>
-      </c>
-      <c r="C154" s="30" t="s">
-        <v>421</v>
-      </c>
-      <c r="D154" s="30" t="s">
-        <v>422</v>
+      <c r="A154" s="3" t="s">
+        <v>568</v>
+      </c>
+      <c r="B154" s="3" t="s">
+        <v>574</v>
+      </c>
+      <c r="C154" s="12" t="n">
+        <v>-38000</v>
+      </c>
+      <c r="D154" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="E154" s="3" t="s">
+        <v>395</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="3" t="s">
-        <v>423</v>
-      </c>
-      <c r="B155" s="12" t="n">
-        <v>267206</v>
+        <v>568</v>
+      </c>
+      <c r="B155" s="3" t="s">
+        <v>553</v>
+      </c>
+      <c r="C155" s="12" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D155" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="E155" s="3" t="s">
+        <v>387</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="3" t="s">
+        <v>568</v>
+      </c>
+      <c r="B156" s="3" t="s">
+        <v>552</v>
+      </c>
+      <c r="C156" s="12" t="n">
+        <v>-70000</v>
+      </c>
+      <c r="D156" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="E156" s="3" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A157" s="3" t="s">
+        <v>568</v>
+      </c>
+      <c r="B157" s="3" t="s">
+        <v>554</v>
+      </c>
+      <c r="C157" s="12" t="n">
+        <v>-120000</v>
+      </c>
+      <c r="D157" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="E157" s="3" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A158" s="3" t="s">
+        <v>568</v>
+      </c>
+      <c r="B158" s="3" t="s">
+        <v>554</v>
+      </c>
+      <c r="C158" s="12" t="n">
+        <v>-3000</v>
+      </c>
+      <c r="D158" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="E158" s="3" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A159" s="3" t="s">
+        <v>568</v>
+      </c>
+      <c r="B159" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="C159" s="12" t="n">
+        <v>-25000</v>
+      </c>
+      <c r="D159" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="E159" s="3" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A160" s="3" t="s">
+        <v>568</v>
+      </c>
+      <c r="B160" s="3" t="s">
+        <v>573</v>
+      </c>
+      <c r="C160" s="12" t="n">
+        <v>-16500</v>
+      </c>
+      <c r="D160" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="E160" s="3" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A161" s="3" t="s">
+        <v>575</v>
+      </c>
+      <c r="B161" s="3" t="s">
+        <v>552</v>
+      </c>
+      <c r="C161" s="12" t="n">
+        <v>-15000</v>
+      </c>
+      <c r="D161" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="E161" s="3" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A162" s="3" t="s">
+        <v>575</v>
+      </c>
+      <c r="B162" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="C162" s="12" t="n">
+        <v>-170000</v>
+      </c>
+      <c r="D162" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="E162" s="3" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A163" s="3" t="s">
+        <v>575</v>
+      </c>
+      <c r="B163" s="3" t="s">
+        <v>576</v>
+      </c>
+      <c r="C163" s="12" t="n">
+        <v>-97000</v>
+      </c>
+      <c r="D163" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="E163" s="3" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A164" s="3" t="s">
+        <v>575</v>
+      </c>
+      <c r="B164" s="3" t="s">
+        <v>554</v>
+      </c>
+      <c r="C164" s="12" t="n">
+        <v>-20000</v>
+      </c>
+      <c r="D164" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="E164" s="3" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A165" s="3" t="s">
+        <v>575</v>
+      </c>
+      <c r="B165" s="3" t="s">
+        <v>577</v>
+      </c>
+      <c r="C165" s="12" t="n">
+        <v>-100000</v>
+      </c>
+      <c r="D165" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="E165" s="3" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A166" s="3" t="s">
+        <v>575</v>
+      </c>
+      <c r="B166" s="3" t="s">
+        <v>578</v>
+      </c>
+      <c r="C166" s="12" t="n">
+        <v>-800000</v>
+      </c>
+      <c r="D166" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="E166" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A167" s="3" t="s">
+        <v>579</v>
+      </c>
+      <c r="B167" s="3" t="s">
+        <v>554</v>
+      </c>
+      <c r="C167" s="12" t="n">
+        <v>-100000</v>
+      </c>
+      <c r="D167" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="E167" s="3" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A168" s="3" t="s">
+        <v>579</v>
+      </c>
+      <c r="B168" s="3" t="s">
+        <v>554</v>
+      </c>
+      <c r="C168" s="12" t="n">
+        <v>-53000</v>
+      </c>
+      <c r="D168" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="E168" s="3" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A169" s="3" t="s">
+        <v>579</v>
+      </c>
+      <c r="B169" s="3" t="s">
+        <v>577</v>
+      </c>
+      <c r="C169" s="12" t="n">
+        <v>-50000</v>
+      </c>
+      <c r="D169" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="E169" s="3" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A171" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="B171" s="2"/>
+      <c r="C171" s="2"/>
+      <c r="D171" s="2"/>
+      <c r="E171" s="2"/>
+      <c r="F171" s="2"/>
+      <c r="G171" s="2"/>
+      <c r="H171" s="2"/>
+      <c r="I171" s="2"/>
+    </row>
+    <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A172" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="B172" s="9" t="s">
+        <v>377</v>
+      </c>
+      <c r="C172" s="30" t="s">
+        <v>421</v>
+      </c>
+      <c r="D172" s="30" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A173" s="3" t="s">
+        <v>423</v>
+      </c>
+      <c r="B173" s="12" t="n">
+        <v>267206</v>
+      </c>
+    </row>
+    <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A174" s="3" t="s">
         <v>424</v>
       </c>
-      <c r="B156" s="12" t="n">
-        <v>14053438</v>
-      </c>
-      <c r="C156" s="31" t="n">
+      <c r="B174" s="12" t="n">
+        <v>14543638</v>
+      </c>
+      <c r="C174" s="31" t="n">
         <f aca="false">F11</f>
         <v>6122312</v>
       </c>
-      <c r="D156" s="31" t="n">
-        <f aca="false">B156-C156</f>
-        <v>7931126</v>
-      </c>
-    </row>
-    <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A157" s="3" t="s">
+      <c r="D174" s="31" t="n">
+        <f aca="false">B174-C174</f>
+        <v>8421326</v>
+      </c>
+    </row>
+    <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A175" s="3" t="s">
         <v>425</v>
       </c>
-      <c r="B157" s="12" t="n">
-        <v>-13156244</v>
-      </c>
-    </row>
-    <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A158" s="18" t="s">
+      <c r="B175" s="12" t="n">
+        <v>-14747473</v>
+      </c>
+    </row>
+    <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A176" s="18" t="s">
         <v>426</v>
       </c>
-      <c r="B158" s="14" t="n">
-        <f aca="false">SUM(B155:B157)</f>
-        <v>1164400</v>
-      </c>
-    </row>
-    <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A159" s="18" t="s">
+      <c r="B176" s="14" t="n">
+        <f aca="false">SUM(B173:B175)</f>
+        <v>63371</v>
+      </c>
+    </row>
+    <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A177" s="18" t="s">
         <v>427</v>
       </c>
-      <c r="B159" s="14" t="n">
-        <v>1164400</v>
-      </c>
-    </row>
-    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A160" s="18" t="s">
+      <c r="B177" s="14" t="n">
+        <v>63371</v>
+      </c>
+    </row>
+    <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A178" s="18" t="s">
         <v>428</v>
       </c>
-      <c r="B160" s="14" t="n">
-        <f aca="false">B158-B159</f>
+      <c r="B178" s="14" t="n">
+        <f aca="false">B176-B177</f>
         <v>0</v>
       </c>
     </row>
-    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A162" s="10" t="s">
+    <row r="180" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A180" s="10" t="s">
         <v>429</v>
       </c>
-      <c r="B162" s="10"/>
-      <c r="C162" s="10"/>
-      <c r="D162" s="10"/>
-      <c r="E162" s="10"/>
-      <c r="F162" s="10"/>
-      <c r="G162" s="10"/>
-      <c r="H162" s="10"/>
+      <c r="B180" s="10"/>
+      <c r="C180" s="10"/>
+      <c r="D180" s="10"/>
+      <c r="E180" s="10"/>
+      <c r="F180" s="10"/>
+      <c r="G180" s="10"/>
+      <c r="H180" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -12920,8 +13280,8 @@
     <mergeCell ref="A4:I4"/>
     <mergeCell ref="A13:I13"/>
     <mergeCell ref="A66:I66"/>
-    <mergeCell ref="A153:I153"/>
-    <mergeCell ref="A162:H162"/>
+    <mergeCell ref="A171:I171"/>
+    <mergeCell ref="A180:H180"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -12948,7 +13308,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>562</v>
+        <v>580</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -12963,7 +13323,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="28" t="s">
-        <v>563</v>
+        <v>581</v>
       </c>
       <c r="B2" s="28"/>
       <c r="C2" s="28"/>
@@ -12978,7 +13338,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>564</v>
+        <v>582</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -12996,34 +13356,34 @@
         <v>153</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>565</v>
+        <v>583</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>566</v>
+        <v>584</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>567</v>
+        <v>585</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>568</v>
+        <v>586</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>569</v>
+        <v>587</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>570</v>
+        <v>588</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>571</v>
+        <v>589</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>572</v>
+        <v>590</v>
       </c>
       <c r="J5" s="9" t="s">
-        <v>573</v>
+        <v>591</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>574</v>
+        <v>592</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13250,7 +13610,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>575</v>
+        <v>593</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -13268,34 +13628,34 @@
         <v>153</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>565</v>
+        <v>583</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>566</v>
+        <v>584</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>567</v>
+        <v>585</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>568</v>
+        <v>586</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>569</v>
+        <v>587</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>570</v>
+        <v>588</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>571</v>
+        <v>589</v>
       </c>
       <c r="I14" s="9" t="s">
-        <v>572</v>
+        <v>590</v>
       </c>
       <c r="J14" s="9" t="s">
-        <v>573</v>
+        <v>591</v>
       </c>
       <c r="K14" s="9" t="s">
-        <v>574</v>
+        <v>592</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13514,7 +13874,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>576</v>
+        <v>594</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -13525,7 +13885,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>577</v>
+        <v>595</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -13535,10 +13895,10 @@
         <v>65</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>578</v>
+        <v>596</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>579</v>
+        <v>597</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13556,7 +13916,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>580</v>
+        <v>598</v>
       </c>
       <c r="B6" s="12" t="n">
         <f aca="false">Consolidado!B6</f>
@@ -13595,7 +13955,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>581</v>
+        <v>599</v>
       </c>
       <c r="B9" s="17" t="n">
         <f aca="false">Consolidado!B10</f>
@@ -13686,7 +14046,7 @@
     </row>
     <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>582</v>
+        <v>600</v>
       </c>
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
@@ -13697,7 +14057,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>583</v>
+        <v>601</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -13708,7 +14068,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="28" t="s">
-        <v>584</v>
+        <v>602</v>
       </c>
       <c r="B21" s="28"/>
       <c r="C21" s="28"/>
@@ -13719,7 +14079,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>585</v>
+        <v>603</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -13733,27 +14093,27 @@
         <v>65</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>586</v>
+        <v>604</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>587</v>
+        <v>605</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>588</v>
+        <v>606</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>589</v>
+        <v>607</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>590</v>
+        <v>608</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>591</v>
+        <v>609</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>592</v>
+        <v>610</v>
       </c>
       <c r="B24" s="33" t="n">
         <f aca="false">Consolidado!B32</f>
@@ -13782,7 +14142,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>593</v>
+        <v>611</v>
       </c>
       <c r="B25" s="33" t="n">
         <f aca="false">Consolidado!C32</f>
@@ -13811,7 +14171,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="18" t="s">
-        <v>594</v>
+        <v>612</v>
       </c>
       <c r="B26" s="14" t="n">
         <f aca="false">B24-B25</f>
@@ -13834,7 +14194,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>595</v>
+        <v>613</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -13848,27 +14208,27 @@
         <v>65</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>586</v>
+        <v>604</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>587</v>
+        <v>605</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>588</v>
+        <v>606</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>589</v>
+        <v>607</v>
       </c>
       <c r="F29" s="9" t="s">
-        <v>590</v>
+        <v>608</v>
       </c>
       <c r="G29" s="9" t="s">
-        <v>591</v>
+        <v>609</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>592</v>
+        <v>610</v>
       </c>
       <c r="B30" s="33" t="n">
         <f aca="false">Consolidado!B41</f>
@@ -13897,7 +14257,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>593</v>
+        <v>611</v>
       </c>
       <c r="B31" s="33" t="n">
         <f aca="false">Consolidado!C41</f>
@@ -13926,7 +14286,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="18" t="s">
-        <v>594</v>
+        <v>612</v>
       </c>
       <c r="B32" s="14" t="n">
         <f aca="false">B30-B31</f>

</xml_diff>

<commit_message>
Agrega hoja Bitacora_Saldo_Diario, lista para partir agosto
</commit_message>
<xml_diff>
--- a/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
+++ b/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
@@ -16,6 +16,7 @@
     <sheet name="Conciliación_Julio" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="Real_vs_Presupuesto" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="Resumen_Ejecutivo" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="Bitácora_Saldo_Diario" sheetId="9" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1924" uniqueCount="614">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1935" uniqueCount="622">
   <si>
     <t xml:space="preserve">SUPUESTOS DEL PRESUPUESTO — SOLLEM + TRAST</t>
   </si>
@@ -1886,6 +1887,33 @@
   </si>
   <si>
     <t xml:space="preserve">SEPTIEMBRE 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BITÁCORA DE SALDO DIARIO — Banco Santander 0-000-3776731-0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Registro diario del "Saldo de Cuentas Corrientes" (reporte simple, sin movimientos). Alerta temprana: compara el saldo real contra el Saldo Acumulado que proyecta Consolidado para esa semana. Al cierre de cada semana, esto se cruza con la conciliación completa (Conciliación_Junio/Julio como plantilla) — la bitácora es la alerta, la conciliación semanal es la confirmación con facturas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saldo Disponible
+(real, del reporte)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Semana
+Consolidado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saldo Acumulado
+Proyectado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diferencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Julio (fuera de Consolidado, mes en curso pre-agosto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saldo real del 29-07-2026, cartola completa conciliada. Punto de partida de la bitácora.</t>
   </si>
 </sst>
 </file>
@@ -2080,7 +2108,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2230,6 +2258,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -14325,4 +14357,363 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F30"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="40"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>614</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="24" t="s">
+        <v>615</v>
+      </c>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+    </row>
+    <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
+        <v>375</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>616</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>617</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>618</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>619</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>579</v>
+      </c>
+      <c r="B5" s="12" t="n">
+        <v>63371</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>620</v>
+      </c>
+      <c r="D5" s="37"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="3" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="38"/>
+      <c r="B6" s="34"/>
+      <c r="C6" s="38"/>
+      <c r="D6" s="34"/>
+      <c r="E6" s="12" t="str">
+        <f aca="false">IF(OR(B6="",D6=""),"",B6-D6)</f>
+        <v/>
+      </c>
+      <c r="F6" s="38"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="38"/>
+      <c r="B7" s="34"/>
+      <c r="C7" s="38"/>
+      <c r="D7" s="34"/>
+      <c r="E7" s="12" t="str">
+        <f aca="false">IF(OR(B7="",D7=""),"",B7-D7)</f>
+        <v/>
+      </c>
+      <c r="F7" s="38"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="38"/>
+      <c r="B8" s="34"/>
+      <c r="C8" s="38"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="12" t="str">
+        <f aca="false">IF(OR(B8="",D8=""),"",B8-D8)</f>
+        <v/>
+      </c>
+      <c r="F8" s="38"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="38"/>
+      <c r="B9" s="34"/>
+      <c r="C9" s="38"/>
+      <c r="D9" s="34"/>
+      <c r="E9" s="12" t="str">
+        <f aca="false">IF(OR(B9="",D9=""),"",B9-D9)</f>
+        <v/>
+      </c>
+      <c r="F9" s="38"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="38"/>
+      <c r="B10" s="34"/>
+      <c r="C10" s="38"/>
+      <c r="D10" s="34"/>
+      <c r="E10" s="12" t="str">
+        <f aca="false">IF(OR(B10="",D10=""),"",B10-D10)</f>
+        <v/>
+      </c>
+      <c r="F10" s="38"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="38"/>
+      <c r="B11" s="34"/>
+      <c r="C11" s="38"/>
+      <c r="D11" s="34"/>
+      <c r="E11" s="12" t="str">
+        <f aca="false">IF(OR(B11="",D11=""),"",B11-D11)</f>
+        <v/>
+      </c>
+      <c r="F11" s="38"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="38"/>
+      <c r="B12" s="34"/>
+      <c r="C12" s="38"/>
+      <c r="D12" s="34"/>
+      <c r="E12" s="12" t="str">
+        <f aca="false">IF(OR(B12="",D12=""),"",B12-D12)</f>
+        <v/>
+      </c>
+      <c r="F12" s="38"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="38"/>
+      <c r="B13" s="34"/>
+      <c r="C13" s="38"/>
+      <c r="D13" s="34"/>
+      <c r="E13" s="12" t="str">
+        <f aca="false">IF(OR(B13="",D13=""),"",B13-D13)</f>
+        <v/>
+      </c>
+      <c r="F13" s="38"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="38"/>
+      <c r="B14" s="34"/>
+      <c r="C14" s="38"/>
+      <c r="D14" s="34"/>
+      <c r="E14" s="12" t="str">
+        <f aca="false">IF(OR(B14="",D14=""),"",B14-D14)</f>
+        <v/>
+      </c>
+      <c r="F14" s="38"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="38"/>
+      <c r="B15" s="34"/>
+      <c r="C15" s="38"/>
+      <c r="D15" s="34"/>
+      <c r="E15" s="12" t="str">
+        <f aca="false">IF(OR(B15="",D15=""),"",B15-D15)</f>
+        <v/>
+      </c>
+      <c r="F15" s="38"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="38"/>
+      <c r="B16" s="34"/>
+      <c r="C16" s="38"/>
+      <c r="D16" s="34"/>
+      <c r="E16" s="12" t="str">
+        <f aca="false">IF(OR(B16="",D16=""),"",B16-D16)</f>
+        <v/>
+      </c>
+      <c r="F16" s="38"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="38"/>
+      <c r="B17" s="34"/>
+      <c r="C17" s="38"/>
+      <c r="D17" s="34"/>
+      <c r="E17" s="12" t="str">
+        <f aca="false">IF(OR(B17="",D17=""),"",B17-D17)</f>
+        <v/>
+      </c>
+      <c r="F17" s="38"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="38"/>
+      <c r="B18" s="34"/>
+      <c r="C18" s="38"/>
+      <c r="D18" s="34"/>
+      <c r="E18" s="12" t="str">
+        <f aca="false">IF(OR(B18="",D18=""),"",B18-D18)</f>
+        <v/>
+      </c>
+      <c r="F18" s="38"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="38"/>
+      <c r="B19" s="34"/>
+      <c r="C19" s="38"/>
+      <c r="D19" s="34"/>
+      <c r="E19" s="12" t="str">
+        <f aca="false">IF(OR(B19="",D19=""),"",B19-D19)</f>
+        <v/>
+      </c>
+      <c r="F19" s="38"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="38"/>
+      <c r="B20" s="34"/>
+      <c r="C20" s="38"/>
+      <c r="D20" s="34"/>
+      <c r="E20" s="12" t="str">
+        <f aca="false">IF(OR(B20="",D20=""),"",B20-D20)</f>
+        <v/>
+      </c>
+      <c r="F20" s="38"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="38"/>
+      <c r="B21" s="34"/>
+      <c r="C21" s="38"/>
+      <c r="D21" s="34"/>
+      <c r="E21" s="12" t="str">
+        <f aca="false">IF(OR(B21="",D21=""),"",B21-D21)</f>
+        <v/>
+      </c>
+      <c r="F21" s="38"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="38"/>
+      <c r="B22" s="34"/>
+      <c r="C22" s="38"/>
+      <c r="D22" s="34"/>
+      <c r="E22" s="12" t="str">
+        <f aca="false">IF(OR(B22="",D22=""),"",B22-D22)</f>
+        <v/>
+      </c>
+      <c r="F22" s="38"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="38"/>
+      <c r="B23" s="34"/>
+      <c r="C23" s="38"/>
+      <c r="D23" s="34"/>
+      <c r="E23" s="12" t="str">
+        <f aca="false">IF(OR(B23="",D23=""),"",B23-D23)</f>
+        <v/>
+      </c>
+      <c r="F23" s="38"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="38"/>
+      <c r="B24" s="34"/>
+      <c r="C24" s="38"/>
+      <c r="D24" s="34"/>
+      <c r="E24" s="12" t="str">
+        <f aca="false">IF(OR(B24="",D24=""),"",B24-D24)</f>
+        <v/>
+      </c>
+      <c r="F24" s="38"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="38"/>
+      <c r="B25" s="34"/>
+      <c r="C25" s="38"/>
+      <c r="D25" s="34"/>
+      <c r="E25" s="12" t="str">
+        <f aca="false">IF(OR(B25="",D25=""),"",B25-D25)</f>
+        <v/>
+      </c>
+      <c r="F25" s="38"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="38"/>
+      <c r="B26" s="34"/>
+      <c r="C26" s="38"/>
+      <c r="D26" s="34"/>
+      <c r="E26" s="12" t="str">
+        <f aca="false">IF(OR(B26="",D26=""),"",B26-D26)</f>
+        <v/>
+      </c>
+      <c r="F26" s="38"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="38"/>
+      <c r="B27" s="34"/>
+      <c r="C27" s="38"/>
+      <c r="D27" s="34"/>
+      <c r="E27" s="12" t="str">
+        <f aca="false">IF(OR(B27="",D27=""),"",B27-D27)</f>
+        <v/>
+      </c>
+      <c r="F27" s="38"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="38"/>
+      <c r="B28" s="34"/>
+      <c r="C28" s="38"/>
+      <c r="D28" s="34"/>
+      <c r="E28" s="12" t="str">
+        <f aca="false">IF(OR(B28="",D28=""),"",B28-D28)</f>
+        <v/>
+      </c>
+      <c r="F28" s="38"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="38"/>
+      <c r="B29" s="34"/>
+      <c r="C29" s="38"/>
+      <c r="D29" s="34"/>
+      <c r="E29" s="12" t="str">
+        <f aca="false">IF(OR(B29="",D29=""),"",B29-D29)</f>
+        <v/>
+      </c>
+      <c r="F29" s="38"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="38"/>
+      <c r="B30" s="34"/>
+      <c r="C30" s="38"/>
+      <c r="D30" s="34"/>
+      <c r="E30" s="12" t="str">
+        <f aca="false">IF(OR(B30="",D30=""),"",B30-D30)</f>
+        <v/>
+      </c>
+      <c r="F30" s="38"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Actualiza Conciliacion_Julio con RCV Compra completo (59 facturas)
</commit_message>
<xml_diff>
--- a/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
+++ b/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1935" uniqueCount="622">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1965" uniqueCount="637">
   <si>
     <t xml:space="preserve">SUPUESTOS DEL PRESUPUESTO — SOLLEM + TRAST</t>
   </si>
@@ -1549,12 +1549,18 @@
     <t xml:space="preserve">Cargo cartola 09-07-2026 — 0153706123 Transf a Francisco Mancilla</t>
   </si>
   <si>
+    <t xml:space="preserve">2732</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2734</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17-07-2026</t>
+  </si>
+  <si>
     <t xml:space="preserve">36566</t>
   </si>
   <si>
-    <t xml:space="preserve">17-07-2026</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cargo cartola 20-07-2026 — Compra Nacional MD ARAMCO</t>
   </si>
   <si>
@@ -1657,10 +1663,73 @@
     <t xml:space="preserve">89054</t>
   </si>
   <si>
+    <t xml:space="preserve">76882569-6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7242</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27-07-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">86887200-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3704825</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cargo cartola 27-07-2026 — Compra Nacional MD APRO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5404067-9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38395</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cargo cartola 27-07-2026 — Compra Nacional MD FEDICAR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">76784703-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3883</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cargo cartola 27-07-2026 — Compra Nacional MD SOLMET SPA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2755582</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28-07-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cargo cartola 28-07-2026 — PAGO EN LINEA ESMAX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7008234-9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">105109</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cargo cartola 28-07-2026 — 0070082349 Transf a VALDES CORNEJO NIBA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">32544416</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2756031</t>
+  </si>
+  <si>
+    <t xml:space="preserve">29-07-2026</t>
+  </si>
+  <si>
     <t xml:space="preserve">20435</t>
   </si>
   <si>
-    <t xml:space="preserve">Identificado: 28 de 49 ($6,200,514)</t>
+    <t xml:space="preserve">Identificado: 33 de 59 ($7,209,342)</t>
   </si>
   <si>
     <t xml:space="preserve">0783031345 Transf. GLOBAL SOLUTIONS SPA</t>
@@ -1717,61 +1786,37 @@
     <t xml:space="preserve">0761971018 Transf. Financia Capital</t>
   </si>
   <si>
+    <t xml:space="preserve">0967985503 Transf a Multiaceros SA</t>
+  </si>
+  <si>
     <t xml:space="preserve">0186584856 Transf. Andoni Luciano Sandova</t>
   </si>
   <si>
-    <t xml:space="preserve">0967985503 Transf a Multiaceros SA</t>
-  </si>
-  <si>
     <t xml:space="preserve">PAGO EN LINEA S.I.I.</t>
   </si>
   <si>
     <t xml:space="preserve">RedGloba*PCY LTDA</t>
   </si>
   <si>
+    <t xml:space="preserve">Compra Nacional MD VULKO</t>
+  </si>
+  <si>
     <t xml:space="preserve">Compra Nacional MD PROSERCOM SPA</t>
   </si>
   <si>
-    <t xml:space="preserve">Compra Nacional MD VULKO</t>
-  </si>
-  <si>
     <t xml:space="preserve">0771337724 PAGO PROVEEDOR Agricola Ge</t>
   </si>
   <si>
-    <t xml:space="preserve">27-07-2026</t>
-  </si>
-  <si>
     <t xml:space="preserve">MERCADOPAGO *ELECTROS</t>
   </si>
   <si>
-    <t xml:space="preserve">Compra Nacional MD FEDICAR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Compra Nacional MD APRO</t>
+    <t xml:space="preserve">GUILLERMO TOBIAS MOLIN</t>
   </si>
   <si>
     <t xml:space="preserve">0140569097 Transf. ANDREA CLEMENTINA ALARCON LARA</t>
   </si>
   <si>
-    <t xml:space="preserve">GUILLERMO TOBIAS MOLIN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Compra Nacional MD SOLMET SPA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">28-07-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0070082349 Transf a VALDES CORNEJO NIBA</t>
-  </si>
-  <si>
     <t xml:space="preserve">0783031345 Transf a Global Solutions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PAGO EN LINEA ESMAX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">29-07-2026</t>
   </si>
   <si>
     <t xml:space="preserve">CONTROL DE CUMPLIMIENTO — REAL vs. PRESUPUESTO Y FLUJO DE CAJA</t>
@@ -9904,7 +9949,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I180"/>
+  <dimension ref="A1:I185"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -10941,48 +10986,48 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="3" t="s">
-        <v>335</v>
+        <v>231</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>505</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>506</v>
+        <v>437</v>
       </c>
       <c r="D45" s="12" t="n">
-        <v>16347</v>
+        <v>63436</v>
       </c>
       <c r="E45" s="12" t="n">
-        <v>2798</v>
+        <v>12053</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>19145</v>
+        <v>75489</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>229</v>
+        <v>196</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>507</v>
+        <v>234</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="D46" s="12" t="n">
-        <v>37807</v>
+        <v>44266</v>
       </c>
       <c r="E46" s="12" t="n">
-        <v>7183</v>
+        <v>8411</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>44990</v>
+        <v>52677</v>
       </c>
       <c r="G46" s="3" t="s">
         <v>196</v>
@@ -10993,74 +11038,74 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
-        <v>235</v>
+        <v>335</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="C47" s="3" t="s">
+        <v>507</v>
+      </c>
+      <c r="D47" s="12" t="n">
+        <v>16347</v>
+      </c>
+      <c r="E47" s="12" t="n">
+        <v>2798</v>
+      </c>
+      <c r="F47" s="12" t="n">
+        <v>19145</v>
+      </c>
+      <c r="G47" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="H47" s="3" t="s">
         <v>509</v>
-      </c>
-      <c r="D47" s="12" t="n">
-        <v>18977</v>
-      </c>
-      <c r="E47" s="12" t="n">
-        <v>3606</v>
-      </c>
-      <c r="F47" s="12" t="n">
-        <v>22583</v>
-      </c>
-      <c r="G47" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="H47" s="3" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="B48" s="3" t="s">
+        <v>510</v>
+      </c>
+      <c r="C48" s="3" t="s">
         <v>511</v>
       </c>
-      <c r="C48" s="3" t="s">
-        <v>512</v>
-      </c>
       <c r="D48" s="12" t="n">
-        <v>811375</v>
+        <v>37807</v>
       </c>
       <c r="E48" s="12" t="n">
-        <v>154161</v>
+        <v>7183</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>1000000</v>
+        <v>44990</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>229</v>
+        <v>196</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>513</v>
+        <v>234</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3" t="s">
-        <v>514</v>
+        <v>235</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="D49" s="12" t="n">
-        <v>983773</v>
+        <v>18977</v>
       </c>
       <c r="E49" s="12" t="n">
-        <v>186918</v>
+        <v>3606</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>1170691</v>
+        <v>22583</v>
       </c>
       <c r="G49" s="3" t="s">
         <v>196</v>
@@ -11071,106 +11116,106 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
-        <v>516</v>
+        <v>226</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>517</v>
+        <v>513</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="D50" s="12" t="n">
-        <v>21008</v>
+        <v>811375</v>
       </c>
       <c r="E50" s="12" t="n">
-        <v>3992</v>
+        <v>154161</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>25000</v>
+        <v>1000000</v>
       </c>
       <c r="G50" s="3" t="s">
         <v>229</v>
       </c>
       <c r="H50" s="3" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
-        <v>255</v>
+        <v>516</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="D51" s="12" t="n">
-        <v>12605</v>
+        <v>983773</v>
       </c>
       <c r="E51" s="12" t="n">
-        <v>2395</v>
+        <v>186918</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>15000</v>
+        <v>1170691</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>229</v>
+        <v>196</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>520</v>
+        <v>234</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>226</v>
+        <v>518</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>522</v>
+        <v>514</v>
       </c>
       <c r="D52" s="12" t="n">
-        <v>121706</v>
+        <v>21008</v>
       </c>
       <c r="E52" s="12" t="n">
-        <v>23124</v>
+        <v>3992</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>150000</v>
+        <v>25000</v>
       </c>
       <c r="G52" s="3" t="s">
         <v>229</v>
       </c>
       <c r="H52" s="3" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
-        <v>226</v>
+        <v>255</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>522</v>
+        <v>514</v>
       </c>
       <c r="D53" s="12" t="n">
-        <v>129820</v>
+        <v>12605</v>
       </c>
       <c r="E53" s="12" t="n">
-        <v>24666</v>
+        <v>2395</v>
       </c>
       <c r="F53" s="12" t="n">
-        <v>160000</v>
+        <v>15000</v>
       </c>
       <c r="G53" s="3" t="s">
         <v>229</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11178,155 +11223,155 @@
         <v>226</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="D54" s="12" t="n">
-        <v>811375</v>
+        <v>121706</v>
       </c>
       <c r="E54" s="12" t="n">
-        <v>154161</v>
+        <v>23124</v>
       </c>
       <c r="F54" s="12" t="n">
-        <v>1000000</v>
+        <v>150000</v>
       </c>
       <c r="G54" s="3" t="s">
         <v>229</v>
       </c>
       <c r="H54" s="3" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>255</v>
+        <v>226</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>528</v>
+        <v>524</v>
       </c>
       <c r="D55" s="12" t="n">
-        <v>44769</v>
+        <v>129820</v>
       </c>
       <c r="E55" s="12" t="n">
-        <v>8507</v>
+        <v>24666</v>
       </c>
       <c r="F55" s="12" t="n">
-        <v>50000</v>
+        <v>160000</v>
       </c>
       <c r="G55" s="3" t="s">
         <v>229</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>529</v>
+        <v>525</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>308</v>
+        <v>226</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>531</v>
+        <v>524</v>
       </c>
       <c r="D56" s="12" t="n">
-        <v>16806</v>
+        <v>811375</v>
       </c>
       <c r="E56" s="12" t="n">
-        <v>3193</v>
+        <v>154161</v>
       </c>
       <c r="F56" s="12" t="n">
-        <v>19999</v>
+        <v>1000000</v>
       </c>
       <c r="G56" s="3" t="s">
         <v>229</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>532</v>
+        <v>528</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
-        <v>308</v>
+        <v>255</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>533</v>
+        <v>529</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="D57" s="12" t="n">
-        <v>16623</v>
+        <v>44769</v>
       </c>
       <c r="E57" s="12" t="n">
-        <v>3158</v>
+        <v>8507</v>
       </c>
       <c r="F57" s="12" t="n">
-        <v>19781</v>
+        <v>50000</v>
       </c>
       <c r="G57" s="3" t="s">
         <v>229</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>255</v>
+        <v>308</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D58" s="12" t="n">
-        <v>53759</v>
+        <v>16806</v>
       </c>
       <c r="E58" s="12" t="n">
-        <v>10215</v>
+        <v>3193</v>
       </c>
       <c r="F58" s="12" t="n">
-        <v>60000</v>
+        <v>19999</v>
       </c>
       <c r="G58" s="3" t="s">
         <v>229</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
-        <v>242</v>
+        <v>308</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D59" s="12" t="n">
-        <v>248771</v>
+        <v>16623</v>
       </c>
       <c r="E59" s="12" t="n">
-        <v>47266</v>
+        <v>3158</v>
       </c>
       <c r="F59" s="12" t="n">
-        <v>296037</v>
+        <v>19781</v>
       </c>
       <c r="G59" s="3" t="s">
         <v>229</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11334,97 +11379,97 @@
         <v>255</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D60" s="12" t="n">
-        <v>71678</v>
+        <v>53759</v>
       </c>
       <c r="E60" s="12" t="n">
-        <v>13620</v>
+        <v>10215</v>
       </c>
       <c r="F60" s="12" t="n">
-        <v>80000</v>
+        <v>60000</v>
       </c>
       <c r="G60" s="3" t="s">
         <v>229</v>
       </c>
       <c r="H60" s="3" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>538</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>533</v>
+      </c>
+      <c r="D61" s="12" t="n">
+        <v>248771</v>
+      </c>
+      <c r="E61" s="12" t="n">
+        <v>47266</v>
+      </c>
+      <c r="F61" s="12" t="n">
+        <v>296037</v>
+      </c>
+      <c r="G61" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="H61" s="3" t="s">
         <v>539</v>
-      </c>
-      <c r="B61" s="3" t="s">
-        <v>540</v>
-      </c>
-      <c r="C61" s="3" t="s">
-        <v>442</v>
-      </c>
-      <c r="D61" s="12" t="n">
-        <v>2479</v>
-      </c>
-      <c r="E61" s="12" t="n">
-        <v>471</v>
-      </c>
-      <c r="F61" s="12" t="n">
-        <v>2950</v>
-      </c>
-      <c r="G61" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="H61" s="3" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>308</v>
+        <v>255</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>451</v>
+        <v>533</v>
       </c>
       <c r="D62" s="12" t="n">
-        <v>18674</v>
+        <v>71678</v>
       </c>
       <c r="E62" s="12" t="n">
-        <v>3548</v>
+        <v>13620</v>
       </c>
       <c r="F62" s="12" t="n">
-        <v>22222</v>
+        <v>80000</v>
       </c>
       <c r="G62" s="3" t="s">
-        <v>196</v>
+        <v>229</v>
       </c>
       <c r="H62" s="3" t="s">
-        <v>234</v>
+        <v>537</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="3" t="s">
-        <v>231</v>
+        <v>541</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>262</v>
+        <v>542</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>497</v>
+        <v>442</v>
       </c>
       <c r="D63" s="12" t="n">
-        <v>20124</v>
+        <v>2479</v>
       </c>
       <c r="E63" s="12" t="n">
-        <v>3824</v>
+        <v>471</v>
       </c>
       <c r="F63" s="12" t="n">
-        <v>23948</v>
+        <v>2950</v>
       </c>
       <c r="G63" s="3" t="s">
         <v>196</v>
@@ -11434,259 +11479,349 @@
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="18" t="s">
-        <v>372</v>
-      </c>
-      <c r="F64" s="14" t="n">
-        <v>8677299</v>
-      </c>
-      <c r="G64" s="29" t="s">
-        <v>542</v>
+      <c r="A64" s="3" t="s">
+        <v>543</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="D64" s="12" t="n">
+        <v>19673</v>
+      </c>
+      <c r="E64" s="12" t="n">
+        <v>3738</v>
+      </c>
+      <c r="F64" s="12" t="n">
+        <v>23411</v>
+      </c>
+      <c r="G64" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="H64" s="3" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="3" t="s">
+        <v>546</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>547</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="D65" s="12" t="n">
+        <v>56200</v>
+      </c>
+      <c r="E65" s="12" t="n">
+        <v>10678</v>
+      </c>
+      <c r="F65" s="12" t="n">
+        <v>66878</v>
+      </c>
+      <c r="G65" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="H65" s="3" t="s">
+        <v>548</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="2" t="s">
-        <v>374</v>
-      </c>
-      <c r="B66" s="2"/>
-      <c r="C66" s="2"/>
-      <c r="D66" s="2"/>
-      <c r="E66" s="2"/>
-      <c r="F66" s="2"/>
-      <c r="G66" s="2"/>
-      <c r="H66" s="2"/>
-      <c r="I66" s="2"/>
+      <c r="A66" s="3" t="s">
+        <v>549</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>550</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="D66" s="12" t="n">
+        <v>5840</v>
+      </c>
+      <c r="E66" s="12" t="n">
+        <v>1110</v>
+      </c>
+      <c r="F66" s="12" t="n">
+        <v>6950</v>
+      </c>
+      <c r="G66" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="H66" s="3" t="s">
+        <v>551</v>
+      </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="9" t="s">
-        <v>375</v>
-      </c>
-      <c r="B67" s="9" t="s">
-        <v>376</v>
-      </c>
-      <c r="C67" s="9" t="s">
-        <v>377</v>
-      </c>
-      <c r="D67" s="9" t="s">
-        <v>378</v>
-      </c>
-      <c r="E67" s="9" t="s">
-        <v>379</v>
+      <c r="A67" s="3" t="s">
+        <v>552</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>553</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="D67" s="12" t="n">
+        <v>31933</v>
+      </c>
+      <c r="E67" s="12" t="n">
+        <v>6067</v>
+      </c>
+      <c r="F67" s="12" t="n">
+        <v>38000</v>
+      </c>
+      <c r="G67" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="H67" s="3" t="s">
+        <v>554</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>434</v>
+        <v>226</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>385</v>
-      </c>
-      <c r="C68" s="12" t="n">
-        <v>-27000</v>
-      </c>
-      <c r="D68" s="3" t="s">
-        <v>386</v>
-      </c>
-      <c r="E68" s="3" t="s">
-        <v>387</v>
+        <v>555</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>556</v>
+      </c>
+      <c r="D68" s="12" t="n">
+        <v>716101</v>
+      </c>
+      <c r="E68" s="12" t="n">
+        <v>136059</v>
+      </c>
+      <c r="F68" s="12" t="n">
+        <v>800000</v>
+      </c>
+      <c r="G68" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="H68" s="3" t="s">
+        <v>557</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="3" t="s">
-        <v>434</v>
+        <v>558</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>543</v>
-      </c>
-      <c r="C69" s="12" t="n">
-        <v>2326472</v>
-      </c>
-      <c r="D69" s="3" t="s">
-        <v>381</v>
-      </c>
-      <c r="E69" s="3" t="s">
-        <v>382</v>
+        <v>559</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>556</v>
+      </c>
+      <c r="D69" s="12" t="n">
+        <v>81513</v>
+      </c>
+      <c r="E69" s="12" t="n">
+        <v>15487</v>
+      </c>
+      <c r="F69" s="12" t="n">
+        <v>97000</v>
+      </c>
+      <c r="G69" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="H69" s="3" t="s">
+        <v>560</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
-        <v>434</v>
+        <v>255</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>544</v>
-      </c>
-      <c r="C70" s="12" t="n">
-        <v>-70000</v>
-      </c>
-      <c r="D70" s="3" t="s">
-        <v>386</v>
-      </c>
-      <c r="E70" s="3" t="s">
-        <v>387</v>
+        <v>561</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="D70" s="12" t="n">
+        <v>89616</v>
+      </c>
+      <c r="E70" s="12" t="n">
+        <v>17028</v>
+      </c>
+      <c r="F70" s="12" t="n">
+        <v>100020</v>
+      </c>
+      <c r="G70" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="H70" s="3" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="3" t="s">
-        <v>434</v>
+        <v>226</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>385</v>
-      </c>
-      <c r="C71" s="12" t="n">
-        <v>-6000</v>
-      </c>
-      <c r="D71" s="3" t="s">
-        <v>386</v>
-      </c>
-      <c r="E71" s="3" t="s">
-        <v>387</v>
+        <v>562</v>
+      </c>
+      <c r="C71" s="3" t="s">
+        <v>563</v>
+      </c>
+      <c r="D71" s="12" t="n">
+        <v>626588</v>
+      </c>
+      <c r="E71" s="12" t="n">
+        <v>119052</v>
+      </c>
+      <c r="F71" s="12" t="n">
+        <v>700000</v>
+      </c>
+      <c r="G71" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="H71" s="3" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>564</v>
+      </c>
+      <c r="C72" s="3" t="s">
         <v>451</v>
       </c>
-      <c r="B72" s="3" t="s">
-        <v>545</v>
-      </c>
-      <c r="C72" s="12" t="n">
-        <v>-2700</v>
-      </c>
-      <c r="D72" s="3" t="s">
-        <v>386</v>
-      </c>
-      <c r="E72" s="3" t="s">
-        <v>408</v>
+      <c r="D72" s="12" t="n">
+        <v>18674</v>
+      </c>
+      <c r="E72" s="12" t="n">
+        <v>3548</v>
+      </c>
+      <c r="F72" s="12" t="n">
+        <v>22222</v>
+      </c>
+      <c r="G72" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="H72" s="3" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="3" t="s">
-        <v>451</v>
+        <v>231</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>546</v>
-      </c>
-      <c r="C73" s="12" t="n">
-        <v>-190000</v>
-      </c>
-      <c r="D73" s="3" t="s">
-        <v>386</v>
-      </c>
-      <c r="E73" s="3" t="s">
-        <v>387</v>
+        <v>262</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>497</v>
+      </c>
+      <c r="D73" s="12" t="n">
+        <v>20124</v>
+      </c>
+      <c r="E73" s="12" t="n">
+        <v>3824</v>
+      </c>
+      <c r="F73" s="12" t="n">
+        <v>23948</v>
+      </c>
+      <c r="G73" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="H73" s="3" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="3" t="s">
-        <v>451</v>
-      </c>
-      <c r="B74" s="3" t="s">
-        <v>547</v>
-      </c>
-      <c r="C74" s="12" t="n">
-        <v>-54000</v>
-      </c>
-      <c r="D74" s="3" t="s">
-        <v>386</v>
-      </c>
-      <c r="E74" s="3" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="3" t="s">
-        <v>451</v>
-      </c>
-      <c r="B75" s="3" t="s">
-        <v>548</v>
-      </c>
-      <c r="C75" s="12" t="n">
-        <v>-225000</v>
-      </c>
-      <c r="D75" s="3" t="s">
-        <v>386</v>
-      </c>
-      <c r="E75" s="3" t="s">
-        <v>387</v>
+      <c r="A74" s="18" t="s">
+        <v>372</v>
+      </c>
+      <c r="F74" s="14" t="n">
+        <v>10637724</v>
+      </c>
+      <c r="G74" s="29" t="s">
+        <v>565</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="3" t="s">
-        <v>465</v>
-      </c>
-      <c r="B76" s="3" t="s">
-        <v>385</v>
-      </c>
-      <c r="C76" s="12" t="n">
-        <v>-17000</v>
-      </c>
-      <c r="D76" s="3" t="s">
-        <v>386</v>
-      </c>
-      <c r="E76" s="3" t="s">
-        <v>387</v>
-      </c>
+      <c r="A76" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="B76" s="2"/>
+      <c r="C76" s="2"/>
+      <c r="D76" s="2"/>
+      <c r="E76" s="2"/>
+      <c r="F76" s="2"/>
+      <c r="G76" s="2"/>
+      <c r="H76" s="2"/>
+      <c r="I76" s="2"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="3" t="s">
-        <v>465</v>
-      </c>
-      <c r="B77" s="3" t="s">
-        <v>549</v>
-      </c>
-      <c r="C77" s="12" t="n">
-        <v>83100</v>
-      </c>
-      <c r="D77" s="3" t="s">
-        <v>381</v>
-      </c>
-      <c r="E77" s="3" t="s">
-        <v>408</v>
+      <c r="A77" s="9" t="s">
+        <v>375</v>
+      </c>
+      <c r="B77" s="9" t="s">
+        <v>376</v>
+      </c>
+      <c r="C77" s="9" t="s">
+        <v>377</v>
+      </c>
+      <c r="D77" s="9" t="s">
+        <v>378</v>
+      </c>
+      <c r="E77" s="9" t="s">
+        <v>379</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="3" t="s">
-        <v>465</v>
+        <v>434</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>550</v>
+        <v>385</v>
       </c>
       <c r="C78" s="12" t="n">
-        <v>270000</v>
+        <v>-27000</v>
       </c>
       <c r="D78" s="3" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="E78" s="3" t="s">
-        <v>408</v>
+        <v>387</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="3" t="s">
-        <v>465</v>
+        <v>434</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>551</v>
+        <v>566</v>
       </c>
       <c r="C79" s="12" t="n">
-        <v>-280000</v>
+        <v>2326472</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="3" t="s">
-        <v>465</v>
+        <v>434</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>552</v>
+        <v>567</v>
       </c>
       <c r="C80" s="12" t="n">
-        <v>-15000</v>
+        <v>-70000</v>
       </c>
       <c r="D80" s="3" t="s">
         <v>386</v>
@@ -11697,16 +11832,16 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="3" t="s">
-        <v>465</v>
+        <v>434</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>553</v>
+        <v>385</v>
       </c>
       <c r="C81" s="12" t="n">
-        <v>1200000</v>
+        <v>-6000</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="E81" s="3" t="s">
         <v>387</v>
@@ -11714,30 +11849,30 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="3" t="s">
-        <v>469</v>
+        <v>451</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>544</v>
+        <v>568</v>
       </c>
       <c r="C82" s="12" t="n">
-        <v>-270000</v>
+        <v>-2700</v>
       </c>
       <c r="D82" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E82" s="3" t="s">
-        <v>387</v>
+        <v>408</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="3" t="s">
-        <v>469</v>
+        <v>451</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>548</v>
+        <v>569</v>
       </c>
       <c r="C83" s="12" t="n">
-        <v>-225000</v>
+        <v>-190000</v>
       </c>
       <c r="D83" s="3" t="s">
         <v>386</v>
@@ -11748,13 +11883,13 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="3" t="s">
-        <v>469</v>
+        <v>451</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>552</v>
+        <v>570</v>
       </c>
       <c r="C84" s="12" t="n">
-        <v>-150000</v>
+        <v>-54000</v>
       </c>
       <c r="D84" s="3" t="s">
         <v>386</v>
@@ -11765,13 +11900,13 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="3" t="s">
-        <v>469</v>
+        <v>451</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>554</v>
+        <v>571</v>
       </c>
       <c r="C85" s="12" t="n">
-        <v>-180000</v>
+        <v>-225000</v>
       </c>
       <c r="D85" s="3" t="s">
         <v>386</v>
@@ -11782,64 +11917,64 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="3" t="s">
-        <v>469</v>
+        <v>465</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>555</v>
+        <v>385</v>
       </c>
       <c r="C86" s="12" t="n">
-        <v>320000</v>
+        <v>-17000</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="E86" s="3" t="s">
-        <v>408</v>
+        <v>387</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="3" t="s">
-        <v>469</v>
+        <v>465</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>385</v>
+        <v>572</v>
       </c>
       <c r="C87" s="12" t="n">
-        <v>-250000</v>
+        <v>83100</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="E87" s="3" t="s">
-        <v>387</v>
+        <v>408</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="3" t="s">
-        <v>469</v>
+        <v>465</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>406</v>
+        <v>573</v>
       </c>
       <c r="C88" s="12" t="n">
-        <v>-100000</v>
+        <v>270000</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="E88" s="3" t="s">
-        <v>387</v>
+        <v>408</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="3" t="s">
-        <v>469</v>
+        <v>465</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>552</v>
+        <v>574</v>
       </c>
       <c r="C89" s="12" t="n">
-        <v>-12000</v>
+        <v>-280000</v>
       </c>
       <c r="D89" s="3" t="s">
         <v>386</v>
@@ -11850,13 +11985,13 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="3" t="s">
-        <v>469</v>
+        <v>465</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>552</v>
+        <v>575</v>
       </c>
       <c r="C90" s="12" t="n">
-        <v>-120000</v>
+        <v>-15000</v>
       </c>
       <c r="D90" s="3" t="s">
         <v>386</v>
@@ -11867,16 +12002,16 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="3" t="s">
-        <v>469</v>
+        <v>465</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>552</v>
+        <v>576</v>
       </c>
       <c r="C91" s="12" t="n">
-        <v>-100000</v>
+        <v>1200000</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="E91" s="3" t="s">
         <v>387</v>
@@ -11884,30 +12019,30 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="3" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>556</v>
+        <v>567</v>
       </c>
       <c r="C92" s="12" t="n">
-        <v>-4700</v>
+        <v>-270000</v>
       </c>
       <c r="D92" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E92" s="3" t="s">
-        <v>408</v>
+        <v>387</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="3" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>393</v>
+        <v>571</v>
       </c>
       <c r="C93" s="12" t="n">
-        <v>-17000</v>
+        <v>-225000</v>
       </c>
       <c r="D93" s="3" t="s">
         <v>386</v>
@@ -11918,13 +12053,13 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="3" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>552</v>
+        <v>575</v>
       </c>
       <c r="C94" s="12" t="n">
-        <v>-12000</v>
+        <v>-150000</v>
       </c>
       <c r="D94" s="3" t="s">
         <v>386</v>
@@ -11935,13 +12070,13 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="3" t="s">
-        <v>473</v>
+        <v>469</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>552</v>
+        <v>577</v>
       </c>
       <c r="C95" s="12" t="n">
-        <v>-8000</v>
+        <v>-180000</v>
       </c>
       <c r="D95" s="3" t="s">
         <v>386</v>
@@ -11952,16 +12087,16 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="3" t="s">
-        <v>473</v>
+        <v>469</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>557</v>
+        <v>578</v>
       </c>
       <c r="C96" s="12" t="n">
-        <v>-14880</v>
+        <v>320000</v>
       </c>
       <c r="D96" s="3" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="E96" s="3" t="s">
         <v>408</v>
@@ -11969,13 +12104,13 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="3" t="s">
-        <v>473</v>
+        <v>469</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>552</v>
+        <v>385</v>
       </c>
       <c r="C97" s="12" t="n">
-        <v>-32000</v>
+        <v>-250000</v>
       </c>
       <c r="D97" s="3" t="s">
         <v>386</v>
@@ -11986,47 +12121,47 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="3" t="s">
-        <v>483</v>
+        <v>469</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>558</v>
+        <v>406</v>
       </c>
       <c r="C98" s="12" t="n">
-        <v>-63065</v>
+        <v>-100000</v>
       </c>
       <c r="D98" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E98" s="3" t="s">
-        <v>408</v>
+        <v>387</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="3" t="s">
-        <v>483</v>
+        <v>469</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>559</v>
+        <v>575</v>
       </c>
       <c r="C99" s="12" t="n">
-        <v>-31955</v>
+        <v>-12000</v>
       </c>
       <c r="D99" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E99" s="3" t="s">
-        <v>408</v>
+        <v>387</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="3" t="s">
-        <v>490</v>
+        <v>469</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>552</v>
+        <v>575</v>
       </c>
       <c r="C100" s="12" t="n">
-        <v>-17000</v>
+        <v>-120000</v>
       </c>
       <c r="D100" s="3" t="s">
         <v>386</v>
@@ -12037,13 +12172,13 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="3" t="s">
-        <v>497</v>
+        <v>469</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>385</v>
+        <v>575</v>
       </c>
       <c r="C101" s="12" t="n">
-        <v>-200000</v>
+        <v>-100000</v>
       </c>
       <c r="D101" s="3" t="s">
         <v>386</v>
@@ -12054,13 +12189,13 @@
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="3" t="s">
-        <v>497</v>
+        <v>471</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>545</v>
+        <v>579</v>
       </c>
       <c r="C102" s="12" t="n">
-        <v>-21470</v>
+        <v>-4700</v>
       </c>
       <c r="D102" s="3" t="s">
         <v>386</v>
@@ -12071,16 +12206,16 @@
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="3" t="s">
-        <v>497</v>
+        <v>471</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>553</v>
+        <v>393</v>
       </c>
       <c r="C103" s="12" t="n">
-        <v>200000</v>
+        <v>-17000</v>
       </c>
       <c r="D103" s="3" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="E103" s="3" t="s">
         <v>387</v>
@@ -12088,30 +12223,30 @@
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="3" t="s">
-        <v>497</v>
+        <v>471</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>543</v>
+        <v>575</v>
       </c>
       <c r="C104" s="12" t="n">
-        <v>1650249</v>
+        <v>-12000</v>
       </c>
       <c r="D104" s="3" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="E104" s="3" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="3" t="s">
-        <v>497</v>
+        <v>473</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>552</v>
+        <v>575</v>
       </c>
       <c r="C105" s="12" t="n">
-        <v>-12000</v>
+        <v>-8000</v>
       </c>
       <c r="D105" s="3" t="s">
         <v>386</v>
@@ -12122,30 +12257,30 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="3" t="s">
-        <v>501</v>
+        <v>473</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>554</v>
+        <v>580</v>
       </c>
       <c r="C106" s="12" t="n">
-        <v>-15000</v>
+        <v>-14880</v>
       </c>
       <c r="D106" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E106" s="3" t="s">
-        <v>387</v>
+        <v>408</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="3" t="s">
-        <v>501</v>
+        <v>473</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>552</v>
+        <v>575</v>
       </c>
       <c r="C107" s="12" t="n">
-        <v>-16000</v>
+        <v>-32000</v>
       </c>
       <c r="D107" s="3" t="s">
         <v>386</v>
@@ -12156,47 +12291,47 @@
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="3" t="s">
-        <v>501</v>
+        <v>483</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>548</v>
+        <v>581</v>
       </c>
       <c r="C108" s="12" t="n">
-        <v>-225000</v>
+        <v>-63065</v>
       </c>
       <c r="D108" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E108" s="3" t="s">
-        <v>387</v>
+        <v>408</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="3" t="s">
-        <v>437</v>
+        <v>483</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>552</v>
+        <v>582</v>
       </c>
       <c r="C109" s="12" t="n">
-        <v>-6800</v>
+        <v>-31955</v>
       </c>
       <c r="D109" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E109" s="3" t="s">
-        <v>387</v>
+        <v>408</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="3" t="s">
-        <v>437</v>
+        <v>490</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>554</v>
+        <v>575</v>
       </c>
       <c r="C110" s="12" t="n">
-        <v>-30000</v>
+        <v>-17000</v>
       </c>
       <c r="D110" s="3" t="s">
         <v>386</v>
@@ -12207,30 +12342,30 @@
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="3" t="s">
-        <v>437</v>
+        <v>497</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>552</v>
+        <v>566</v>
       </c>
       <c r="C111" s="12" t="n">
-        <v>-6000</v>
+        <v>1650249</v>
       </c>
       <c r="D111" s="3" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="E111" s="3" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="3" t="s">
-        <v>437</v>
+        <v>497</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>554</v>
+        <v>575</v>
       </c>
       <c r="C112" s="12" t="n">
-        <v>-15000</v>
+        <v>-12000</v>
       </c>
       <c r="D112" s="3" t="s">
         <v>386</v>
@@ -12241,30 +12376,30 @@
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="3" t="s">
-        <v>437</v>
+        <v>497</v>
       </c>
       <c r="B113" s="3" t="s">
-        <v>552</v>
+        <v>568</v>
       </c>
       <c r="C113" s="12" t="n">
-        <v>-50000</v>
+        <v>-21470</v>
       </c>
       <c r="D113" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E113" s="3" t="s">
-        <v>387</v>
+        <v>408</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="3" t="s">
-        <v>506</v>
+        <v>497</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>554</v>
+        <v>385</v>
       </c>
       <c r="C114" s="12" t="n">
-        <v>-50000</v>
+        <v>-200000</v>
       </c>
       <c r="D114" s="3" t="s">
         <v>386</v>
@@ -12275,30 +12410,30 @@
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="3" t="s">
-        <v>506</v>
+        <v>497</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>560</v>
+        <v>576</v>
       </c>
       <c r="C115" s="12" t="n">
-        <v>2813595</v>
+        <v>200000</v>
       </c>
       <c r="D115" s="3" t="s">
         <v>381</v>
       </c>
       <c r="E115" s="3" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="3" t="s">
-        <v>512</v>
+        <v>501</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>385</v>
+        <v>575</v>
       </c>
       <c r="C116" s="12" t="n">
-        <v>-400000</v>
+        <v>-16000</v>
       </c>
       <c r="D116" s="3" t="s">
         <v>386</v>
@@ -12309,30 +12444,30 @@
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="3" t="s">
-        <v>512</v>
+        <v>501</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>561</v>
+        <v>571</v>
       </c>
       <c r="C117" s="12" t="n">
-        <v>760000</v>
+        <v>-225000</v>
       </c>
       <c r="D117" s="3" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="E117" s="3" t="s">
-        <v>408</v>
+        <v>387</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="3" t="s">
-        <v>512</v>
+        <v>501</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>552</v>
+        <v>577</v>
       </c>
       <c r="C118" s="12" t="n">
-        <v>-250000</v>
+        <v>-15000</v>
       </c>
       <c r="D118" s="3" t="s">
         <v>386</v>
@@ -12343,13 +12478,13 @@
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="3" t="s">
-        <v>512</v>
+        <v>437</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>393</v>
+        <v>575</v>
       </c>
       <c r="C119" s="12" t="n">
-        <v>-300000</v>
+        <v>-6800</v>
       </c>
       <c r="D119" s="3" t="s">
         <v>386</v>
@@ -12360,13 +12495,13 @@
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="3" t="s">
-        <v>512</v>
+        <v>437</v>
       </c>
       <c r="B120" s="3" t="s">
-        <v>544</v>
+        <v>577</v>
       </c>
       <c r="C120" s="12" t="n">
-        <v>-300000</v>
+        <v>-30000</v>
       </c>
       <c r="D120" s="3" t="s">
         <v>386</v>
@@ -12377,13 +12512,13 @@
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="3" t="s">
-        <v>512</v>
+        <v>437</v>
       </c>
       <c r="B121" s="3" t="s">
-        <v>406</v>
+        <v>575</v>
       </c>
       <c r="C121" s="12" t="n">
-        <v>-150000</v>
+        <v>-6000</v>
       </c>
       <c r="D121" s="3" t="s">
         <v>386</v>
@@ -12394,13 +12529,13 @@
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="3" t="s">
-        <v>512</v>
+        <v>437</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>562</v>
+        <v>577</v>
       </c>
       <c r="C122" s="12" t="n">
-        <v>-1000000</v>
+        <v>-15000</v>
       </c>
       <c r="D122" s="3" t="s">
         <v>386</v>
@@ -12411,13 +12546,13 @@
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="3" t="s">
-        <v>512</v>
+        <v>437</v>
       </c>
       <c r="B123" s="3" t="s">
-        <v>548</v>
+        <v>575</v>
       </c>
       <c r="C123" s="12" t="n">
-        <v>-55000</v>
+        <v>-50000</v>
       </c>
       <c r="D123" s="3" t="s">
         <v>386</v>
@@ -12428,13 +12563,13 @@
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="3" t="s">
-        <v>512</v>
+        <v>507</v>
       </c>
       <c r="B124" s="3" t="s">
-        <v>554</v>
+        <v>577</v>
       </c>
       <c r="C124" s="12" t="n">
-        <v>-70000</v>
+        <v>-50000</v>
       </c>
       <c r="D124" s="3" t="s">
         <v>386</v>
@@ -12445,30 +12580,30 @@
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="3" t="s">
-        <v>439</v>
+        <v>507</v>
       </c>
       <c r="B125" s="3" t="s">
-        <v>554</v>
+        <v>583</v>
       </c>
       <c r="C125" s="12" t="n">
-        <v>-17000</v>
+        <v>2813595</v>
       </c>
       <c r="D125" s="3" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="E125" s="3" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="3" t="s">
-        <v>439</v>
+        <v>514</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>393</v>
+        <v>385</v>
       </c>
       <c r="C126" s="12" t="n">
-        <v>-32000</v>
+        <v>-400000</v>
       </c>
       <c r="D126" s="3" t="s">
         <v>386</v>
@@ -12479,64 +12614,64 @@
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="3" t="s">
-        <v>439</v>
+        <v>514</v>
       </c>
       <c r="B127" s="3" t="s">
-        <v>563</v>
+        <v>575</v>
       </c>
       <c r="C127" s="12" t="n">
-        <v>-9471</v>
+        <v>-250000</v>
       </c>
       <c r="D127" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E127" s="3" t="s">
-        <v>408</v>
+        <v>387</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="3" t="s">
-        <v>522</v>
+        <v>514</v>
       </c>
       <c r="B128" s="3" t="s">
-        <v>564</v>
+        <v>571</v>
       </c>
       <c r="C128" s="12" t="n">
-        <v>-31319</v>
+        <v>-55000</v>
       </c>
       <c r="D128" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E128" s="3" t="s">
-        <v>408</v>
+        <v>387</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="3" t="s">
-        <v>522</v>
+        <v>514</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>543</v>
+        <v>584</v>
       </c>
       <c r="C129" s="12" t="n">
-        <v>198000</v>
+        <v>-1000000</v>
       </c>
       <c r="D129" s="3" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="E129" s="3" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="3" t="s">
-        <v>522</v>
+        <v>514</v>
       </c>
       <c r="B130" s="3" t="s">
-        <v>552</v>
+        <v>406</v>
       </c>
       <c r="C130" s="12" t="n">
-        <v>-12000</v>
+        <v>-150000</v>
       </c>
       <c r="D130" s="3" t="s">
         <v>386</v>
@@ -12547,47 +12682,47 @@
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="3" t="s">
-        <v>522</v>
+        <v>514</v>
       </c>
       <c r="B131" s="3" t="s">
-        <v>554</v>
+        <v>585</v>
       </c>
       <c r="C131" s="12" t="n">
-        <v>-12000</v>
+        <v>760000</v>
       </c>
       <c r="D131" s="3" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="E131" s="3" t="s">
-        <v>387</v>
+        <v>408</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="3" t="s">
-        <v>522</v>
+        <v>514</v>
       </c>
       <c r="B132" s="3" t="s">
-        <v>560</v>
+        <v>577</v>
       </c>
       <c r="C132" s="12" t="n">
-        <v>2234722</v>
+        <v>-70000</v>
       </c>
       <c r="D132" s="3" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="E132" s="3" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="3" t="s">
-        <v>528</v>
+        <v>514</v>
       </c>
       <c r="B133" s="3" t="s">
-        <v>548</v>
+        <v>393</v>
       </c>
       <c r="C133" s="12" t="n">
-        <v>-350000</v>
+        <v>-300000</v>
       </c>
       <c r="D133" s="3" t="s">
         <v>386</v>
@@ -12598,13 +12733,13 @@
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="3" t="s">
-        <v>528</v>
+        <v>514</v>
       </c>
       <c r="B134" s="3" t="s">
-        <v>552</v>
+        <v>567</v>
       </c>
       <c r="C134" s="12" t="n">
-        <v>-16000</v>
+        <v>-300000</v>
       </c>
       <c r="D134" s="3" t="s">
         <v>386</v>
@@ -12615,30 +12750,30 @@
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="3" t="s">
-        <v>528</v>
+        <v>439</v>
       </c>
       <c r="B135" s="3" t="s">
-        <v>565</v>
+        <v>577</v>
       </c>
       <c r="C135" s="12" t="n">
-        <v>-5770</v>
+        <v>-17000</v>
       </c>
       <c r="D135" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E135" s="3" t="s">
-        <v>395</v>
+        <v>387</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="3" t="s">
-        <v>528</v>
+        <v>439</v>
       </c>
       <c r="B136" s="3" t="s">
-        <v>554</v>
+        <v>393</v>
       </c>
       <c r="C136" s="12" t="n">
-        <v>-20000</v>
+        <v>-32000</v>
       </c>
       <c r="D136" s="3" t="s">
         <v>386</v>
@@ -12649,30 +12784,30 @@
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="3" t="s">
-        <v>528</v>
+        <v>439</v>
       </c>
       <c r="B137" s="3" t="s">
-        <v>566</v>
+        <v>586</v>
       </c>
       <c r="C137" s="12" t="n">
-        <v>-405600</v>
+        <v>-9471</v>
       </c>
       <c r="D137" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E137" s="3" t="s">
-        <v>395</v>
+        <v>408</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="3" t="s">
-        <v>528</v>
+        <v>524</v>
       </c>
       <c r="B138" s="3" t="s">
-        <v>393</v>
+        <v>577</v>
       </c>
       <c r="C138" s="12" t="n">
-        <v>-15000</v>
+        <v>-12000</v>
       </c>
       <c r="D138" s="3" t="s">
         <v>386</v>
@@ -12683,81 +12818,81 @@
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="3" t="s">
-        <v>531</v>
+        <v>524</v>
       </c>
       <c r="B139" s="3" t="s">
-        <v>554</v>
+        <v>583</v>
       </c>
       <c r="C139" s="12" t="n">
-        <v>-20000</v>
+        <v>2234722</v>
       </c>
       <c r="D139" s="3" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="E139" s="3" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="3" t="s">
-        <v>531</v>
+        <v>524</v>
       </c>
       <c r="B140" s="3" t="s">
-        <v>552</v>
+        <v>587</v>
       </c>
       <c r="C140" s="12" t="n">
-        <v>-20000</v>
+        <v>-31319</v>
       </c>
       <c r="D140" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E140" s="3" t="s">
-        <v>387</v>
+        <v>408</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="3" t="s">
-        <v>531</v>
+        <v>524</v>
       </c>
       <c r="B141" s="3" t="s">
-        <v>567</v>
+        <v>575</v>
       </c>
       <c r="C141" s="12" t="n">
-        <v>357000</v>
+        <v>-12000</v>
       </c>
       <c r="D141" s="3" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="E141" s="3" t="s">
-        <v>408</v>
+        <v>387</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="3" t="s">
-        <v>531</v>
+        <v>524</v>
       </c>
       <c r="B142" s="3" t="s">
-        <v>393</v>
+        <v>566</v>
       </c>
       <c r="C142" s="12" t="n">
-        <v>-29000</v>
+        <v>198000</v>
       </c>
       <c r="D142" s="3" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="E142" s="3" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="3" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B143" s="3" t="s">
-        <v>544</v>
+        <v>393</v>
       </c>
       <c r="C143" s="12" t="n">
-        <v>-20000</v>
+        <v>-15000</v>
       </c>
       <c r="D143" s="3" t="s">
         <v>386</v>
@@ -12768,47 +12903,47 @@
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="3" t="s">
-        <v>568</v>
+        <v>530</v>
       </c>
       <c r="B144" s="3" t="s">
-        <v>554</v>
+        <v>588</v>
       </c>
       <c r="C144" s="12" t="n">
-        <v>-12000</v>
+        <v>-405600</v>
       </c>
       <c r="D144" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E144" s="3" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="3" t="s">
-        <v>568</v>
+        <v>530</v>
       </c>
       <c r="B145" s="3" t="s">
-        <v>569</v>
+        <v>577</v>
       </c>
       <c r="C145" s="12" t="n">
-        <v>-58001</v>
+        <v>-20000</v>
       </c>
       <c r="D145" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E145" s="3" t="s">
-        <v>408</v>
+        <v>387</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="3" t="s">
-        <v>568</v>
+        <v>530</v>
       </c>
       <c r="B146" s="3" t="s">
-        <v>570</v>
+        <v>589</v>
       </c>
       <c r="C146" s="12" t="n">
-        <v>-6950</v>
+        <v>-5770</v>
       </c>
       <c r="D146" s="3" t="s">
         <v>386</v>
@@ -12819,13 +12954,13 @@
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="3" t="s">
-        <v>568</v>
+        <v>530</v>
       </c>
       <c r="B147" s="3" t="s">
-        <v>552</v>
+        <v>575</v>
       </c>
       <c r="C147" s="12" t="n">
-        <v>-15000</v>
+        <v>-16000</v>
       </c>
       <c r="D147" s="3" t="s">
         <v>386</v>
@@ -12836,67 +12971,67 @@
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="3" t="s">
-        <v>568</v>
+        <v>530</v>
       </c>
       <c r="B148" s="3" t="s">
         <v>571</v>
       </c>
       <c r="C148" s="12" t="n">
-        <v>-66878</v>
+        <v>-350000</v>
       </c>
       <c r="D148" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E148" s="3" t="s">
-        <v>395</v>
+        <v>387</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="3" t="s">
-        <v>568</v>
+        <v>533</v>
       </c>
       <c r="B149" s="3" t="s">
-        <v>572</v>
+        <v>393</v>
       </c>
       <c r="C149" s="12" t="n">
-        <v>490200</v>
+        <v>-29000</v>
       </c>
       <c r="D149" s="3" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="E149" s="3" t="s">
-        <v>408</v>
+        <v>387</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="3" t="s">
-        <v>568</v>
+        <v>533</v>
       </c>
       <c r="B150" s="3" t="s">
-        <v>573</v>
+        <v>567</v>
       </c>
       <c r="C150" s="12" t="n">
-        <v>-4200</v>
+        <v>-20000</v>
       </c>
       <c r="D150" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E150" s="3" t="s">
-        <v>408</v>
+        <v>387</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="3" t="s">
-        <v>568</v>
+        <v>533</v>
       </c>
       <c r="B151" s="3" t="s">
-        <v>573</v>
+        <v>590</v>
       </c>
       <c r="C151" s="12" t="n">
-        <v>-6700</v>
+        <v>357000</v>
       </c>
       <c r="D151" s="3" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="E151" s="3" t="s">
         <v>408</v>
@@ -12904,13 +13039,13 @@
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="3" t="s">
-        <v>568</v>
+        <v>533</v>
       </c>
       <c r="B152" s="3" t="s">
-        <v>548</v>
+        <v>577</v>
       </c>
       <c r="C152" s="12" t="n">
-        <v>-18000</v>
+        <v>-20000</v>
       </c>
       <c r="D152" s="3" t="s">
         <v>386</v>
@@ -12921,64 +13056,64 @@
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="3" t="s">
-        <v>568</v>
+        <v>533</v>
       </c>
       <c r="B153" s="3" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="C153" s="12" t="n">
-        <v>200000</v>
+        <v>-20000</v>
       </c>
       <c r="D153" s="3" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="E153" s="3" t="s">
-        <v>408</v>
+        <v>387</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="3" t="s">
-        <v>568</v>
+        <v>545</v>
       </c>
       <c r="B154" s="3" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="C154" s="12" t="n">
-        <v>-38000</v>
+        <v>-12000</v>
       </c>
       <c r="D154" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E154" s="3" t="s">
-        <v>395</v>
+        <v>387</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="3" t="s">
-        <v>568</v>
+        <v>545</v>
       </c>
       <c r="B155" s="3" t="s">
-        <v>553</v>
+        <v>591</v>
       </c>
       <c r="C155" s="12" t="n">
-        <v>1000000</v>
+        <v>-58001</v>
       </c>
       <c r="D155" s="3" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="E155" s="3" t="s">
-        <v>387</v>
+        <v>408</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="3" t="s">
-        <v>568</v>
+        <v>545</v>
       </c>
       <c r="B156" s="3" t="s">
-        <v>552</v>
+        <v>575</v>
       </c>
       <c r="C156" s="12" t="n">
-        <v>-70000</v>
+        <v>-15000</v>
       </c>
       <c r="D156" s="3" t="s">
         <v>386</v>
@@ -12989,67 +13124,67 @@
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="3" t="s">
-        <v>568</v>
+        <v>545</v>
       </c>
       <c r="B157" s="3" t="s">
-        <v>554</v>
+        <v>592</v>
       </c>
       <c r="C157" s="12" t="n">
-        <v>-120000</v>
+        <v>-4200</v>
       </c>
       <c r="D157" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E157" s="3" t="s">
-        <v>387</v>
+        <v>408</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="3" t="s">
-        <v>568</v>
+        <v>545</v>
       </c>
       <c r="B158" s="3" t="s">
-        <v>554</v>
+        <v>592</v>
       </c>
       <c r="C158" s="12" t="n">
-        <v>-3000</v>
+        <v>-6700</v>
       </c>
       <c r="D158" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E158" s="3" t="s">
-        <v>387</v>
+        <v>408</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="3" t="s">
-        <v>568</v>
+        <v>545</v>
       </c>
       <c r="B159" s="3" t="s">
-        <v>544</v>
+        <v>592</v>
       </c>
       <c r="C159" s="12" t="n">
-        <v>-25000</v>
+        <v>-16500</v>
       </c>
       <c r="D159" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E159" s="3" t="s">
-        <v>387</v>
+        <v>408</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="3" t="s">
-        <v>568</v>
+        <v>545</v>
       </c>
       <c r="B160" s="3" t="s">
-        <v>573</v>
+        <v>593</v>
       </c>
       <c r="C160" s="12" t="n">
-        <v>-16500</v>
+        <v>490200</v>
       </c>
       <c r="D160" s="3" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="E160" s="3" t="s">
         <v>408</v>
@@ -13057,16 +13192,16 @@
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="3" t="s">
-        <v>575</v>
+        <v>545</v>
       </c>
       <c r="B161" s="3" t="s">
-        <v>552</v>
+        <v>576</v>
       </c>
       <c r="C161" s="12" t="n">
-        <v>-15000</v>
+        <v>1000000</v>
       </c>
       <c r="D161" s="3" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="E161" s="3" t="s">
         <v>387</v>
@@ -13074,13 +13209,13 @@
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="B162" s="3" t="s">
         <v>575</v>
       </c>
-      <c r="B162" s="3" t="s">
-        <v>544</v>
-      </c>
       <c r="C162" s="12" t="n">
-        <v>-170000</v>
+        <v>-70000</v>
       </c>
       <c r="D162" s="3" t="s">
         <v>386</v>
@@ -13091,13 +13226,13 @@
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="3" t="s">
-        <v>575</v>
+        <v>545</v>
       </c>
       <c r="B163" s="3" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="C163" s="12" t="n">
-        <v>-97000</v>
+        <v>-120000</v>
       </c>
       <c r="D163" s="3" t="s">
         <v>386</v>
@@ -13108,13 +13243,13 @@
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="3" t="s">
-        <v>575</v>
+        <v>545</v>
       </c>
       <c r="B164" s="3" t="s">
-        <v>554</v>
+        <v>577</v>
       </c>
       <c r="C164" s="12" t="n">
-        <v>-20000</v>
+        <v>-3000</v>
       </c>
       <c r="D164" s="3" t="s">
         <v>386</v>
@@ -13125,13 +13260,13 @@
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="3" t="s">
-        <v>575</v>
+        <v>545</v>
       </c>
       <c r="B165" s="3" t="s">
-        <v>577</v>
+        <v>571</v>
       </c>
       <c r="C165" s="12" t="n">
-        <v>-100000</v>
+        <v>-18000</v>
       </c>
       <c r="D165" s="3" t="s">
         <v>386</v>
@@ -13142,47 +13277,47 @@
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="3" t="s">
-        <v>575</v>
+        <v>545</v>
       </c>
       <c r="B166" s="3" t="s">
-        <v>578</v>
+        <v>567</v>
       </c>
       <c r="C166" s="12" t="n">
-        <v>-800000</v>
+        <v>-25000</v>
       </c>
       <c r="D166" s="3" t="s">
         <v>386</v>
       </c>
       <c r="E166" s="3" t="s">
-        <v>77</v>
+        <v>387</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="3" t="s">
-        <v>579</v>
+        <v>545</v>
       </c>
       <c r="B167" s="3" t="s">
-        <v>554</v>
+        <v>593</v>
       </c>
       <c r="C167" s="12" t="n">
-        <v>-100000</v>
+        <v>200000</v>
       </c>
       <c r="D167" s="3" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="E167" s="3" t="s">
-        <v>387</v>
+        <v>408</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="3" t="s">
-        <v>579</v>
+        <v>556</v>
       </c>
       <c r="B168" s="3" t="s">
-        <v>554</v>
+        <v>594</v>
       </c>
       <c r="C168" s="12" t="n">
-        <v>-53000</v>
+        <v>-100000</v>
       </c>
       <c r="D168" s="3" t="s">
         <v>386</v>
@@ -13193,13 +13328,13 @@
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="3" t="s">
-        <v>579</v>
+        <v>556</v>
       </c>
       <c r="B169" s="3" t="s">
         <v>577</v>
       </c>
       <c r="C169" s="12" t="n">
-        <v>-50000</v>
+        <v>-20000</v>
       </c>
       <c r="D169" s="3" t="s">
         <v>386</v>
@@ -13208,102 +13343,187 @@
         <v>387</v>
       </c>
     </row>
+    <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A170" s="3" t="s">
+        <v>556</v>
+      </c>
+      <c r="B170" s="3" t="s">
+        <v>567</v>
+      </c>
+      <c r="C170" s="12" t="n">
+        <v>-170000</v>
+      </c>
+      <c r="D170" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="E170" s="3" t="s">
+        <v>387</v>
+      </c>
+    </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A171" s="2" t="s">
-        <v>420</v>
-      </c>
-      <c r="B171" s="2"/>
-      <c r="C171" s="2"/>
-      <c r="D171" s="2"/>
-      <c r="E171" s="2"/>
-      <c r="F171" s="2"/>
-      <c r="G171" s="2"/>
-      <c r="H171" s="2"/>
-      <c r="I171" s="2"/>
+      <c r="A171" s="3" t="s">
+        <v>556</v>
+      </c>
+      <c r="B171" s="3" t="s">
+        <v>575</v>
+      </c>
+      <c r="C171" s="12" t="n">
+        <v>-15000</v>
+      </c>
+      <c r="D171" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="E171" s="3" t="s">
+        <v>387</v>
+      </c>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A172" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="B172" s="9" t="s">
-        <v>377</v>
-      </c>
-      <c r="C172" s="30" t="s">
-        <v>421</v>
-      </c>
-      <c r="D172" s="30" t="s">
-        <v>422</v>
+      <c r="A172" s="3" t="s">
+        <v>563</v>
+      </c>
+      <c r="B172" s="3" t="s">
+        <v>577</v>
+      </c>
+      <c r="C172" s="12" t="n">
+        <v>-100000</v>
+      </c>
+      <c r="D172" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="E172" s="3" t="s">
+        <v>387</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="3" t="s">
-        <v>423</v>
-      </c>
-      <c r="B173" s="12" t="n">
-        <v>267206</v>
+        <v>563</v>
+      </c>
+      <c r="B173" s="3" t="s">
+        <v>577</v>
+      </c>
+      <c r="C173" s="12" t="n">
+        <v>-53000</v>
+      </c>
+      <c r="D173" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="E173" s="3" t="s">
+        <v>387</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="3" t="s">
+        <v>563</v>
+      </c>
+      <c r="B174" s="3" t="s">
+        <v>594</v>
+      </c>
+      <c r="C174" s="12" t="n">
+        <v>-50000</v>
+      </c>
+      <c r="D174" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="E174" s="3" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A176" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="B176" s="2"/>
+      <c r="C176" s="2"/>
+      <c r="D176" s="2"/>
+      <c r="E176" s="2"/>
+      <c r="F176" s="2"/>
+      <c r="G176" s="2"/>
+      <c r="H176" s="2"/>
+      <c r="I176" s="2"/>
+    </row>
+    <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A177" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="B177" s="9" t="s">
+        <v>377</v>
+      </c>
+      <c r="C177" s="30" t="s">
+        <v>421</v>
+      </c>
+      <c r="D177" s="30" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A178" s="3" t="s">
+        <v>423</v>
+      </c>
+      <c r="B178" s="12" t="n">
+        <v>267206</v>
+      </c>
+    </row>
+    <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A179" s="3" t="s">
         <v>424</v>
       </c>
-      <c r="B174" s="12" t="n">
+      <c r="B179" s="12" t="n">
         <v>14543638</v>
       </c>
-      <c r="C174" s="31" t="n">
+      <c r="C179" s="31" t="n">
         <f aca="false">F11</f>
         <v>6122312</v>
       </c>
-      <c r="D174" s="31" t="n">
-        <f aca="false">B174-C174</f>
+      <c r="D179" s="31" t="n">
+        <f aca="false">B179-C179</f>
         <v>8421326</v>
       </c>
     </row>
-    <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A175" s="3" t="s">
+    <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A180" s="3" t="s">
         <v>425</v>
       </c>
-      <c r="B175" s="12" t="n">
+      <c r="B180" s="12" t="n">
         <v>-14747473</v>
       </c>
     </row>
-    <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A176" s="18" t="s">
+    <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A181" s="18" t="s">
         <v>426</v>
       </c>
-      <c r="B176" s="14" t="n">
-        <f aca="false">SUM(B173:B175)</f>
+      <c r="B181" s="14" t="n">
+        <f aca="false">SUM(B178:B180)</f>
         <v>63371</v>
       </c>
     </row>
-    <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A177" s="18" t="s">
+    <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A182" s="18" t="s">
         <v>427</v>
       </c>
-      <c r="B177" s="14" t="n">
+      <c r="B182" s="14" t="n">
         <v>63371</v>
       </c>
     </row>
-    <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A178" s="18" t="s">
+    <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A183" s="18" t="s">
         <v>428</v>
       </c>
-      <c r="B178" s="14" t="n">
-        <f aca="false">B176-B177</f>
+      <c r="B183" s="14" t="n">
+        <f aca="false">B181-B182</f>
         <v>0</v>
       </c>
     </row>
-    <row r="180" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A180" s="10" t="s">
+    <row r="185" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A185" s="10" t="s">
         <v>429</v>
       </c>
-      <c r="B180" s="10"/>
-      <c r="C180" s="10"/>
-      <c r="D180" s="10"/>
-      <c r="E180" s="10"/>
-      <c r="F180" s="10"/>
-      <c r="G180" s="10"/>
-      <c r="H180" s="10"/>
+      <c r="B185" s="10"/>
+      <c r="C185" s="10"/>
+      <c r="D185" s="10"/>
+      <c r="E185" s="10"/>
+      <c r="F185" s="10"/>
+      <c r="G185" s="10"/>
+      <c r="H185" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -13311,9 +13531,9 @@
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A4:I4"/>
     <mergeCell ref="A13:I13"/>
-    <mergeCell ref="A66:I66"/>
-    <mergeCell ref="A171:I171"/>
-    <mergeCell ref="A180:H180"/>
+    <mergeCell ref="A76:I76"/>
+    <mergeCell ref="A176:I176"/>
+    <mergeCell ref="A185:H185"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -13340,7 +13560,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>580</v>
+        <v>595</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -13355,7 +13575,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="28" t="s">
-        <v>581</v>
+        <v>596</v>
       </c>
       <c r="B2" s="28"/>
       <c r="C2" s="28"/>
@@ -13370,7 +13590,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>582</v>
+        <v>597</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -13388,34 +13608,34 @@
         <v>153</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>583</v>
+        <v>598</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>584</v>
+        <v>599</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>585</v>
+        <v>600</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>586</v>
+        <v>601</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>587</v>
+        <v>602</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>588</v>
+        <v>603</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>589</v>
+        <v>604</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>590</v>
+        <v>605</v>
       </c>
       <c r="J5" s="9" t="s">
-        <v>591</v>
+        <v>606</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>592</v>
+        <v>607</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13642,7 +13862,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>593</v>
+        <v>608</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -13660,34 +13880,34 @@
         <v>153</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>583</v>
+        <v>598</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>584</v>
+        <v>599</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>585</v>
+        <v>600</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>586</v>
+        <v>601</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>587</v>
+        <v>602</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>588</v>
+        <v>603</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>589</v>
+        <v>604</v>
       </c>
       <c r="I14" s="9" t="s">
-        <v>590</v>
+        <v>605</v>
       </c>
       <c r="J14" s="9" t="s">
-        <v>591</v>
+        <v>606</v>
       </c>
       <c r="K14" s="9" t="s">
-        <v>592</v>
+        <v>607</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13906,7 +14126,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>594</v>
+        <v>609</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -13917,7 +14137,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>595</v>
+        <v>610</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -13927,10 +14147,10 @@
         <v>65</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>596</v>
+        <v>611</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>597</v>
+        <v>612</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13948,7 +14168,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>598</v>
+        <v>613</v>
       </c>
       <c r="B6" s="12" t="n">
         <f aca="false">Consolidado!B6</f>
@@ -13987,7 +14207,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>599</v>
+        <v>614</v>
       </c>
       <c r="B9" s="17" t="n">
         <f aca="false">Consolidado!B10</f>
@@ -14078,7 +14298,7 @@
     </row>
     <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>600</v>
+        <v>615</v>
       </c>
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
@@ -14089,7 +14309,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>601</v>
+        <v>616</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -14100,7 +14320,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="28" t="s">
-        <v>602</v>
+        <v>617</v>
       </c>
       <c r="B21" s="28"/>
       <c r="C21" s="28"/>
@@ -14111,7 +14331,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>603</v>
+        <v>618</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -14125,27 +14345,27 @@
         <v>65</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>604</v>
+        <v>619</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>605</v>
+        <v>620</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>606</v>
+        <v>621</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>607</v>
+        <v>622</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>608</v>
+        <v>623</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>609</v>
+        <v>624</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>610</v>
+        <v>625</v>
       </c>
       <c r="B24" s="33" t="n">
         <f aca="false">Consolidado!B32</f>
@@ -14174,7 +14394,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>611</v>
+        <v>626</v>
       </c>
       <c r="B25" s="33" t="n">
         <f aca="false">Consolidado!C32</f>
@@ -14203,7 +14423,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="18" t="s">
-        <v>612</v>
+        <v>627</v>
       </c>
       <c r="B26" s="14" t="n">
         <f aca="false">B24-B25</f>
@@ -14226,7 +14446,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>613</v>
+        <v>628</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -14240,27 +14460,27 @@
         <v>65</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>604</v>
+        <v>619</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>605</v>
+        <v>620</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>606</v>
+        <v>621</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>607</v>
+        <v>622</v>
       </c>
       <c r="F29" s="9" t="s">
-        <v>608</v>
+        <v>623</v>
       </c>
       <c r="G29" s="9" t="s">
-        <v>609</v>
+        <v>624</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>610</v>
+        <v>625</v>
       </c>
       <c r="B30" s="33" t="n">
         <f aca="false">Consolidado!B41</f>
@@ -14289,7 +14509,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>611</v>
+        <v>626</v>
       </c>
       <c r="B31" s="33" t="n">
         <f aca="false">Consolidado!C41</f>
@@ -14318,7 +14538,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="18" t="s">
-        <v>612</v>
+        <v>627</v>
       </c>
       <c r="B32" s="14" t="n">
         <f aca="false">B30-B31</f>
@@ -14374,7 +14594,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>614</v>
+        <v>629</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -14384,7 +14604,7 @@
     </row>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="24" t="s">
-        <v>615</v>
+        <v>630</v>
       </c>
       <c r="B2" s="24"/>
       <c r="C2" s="24"/>
@@ -14397,16 +14617,16 @@
         <v>375</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>616</v>
+        <v>631</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>617</v>
+        <v>632</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>618</v>
+        <v>633</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>619</v>
+        <v>634</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>187</v>
@@ -14414,18 +14634,18 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>579</v>
+        <v>563</v>
       </c>
       <c r="B5" s="12" t="n">
         <v>63371</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>620</v>
+        <v>635</v>
       </c>
       <c r="D5" s="37"/>
       <c r="E5" s="37"/>
       <c r="F5" s="3" t="s">
-        <v>621</v>
+        <v>636</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Agrega saldo 01-08, Aramco completo julio, Copec resumen; actualiza Bitacora
</commit_message>
<xml_diff>
--- a/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
+++ b/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2018" uniqueCount="643">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2021" uniqueCount="646">
   <si>
     <t xml:space="preserve">SUPUESTOS DEL PRESUPUESTO — SOLLEM + TRAST</t>
   </si>
@@ -1977,6 +1977,15 @@
   </si>
   <si>
     <t xml:space="preserve">Saldo real del 29-07-2026, cartola completa conciliada. Punto de partida de la bitácora.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01-08-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agosto S0 (01-02 ago)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saldo real 01-08-2026, 18:21hrs. Primer dato ya dentro de agosto — falta cargar el Saldo Acumulado Proyectado de la semana S0 en Consolidado (columna D) para activar la comparación.</t>
   </si>
 </sst>
 </file>
@@ -14864,7 +14873,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -14929,15 +14938,23 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="38"/>
-      <c r="B6" s="34"/>
-      <c r="C6" s="38"/>
+      <c r="A6" s="3" t="s">
+        <v>643</v>
+      </c>
+      <c r="B6" s="12" t="n">
+        <v>1275801</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>644</v>
+      </c>
       <c r="D6" s="34"/>
       <c r="E6" s="12" t="str">
-        <f aca="false">IF(OR(B6="",D6=""),"",B6-D6)</f>
+        <f aca="false">IF(D6="","",B6-D6)</f>
         <v/>
       </c>
-      <c r="F6" s="38"/>
+      <c r="F6" s="3" t="s">
+        <v>645</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="38"/>
@@ -15202,6 +15219,17 @@
         <v/>
       </c>
       <c r="F30" s="38"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="38"/>
+      <c r="B31" s="34"/>
+      <c r="C31" s="38"/>
+      <c r="D31" s="34"/>
+      <c r="E31" s="12" t="str">
+        <f aca="false">IF(OR(B31="",D31=""),"",B31-D31)</f>
+        <v/>
+      </c>
+      <c r="F31" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
CIERRE JULIO 2026: cartola definitiva completa, cuadre exacto
</commit_message>
<xml_diff>
--- a/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
+++ b/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2076" uniqueCount="669">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2096" uniqueCount="669">
   <si>
     <t xml:space="preserve">SUPUESTOS DEL PRESUPUESTO — SOLLEM + TRAST</t>
   </si>
@@ -1327,10 +1327,10 @@
     <t xml:space="preserve">Nota: comparación agregada entre Abonos reales de la cartola y total facturado en Ventas RCV del mismo mes.</t>
   </si>
   <si>
-    <t xml:space="preserve">CONCILIACIÓN BANCARIA — JULIO 2026 (Global Solutions SPA, cartola provisoria N°3 al 30-07-2026)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuente: Cartola provisoria (30/06 al 30/07/2026, 140 movimientos) + RCV Compra/Venta SII período 202607. Mes prácticamente cerrado (falta 1 día hábil), repetir con la cartola de cierre definitivo.</t>
+    <t xml:space="preserve">CONCILIACIÓN BANCARIA — JULIO 2026 CERRADO (Global Solutions SPA, cartola histórica N°3 definitiva)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuente: Cartola histórica definitiva (30/06 al 31/07/2026, mes cerrado completo) + RCV Compra/Venta SII período 202607.</t>
   </si>
   <si>
     <t xml:space="preserve">LOGÍSTICA Y TRANSPORTES ALFA JAM SPA</t>
@@ -1423,7 +1423,7 @@
     <t xml:space="preserve">299681</t>
   </si>
   <si>
-    <t xml:space="preserve">Cargo cartola 03-07-2026 — COMERCIAL RIHE LTDA</t>
+    <t xml:space="preserve">Cargo cartola 03-07-2026 — Compra Nacional MD COMERCIAL RIHE</t>
   </si>
   <si>
     <t xml:space="preserve">299686</t>
@@ -1438,7 +1438,7 @@
     <t xml:space="preserve">6711841</t>
   </si>
   <si>
-    <t xml:space="preserve">Cargo cartola 03-07-2026 — IMPLEMENTOS S.A.</t>
+    <t xml:space="preserve">Cargo cartola 03-07-2026 — Compra Nacional MD IMPLEMENTOS S.A</t>
   </si>
   <si>
     <t xml:space="preserve">99581430-7</t>
@@ -1480,7 +1480,7 @@
     <t xml:space="preserve">08-07-2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Cargo cartola 09-07-2026 — COMERCIAL ECUADOR SPA</t>
+    <t xml:space="preserve">Cargo cartola 09-07-2026 — Compra Nacional MD COMERCIAL ECUAD</t>
   </si>
   <si>
     <t xml:space="preserve">300297</t>
@@ -1501,7 +1501,7 @@
     <t xml:space="preserve">350990</t>
   </si>
   <si>
-    <t xml:space="preserve">Cargo cartola 09-07-2026 — TTP S.A RANCAGUA</t>
+    <t xml:space="preserve">Cargo cartola 09-07-2026 — Compra Nacional MD TTP S.A RANCAGU</t>
   </si>
   <si>
     <t xml:space="preserve">6729429</t>
@@ -1603,7 +1603,7 @@
     <t xml:space="preserve">20-07-2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Cargo cartola 20-07-2026 — 0967985503 Transf a Multiaceros SA</t>
+    <t xml:space="preserve">Cargo cartola 20-07-2026 — PAGO EN LINEA ESMAX</t>
   </si>
   <si>
     <t xml:space="preserve">96798550-3</t>
@@ -1618,7 +1618,7 @@
     <t xml:space="preserve">678717</t>
   </si>
   <si>
-    <t xml:space="preserve">Cargo cartola 20-07-2026 — TRANSAGRO RANCAGUA</t>
+    <t xml:space="preserve">Cargo cartola 20-07-2026 — Compra Nacional MD TRANSAGRO RANCA</t>
   </si>
   <si>
     <t xml:space="preserve">32186742</t>
@@ -1675,7 +1675,7 @@
     <t xml:space="preserve">24-07-2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Cargo cartola 24-07-2026 — COMERCIAL RIHE LTDA</t>
+    <t xml:space="preserve">Cargo cartola 24-07-2026 — Compra Nacional MD COMERCIAL RIHE</t>
   </si>
   <si>
     <t xml:space="preserve">301680</t>
@@ -1690,7 +1690,7 @@
     <t xml:space="preserve">22908735</t>
   </si>
   <si>
-    <t xml:space="preserve">Cargo cartola 27-07-2026 — CONSTRU-MART RANCAGUA</t>
+    <t xml:space="preserve">Cargo cartola 27-07-2026 — Compra Nacional MD CONSTRU-MART RA</t>
   </si>
   <si>
     <t xml:space="preserve">119346</t>
@@ -1744,7 +1744,7 @@
     <t xml:space="preserve">6299</t>
   </si>
   <si>
-    <t xml:space="preserve">Cargo cartola 27-07-2026 — MERCADOPAGO *ELECTROS</t>
+    <t xml:space="preserve">Cargo cartola 27-07-2026 — Compra Nacional MD MERCADOPAGO *EL</t>
   </si>
   <si>
     <t xml:space="preserve">2755582</t>
@@ -1780,7 +1780,7 @@
     <t xml:space="preserve">302126</t>
   </si>
   <si>
-    <t xml:space="preserve">Cargo cartola 29-07-2026 — COMERCIAL RIHE LTDA</t>
+    <t xml:space="preserve">Cargo cartola 29-07-2026 — Compra Nacional MD COMERCIAL RIHE</t>
   </si>
   <si>
     <t xml:space="preserve">6767525</t>
@@ -1789,7 +1789,7 @@
     <t xml:space="preserve">9363</t>
   </si>
   <si>
-    <t xml:space="preserve">Cargo cartola 27-07-2026 — GUILLERMO TOBIAS MOLIN</t>
+    <t xml:space="preserve">Cargo cartola 27-07-2026 — Compra Nacional MD GUILLERMO TOBIA</t>
   </si>
   <si>
     <t xml:space="preserve">9364</t>
@@ -1819,6 +1819,9 @@
     <t xml:space="preserve">103907</t>
   </si>
   <si>
+    <t xml:space="preserve">Cargo cartola 31-07-2026 — Compra Nacional MD CARDANICA PACIF</t>
+  </si>
+  <si>
     <t xml:space="preserve">76288622-7</t>
   </si>
   <si>
@@ -1828,6 +1831,9 @@
     <t xml:space="preserve">302316</t>
   </si>
   <si>
+    <t xml:space="preserve">Cargo cartola 31-07-2026 — Compra Nacional MD COMERCIAL RIHE</t>
+  </si>
+  <si>
     <t xml:space="preserve">32558596</t>
   </si>
   <si>
@@ -1852,7 +1858,7 @@
     <t xml:space="preserve">20435</t>
   </si>
   <si>
-    <t xml:space="preserve">Identificado: 44 de 79 ($8,960,511)</t>
+    <t xml:space="preserve">Identificado: 46 de 79 ($9,078,883)</t>
   </si>
   <si>
     <t xml:space="preserve">0175020268 Transf a Nicolás Carval</t>
@@ -1861,37 +1867,31 @@
     <t xml:space="preserve">0119944848 Transf a José Acevedo</t>
   </si>
   <si>
-    <t xml:space="preserve">TUU*COMERCIAL ESCORPIO</t>
-  </si>
-  <si>
     <t xml:space="preserve">0197068833 Transf a Felipe Tapia D</t>
   </si>
   <si>
     <t xml:space="preserve">019591141K Transf. Nicolas Matias</t>
   </si>
   <si>
-    <t xml:space="preserve">TUU*comercialEscorpion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">40574-SBX ROSARIO 100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COMERCIAL RIHE LTDA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EL PALACIO DEL POROTO</t>
+    <t xml:space="preserve">Compra Nacional MD 40574-SBX ROSAR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compra Nacional MD COMERCIAL RIHE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compra Nacional MD EL PALACIO DEL</t>
   </si>
   <si>
     <t xml:space="preserve">0761971018 Transf. Financia Capita</t>
   </si>
   <si>
-    <t xml:space="preserve">PAGO EN LINEA ESMAX</t>
+    <t xml:space="preserve">0967985503 Transf a Multiaceros SA</t>
   </si>
   <si>
     <t xml:space="preserve">PAGO EN LINEA S.I.I.</t>
   </si>
   <si>
-    <t xml:space="preserve">RedGloba*PCY LTDA</t>
+    <t xml:space="preserve">Compra Nacional MD RedGloba*PCY LT</t>
   </si>
   <si>
     <t xml:space="preserve">Compra Nacional MD PROSERCOM SPA</t>
@@ -1903,7 +1903,7 @@
     <t xml:space="preserve">0140569097 Transf. ANDREA CLEMENTI</t>
   </si>
   <si>
-    <t xml:space="preserve">GUILLERMO TOBIAS MOLIN</t>
+    <t xml:space="preserve">Compra Nacional MD GUILLERMO TOBIA</t>
   </si>
   <si>
     <t xml:space="preserve">CONTROL DE CUMPLIMIENTO — REAL vs. PRESUPUESTO Y FLUJO DE CAJA</t>
@@ -10048,7 +10048,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I206"/>
+  <dimension ref="A1:I211"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -12221,18 +12221,18 @@
         <v>46550</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>197</v>
+        <v>230</v>
       </c>
       <c r="H88" s="3" t="s">
-        <v>235</v>
+        <v>595</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="3" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="C89" s="3" t="s">
         <v>448</v>
@@ -12258,7 +12258,7 @@
         <v>309</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="C90" s="3" t="s">
         <v>448</v>
@@ -12273,10 +12273,10 @@
         <v>71822</v>
       </c>
       <c r="G90" s="3" t="s">
-        <v>197</v>
+        <v>230</v>
       </c>
       <c r="H90" s="3" t="s">
-        <v>235</v>
+        <v>599</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12284,7 +12284,7 @@
         <v>256</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="C91" s="3" t="s">
         <v>448</v>
@@ -12302,7 +12302,7 @@
         <v>230</v>
       </c>
       <c r="H91" s="3" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12310,7 +12310,7 @@
         <v>362</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="C92" s="3" t="s">
         <v>450</v>
@@ -12336,7 +12336,7 @@
         <v>227</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="C93" s="3" t="s">
         <v>450</v>
@@ -12359,10 +12359,10 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="3" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="C94" s="3" t="s">
         <v>450</v>
@@ -12380,7 +12380,7 @@
         <v>230</v>
       </c>
       <c r="H94" s="3" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12388,7 +12388,7 @@
         <v>309</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="C95" s="3" t="s">
         <v>459</v>
@@ -12443,7 +12443,7 @@
         <v>13552571</v>
       </c>
       <c r="G97" s="29" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12481,16 +12481,16 @@
         <v>435</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="C101" s="12" t="n">
-        <v>-27000</v>
+        <v>2326472</v>
       </c>
       <c r="D101" s="3" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="E101" s="3" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12518,7 +12518,7 @@
         <v>386</v>
       </c>
       <c r="C103" s="12" t="n">
-        <v>-6000</v>
+        <v>-27000</v>
       </c>
       <c r="D103" s="3" t="s">
         <v>387</v>
@@ -12532,16 +12532,16 @@
         <v>435</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="C104" s="12" t="n">
-        <v>2326472</v>
+        <v>-6000</v>
       </c>
       <c r="D104" s="3" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="E104" s="3" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12549,10 +12549,10 @@
         <v>459</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>607</v>
+        <v>406</v>
       </c>
       <c r="C105" s="12" t="n">
-        <v>-190000</v>
+        <v>-225000</v>
       </c>
       <c r="D105" s="3" t="s">
         <v>387</v>
@@ -12566,10 +12566,10 @@
         <v>459</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="C106" s="12" t="n">
-        <v>-54000</v>
+        <v>-190000</v>
       </c>
       <c r="D106" s="3" t="s">
         <v>387</v>
@@ -12583,10 +12583,10 @@
         <v>459</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>406</v>
+        <v>610</v>
       </c>
       <c r="C107" s="12" t="n">
-        <v>-225000</v>
+        <v>-54000</v>
       </c>
       <c r="D107" s="3" t="s">
         <v>387</v>
@@ -12600,7 +12600,7 @@
         <v>459</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>609</v>
+        <v>405</v>
       </c>
       <c r="C108" s="12" t="n">
         <v>-2700</v>
@@ -12609,7 +12609,7 @@
         <v>387</v>
       </c>
       <c r="E108" s="3" t="s">
-        <v>409</v>
+        <v>396</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12617,13 +12617,13 @@
         <v>473</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>410</v>
+        <v>393</v>
       </c>
       <c r="C109" s="12" t="n">
-        <v>1200000</v>
+        <v>-15000</v>
       </c>
       <c r="D109" s="3" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="E109" s="3" t="s">
         <v>388</v>
@@ -12634,7 +12634,7 @@
         <v>473</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="C110" s="12" t="n">
         <v>-280000</v>
@@ -12651,10 +12651,10 @@
         <v>473</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>393</v>
+        <v>386</v>
       </c>
       <c r="C111" s="12" t="n">
-        <v>-15000</v>
+        <v>-17000</v>
       </c>
       <c r="D111" s="3" t="s">
         <v>387</v>
@@ -12668,10 +12668,10 @@
         <v>473</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>420</v>
+        <v>408</v>
       </c>
       <c r="C112" s="12" t="n">
-        <v>83100</v>
+        <v>270000</v>
       </c>
       <c r="D112" s="3" t="s">
         <v>382</v>
@@ -12685,13 +12685,13 @@
         <v>473</v>
       </c>
       <c r="B113" s="3" t="s">
-        <v>386</v>
+        <v>410</v>
       </c>
       <c r="C113" s="12" t="n">
-        <v>-17000</v>
+        <v>1200000</v>
       </c>
       <c r="D113" s="3" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="E113" s="3" t="s">
         <v>388</v>
@@ -12702,10 +12702,10 @@
         <v>473</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>408</v>
+        <v>420</v>
       </c>
       <c r="C114" s="12" t="n">
-        <v>270000</v>
+        <v>83100</v>
       </c>
       <c r="D114" s="3" t="s">
         <v>382</v>
@@ -12736,16 +12736,16 @@
         <v>477</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>393</v>
+        <v>612</v>
       </c>
       <c r="C116" s="12" t="n">
-        <v>-100000</v>
+        <v>320000</v>
       </c>
       <c r="D116" s="3" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="E116" s="3" t="s">
-        <v>388</v>
+        <v>409</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12753,16 +12753,16 @@
         <v>477</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>611</v>
+        <v>390</v>
       </c>
       <c r="C117" s="12" t="n">
-        <v>320000</v>
+        <v>-270000</v>
       </c>
       <c r="D117" s="3" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="E117" s="3" t="s">
-        <v>409</v>
+        <v>388</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12770,10 +12770,10 @@
         <v>477</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>407</v>
+        <v>386</v>
       </c>
       <c r="C118" s="12" t="n">
-        <v>-100000</v>
+        <v>-250000</v>
       </c>
       <c r="D118" s="3" t="s">
         <v>387</v>
@@ -12787,10 +12787,10 @@
         <v>477</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>386</v>
+        <v>406</v>
       </c>
       <c r="C119" s="12" t="n">
-        <v>-250000</v>
+        <v>-225000</v>
       </c>
       <c r="D119" s="3" t="s">
         <v>387</v>
@@ -12804,10 +12804,10 @@
         <v>477</v>
       </c>
       <c r="B120" s="3" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="C120" s="12" t="n">
-        <v>-120000</v>
+        <v>-180000</v>
       </c>
       <c r="D120" s="3" t="s">
         <v>387</v>
@@ -12821,10 +12821,10 @@
         <v>477</v>
       </c>
       <c r="B121" s="3" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="C121" s="12" t="n">
-        <v>-180000</v>
+        <v>-150000</v>
       </c>
       <c r="D121" s="3" t="s">
         <v>387</v>
@@ -12841,7 +12841,7 @@
         <v>393</v>
       </c>
       <c r="C122" s="12" t="n">
-        <v>-150000</v>
+        <v>-120000</v>
       </c>
       <c r="D122" s="3" t="s">
         <v>387</v>
@@ -12855,10 +12855,10 @@
         <v>477</v>
       </c>
       <c r="B123" s="3" t="s">
-        <v>406</v>
+        <v>393</v>
       </c>
       <c r="C123" s="12" t="n">
-        <v>-225000</v>
+        <v>-100000</v>
       </c>
       <c r="D123" s="3" t="s">
         <v>387</v>
@@ -12872,10 +12872,10 @@
         <v>477</v>
       </c>
       <c r="B124" s="3" t="s">
-        <v>390</v>
+        <v>407</v>
       </c>
       <c r="C124" s="12" t="n">
-        <v>-270000</v>
+        <v>-100000</v>
       </c>
       <c r="D124" s="3" t="s">
         <v>387</v>
@@ -12889,7 +12889,7 @@
         <v>479</v>
       </c>
       <c r="B125" s="3" t="s">
-        <v>612</v>
+        <v>395</v>
       </c>
       <c r="C125" s="12" t="n">
         <v>-4700</v>
@@ -12898,7 +12898,7 @@
         <v>387</v>
       </c>
       <c r="E125" s="3" t="s">
-        <v>409</v>
+        <v>396</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12943,7 +12943,7 @@
         <v>393</v>
       </c>
       <c r="C128" s="12" t="n">
-        <v>-8000</v>
+        <v>-32000</v>
       </c>
       <c r="D128" s="3" t="s">
         <v>387</v>
@@ -12966,7 +12966,7 @@
         <v>387</v>
       </c>
       <c r="E129" s="3" t="s">
-        <v>409</v>
+        <v>396</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12977,7 +12977,7 @@
         <v>393</v>
       </c>
       <c r="C130" s="12" t="n">
-        <v>-32000</v>
+        <v>-8000</v>
       </c>
       <c r="D130" s="3" t="s">
         <v>387</v>
@@ -13000,7 +13000,7 @@
         <v>387</v>
       </c>
       <c r="E131" s="3" t="s">
-        <v>409</v>
+        <v>396</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13017,7 +13017,7 @@
         <v>387</v>
       </c>
       <c r="E132" s="3" t="s">
-        <v>409</v>
+        <v>396</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13059,16 +13059,16 @@
         <v>505</v>
       </c>
       <c r="B135" s="3" t="s">
-        <v>609</v>
+        <v>381</v>
       </c>
       <c r="C135" s="12" t="n">
-        <v>-21470</v>
+        <v>1650249</v>
       </c>
       <c r="D135" s="3" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="E135" s="3" t="s">
-        <v>409</v>
+        <v>383</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13093,16 +13093,16 @@
         <v>505</v>
       </c>
       <c r="B137" s="3" t="s">
-        <v>381</v>
+        <v>405</v>
       </c>
       <c r="C137" s="12" t="n">
-        <v>1650249</v>
+        <v>-21470</v>
       </c>
       <c r="D137" s="3" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="E137" s="3" t="s">
-        <v>383</v>
+        <v>396</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13127,10 +13127,10 @@
         <v>509</v>
       </c>
       <c r="B139" s="3" t="s">
-        <v>393</v>
+        <v>406</v>
       </c>
       <c r="C139" s="12" t="n">
-        <v>-16000</v>
+        <v>-225000</v>
       </c>
       <c r="D139" s="3" t="s">
         <v>387</v>
@@ -13144,10 +13144,10 @@
         <v>509</v>
       </c>
       <c r="B140" s="3" t="s">
-        <v>406</v>
+        <v>393</v>
       </c>
       <c r="C140" s="12" t="n">
-        <v>-225000</v>
+        <v>-16000</v>
       </c>
       <c r="D140" s="3" t="s">
         <v>387</v>
@@ -13164,7 +13164,7 @@
         <v>393</v>
       </c>
       <c r="C141" s="12" t="n">
-        <v>-6800</v>
+        <v>-50000</v>
       </c>
       <c r="D141" s="3" t="s">
         <v>387</v>
@@ -13195,10 +13195,10 @@
         <v>438</v>
       </c>
       <c r="B143" s="3" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="C143" s="12" t="n">
-        <v>-6000</v>
+        <v>-15000</v>
       </c>
       <c r="D143" s="3" t="s">
         <v>387</v>
@@ -13212,10 +13212,10 @@
         <v>438</v>
       </c>
       <c r="B144" s="3" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="C144" s="12" t="n">
-        <v>-15000</v>
+        <v>-6800</v>
       </c>
       <c r="D144" s="3" t="s">
         <v>387</v>
@@ -13232,7 +13232,7 @@
         <v>393</v>
       </c>
       <c r="C145" s="12" t="n">
-        <v>-50000</v>
+        <v>-6000</v>
       </c>
       <c r="D145" s="3" t="s">
         <v>387</v>
@@ -13263,16 +13263,16 @@
         <v>522</v>
       </c>
       <c r="B147" s="3" t="s">
-        <v>617</v>
+        <v>389</v>
       </c>
       <c r="C147" s="12" t="n">
-        <v>-1000000</v>
+        <v>-70000</v>
       </c>
       <c r="D147" s="3" t="s">
         <v>387</v>
       </c>
       <c r="E147" s="3" t="s">
-        <v>78</v>
+        <v>388</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13314,10 +13314,10 @@
         <v>522</v>
       </c>
       <c r="B150" s="3" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="C150" s="12" t="n">
-        <v>-300000</v>
+        <v>-250000</v>
       </c>
       <c r="D150" s="3" t="s">
         <v>387</v>
@@ -13331,16 +13331,16 @@
         <v>522</v>
       </c>
       <c r="B151" s="3" t="s">
-        <v>418</v>
+        <v>394</v>
       </c>
       <c r="C151" s="12" t="n">
-        <v>760000</v>
+        <v>-300000</v>
       </c>
       <c r="D151" s="3" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="E151" s="3" t="s">
-        <v>409</v>
+        <v>388</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13348,7 +13348,7 @@
         <v>522</v>
       </c>
       <c r="B152" s="3" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="C152" s="12" t="n">
         <v>-300000</v>
@@ -13365,10 +13365,10 @@
         <v>522</v>
       </c>
       <c r="B153" s="3" t="s">
-        <v>393</v>
+        <v>386</v>
       </c>
       <c r="C153" s="12" t="n">
-        <v>-250000</v>
+        <v>-400000</v>
       </c>
       <c r="D153" s="3" t="s">
         <v>387</v>
@@ -13382,10 +13382,10 @@
         <v>522</v>
       </c>
       <c r="B154" s="3" t="s">
-        <v>389</v>
+        <v>617</v>
       </c>
       <c r="C154" s="12" t="n">
-        <v>-70000</v>
+        <v>-1000000</v>
       </c>
       <c r="D154" s="3" t="s">
         <v>387</v>
@@ -13399,16 +13399,16 @@
         <v>522</v>
       </c>
       <c r="B155" s="3" t="s">
-        <v>386</v>
+        <v>418</v>
       </c>
       <c r="C155" s="12" t="n">
-        <v>-400000</v>
+        <v>760000</v>
       </c>
       <c r="D155" s="3" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="E155" s="3" t="s">
-        <v>388</v>
+        <v>409</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13416,10 +13416,10 @@
         <v>440</v>
       </c>
       <c r="B156" s="3" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="C156" s="12" t="n">
-        <v>-17000</v>
+        <v>-32000</v>
       </c>
       <c r="D156" s="3" t="s">
         <v>387</v>
@@ -13433,10 +13433,10 @@
         <v>440</v>
       </c>
       <c r="B157" s="3" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
       <c r="C157" s="12" t="n">
-        <v>-32000</v>
+        <v>-17000</v>
       </c>
       <c r="D157" s="3" t="s">
         <v>387</v>
@@ -13467,16 +13467,16 @@
         <v>532</v>
       </c>
       <c r="B159" s="3" t="s">
-        <v>616</v>
+        <v>393</v>
       </c>
       <c r="C159" s="12" t="n">
-        <v>2234722</v>
+        <v>-12000</v>
       </c>
       <c r="D159" s="3" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="E159" s="3" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13484,16 +13484,16 @@
         <v>532</v>
       </c>
       <c r="B160" s="3" t="s">
-        <v>389</v>
+        <v>619</v>
       </c>
       <c r="C160" s="12" t="n">
-        <v>-12000</v>
+        <v>-31319</v>
       </c>
       <c r="D160" s="3" t="s">
         <v>387</v>
       </c>
       <c r="E160" s="3" t="s">
-        <v>388</v>
+        <v>396</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13501,7 +13501,7 @@
         <v>532</v>
       </c>
       <c r="B161" s="3" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="C161" s="12" t="n">
         <v>-12000</v>
@@ -13518,16 +13518,16 @@
         <v>532</v>
       </c>
       <c r="B162" s="3" t="s">
-        <v>381</v>
+        <v>616</v>
       </c>
       <c r="C162" s="12" t="n">
-        <v>198000</v>
+        <v>2234722</v>
       </c>
       <c r="D162" s="3" t="s">
         <v>382</v>
       </c>
       <c r="E162" s="3" t="s">
-        <v>383</v>
+        <v>392</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13535,16 +13535,16 @@
         <v>532</v>
       </c>
       <c r="B163" s="3" t="s">
-        <v>619</v>
+        <v>381</v>
       </c>
       <c r="C163" s="12" t="n">
-        <v>-31319</v>
+        <v>198000</v>
       </c>
       <c r="D163" s="3" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="E163" s="3" t="s">
-        <v>409</v>
+        <v>383</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13552,10 +13552,10 @@
         <v>542</v>
       </c>
       <c r="B164" s="3" t="s">
-        <v>394</v>
+        <v>406</v>
       </c>
       <c r="C164" s="12" t="n">
-        <v>-15000</v>
+        <v>-350000</v>
       </c>
       <c r="D164" s="3" t="s">
         <v>387</v>
@@ -13569,10 +13569,10 @@
         <v>542</v>
       </c>
       <c r="B165" s="3" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="C165" s="12" t="n">
-        <v>-20000</v>
+        <v>-16000</v>
       </c>
       <c r="D165" s="3" t="s">
         <v>387</v>
@@ -13586,16 +13586,16 @@
         <v>542</v>
       </c>
       <c r="B166" s="3" t="s">
-        <v>620</v>
+        <v>394</v>
       </c>
       <c r="C166" s="12" t="n">
-        <v>-5770</v>
+        <v>-15000</v>
       </c>
       <c r="D166" s="3" t="s">
         <v>387</v>
       </c>
       <c r="E166" s="3" t="s">
-        <v>396</v>
+        <v>388</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13603,16 +13603,16 @@
         <v>542</v>
       </c>
       <c r="B167" s="3" t="s">
-        <v>393</v>
+        <v>620</v>
       </c>
       <c r="C167" s="12" t="n">
-        <v>-16000</v>
+        <v>-5770</v>
       </c>
       <c r="D167" s="3" t="s">
         <v>387</v>
       </c>
       <c r="E167" s="3" t="s">
-        <v>388</v>
+        <v>396</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13620,10 +13620,10 @@
         <v>542</v>
       </c>
       <c r="B168" s="3" t="s">
-        <v>406</v>
+        <v>389</v>
       </c>
       <c r="C168" s="12" t="n">
-        <v>-350000</v>
+        <v>-20000</v>
       </c>
       <c r="D168" s="3" t="s">
         <v>387</v>
@@ -13637,10 +13637,10 @@
         <v>546</v>
       </c>
       <c r="B169" s="3" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="C169" s="12" t="n">
-        <v>-29000</v>
+        <v>-20000</v>
       </c>
       <c r="D169" s="3" t="s">
         <v>387</v>
@@ -13671,10 +13671,10 @@
         <v>546</v>
       </c>
       <c r="B171" s="3" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="C171" s="12" t="n">
-        <v>-20000</v>
+        <v>-29000</v>
       </c>
       <c r="D171" s="3" t="s">
         <v>387</v>
@@ -13722,10 +13722,10 @@
         <v>559</v>
       </c>
       <c r="B174" s="3" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="C174" s="12" t="n">
-        <v>-12000</v>
+        <v>-15000</v>
       </c>
       <c r="D174" s="3" t="s">
         <v>387</v>
@@ -13742,7 +13742,7 @@
         <v>622</v>
       </c>
       <c r="C175" s="12" t="n">
-        <v>490200</v>
+        <v>200000</v>
       </c>
       <c r="D175" s="3" t="s">
         <v>382</v>
@@ -13756,16 +13756,16 @@
         <v>559</v>
       </c>
       <c r="B176" s="3" t="s">
-        <v>623</v>
+        <v>389</v>
       </c>
       <c r="C176" s="12" t="n">
-        <v>-16500</v>
+        <v>-3000</v>
       </c>
       <c r="D176" s="3" t="s">
         <v>387</v>
       </c>
       <c r="E176" s="3" t="s">
-        <v>409</v>
+        <v>388</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13773,16 +13773,16 @@
         <v>559</v>
       </c>
       <c r="B177" s="3" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="C177" s="12" t="n">
-        <v>200000</v>
+        <v>-16500</v>
       </c>
       <c r="D177" s="3" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="E177" s="3" t="s">
-        <v>409</v>
+        <v>396</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13790,13 +13790,13 @@
         <v>559</v>
       </c>
       <c r="B178" s="3" t="s">
-        <v>410</v>
+        <v>389</v>
       </c>
       <c r="C178" s="12" t="n">
-        <v>1000000</v>
+        <v>-12000</v>
       </c>
       <c r="D178" s="3" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="E178" s="3" t="s">
         <v>388</v>
@@ -13807,10 +13807,10 @@
         <v>559</v>
       </c>
       <c r="B179" s="3" t="s">
-        <v>393</v>
+        <v>406</v>
       </c>
       <c r="C179" s="12" t="n">
-        <v>-15000</v>
+        <v>-18000</v>
       </c>
       <c r="D179" s="3" t="s">
         <v>387</v>
@@ -13824,13 +13824,13 @@
         <v>559</v>
       </c>
       <c r="B180" s="3" t="s">
-        <v>389</v>
+        <v>410</v>
       </c>
       <c r="C180" s="12" t="n">
-        <v>-120000</v>
+        <v>1000000</v>
       </c>
       <c r="D180" s="3" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="E180" s="3" t="s">
         <v>388</v>
@@ -13841,10 +13841,10 @@
         <v>559</v>
       </c>
       <c r="B181" s="3" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="C181" s="12" t="n">
-        <v>-3000</v>
+        <v>-70000</v>
       </c>
       <c r="D181" s="3" t="s">
         <v>387</v>
@@ -13858,10 +13858,10 @@
         <v>559</v>
       </c>
       <c r="B182" s="3" t="s">
-        <v>406</v>
+        <v>389</v>
       </c>
       <c r="C182" s="12" t="n">
-        <v>-18000</v>
+        <v>-120000</v>
       </c>
       <c r="D182" s="3" t="s">
         <v>387</v>
@@ -13875,16 +13875,16 @@
         <v>559</v>
       </c>
       <c r="B183" s="3" t="s">
-        <v>390</v>
+        <v>622</v>
       </c>
       <c r="C183" s="12" t="n">
-        <v>-25000</v>
+        <v>490200</v>
       </c>
       <c r="D183" s="3" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="E183" s="3" t="s">
-        <v>388</v>
+        <v>409</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13892,10 +13892,10 @@
         <v>559</v>
       </c>
       <c r="B184" s="3" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="C184" s="12" t="n">
-        <v>-70000</v>
+        <v>-25000</v>
       </c>
       <c r="D184" s="3" t="s">
         <v>387</v>
@@ -13909,10 +13909,10 @@
         <v>572</v>
       </c>
       <c r="B185" s="3" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C185" s="12" t="n">
-        <v>-20000</v>
+        <v>-170000</v>
       </c>
       <c r="D185" s="3" t="s">
         <v>387</v>
@@ -13926,10 +13926,10 @@
         <v>572</v>
       </c>
       <c r="B186" s="3" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C186" s="12" t="n">
-        <v>-170000</v>
+        <v>-20000</v>
       </c>
       <c r="D186" s="3" t="s">
         <v>387</v>
@@ -13960,13 +13960,13 @@
         <v>445</v>
       </c>
       <c r="B188" s="3" t="s">
-        <v>389</v>
+        <v>410</v>
       </c>
       <c r="C188" s="12" t="n">
-        <v>-53000</v>
+        <v>500000</v>
       </c>
       <c r="D188" s="3" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="E188" s="3" t="s">
         <v>388</v>
@@ -13977,16 +13977,16 @@
         <v>445</v>
       </c>
       <c r="B189" s="3" t="s">
-        <v>393</v>
+        <v>381</v>
       </c>
       <c r="C189" s="12" t="n">
-        <v>-12000</v>
+        <v>500000</v>
       </c>
       <c r="D189" s="3" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="E189" s="3" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13997,7 +13997,7 @@
         <v>389</v>
       </c>
       <c r="C190" s="12" t="n">
-        <v>-12000</v>
+        <v>-53000</v>
       </c>
       <c r="D190" s="3" t="s">
         <v>387</v>
@@ -14028,16 +14028,16 @@
         <v>445</v>
       </c>
       <c r="B192" s="3" t="s">
-        <v>381</v>
+        <v>393</v>
       </c>
       <c r="C192" s="12" t="n">
-        <v>500000</v>
+        <v>-12000</v>
       </c>
       <c r="D192" s="3" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="E192" s="3" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14045,13 +14045,13 @@
         <v>445</v>
       </c>
       <c r="B193" s="3" t="s">
-        <v>410</v>
+        <v>389</v>
       </c>
       <c r="C193" s="12" t="n">
-        <v>500000</v>
+        <v>-12000</v>
       </c>
       <c r="D193" s="3" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="E193" s="3" t="s">
         <v>388</v>
@@ -14062,7 +14062,7 @@
         <v>448</v>
       </c>
       <c r="B194" s="3" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="C194" s="12" t="n">
         <v>-20000</v>
@@ -14079,7 +14079,7 @@
         <v>448</v>
       </c>
       <c r="B195" s="3" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="C195" s="12" t="n">
         <v>-20000</v>
@@ -14091,102 +14091,187 @@
         <v>388</v>
       </c>
     </row>
+    <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A196" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="B196" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C196" s="12" t="n">
+        <v>-30000</v>
+      </c>
+      <c r="D196" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E196" s="3" t="s">
+        <v>388</v>
+      </c>
+    </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A197" s="2" t="s">
-        <v>421</v>
-      </c>
-      <c r="B197" s="2"/>
-      <c r="C197" s="2"/>
-      <c r="D197" s="2"/>
-      <c r="E197" s="2"/>
-      <c r="F197" s="2"/>
-      <c r="G197" s="2"/>
-      <c r="H197" s="2"/>
-      <c r="I197" s="2"/>
+      <c r="A197" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="B197" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="C197" s="12" t="n">
+        <v>-24000</v>
+      </c>
+      <c r="D197" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E197" s="3" t="s">
+        <v>388</v>
+      </c>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A198" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="B198" s="9" t="s">
-        <v>378</v>
-      </c>
-      <c r="C198" s="30" t="s">
-        <v>422</v>
-      </c>
-      <c r="D198" s="30" t="s">
-        <v>423</v>
+      <c r="A198" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="B198" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="C198" s="12" t="n">
+        <v>4625470</v>
+      </c>
+      <c r="D198" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="E198" s="3" t="s">
+        <v>392</v>
       </c>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A199" s="3" t="s">
-        <v>424</v>
-      </c>
-      <c r="B199" s="12" t="n">
-        <v>267206</v>
+        <v>450</v>
+      </c>
+      <c r="B199" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C199" s="12" t="n">
+        <v>-250000</v>
+      </c>
+      <c r="D199" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E199" s="3" t="s">
+        <v>388</v>
       </c>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="B200" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C200" s="12" t="n">
+        <v>-6000</v>
+      </c>
+      <c r="D200" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E200" s="3" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A202" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="B202" s="2"/>
+      <c r="C202" s="2"/>
+      <c r="D202" s="2"/>
+      <c r="E202" s="2"/>
+      <c r="F202" s="2"/>
+      <c r="G202" s="2"/>
+      <c r="H202" s="2"/>
+      <c r="I202" s="2"/>
+    </row>
+    <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A203" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B203" s="9" t="s">
+        <v>378</v>
+      </c>
+      <c r="C203" s="30" t="s">
+        <v>422</v>
+      </c>
+      <c r="D203" s="30" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A204" s="3" t="s">
+        <v>424</v>
+      </c>
+      <c r="B204" s="12" t="n">
+        <v>267206</v>
+      </c>
+    </row>
+    <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A205" s="3" t="s">
         <v>425</v>
       </c>
-      <c r="B200" s="12" t="n">
-        <v>15543638</v>
-      </c>
-      <c r="C200" s="31" t="n">
+      <c r="B205" s="12" t="n">
+        <v>20169108</v>
+      </c>
+      <c r="C205" s="31" t="n">
         <f aca="false">F14</f>
         <v>14685671</v>
       </c>
-      <c r="D200" s="31" t="n">
-        <f aca="false">B200-C200</f>
-        <v>857967</v>
-      </c>
-    </row>
-    <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A201" s="3" t="s">
+      <c r="D205" s="31" t="n">
+        <f aca="false">B205-C205</f>
+        <v>5483437</v>
+      </c>
+    </row>
+    <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A206" s="3" t="s">
         <v>426</v>
       </c>
-      <c r="B201" s="12" t="n">
-        <v>-15627141</v>
-      </c>
-    </row>
-    <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A202" s="18" t="s">
+      <c r="B206" s="12" t="n">
+        <v>-16055513</v>
+      </c>
+    </row>
+    <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A207" s="18" t="s">
         <v>427</v>
       </c>
-      <c r="B202" s="14" t="n">
-        <f aca="false">SUM(B199:B201)</f>
-        <v>183703</v>
-      </c>
-    </row>
-    <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A203" s="18" t="s">
+      <c r="B207" s="14" t="n">
+        <f aca="false">SUM(B204:B206)</f>
+        <v>4380801</v>
+      </c>
+    </row>
+    <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A208" s="18" t="s">
         <v>428</v>
       </c>
-      <c r="B203" s="14" t="n">
-        <v>183703</v>
-      </c>
-    </row>
-    <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A204" s="18" t="s">
+      <c r="B208" s="14" t="n">
+        <v>4380801</v>
+      </c>
+    </row>
+    <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A209" s="18" t="s">
         <v>429</v>
       </c>
-      <c r="B204" s="14" t="n">
-        <f aca="false">B202-B203</f>
+      <c r="B209" s="14" t="n">
+        <f aca="false">B207-B208</f>
         <v>0</v>
       </c>
     </row>
-    <row r="206" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A206" s="10" t="s">
+    <row r="211" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A211" s="10" t="s">
         <v>430</v>
       </c>
-      <c r="B206" s="10"/>
-      <c r="C206" s="10"/>
-      <c r="D206" s="10"/>
-      <c r="E206" s="10"/>
-      <c r="F206" s="10"/>
-      <c r="G206" s="10"/>
-      <c r="H206" s="10"/>
+      <c r="B211" s="10"/>
+      <c r="C211" s="10"/>
+      <c r="D211" s="10"/>
+      <c r="E211" s="10"/>
+      <c r="F211" s="10"/>
+      <c r="G211" s="10"/>
+      <c r="H211" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -14195,8 +14280,8 @@
     <mergeCell ref="A4:I4"/>
     <mergeCell ref="A16:I16"/>
     <mergeCell ref="A99:I99"/>
-    <mergeCell ref="A197:I197"/>
-    <mergeCell ref="A206:H206"/>
+    <mergeCell ref="A202:I202"/>
+    <mergeCell ref="A211:H211"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Agrega hoja Categorizacion_Cartola_Julio (26 categorias reales kaptura_categorias_costo) para revision previa a cargar Supabase
</commit_message>
<xml_diff>
--- a/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
+++ b/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
@@ -16,7 +16,8 @@
     <sheet name="Conciliación_Julio" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="Real_vs_Presupuesto" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="Resumen_Ejecutivo" sheetId="8" state="visible" r:id="rId10"/>
-    <sheet name="Bitácora_Saldo_Diario" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="Categorizacion_Cartola_Julio" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="Bitácora_Saldo_Diario" sheetId="10" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2096" uniqueCount="669">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3000" uniqueCount="714">
   <si>
     <t xml:space="preserve">SUPUESTOS DEL PRESUPUESTO — SOLLEM + TRAST</t>
   </si>
@@ -2019,6 +2020,142 @@
   </si>
   <si>
     <t xml:space="preserve">SEPTIEMBRE 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CATEGORIZACIÓN CARTOLA JULIO 2026 — para revisión antes de cargar a kaptura_estado_resultados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cartola histórica definitiva N°3 (30/06 al 31/07/2026, 152 movimientos). Categorías = las 26 reales de kaptura_categorias_costo (Supabase), no un esquema aparte. Columna "Revisar" queda en amarillo para las categorías de menor confianza (heurística por monto, o "otro_por_clasificar") — confírmelas o corríjalas acá antes de que se carguen a Supabase.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Descripción Movimiento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cargo/
+Abono</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Categoría (kaptura_categorias_costo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Centro de Costo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confianza / Revisar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">transferencia_interna_por_confirmar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">administracion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Media</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PAGO EN LINEA ESMAX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">combustible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flota</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">remuneracion_administrativa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baja — sin desglose exacto, revisar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">076630639K Transf a Servicios inte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">otro_por_clasificar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baja — revisar manualmente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compra Nacional MD VALPAR LTDA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compra Nacional MD IMPLEMENTOS S.A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mantencion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aporte_retiro_socio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">viatico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Media — heurística por monto múltiplo $12.000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0780993812 Transf. LOGISTICA Y TRA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compra Nacional MD TTP S.A RANCAGU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compra Nacional MD COMERCIAL ECUAD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0772640749 Transf a Fijasur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">factoring</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alta — confirmado con comprobante real</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compra Nacional MD TRANSAGRO RANCA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">iva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compra Nacional MD VULKO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compra Nacional MD FEDICAR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compra Nacional MD SOLMET SPA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compra Nacional MD APRO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compra Nacional MD CONSTRU-MART RA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compra Nacional MD MERCADOPAGO *EL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0070082349 Transf a VALDES CORNEJO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compra Nacional MD CARDANICA PACIF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RESUMEN POR CATEGORÍA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Categoría</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N° movimientos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total</t>
   </si>
   <si>
     <t xml:space="preserve">BITÁCORA DE SALDO DIARIO — Banco Santander 0-000-3776731-0</t>
@@ -2249,7 +2386,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2399,6 +2536,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3090,6 +3231,384 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F31"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="40"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>703</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="24" t="s">
+        <v>704</v>
+      </c>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+    </row>
+    <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
+        <v>376</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>705</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>706</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>707</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>708</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="B5" s="12" t="n">
+        <v>63371</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>709</v>
+      </c>
+      <c r="D5" s="37"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="3" t="s">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>711</v>
+      </c>
+      <c r="B6" s="12" t="n">
+        <v>1275801</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>712</v>
+      </c>
+      <c r="D6" s="34"/>
+      <c r="E6" s="12" t="str">
+        <f aca="false">IF(D6="","",B6-D6)</f>
+        <v/>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="39"/>
+      <c r="B7" s="34"/>
+      <c r="C7" s="39"/>
+      <c r="D7" s="34"/>
+      <c r="E7" s="12" t="str">
+        <f aca="false">IF(OR(B7="",D7=""),"",B7-D7)</f>
+        <v/>
+      </c>
+      <c r="F7" s="39"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="39"/>
+      <c r="B8" s="34"/>
+      <c r="C8" s="39"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="12" t="str">
+        <f aca="false">IF(OR(B8="",D8=""),"",B8-D8)</f>
+        <v/>
+      </c>
+      <c r="F8" s="39"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="39"/>
+      <c r="B9" s="34"/>
+      <c r="C9" s="39"/>
+      <c r="D9" s="34"/>
+      <c r="E9" s="12" t="str">
+        <f aca="false">IF(OR(B9="",D9=""),"",B9-D9)</f>
+        <v/>
+      </c>
+      <c r="F9" s="39"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="39"/>
+      <c r="B10" s="34"/>
+      <c r="C10" s="39"/>
+      <c r="D10" s="34"/>
+      <c r="E10" s="12" t="str">
+        <f aca="false">IF(OR(B10="",D10=""),"",B10-D10)</f>
+        <v/>
+      </c>
+      <c r="F10" s="39"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="39"/>
+      <c r="B11" s="34"/>
+      <c r="C11" s="39"/>
+      <c r="D11" s="34"/>
+      <c r="E11" s="12" t="str">
+        <f aca="false">IF(OR(B11="",D11=""),"",B11-D11)</f>
+        <v/>
+      </c>
+      <c r="F11" s="39"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="39"/>
+      <c r="B12" s="34"/>
+      <c r="C12" s="39"/>
+      <c r="D12" s="34"/>
+      <c r="E12" s="12" t="str">
+        <f aca="false">IF(OR(B12="",D12=""),"",B12-D12)</f>
+        <v/>
+      </c>
+      <c r="F12" s="39"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="39"/>
+      <c r="B13" s="34"/>
+      <c r="C13" s="39"/>
+      <c r="D13" s="34"/>
+      <c r="E13" s="12" t="str">
+        <f aca="false">IF(OR(B13="",D13=""),"",B13-D13)</f>
+        <v/>
+      </c>
+      <c r="F13" s="39"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="39"/>
+      <c r="B14" s="34"/>
+      <c r="C14" s="39"/>
+      <c r="D14" s="34"/>
+      <c r="E14" s="12" t="str">
+        <f aca="false">IF(OR(B14="",D14=""),"",B14-D14)</f>
+        <v/>
+      </c>
+      <c r="F14" s="39"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="39"/>
+      <c r="B15" s="34"/>
+      <c r="C15" s="39"/>
+      <c r="D15" s="34"/>
+      <c r="E15" s="12" t="str">
+        <f aca="false">IF(OR(B15="",D15=""),"",B15-D15)</f>
+        <v/>
+      </c>
+      <c r="F15" s="39"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="39"/>
+      <c r="B16" s="34"/>
+      <c r="C16" s="39"/>
+      <c r="D16" s="34"/>
+      <c r="E16" s="12" t="str">
+        <f aca="false">IF(OR(B16="",D16=""),"",B16-D16)</f>
+        <v/>
+      </c>
+      <c r="F16" s="39"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="39"/>
+      <c r="B17" s="34"/>
+      <c r="C17" s="39"/>
+      <c r="D17" s="34"/>
+      <c r="E17" s="12" t="str">
+        <f aca="false">IF(OR(B17="",D17=""),"",B17-D17)</f>
+        <v/>
+      </c>
+      <c r="F17" s="39"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="39"/>
+      <c r="B18" s="34"/>
+      <c r="C18" s="39"/>
+      <c r="D18" s="34"/>
+      <c r="E18" s="12" t="str">
+        <f aca="false">IF(OR(B18="",D18=""),"",B18-D18)</f>
+        <v/>
+      </c>
+      <c r="F18" s="39"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="39"/>
+      <c r="B19" s="34"/>
+      <c r="C19" s="39"/>
+      <c r="D19" s="34"/>
+      <c r="E19" s="12" t="str">
+        <f aca="false">IF(OR(B19="",D19=""),"",B19-D19)</f>
+        <v/>
+      </c>
+      <c r="F19" s="39"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="39"/>
+      <c r="B20" s="34"/>
+      <c r="C20" s="39"/>
+      <c r="D20" s="34"/>
+      <c r="E20" s="12" t="str">
+        <f aca="false">IF(OR(B20="",D20=""),"",B20-D20)</f>
+        <v/>
+      </c>
+      <c r="F20" s="39"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="39"/>
+      <c r="B21" s="34"/>
+      <c r="C21" s="39"/>
+      <c r="D21" s="34"/>
+      <c r="E21" s="12" t="str">
+        <f aca="false">IF(OR(B21="",D21=""),"",B21-D21)</f>
+        <v/>
+      </c>
+      <c r="F21" s="39"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="39"/>
+      <c r="B22" s="34"/>
+      <c r="C22" s="39"/>
+      <c r="D22" s="34"/>
+      <c r="E22" s="12" t="str">
+        <f aca="false">IF(OR(B22="",D22=""),"",B22-D22)</f>
+        <v/>
+      </c>
+      <c r="F22" s="39"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="39"/>
+      <c r="B23" s="34"/>
+      <c r="C23" s="39"/>
+      <c r="D23" s="34"/>
+      <c r="E23" s="12" t="str">
+        <f aca="false">IF(OR(B23="",D23=""),"",B23-D23)</f>
+        <v/>
+      </c>
+      <c r="F23" s="39"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="39"/>
+      <c r="B24" s="34"/>
+      <c r="C24" s="39"/>
+      <c r="D24" s="34"/>
+      <c r="E24" s="12" t="str">
+        <f aca="false">IF(OR(B24="",D24=""),"",B24-D24)</f>
+        <v/>
+      </c>
+      <c r="F24" s="39"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="39"/>
+      <c r="B25" s="34"/>
+      <c r="C25" s="39"/>
+      <c r="D25" s="34"/>
+      <c r="E25" s="12" t="str">
+        <f aca="false">IF(OR(B25="",D25=""),"",B25-D25)</f>
+        <v/>
+      </c>
+      <c r="F25" s="39"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="39"/>
+      <c r="B26" s="34"/>
+      <c r="C26" s="39"/>
+      <c r="D26" s="34"/>
+      <c r="E26" s="12" t="str">
+        <f aca="false">IF(OR(B26="",D26=""),"",B26-D26)</f>
+        <v/>
+      </c>
+      <c r="F26" s="39"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="39"/>
+      <c r="B27" s="34"/>
+      <c r="C27" s="39"/>
+      <c r="D27" s="34"/>
+      <c r="E27" s="12" t="str">
+        <f aca="false">IF(OR(B27="",D27=""),"",B27-D27)</f>
+        <v/>
+      </c>
+      <c r="F27" s="39"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="39"/>
+      <c r="B28" s="34"/>
+      <c r="C28" s="39"/>
+      <c r="D28" s="34"/>
+      <c r="E28" s="12" t="str">
+        <f aca="false">IF(OR(B28="",D28=""),"",B28-D28)</f>
+        <v/>
+      </c>
+      <c r="F28" s="39"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="39"/>
+      <c r="B29" s="34"/>
+      <c r="C29" s="39"/>
+      <c r="D29" s="34"/>
+      <c r="E29" s="12" t="str">
+        <f aca="false">IF(OR(B29="",D29=""),"",B29-D29)</f>
+        <v/>
+      </c>
+      <c r="F29" s="39"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="39"/>
+      <c r="B30" s="34"/>
+      <c r="C30" s="39"/>
+      <c r="D30" s="34"/>
+      <c r="E30" s="12" t="str">
+        <f aca="false">IF(OR(B30="",D30=""),"",B30-D30)</f>
+        <v/>
+      </c>
+      <c r="F30" s="39"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="39"/>
+      <c r="B31" s="34"/>
+      <c r="C31" s="39"/>
+      <c r="D31" s="34"/>
+      <c r="E31" s="12" t="str">
+        <f aca="false">IF(OR(B31="",D31=""),"",B31-D31)</f>
+        <v/>
+      </c>
+      <c r="F31" s="39"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
@@ -15332,12 +15851,16 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:G163"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="40"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15349,8 +15872,9 @@
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="G1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="24" t="s">
         <v>659</v>
       </c>
@@ -15359,6 +15883,7 @@
       <c r="D2" s="24"/>
       <c r="E2" s="24"/>
       <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
@@ -15368,332 +15893,3528 @@
         <v>660</v>
       </c>
       <c r="C4" s="9" t="s">
+        <v>378</v>
+      </c>
+      <c r="D4" s="9" t="s">
         <v>661</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="E4" s="9" t="s">
         <v>662</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="F4" s="9" t="s">
         <v>663</v>
       </c>
-      <c r="F4" s="9" t="s">
-        <v>188</v>
+      <c r="G4" s="9" t="s">
+        <v>664</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>445</v>
-      </c>
-      <c r="B5" s="12" t="n">
-        <v>63371</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>664</v>
-      </c>
-      <c r="D5" s="37"/>
-      <c r="E5" s="37"/>
+        <v>435</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>2326472</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="E5" s="38" t="s">
+        <v>665</v>
+      </c>
       <c r="F5" s="3" t="s">
-        <v>665</v>
+        <v>666</v>
+      </c>
+      <c r="G5" s="38" t="s">
+        <v>667</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>668</v>
+      </c>
+      <c r="C6" s="12" t="n">
+        <v>-1300000</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>669</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="C7" s="12" t="n">
+        <v>-70000</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E7" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>666</v>
       </c>
-      <c r="B6" s="12" t="n">
-        <v>1275801</v>
-      </c>
-      <c r="C6" s="3" t="s">
+      <c r="G7" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>-27000</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E8" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G8" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="C9" s="12" t="n">
+        <v>-6000</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E9" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G9" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="C10" s="12" t="n">
+        <v>-225000</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E10" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G10" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>609</v>
+      </c>
+      <c r="C11" s="12" t="n">
+        <v>-190000</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E11" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G11" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>610</v>
+      </c>
+      <c r="C12" s="12" t="n">
+        <v>-54000</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E12" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G12" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>674</v>
+      </c>
+      <c r="C13" s="12" t="n">
+        <v>-30000</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E13" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G13" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="C14" s="12" t="n">
+        <v>-2700</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E14" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G14" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C15" s="12" t="n">
+        <v>-15000</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E15" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G15" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="C16" s="12" t="n">
+        <v>-17000</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E16" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G16" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>677</v>
+      </c>
+      <c r="C17" s="12" t="n">
+        <v>-92344</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E17" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G17" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>611</v>
+      </c>
+      <c r="C18" s="12" t="n">
+        <v>-280000</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E18" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G18" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>678</v>
+      </c>
+      <c r="C19" s="12" t="n">
+        <v>-17980</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E19" s="38" t="s">
+        <v>679</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G19" s="38" t="s">
         <v>667</v>
       </c>
-      <c r="D6" s="34"/>
-      <c r="E6" s="12" t="str">
-        <f aca="false">IF(D6="","",B6-D6)</f>
-        <v/>
-      </c>
-      <c r="F6" s="3" t="s">
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="C20" s="12" t="n">
+        <v>83100</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="E20" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G20" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="C21" s="12" t="n">
+        <v>270000</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="E21" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G21" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="C22" s="12" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="E22" s="38" t="s">
+        <v>680</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G22" s="38" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>614</v>
+      </c>
+      <c r="C23" s="12" t="n">
+        <v>-299606</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E23" s="38" t="s">
+        <v>679</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G23" s="38" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C24" s="12" t="n">
+        <v>-12000</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E24" s="38" t="s">
+        <v>681</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G24" s="38" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C25" s="12" t="n">
+        <v>-50000</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E25" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G25" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="C26" s="12" t="n">
+        <v>-100000</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E26" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G26" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C27" s="12" t="n">
+        <v>-100000</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E27" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G27" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C28" s="12" t="n">
+        <v>-120000</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E28" s="38" t="s">
+        <v>681</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G28" s="38" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C29" s="12" t="n">
+        <v>-150000</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E29" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G29" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="C30" s="12" t="n">
+        <v>-225000</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E30" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G30" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="C31" s="12" t="n">
+        <v>-250000</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E31" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G31" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="C32" s="12" t="n">
+        <v>-270000</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E32" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G32" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>612</v>
+      </c>
+      <c r="C33" s="12" t="n">
+        <v>320000</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="E33" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G33" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C34" s="12" t="n">
+        <v>-180000</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E34" s="38" t="s">
+        <v>681</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G34" s="38" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="C35" s="12" t="n">
+        <v>-4700</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E35" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G35" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="C36" s="12" t="n">
+        <v>-17000</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E36" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G36" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C37" s="12" t="n">
+        <v>-12000</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E37" s="38" t="s">
+        <v>681</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G37" s="38" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C38" s="12" t="n">
+        <v>-8000</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E38" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G38" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>613</v>
+      </c>
+      <c r="C39" s="12" t="n">
+        <v>-14880</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E39" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G39" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C40" s="12" t="n">
+        <v>-32000</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E40" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G40" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>683</v>
+      </c>
+      <c r="C41" s="12" t="n">
+        <v>440300</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="E41" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G41" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C42" s="12" t="n">
+        <v>-100000</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E42" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F42" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G42" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>684</v>
+      </c>
+      <c r="C43" s="12" t="n">
+        <v>-88073</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E43" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F43" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G43" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>614</v>
+      </c>
+      <c r="C44" s="12" t="n">
+        <v>-63065</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E44" s="38" t="s">
+        <v>679</v>
+      </c>
+      <c r="F44" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G44" s="38" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>685</v>
+      </c>
+      <c r="C45" s="12" t="n">
+        <v>-36259</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E45" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F45" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G45" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>615</v>
+      </c>
+      <c r="C46" s="12" t="n">
+        <v>-31955</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E46" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F46" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G46" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="3" t="s">
+        <v>498</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>678</v>
+      </c>
+      <c r="C47" s="12" t="n">
+        <v>-77990</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E47" s="38" t="s">
+        <v>679</v>
+      </c>
+      <c r="F47" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G47" s="38" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="3" t="s">
+        <v>498</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C48" s="12" t="n">
+        <v>-17000</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E48" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F48" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G48" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="3" t="s">
+        <v>505</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C49" s="12" t="n">
+        <v>-12000</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E49" s="38" t="s">
+        <v>681</v>
+      </c>
+      <c r="F49" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G49" s="38" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="3" t="s">
+        <v>505</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="C50" s="12" t="n">
+        <v>-21470</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E50" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F50" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G50" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="3" t="s">
+        <v>505</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C51" s="12" t="n">
+        <v>-50000</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E51" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F51" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G51" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="3" t="s">
+        <v>505</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C52" s="12" t="n">
+        <v>-50000</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E52" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F52" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G52" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="3" t="s">
+        <v>505</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="C53" s="12" t="n">
+        <v>-30000</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>669</v>
+      </c>
+      <c r="F53" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G53" s="3" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="3" t="s">
+        <v>505</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="C54" s="12" t="n">
+        <v>-200000</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E54" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F54" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G54" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="3" t="s">
+        <v>505</v>
+      </c>
+      <c r="B55" s="3" t="s">
         <v>668</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="38"/>
-      <c r="B7" s="34"/>
-      <c r="C7" s="38"/>
-      <c r="D7" s="34"/>
-      <c r="E7" s="12" t="str">
-        <f aca="false">IF(OR(B7="",D7=""),"",B7-D7)</f>
-        <v/>
-      </c>
-      <c r="F7" s="38"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="38"/>
-      <c r="B8" s="34"/>
-      <c r="C8" s="38"/>
-      <c r="D8" s="34"/>
-      <c r="E8" s="12" t="str">
-        <f aca="false">IF(OR(B8="",D8=""),"",B8-D8)</f>
-        <v/>
-      </c>
-      <c r="F8" s="38"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="38"/>
-      <c r="B9" s="34"/>
-      <c r="C9" s="38"/>
-      <c r="D9" s="34"/>
-      <c r="E9" s="12" t="str">
-        <f aca="false">IF(OR(B9="",D9=""),"",B9-D9)</f>
-        <v/>
-      </c>
-      <c r="F9" s="38"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="38"/>
-      <c r="B10" s="34"/>
-      <c r="C10" s="38"/>
-      <c r="D10" s="34"/>
-      <c r="E10" s="12" t="str">
-        <f aca="false">IF(OR(B10="",D10=""),"",B10-D10)</f>
-        <v/>
-      </c>
-      <c r="F10" s="38"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="38"/>
-      <c r="B11" s="34"/>
-      <c r="C11" s="38"/>
-      <c r="D11" s="34"/>
-      <c r="E11" s="12" t="str">
-        <f aca="false">IF(OR(B11="",D11=""),"",B11-D11)</f>
-        <v/>
-      </c>
-      <c r="F11" s="38"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="38"/>
-      <c r="B12" s="34"/>
-      <c r="C12" s="38"/>
-      <c r="D12" s="34"/>
-      <c r="E12" s="12" t="str">
-        <f aca="false">IF(OR(B12="",D12=""),"",B12-D12)</f>
-        <v/>
-      </c>
-      <c r="F12" s="38"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="38"/>
-      <c r="B13" s="34"/>
-      <c r="C13" s="38"/>
-      <c r="D13" s="34"/>
-      <c r="E13" s="12" t="str">
-        <f aca="false">IF(OR(B13="",D13=""),"",B13-D13)</f>
-        <v/>
-      </c>
-      <c r="F13" s="38"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="38"/>
-      <c r="B14" s="34"/>
-      <c r="C14" s="38"/>
-      <c r="D14" s="34"/>
-      <c r="E14" s="12" t="str">
-        <f aca="false">IF(OR(B14="",D14=""),"",B14-D14)</f>
-        <v/>
-      </c>
-      <c r="F14" s="38"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="38"/>
-      <c r="B15" s="34"/>
-      <c r="C15" s="38"/>
-      <c r="D15" s="34"/>
-      <c r="E15" s="12" t="str">
-        <f aca="false">IF(OR(B15="",D15=""),"",B15-D15)</f>
-        <v/>
-      </c>
-      <c r="F15" s="38"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="38"/>
-      <c r="B16" s="34"/>
-      <c r="C16" s="38"/>
-      <c r="D16" s="34"/>
-      <c r="E16" s="12" t="str">
-        <f aca="false">IF(OR(B16="",D16=""),"",B16-D16)</f>
-        <v/>
-      </c>
-      <c r="F16" s="38"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="38"/>
-      <c r="B17" s="34"/>
-      <c r="C17" s="38"/>
-      <c r="D17" s="34"/>
-      <c r="E17" s="12" t="str">
-        <f aca="false">IF(OR(B17="",D17=""),"",B17-D17)</f>
-        <v/>
-      </c>
-      <c r="F17" s="38"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="38"/>
-      <c r="B18" s="34"/>
-      <c r="C18" s="38"/>
-      <c r="D18" s="34"/>
-      <c r="E18" s="12" t="str">
-        <f aca="false">IF(OR(B18="",D18=""),"",B18-D18)</f>
-        <v/>
-      </c>
-      <c r="F18" s="38"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="38"/>
-      <c r="B19" s="34"/>
-      <c r="C19" s="38"/>
-      <c r="D19" s="34"/>
-      <c r="E19" s="12" t="str">
-        <f aca="false">IF(OR(B19="",D19=""),"",B19-D19)</f>
-        <v/>
-      </c>
-      <c r="F19" s="38"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="38"/>
-      <c r="B20" s="34"/>
-      <c r="C20" s="38"/>
-      <c r="D20" s="34"/>
-      <c r="E20" s="12" t="str">
-        <f aca="false">IF(OR(B20="",D20=""),"",B20-D20)</f>
-        <v/>
-      </c>
-      <c r="F20" s="38"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="38"/>
-      <c r="B21" s="34"/>
-      <c r="C21" s="38"/>
-      <c r="D21" s="34"/>
-      <c r="E21" s="12" t="str">
-        <f aca="false">IF(OR(B21="",D21=""),"",B21-D21)</f>
-        <v/>
-      </c>
-      <c r="F21" s="38"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="38"/>
-      <c r="B22" s="34"/>
-      <c r="C22" s="38"/>
-      <c r="D22" s="34"/>
-      <c r="E22" s="12" t="str">
-        <f aca="false">IF(OR(B22="",D22=""),"",B22-D22)</f>
-        <v/>
-      </c>
-      <c r="F22" s="38"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="38"/>
-      <c r="B23" s="34"/>
-      <c r="C23" s="38"/>
-      <c r="D23" s="34"/>
-      <c r="E23" s="12" t="str">
-        <f aca="false">IF(OR(B23="",D23=""),"",B23-D23)</f>
-        <v/>
-      </c>
-      <c r="F23" s="38"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="38"/>
-      <c r="B24" s="34"/>
-      <c r="C24" s="38"/>
-      <c r="D24" s="34"/>
-      <c r="E24" s="12" t="str">
-        <f aca="false">IF(OR(B24="",D24=""),"",B24-D24)</f>
-        <v/>
-      </c>
-      <c r="F24" s="38"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="38"/>
-      <c r="B25" s="34"/>
-      <c r="C25" s="38"/>
-      <c r="D25" s="34"/>
-      <c r="E25" s="12" t="str">
-        <f aca="false">IF(OR(B25="",D25=""),"",B25-D25)</f>
-        <v/>
-      </c>
-      <c r="F25" s="38"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="38"/>
-      <c r="B26" s="34"/>
-      <c r="C26" s="38"/>
-      <c r="D26" s="34"/>
-      <c r="E26" s="12" t="str">
-        <f aca="false">IF(OR(B26="",D26=""),"",B26-D26)</f>
-        <v/>
-      </c>
-      <c r="F26" s="38"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="38"/>
-      <c r="B27" s="34"/>
-      <c r="C27" s="38"/>
-      <c r="D27" s="34"/>
-      <c r="E27" s="12" t="str">
-        <f aca="false">IF(OR(B27="",D27=""),"",B27-D27)</f>
-        <v/>
-      </c>
-      <c r="F27" s="38"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="38"/>
-      <c r="B28" s="34"/>
-      <c r="C28" s="38"/>
-      <c r="D28" s="34"/>
-      <c r="E28" s="12" t="str">
-        <f aca="false">IF(OR(B28="",D28=""),"",B28-D28)</f>
-        <v/>
-      </c>
-      <c r="F28" s="38"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="38"/>
-      <c r="B29" s="34"/>
-      <c r="C29" s="38"/>
-      <c r="D29" s="34"/>
-      <c r="E29" s="12" t="str">
-        <f aca="false">IF(OR(B29="",D29=""),"",B29-D29)</f>
-        <v/>
-      </c>
-      <c r="F29" s="38"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="38"/>
-      <c r="B30" s="34"/>
-      <c r="C30" s="38"/>
-      <c r="D30" s="34"/>
-      <c r="E30" s="12" t="str">
-        <f aca="false">IF(OR(B30="",D30=""),"",B30-D30)</f>
-        <v/>
-      </c>
-      <c r="F30" s="38"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="38"/>
-      <c r="B31" s="34"/>
-      <c r="C31" s="38"/>
-      <c r="D31" s="34"/>
-      <c r="E31" s="12" t="str">
-        <f aca="false">IF(OR(B31="",D31=""),"",B31-D31)</f>
-        <v/>
-      </c>
-      <c r="F31" s="38"/>
+      <c r="C55" s="12" t="n">
+        <v>-1000000</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E55" s="3" t="s">
+        <v>669</v>
+      </c>
+      <c r="F55" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G55" s="3" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="3" t="s">
+        <v>505</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="C56" s="12" t="n">
+        <v>200000</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="E56" s="38" t="s">
+        <v>680</v>
+      </c>
+      <c r="F56" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G56" s="38" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="3" t="s">
+        <v>505</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="C57" s="12" t="n">
+        <v>1650249</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="E57" s="38" t="s">
+        <v>665</v>
+      </c>
+      <c r="F57" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G57" s="38" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="3" t="s">
+        <v>505</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>686</v>
+      </c>
+      <c r="C58" s="12" t="n">
+        <v>-83300</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E58" s="38" t="s">
+        <v>679</v>
+      </c>
+      <c r="F58" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G58" s="38" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="C59" s="12" t="n">
+        <v>-225000</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E59" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F59" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G59" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C60" s="12" t="n">
+        <v>-16000</v>
+      </c>
+      <c r="D60" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E60" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F60" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G60" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C61" s="12" t="n">
+        <v>-15000</v>
+      </c>
+      <c r="D61" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E61" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F61" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G61" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="3" t="s">
+        <v>438</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C62" s="12" t="n">
+        <v>-6000</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E62" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F62" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G62" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="3" t="s">
+        <v>438</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C63" s="12" t="n">
+        <v>-6800</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E63" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F63" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G63" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="3" t="s">
+        <v>438</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C64" s="12" t="n">
+        <v>-30000</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E64" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F64" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G64" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="3" t="s">
+        <v>438</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C65" s="12" t="n">
+        <v>-50000</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E65" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F65" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G65" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="3" t="s">
+        <v>438</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C66" s="12" t="n">
+        <v>-15000</v>
+      </c>
+      <c r="D66" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E66" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F66" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G66" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>616</v>
+      </c>
+      <c r="C67" s="12" t="n">
+        <v>2813595</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="E67" s="3" t="s">
+        <v>687</v>
+      </c>
+      <c r="F67" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G67" s="3" t="s">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C68" s="12" t="n">
+        <v>-50000</v>
+      </c>
+      <c r="D68" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E68" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F68" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G68" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="C69" s="12" t="n">
+        <v>-150000</v>
+      </c>
+      <c r="D69" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E69" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F69" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G69" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="C70" s="12" t="n">
+        <v>-19145</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E70" s="3" t="s">
+        <v>669</v>
+      </c>
+      <c r="F70" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G70" s="3" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>689</v>
+      </c>
+      <c r="C71" s="12" t="n">
+        <v>-25000</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E71" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F71" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G71" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C72" s="12" t="n">
+        <v>-70000</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E72" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F72" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G72" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C73" s="12" t="n">
+        <v>-250000</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E73" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F73" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G73" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="C74" s="12" t="n">
+        <v>-55000</v>
+      </c>
+      <c r="D74" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E74" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F74" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G74" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="C75" s="12" t="n">
+        <v>-300000</v>
+      </c>
+      <c r="D75" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E75" s="38" t="s">
+        <v>681</v>
+      </c>
+      <c r="F75" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G75" s="38" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="C76" s="12" t="n">
+        <v>-400000</v>
+      </c>
+      <c r="D76" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E76" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F76" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G76" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="B77" s="3" t="s">
+        <v>617</v>
+      </c>
+      <c r="C77" s="12" t="n">
+        <v>-1000000</v>
+      </c>
+      <c r="D77" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E77" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F77" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G77" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="C78" s="12" t="n">
+        <v>-300000</v>
+      </c>
+      <c r="D78" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E78" s="38" t="s">
+        <v>681</v>
+      </c>
+      <c r="F78" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G78" s="38" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>668</v>
+      </c>
+      <c r="C79" s="12" t="n">
+        <v>-1000000</v>
+      </c>
+      <c r="D79" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E79" s="3" t="s">
+        <v>669</v>
+      </c>
+      <c r="F79" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G79" s="3" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="B80" s="3" t="s">
+        <v>418</v>
+      </c>
+      <c r="C80" s="12" t="n">
+        <v>760000</v>
+      </c>
+      <c r="D80" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="E80" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F80" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G80" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="3" t="s">
+        <v>440</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="C81" s="12" t="n">
+        <v>-32000</v>
+      </c>
+      <c r="D81" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E81" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F81" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G81" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="3" t="s">
+        <v>440</v>
+      </c>
+      <c r="B82" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C82" s="12" t="n">
+        <v>-17000</v>
+      </c>
+      <c r="D82" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E82" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F82" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G82" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="3" t="s">
+        <v>440</v>
+      </c>
+      <c r="B83" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C83" s="12" t="n">
+        <v>-15000</v>
+      </c>
+      <c r="D83" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E83" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F83" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G83" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="3" t="s">
+        <v>440</v>
+      </c>
+      <c r="B84" s="3" t="s">
+        <v>618</v>
+      </c>
+      <c r="C84" s="12" t="n">
+        <v>-9471</v>
+      </c>
+      <c r="D84" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E84" s="3" t="s">
+        <v>690</v>
+      </c>
+      <c r="F84" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G84" s="3" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="3" t="s">
+        <v>532</v>
+      </c>
+      <c r="B85" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C85" s="12" t="n">
+        <v>-12000</v>
+      </c>
+      <c r="D85" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E85" s="38" t="s">
+        <v>681</v>
+      </c>
+      <c r="F85" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G85" s="38" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="3" t="s">
+        <v>532</v>
+      </c>
+      <c r="B86" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C86" s="12" t="n">
+        <v>-12000</v>
+      </c>
+      <c r="D86" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E86" s="38" t="s">
+        <v>681</v>
+      </c>
+      <c r="F86" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G86" s="38" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="3" t="s">
+        <v>532</v>
+      </c>
+      <c r="B87" s="3" t="s">
+        <v>619</v>
+      </c>
+      <c r="C87" s="12" t="n">
+        <v>-31319</v>
+      </c>
+      <c r="D87" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E87" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F87" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G87" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="3" t="s">
+        <v>532</v>
+      </c>
+      <c r="B88" s="3" t="s">
+        <v>616</v>
+      </c>
+      <c r="C88" s="12" t="n">
+        <v>2234722</v>
+      </c>
+      <c r="D88" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="E88" s="3" t="s">
+        <v>687</v>
+      </c>
+      <c r="F88" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G88" s="3" t="s">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="3" t="s">
+        <v>532</v>
+      </c>
+      <c r="B89" s="3" t="s">
+        <v>668</v>
+      </c>
+      <c r="C89" s="12" t="n">
+        <v>-160000</v>
+      </c>
+      <c r="D89" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E89" s="3" t="s">
+        <v>669</v>
+      </c>
+      <c r="F89" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G89" s="3" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="3" t="s">
+        <v>532</v>
+      </c>
+      <c r="B90" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="C90" s="12" t="n">
+        <v>198000</v>
+      </c>
+      <c r="D90" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="E90" s="38" t="s">
+        <v>665</v>
+      </c>
+      <c r="F90" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G90" s="38" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="3" t="s">
+        <v>532</v>
+      </c>
+      <c r="B91" s="3" t="s">
+        <v>668</v>
+      </c>
+      <c r="C91" s="12" t="n">
+        <v>-150000</v>
+      </c>
+      <c r="D91" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E91" s="3" t="s">
+        <v>669</v>
+      </c>
+      <c r="F91" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G91" s="3" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="3" t="s">
+        <v>542</v>
+      </c>
+      <c r="B92" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C92" s="12" t="n">
+        <v>-16000</v>
+      </c>
+      <c r="D92" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E92" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F92" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G92" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="3" t="s">
+        <v>542</v>
+      </c>
+      <c r="B93" s="3" t="s">
+        <v>620</v>
+      </c>
+      <c r="C93" s="12" t="n">
+        <v>-5770</v>
+      </c>
+      <c r="D93" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E93" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F93" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G93" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="3" t="s">
+        <v>542</v>
+      </c>
+      <c r="B94" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="C94" s="12" t="n">
+        <v>-15000</v>
+      </c>
+      <c r="D94" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E94" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F94" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G94" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="3" t="s">
+        <v>542</v>
+      </c>
+      <c r="B95" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C95" s="12" t="n">
+        <v>-20000</v>
+      </c>
+      <c r="D95" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E95" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F95" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G95" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="3" t="s">
+        <v>542</v>
+      </c>
+      <c r="B96" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="C96" s="12" t="n">
+        <v>-50000</v>
+      </c>
+      <c r="D96" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E96" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F96" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G96" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="3" t="s">
+        <v>542</v>
+      </c>
+      <c r="B97" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="C97" s="12" t="n">
+        <v>-350000</v>
+      </c>
+      <c r="D97" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E97" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F97" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G97" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="3" t="s">
+        <v>542</v>
+      </c>
+      <c r="B98" s="3" t="s">
+        <v>691</v>
+      </c>
+      <c r="C98" s="12" t="n">
+        <v>-405600</v>
+      </c>
+      <c r="D98" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E98" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F98" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G98" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="3" t="s">
+        <v>542</v>
+      </c>
+      <c r="B99" s="3" t="s">
+        <v>668</v>
+      </c>
+      <c r="C99" s="12" t="n">
+        <v>-1000000</v>
+      </c>
+      <c r="D99" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E99" s="3" t="s">
+        <v>669</v>
+      </c>
+      <c r="F99" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G99" s="3" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="3" t="s">
+        <v>546</v>
+      </c>
+      <c r="B100" s="3" t="s">
+        <v>614</v>
+      </c>
+      <c r="C100" s="12" t="n">
+        <v>-19999</v>
+      </c>
+      <c r="D100" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E100" s="38" t="s">
+        <v>679</v>
+      </c>
+      <c r="F100" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G100" s="38" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="3" t="s">
+        <v>546</v>
+      </c>
+      <c r="B101" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="C101" s="12" t="n">
+        <v>-20000</v>
+      </c>
+      <c r="D101" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E101" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F101" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G101" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="3" t="s">
+        <v>546</v>
+      </c>
+      <c r="B102" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C102" s="12" t="n">
+        <v>-20000</v>
+      </c>
+      <c r="D102" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E102" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F102" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G102" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="3" t="s">
+        <v>546</v>
+      </c>
+      <c r="B103" s="3" t="s">
+        <v>614</v>
+      </c>
+      <c r="C103" s="12" t="n">
+        <v>-19781</v>
+      </c>
+      <c r="D103" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E103" s="38" t="s">
+        <v>679</v>
+      </c>
+      <c r="F103" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G103" s="38" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="3" t="s">
+        <v>546</v>
+      </c>
+      <c r="B104" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="C104" s="12" t="n">
+        <v>-29000</v>
+      </c>
+      <c r="D104" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E104" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F104" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G104" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="3" t="s">
+        <v>546</v>
+      </c>
+      <c r="B105" s="3" t="s">
+        <v>621</v>
+      </c>
+      <c r="C105" s="12" t="n">
+        <v>357000</v>
+      </c>
+      <c r="D105" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="E105" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F105" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G105" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="3" t="s">
+        <v>546</v>
+      </c>
+      <c r="B106" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C106" s="12" t="n">
+        <v>-20000</v>
+      </c>
+      <c r="D106" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E106" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F106" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G106" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="B107" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="C107" s="12" t="n">
+        <v>-25000</v>
+      </c>
+      <c r="D107" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E107" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F107" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G107" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="B108" s="3" t="s">
+        <v>623</v>
+      </c>
+      <c r="C108" s="12" t="n">
+        <v>-4200</v>
+      </c>
+      <c r="D108" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E108" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F108" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G108" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="B109" s="3" t="s">
+        <v>623</v>
+      </c>
+      <c r="C109" s="12" t="n">
+        <v>-6700</v>
+      </c>
+      <c r="D109" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E109" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F109" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G109" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="B110" s="3" t="s">
+        <v>692</v>
+      </c>
+      <c r="C110" s="12" t="n">
+        <v>-6950</v>
+      </c>
+      <c r="D110" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E110" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F110" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G110" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="B111" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C111" s="12" t="n">
+        <v>-12000</v>
+      </c>
+      <c r="D111" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E111" s="38" t="s">
+        <v>681</v>
+      </c>
+      <c r="F111" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G111" s="38" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="B112" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C112" s="12" t="n">
+        <v>-15000</v>
+      </c>
+      <c r="D112" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E112" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F112" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G112" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="B113" s="3" t="s">
+        <v>623</v>
+      </c>
+      <c r="C113" s="12" t="n">
+        <v>-16500</v>
+      </c>
+      <c r="D113" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E113" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F113" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G113" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="B114" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C114" s="12" t="n">
+        <v>-3000</v>
+      </c>
+      <c r="D114" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E114" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F114" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G114" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="B115" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="C115" s="12" t="n">
+        <v>-18000</v>
+      </c>
+      <c r="D115" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E115" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F115" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G115" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="B116" s="3" t="s">
+        <v>693</v>
+      </c>
+      <c r="C116" s="12" t="n">
+        <v>-38000</v>
+      </c>
+      <c r="D116" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E116" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F116" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G116" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="B117" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C117" s="12" t="n">
+        <v>-70000</v>
+      </c>
+      <c r="D117" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E117" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F117" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G117" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="B118" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="C118" s="12" t="n">
+        <v>-60000</v>
+      </c>
+      <c r="D118" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E118" s="38" t="s">
+        <v>681</v>
+      </c>
+      <c r="F118" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G118" s="38" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="B119" s="3" t="s">
+        <v>694</v>
+      </c>
+      <c r="C119" s="12" t="n">
+        <v>-66878</v>
+      </c>
+      <c r="D119" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E119" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F119" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G119" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="B120" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="C120" s="12" t="n">
+        <v>-80000</v>
+      </c>
+      <c r="D120" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E120" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F120" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G120" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="B121" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C121" s="12" t="n">
+        <v>-120000</v>
+      </c>
+      <c r="D121" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E121" s="38" t="s">
+        <v>681</v>
+      </c>
+      <c r="F121" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G121" s="38" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="B122" s="3" t="s">
+        <v>695</v>
+      </c>
+      <c r="C122" s="12" t="n">
+        <v>-296037</v>
+      </c>
+      <c r="D122" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E122" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F122" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G122" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="B123" s="3" t="s">
+        <v>622</v>
+      </c>
+      <c r="C123" s="12" t="n">
+        <v>200000</v>
+      </c>
+      <c r="D123" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="E123" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F123" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G123" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="B124" s="3" t="s">
+        <v>622</v>
+      </c>
+      <c r="C124" s="12" t="n">
+        <v>490200</v>
+      </c>
+      <c r="D124" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="E124" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F124" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G124" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A125" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="B125" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="C125" s="12" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D125" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="E125" s="38" t="s">
+        <v>680</v>
+      </c>
+      <c r="F125" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G125" s="38" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A126" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="B126" s="3" t="s">
+        <v>696</v>
+      </c>
+      <c r="C126" s="12" t="n">
+        <v>-58001</v>
+      </c>
+      <c r="D126" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E126" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F126" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G126" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="3" t="s">
+        <v>572</v>
+      </c>
+      <c r="B127" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C127" s="12" t="n">
+        <v>-15000</v>
+      </c>
+      <c r="D127" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E127" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F127" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G127" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A128" s="3" t="s">
+        <v>572</v>
+      </c>
+      <c r="B128" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C128" s="12" t="n">
+        <v>-20000</v>
+      </c>
+      <c r="D128" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E128" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F128" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G128" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="3" t="s">
+        <v>572</v>
+      </c>
+      <c r="B129" s="3" t="s">
+        <v>697</v>
+      </c>
+      <c r="C129" s="12" t="n">
+        <v>-97000</v>
+      </c>
+      <c r="D129" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E129" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F129" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G129" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="3" t="s">
+        <v>572</v>
+      </c>
+      <c r="B130" s="3" t="s">
+        <v>668</v>
+      </c>
+      <c r="C130" s="12" t="n">
+        <v>-800000</v>
+      </c>
+      <c r="D130" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E130" s="3" t="s">
+        <v>669</v>
+      </c>
+      <c r="F130" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G130" s="3" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A131" s="3" t="s">
+        <v>572</v>
+      </c>
+      <c r="B131" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="C131" s="12" t="n">
+        <v>-170000</v>
+      </c>
+      <c r="D131" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E131" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F131" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G131" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="3" t="s">
+        <v>572</v>
+      </c>
+      <c r="B132" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="C132" s="12" t="n">
+        <v>-100000</v>
+      </c>
+      <c r="D132" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E132" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F132" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G132" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="B133" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="C133" s="12" t="n">
+        <v>-50000</v>
+      </c>
+      <c r="D133" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E133" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F133" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G133" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A134" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="B134" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C134" s="12" t="n">
+        <v>-12000</v>
+      </c>
+      <c r="D134" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E134" s="38" t="s">
+        <v>681</v>
+      </c>
+      <c r="F134" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G134" s="38" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A135" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="B135" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C135" s="12" t="n">
+        <v>-12000</v>
+      </c>
+      <c r="D135" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E135" s="38" t="s">
+        <v>681</v>
+      </c>
+      <c r="F135" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G135" s="38" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A136" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="B136" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="C136" s="12" t="n">
+        <v>-39000</v>
+      </c>
+      <c r="D136" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E136" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F136" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G136" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="B137" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C137" s="12" t="n">
+        <v>-53000</v>
+      </c>
+      <c r="D137" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E137" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F137" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G137" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A138" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="B138" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="C138" s="12" t="n">
+        <v>500000</v>
+      </c>
+      <c r="D138" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="E138" s="38" t="s">
+        <v>665</v>
+      </c>
+      <c r="F138" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G138" s="38" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A139" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="B139" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C139" s="12" t="n">
+        <v>-100000</v>
+      </c>
+      <c r="D139" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E139" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F139" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G139" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A140" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="B140" s="3" t="s">
+        <v>668</v>
+      </c>
+      <c r="C140" s="12" t="n">
+        <v>-700000</v>
+      </c>
+      <c r="D140" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E140" s="3" t="s">
+        <v>669</v>
+      </c>
+      <c r="F140" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G140" s="3" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A141" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="B141" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="C141" s="12" t="n">
+        <v>500000</v>
+      </c>
+      <c r="D141" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="E141" s="38" t="s">
+        <v>680</v>
+      </c>
+      <c r="F141" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G141" s="38" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A142" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="B142" s="3" t="s">
+        <v>614</v>
+      </c>
+      <c r="C142" s="12" t="n">
+        <v>-76668</v>
+      </c>
+      <c r="D142" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E142" s="38" t="s">
+        <v>679</v>
+      </c>
+      <c r="F142" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G142" s="38" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A143" s="3" t="s">
+        <v>448</v>
+      </c>
+      <c r="B143" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C143" s="12" t="n">
+        <v>-20000</v>
+      </c>
+      <c r="D143" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E143" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F143" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G143" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A144" s="3" t="s">
+        <v>448</v>
+      </c>
+      <c r="B144" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C144" s="12" t="n">
+        <v>-20000</v>
+      </c>
+      <c r="D144" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E144" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F144" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G144" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A145" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="B145" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="C145" s="12" t="n">
+        <v>-24000</v>
+      </c>
+      <c r="D145" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E145" s="38" t="s">
+        <v>681</v>
+      </c>
+      <c r="F145" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G145" s="38" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A146" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="B146" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="C146" s="12" t="n">
+        <v>4625470</v>
+      </c>
+      <c r="D146" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="E146" s="3" t="s">
+        <v>687</v>
+      </c>
+      <c r="F146" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G146" s="3" t="s">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A147" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="B147" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C147" s="12" t="n">
+        <v>-250000</v>
+      </c>
+      <c r="D147" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E147" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F147" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G147" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A148" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="B148" s="3" t="s">
+        <v>614</v>
+      </c>
+      <c r="C148" s="12" t="n">
+        <v>-71822</v>
+      </c>
+      <c r="D148" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E148" s="38" t="s">
+        <v>679</v>
+      </c>
+      <c r="F148" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="G148" s="38" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A149" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="B149" s="3" t="s">
+        <v>698</v>
+      </c>
+      <c r="C149" s="12" t="n">
+        <v>-46550</v>
+      </c>
+      <c r="D149" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E149" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="F149" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G149" s="38" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A150" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="B150" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C150" s="12" t="n">
+        <v>-30000</v>
+      </c>
+      <c r="D150" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E150" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F150" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G150" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A151" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="B151" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C151" s="12" t="n">
+        <v>-6000</v>
+      </c>
+      <c r="D151" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E151" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="F151" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="G151" s="38" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A153" s="2" t="s">
+        <v>699</v>
+      </c>
+      <c r="B153" s="2"/>
+      <c r="C153" s="2"/>
+      <c r="D153" s="2"/>
+      <c r="E153" s="2"/>
+      <c r="F153" s="2"/>
+      <c r="G153" s="2"/>
+    </row>
+    <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A154" s="9" t="s">
+        <v>700</v>
+      </c>
+      <c r="B154" s="9" t="s">
+        <v>701</v>
+      </c>
+      <c r="C154" s="9" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A155" s="3" t="s">
+        <v>672</v>
+      </c>
+      <c r="B155" s="3" t="n">
+        <v>72</v>
+      </c>
+      <c r="C155" s="12" t="n">
+        <v>-6656800</v>
+      </c>
+    </row>
+    <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A156" s="3" t="s">
+        <v>669</v>
+      </c>
+      <c r="B156" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C156" s="12" t="n">
+        <v>-6159145</v>
+      </c>
+    </row>
+    <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A157" s="3" t="s">
+        <v>681</v>
+      </c>
+      <c r="B157" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="C157" s="12" t="n">
+        <v>-1200000</v>
+      </c>
+    </row>
+    <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A158" s="3" t="s">
+        <v>679</v>
+      </c>
+      <c r="B158" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="C158" s="12" t="n">
+        <v>-730211</v>
+      </c>
+    </row>
+    <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A159" s="3" t="s">
+        <v>690</v>
+      </c>
+      <c r="B159" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C159" s="12" t="n">
+        <v>-9471</v>
+      </c>
+    </row>
+    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A160" s="3" t="s">
+        <v>675</v>
+      </c>
+      <c r="B160" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="C160" s="12" t="n">
+        <v>1620714</v>
+      </c>
+    </row>
+    <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A161" s="3" t="s">
+        <v>680</v>
+      </c>
+      <c r="B161" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C161" s="12" t="n">
+        <v>2900000</v>
+      </c>
+    </row>
+    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A162" s="3" t="s">
+        <v>665</v>
+      </c>
+      <c r="B162" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C162" s="12" t="n">
+        <v>4674721</v>
+      </c>
+    </row>
+    <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A163" s="3" t="s">
+        <v>687</v>
+      </c>
+      <c r="B163" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C163" s="12" t="n">
+        <v>9673787</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:F2"/>
+  <mergeCells count="3">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A153:G153"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Categorizacion final (RCV+web cruzados) e Informe de Resultados Julio 2026 real en Resumen_Ejecutivo
</commit_message>
<xml_diff>
--- a/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
+++ b/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3000" uniqueCount="714">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3025" uniqueCount="739">
   <si>
     <t xml:space="preserve">SUPUESTOS DEL PRESUPUESTO — SOLLEM + TRAST</t>
   </si>
@@ -1978,6 +1978,51 @@
     <t xml:space="preserve">Este informe usa valores NETOS (sin IVA) — es la utilidad real, distinta del Saldo de caja semanal (que incluye IVA cobrado, aún no pagado al Fisco). Ver hoja Consolidado para el detalle completo.</t>
   </si>
   <si>
+    <t xml:space="preserve">INFORME DE RESULTADOS FINANCIEROS — JULIO 2026 (REAL, mes cerrado)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Julio 2026 (Real)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingreso Neto (ventas, RCV 8 facturas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Combustible (real, Aramco+Copec vía cartola)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neumáticos (real, Vulko SPA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mantención (real, RCV cruzado)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viático (real, cartola)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gastos de Representación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remuneración Administrativa (sin desglose exacto — ver nota)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Factoring (costo real: 3 comprobantes reales)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Julio NO tiene presupuesto formal (el sistema de presupuesto formal parte en Agosto) — por eso esta tabla no tiene columna de comparación, solo el real.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costos en base CASH (lo que efectivamente salió del banco en julio), cruzados 1 a 1 contra RCV Compra/Venta y comprobantes reales donde existen (Vulko, Construmart, Cardánica, factoring) — no son supuestos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Remuneración Administrativa' ($6.656.800) es el bloque menos confiable: son 72 transferencias a personas sin desglose exacto de si son sueldo, viático o anticipo — la heurística solo separó Viático cuando el monto era múltiplo exacto de $12.000. Es probable que parte de este monto sea realmente Sueldo Conductor mal clasificado, lo que subestimaría el margen real un poco menos negativo de lo mostrado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo de Factoring ($459.420) = suma de los 3 comprobantes reales de julio: folio 20+bundle $158.549, folio 22 $152.894 (dato previo de Kaptura, sin comprobante propio revisado esta sesión), folio 28 $147.977 (LATAM Trade Capital, comprobante real).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Utilidad negativa es consistente con el subregistro ya documentado: el Ingreso Neto usado (RCV, $12.340.900) probablemente no refleja todos los servicios reales ejecutados en julio — cargar los servicios de julio en Kaptura sigue siendo el pendiente que más cambiaría este número.</t>
+  </si>
+  <si>
     <t xml:space="preserve">PLAN vs. REAL vs. REPROYECCIÓN (flujo de caja semanal)</t>
   </si>
   <si>
@@ -2077,16 +2122,28 @@
     <t xml:space="preserve">otro_por_clasificar</t>
   </si>
   <si>
-    <t xml:space="preserve">Baja — revisar manualmente</t>
+    <t xml:space="preserve">Baja — evidencia agotada (RCV+web), sin identificar</t>
   </si>
   <si>
     <t xml:space="preserve">Compra Nacional MD VALPAR LTDA.</t>
   </si>
   <si>
+    <t xml:space="preserve">mantencion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alta — RCV exacto o proveedor confirmado</t>
+  </si>
+  <si>
     <t xml:space="preserve">Compra Nacional MD IMPLEMENTOS S.A</t>
   </si>
   <si>
-    <t xml:space="preserve">mantencion</t>
+    <t xml:space="preserve">cobro_cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">comercial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alta — pago parcial El Enano SPA, RCV folio 12 junio</t>
   </si>
   <si>
     <t xml:space="preserve">aporte_retiro_socio</t>
@@ -2098,15 +2155,27 @@
     <t xml:space="preserve">Media — heurística por monto múltiplo $12.000</t>
   </si>
   <si>
+    <t xml:space="preserve">Sin clasificar — instrucción explícita del usuario</t>
+  </si>
+  <si>
     <t xml:space="preserve">0780993812 Transf. LOGISTICA Y TRA</t>
   </si>
   <si>
+    <t xml:space="preserve">Alta — RCV folio 19/2, Alfa Jam / Santa Berenice</t>
+  </si>
+  <si>
     <t xml:space="preserve">Compra Nacional MD TTP S.A RANCAGU</t>
   </si>
   <si>
     <t xml:space="preserve">Compra Nacional MD COMERCIAL ECUAD</t>
   </si>
   <si>
+    <t xml:space="preserve">gastos_representacion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alta — confirmado por el usuario (alimentación)</t>
+  </si>
+  <si>
     <t xml:space="preserve">0772640749 Transf a Fijasur</t>
   </si>
   <si>
@@ -2123,6 +2192,12 @@
   </si>
   <si>
     <t xml:space="preserve">Compra Nacional MD VULKO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">neumaticos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alta — RCV exacto folio 119271, Vulko SPA (vulcanización)</t>
   </si>
   <si>
     <t xml:space="preserve">Compra Nacional MD FEDICAR</t>
@@ -3246,7 +3321,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>703</v>
+        <v>728</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3256,7 +3331,7 @@
     </row>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="24" t="s">
-        <v>704</v>
+        <v>729</v>
       </c>
       <c r="B2" s="24"/>
       <c r="C2" s="24"/>
@@ -3269,16 +3344,16 @@
         <v>376</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>705</v>
+        <v>730</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>706</v>
+        <v>731</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>707</v>
+        <v>732</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>708</v>
+        <v>733</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>188</v>
@@ -3292,23 +3367,23 @@
         <v>63371</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>709</v>
+        <v>734</v>
       </c>
       <c r="D5" s="37"/>
       <c r="E5" s="37"/>
       <c r="F5" s="3" t="s">
-        <v>710</v>
+        <v>735</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>711</v>
+        <v>736</v>
       </c>
       <c r="B6" s="12" t="n">
         <v>1275801</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>712</v>
+        <v>737</v>
       </c>
       <c r="D6" s="34"/>
       <c r="E6" s="12" t="str">
@@ -3316,7 +3391,7 @@
         <v/>
       </c>
       <c r="F6" s="3" t="s">
-        <v>713</v>
+        <v>738</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15384,7 +15459,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -15580,261 +15655,479 @@
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="28" t="s">
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B21" s="9" t="s">
         <v>646</v>
       </c>
-      <c r="B21" s="28"/>
-      <c r="C21" s="28"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="28"/>
-      <c r="F21" s="28"/>
-      <c r="G21" s="28"/>
+      <c r="C21" s="9"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="3" t="s">
         <v>647</v>
       </c>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-    </row>
-    <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="9" t="s">
+      <c r="B22" s="12" t="n">
+        <v>12340900</v>
+      </c>
+      <c r="C22" s="12"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
+        <v>642</v>
+      </c>
+      <c r="B23" s="12" t="n">
+        <v>2344771</v>
+      </c>
+      <c r="C23" s="12"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="B24" s="17" t="n">
+        <v>14685671</v>
+      </c>
+      <c r="C24" s="17"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="s">
+        <v>648</v>
+      </c>
+      <c r="B25" s="12" t="n">
+        <v>-6159145</v>
+      </c>
+      <c r="C25" s="12"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="s">
+        <v>649</v>
+      </c>
+      <c r="B26" s="12" t="n">
+        <v>-405600</v>
+      </c>
+      <c r="C26" s="12"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="3" t="s">
+        <v>650</v>
+      </c>
+      <c r="B27" s="12" t="n">
+        <v>-1385644</v>
+      </c>
+      <c r="C27" s="12"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="3" t="s">
+        <v>651</v>
+      </c>
+      <c r="B28" s="12" t="n">
+        <v>-1200000</v>
+      </c>
+      <c r="C28" s="12"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="3" t="s">
+        <v>652</v>
+      </c>
+      <c r="B29" s="12" t="n">
+        <v>-31955</v>
+      </c>
+      <c r="C29" s="12"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="B30" s="17" t="n">
+        <v>-9182344</v>
+      </c>
+      <c r="C30" s="17"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="15" t="s">
+        <v>643</v>
+      </c>
+      <c r="B31" s="17" t="n">
+        <v>3158556</v>
+      </c>
+      <c r="C31" s="17"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="3" t="s">
+        <v>653</v>
+      </c>
+      <c r="B32" s="12" t="n">
+        <v>-6656800</v>
+      </c>
+      <c r="C32" s="12"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="3" t="s">
+        <v>654</v>
+      </c>
+      <c r="B33" s="12" t="n">
+        <v>-459420</v>
+      </c>
+      <c r="C33" s="12"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="B34" s="17" t="n">
+        <v>-3957664</v>
+      </c>
+      <c r="C34" s="17"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="B35" s="27" t="n">
+        <v>-0.269491533618042</v>
+      </c>
+      <c r="C35" s="27"/>
+    </row>
+    <row r="37" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="24" t="s">
+        <v>655</v>
+      </c>
+      <c r="B37" s="24"/>
+      <c r="C37" s="24"/>
+      <c r="D37" s="24"/>
+      <c r="E37" s="24"/>
+      <c r="F37" s="24"/>
+      <c r="G37" s="24"/>
+    </row>
+    <row r="38" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="24" t="s">
+        <v>656</v>
+      </c>
+      <c r="B38" s="24"/>
+      <c r="C38" s="24"/>
+      <c r="D38" s="24"/>
+      <c r="E38" s="24"/>
+      <c r="F38" s="24"/>
+      <c r="G38" s="24"/>
+    </row>
+    <row r="39" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="24" t="s">
+        <v>657</v>
+      </c>
+      <c r="B39" s="24"/>
+      <c r="C39" s="24"/>
+      <c r="D39" s="24"/>
+      <c r="E39" s="24"/>
+      <c r="F39" s="24"/>
+      <c r="G39" s="24"/>
+    </row>
+    <row r="40" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="24" t="s">
+        <v>658</v>
+      </c>
+      <c r="B40" s="24"/>
+      <c r="C40" s="24"/>
+      <c r="D40" s="24"/>
+      <c r="E40" s="24"/>
+      <c r="F40" s="24"/>
+      <c r="G40" s="24"/>
+    </row>
+    <row r="41" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="24" t="s">
+        <v>659</v>
+      </c>
+      <c r="B41" s="24"/>
+      <c r="C41" s="24"/>
+      <c r="D41" s="24"/>
+      <c r="E41" s="24"/>
+      <c r="F41" s="24"/>
+      <c r="G41" s="24"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="2" t="s">
+        <v>660</v>
+      </c>
+      <c r="B43" s="2"/>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+      <c r="E43" s="2"/>
+      <c r="F43" s="2"/>
+      <c r="G43" s="2"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="28" t="s">
+        <v>661</v>
+      </c>
+      <c r="B44" s="28"/>
+      <c r="C44" s="28"/>
+      <c r="D44" s="28"/>
+      <c r="E44" s="28"/>
+      <c r="F44" s="28"/>
+      <c r="G44" s="28"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="2" t="s">
+        <v>662</v>
+      </c>
+      <c r="B45" s="2"/>
+      <c r="C45" s="2"/>
+      <c r="D45" s="2"/>
+      <c r="E45" s="2"/>
+      <c r="F45" s="2"/>
+      <c r="G45" s="2"/>
+    </row>
+    <row r="46" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="B23" s="9" t="s">
-        <v>648</v>
-      </c>
-      <c r="C23" s="9" t="s">
-        <v>649</v>
-      </c>
-      <c r="D23" s="9" t="s">
-        <v>650</v>
-      </c>
-      <c r="E23" s="9" t="s">
-        <v>651</v>
-      </c>
-      <c r="F23" s="9" t="s">
-        <v>652</v>
-      </c>
-      <c r="G23" s="9" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="s">
-        <v>654</v>
-      </c>
-      <c r="B24" s="33" t="n">
+      <c r="B46" s="9" t="s">
+        <v>663</v>
+      </c>
+      <c r="C46" s="9" t="s">
+        <v>664</v>
+      </c>
+      <c r="D46" s="9" t="s">
+        <v>665</v>
+      </c>
+      <c r="E46" s="9" t="s">
+        <v>666</v>
+      </c>
+      <c r="F46" s="9" t="s">
+        <v>667</v>
+      </c>
+      <c r="G46" s="9" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="3" t="s">
+        <v>669</v>
+      </c>
+      <c r="B47" s="33" t="n">
         <f aca="false">Consolidado!B32</f>
         <v>29402660.3612933</v>
       </c>
-      <c r="C24" s="12" t="n">
+      <c r="C47" s="12" t="n">
         <f aca="false">SUM(Real_vs_Presupuesto!C6:C11)</f>
         <v>0</v>
       </c>
-      <c r="D24" s="35" t="str">
+      <c r="D47" s="35" t="str">
         <f aca="false">COUNT(Real_vs_Presupuesto!C6:C11)&amp;" de 6"</f>
         <v>0 de 6</v>
       </c>
-      <c r="E24" s="12" t="n">
+      <c r="E47" s="12" t="n">
         <f aca="false">SUMIF(Real_vs_Presupuesto!C6:C11,"",Real_vs_Presupuesto!B6:B11)</f>
         <v>29402660.3612933</v>
       </c>
-      <c r="F24" s="14" t="n">
-        <f aca="false">C24+E24</f>
+      <c r="F47" s="14" t="n">
+        <f aca="false">C47+E47</f>
         <v>29402660.3612933</v>
       </c>
-      <c r="G24" s="27" t="n">
-        <f aca="false">F24/B24</f>
+      <c r="G47" s="27" t="n">
+        <f aca="false">F47/B47</f>
         <v>1</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
-        <v>655</v>
-      </c>
-      <c r="B25" s="33" t="n">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="B48" s="33" t="n">
         <f aca="false">Consolidado!C32</f>
         <v>26434798.4092921</v>
       </c>
-      <c r="C25" s="12" t="n">
+      <c r="C48" s="12" t="n">
         <f aca="false">SUM(Real_vs_Presupuesto!F6:F11)</f>
         <v>0</v>
       </c>
-      <c r="D25" s="35" t="str">
+      <c r="D48" s="35" t="str">
         <f aca="false">COUNT(Real_vs_Presupuesto!F6:F11)&amp;" de 6"</f>
         <v>0 de 6</v>
       </c>
-      <c r="E25" s="12" t="n">
+      <c r="E48" s="12" t="n">
         <f aca="false">SUMIF(Real_vs_Presupuesto!F6:F11,"",Real_vs_Presupuesto!E6:E11)</f>
         <v>26434798.4092921</v>
       </c>
-      <c r="F25" s="14" t="n">
-        <f aca="false">C25+E25</f>
+      <c r="F48" s="14" t="n">
+        <f aca="false">C48+E48</f>
         <v>26434798.4092921</v>
       </c>
-      <c r="G25" s="27" t="n">
-        <f aca="false">F25/B25</f>
+      <c r="G48" s="27" t="n">
+        <f aca="false">F48/B48</f>
         <v>1</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="18" t="s">
-        <v>656</v>
-      </c>
-      <c r="B26" s="14" t="n">
-        <f aca="false">B24-B25</f>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="18" t="s">
+        <v>671</v>
+      </c>
+      <c r="B49" s="14" t="n">
+        <f aca="false">B47-B48</f>
         <v>2967861.9520012</v>
       </c>
-      <c r="C26" s="14" t="n">
-        <f aca="false">C24-C25</f>
+      <c r="C49" s="14" t="n">
+        <f aca="false">C47-C48</f>
         <v>0</v>
       </c>
-      <c r="D26" s="37"/>
-      <c r="E26" s="14" t="n">
-        <f aca="false">E24-E25</f>
+      <c r="D49" s="37"/>
+      <c r="E49" s="14" t="n">
+        <f aca="false">E47-E48</f>
         <v>2967861.9520012</v>
       </c>
-      <c r="F26" s="14" t="n">
-        <f aca="false">F24-F25</f>
+      <c r="F49" s="14" t="n">
+        <f aca="false">F47-F48</f>
         <v>2967861.9520012</v>
       </c>
-      <c r="G26" s="37"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="s">
-        <v>657</v>
-      </c>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-    </row>
-    <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="9" t="s">
+      <c r="G49" s="37"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="2" t="s">
+        <v>672</v>
+      </c>
+      <c r="B51" s="2"/>
+      <c r="C51" s="2"/>
+      <c r="D51" s="2"/>
+      <c r="E51" s="2"/>
+      <c r="F51" s="2"/>
+      <c r="G51" s="2"/>
+    </row>
+    <row r="52" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="B29" s="9" t="s">
-        <v>648</v>
-      </c>
-      <c r="C29" s="9" t="s">
-        <v>649</v>
-      </c>
-      <c r="D29" s="9" t="s">
-        <v>650</v>
-      </c>
-      <c r="E29" s="9" t="s">
-        <v>651</v>
-      </c>
-      <c r="F29" s="9" t="s">
-        <v>652</v>
-      </c>
-      <c r="G29" s="9" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3" t="s">
-        <v>654</v>
-      </c>
-      <c r="B30" s="33" t="n">
+      <c r="B52" s="9" t="s">
+        <v>663</v>
+      </c>
+      <c r="C52" s="9" t="s">
+        <v>664</v>
+      </c>
+      <c r="D52" s="9" t="s">
+        <v>665</v>
+      </c>
+      <c r="E52" s="9" t="s">
+        <v>666</v>
+      </c>
+      <c r="F52" s="9" t="s">
+        <v>667</v>
+      </c>
+      <c r="G52" s="9" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="3" t="s">
+        <v>669</v>
+      </c>
+      <c r="B53" s="33" t="n">
         <f aca="false">Consolidado!B41</f>
         <v>38030368.58194</v>
       </c>
-      <c r="C30" s="12" t="n">
+      <c r="C53" s="12" t="n">
         <f aca="false">SUM(Real_vs_Presupuesto!C15:C19)</f>
         <v>0</v>
       </c>
-      <c r="D30" s="35" t="str">
+      <c r="D53" s="35" t="str">
         <f aca="false">COUNT(Real_vs_Presupuesto!C15:C19)&amp;" de 5"</f>
         <v>0 de 5</v>
       </c>
-      <c r="E30" s="12" t="n">
+      <c r="E53" s="12" t="n">
         <f aca="false">SUMIF(Real_vs_Presupuesto!C15:C19,"",Real_vs_Presupuesto!B15:B19)</f>
         <v>38030368.58194</v>
       </c>
-      <c r="F30" s="14" t="n">
-        <f aca="false">C30+E30</f>
+      <c r="F53" s="14" t="n">
+        <f aca="false">C53+E53</f>
         <v>38030368.58194</v>
       </c>
-      <c r="G30" s="27" t="n">
-        <f aca="false">F30/B30</f>
+      <c r="G53" s="27" t="n">
+        <f aca="false">F53/B53</f>
         <v>1</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="3" t="s">
-        <v>655</v>
-      </c>
-      <c r="B31" s="33" t="n">
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="B54" s="33" t="n">
         <f aca="false">Consolidado!C41</f>
         <v>33067690.8539382</v>
       </c>
-      <c r="C31" s="12" t="n">
+      <c r="C54" s="12" t="n">
         <f aca="false">SUM(Real_vs_Presupuesto!F15:F19)</f>
         <v>0</v>
       </c>
-      <c r="D31" s="35" t="str">
+      <c r="D54" s="35" t="str">
         <f aca="false">COUNT(Real_vs_Presupuesto!F15:F19)&amp;" de 5"</f>
         <v>0 de 5</v>
       </c>
-      <c r="E31" s="12" t="n">
+      <c r="E54" s="12" t="n">
         <f aca="false">SUMIF(Real_vs_Presupuesto!F15:F19,"",Real_vs_Presupuesto!E15:E19)</f>
         <v>33067690.8539382</v>
       </c>
-      <c r="F31" s="14" t="n">
-        <f aca="false">C31+E31</f>
+      <c r="F54" s="14" t="n">
+        <f aca="false">C54+E54</f>
         <v>33067690.8539382</v>
       </c>
-      <c r="G31" s="27" t="n">
-        <f aca="false">F31/B31</f>
+      <c r="G54" s="27" t="n">
+        <f aca="false">F54/B54</f>
         <v>1</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="18" t="s">
-        <v>656</v>
-      </c>
-      <c r="B32" s="14" t="n">
-        <f aca="false">B30-B31</f>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="18" t="s">
+        <v>671</v>
+      </c>
+      <c r="B55" s="14" t="n">
+        <f aca="false">B53-B54</f>
         <v>4962677.7280018</v>
       </c>
-      <c r="C32" s="14" t="n">
-        <f aca="false">C30-C31</f>
+      <c r="C55" s="14" t="n">
+        <f aca="false">C53-C54</f>
         <v>0</v>
       </c>
-      <c r="D32" s="37"/>
-      <c r="E32" s="14" t="n">
-        <f aca="false">E30-E31</f>
+      <c r="D55" s="37"/>
+      <c r="E55" s="14" t="n">
+        <f aca="false">E53-E54</f>
         <v>4962677.7280018</v>
       </c>
-      <c r="F32" s="14" t="n">
-        <f aca="false">F30-F31</f>
+      <c r="F55" s="14" t="n">
+        <f aca="false">F53-F54</f>
         <v>4962677.7280018</v>
       </c>
-      <c r="G32" s="37"/>
+      <c r="G55" s="37"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="28">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A17:G17"/>
-    <mergeCell ref="A20:G20"/>
-    <mergeCell ref="A21:G21"/>
-    <mergeCell ref="A22:G22"/>
-    <mergeCell ref="A28:G28"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="A38:G38"/>
+    <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A40:G40"/>
+    <mergeCell ref="A41:G41"/>
+    <mergeCell ref="A43:G43"/>
+    <mergeCell ref="A44:G44"/>
+    <mergeCell ref="A45:G45"/>
+    <mergeCell ref="A51:G51"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -15851,7 +16144,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G163"/>
+  <dimension ref="A1:G166"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -15865,7 +16158,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>658</v>
+        <v>673</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -15876,7 +16169,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="24" t="s">
-        <v>659</v>
+        <v>674</v>
       </c>
       <c r="B2" s="24"/>
       <c r="C2" s="24"/>
@@ -15890,22 +16183,22 @@
         <v>376</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>660</v>
+        <v>675</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>378</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>661</v>
+        <v>676</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>662</v>
+        <v>677</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>663</v>
+        <v>678</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>664</v>
+        <v>679</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15922,13 +16215,13 @@
         <v>382</v>
       </c>
       <c r="E5" s="38" t="s">
-        <v>665</v>
+        <v>680</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G5" s="38" t="s">
-        <v>667</v>
+        <v>682</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15936,7 +16229,7 @@
         <v>435</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>668</v>
+        <v>683</v>
       </c>
       <c r="C6" s="12" t="n">
         <v>-1300000</v>
@@ -15945,13 +16238,13 @@
         <v>387</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>669</v>
+        <v>684</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>670</v>
+        <v>685</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>671</v>
+        <v>686</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15968,13 +16261,13 @@
         <v>387</v>
       </c>
       <c r="E7" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G7" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15991,13 +16284,13 @@
         <v>387</v>
       </c>
       <c r="E8" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G8" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16014,13 +16307,13 @@
         <v>387</v>
       </c>
       <c r="E9" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G9" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16037,13 +16330,13 @@
         <v>387</v>
       </c>
       <c r="E10" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G10" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16060,13 +16353,13 @@
         <v>387</v>
       </c>
       <c r="E11" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G11" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16083,13 +16376,13 @@
         <v>387</v>
       </c>
       <c r="E12" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G12" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16097,7 +16390,7 @@
         <v>459</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>674</v>
+        <v>689</v>
       </c>
       <c r="C13" s="12" t="n">
         <v>-30000</v>
@@ -16106,13 +16399,13 @@
         <v>387</v>
       </c>
       <c r="E13" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G13" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16129,13 +16422,13 @@
         <v>387</v>
       </c>
       <c r="E14" s="38" t="s">
-        <v>675</v>
+        <v>690</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G14" s="38" t="s">
-        <v>676</v>
+        <v>691</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16152,13 +16445,13 @@
         <v>387</v>
       </c>
       <c r="E15" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G15" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16175,13 +16468,13 @@
         <v>387</v>
       </c>
       <c r="E16" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G16" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16189,7 +16482,7 @@
         <v>473</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>677</v>
+        <v>692</v>
       </c>
       <c r="C17" s="12" t="n">
         <v>-92344</v>
@@ -16197,14 +16490,14 @@
       <c r="D17" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E17" s="38" t="s">
-        <v>675</v>
+      <c r="E17" s="3" t="s">
+        <v>693</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>666</v>
-      </c>
-      <c r="G17" s="38" t="s">
-        <v>676</v>
+        <v>685</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>694</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16221,13 +16514,13 @@
         <v>387</v>
       </c>
       <c r="E18" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G18" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16235,7 +16528,7 @@
         <v>473</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>678</v>
+        <v>695</v>
       </c>
       <c r="C19" s="12" t="n">
         <v>-17980</v>
@@ -16243,14 +16536,14 @@
       <c r="D19" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E19" s="38" t="s">
-        <v>679</v>
+      <c r="E19" s="3" t="s">
+        <v>693</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>670</v>
-      </c>
-      <c r="G19" s="38" t="s">
-        <v>667</v>
+        <v>685</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>694</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16266,14 +16559,14 @@
       <c r="D20" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="E20" s="38" t="s">
-        <v>675</v>
+      <c r="E20" s="3" t="s">
+        <v>696</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>666</v>
-      </c>
-      <c r="G20" s="38" t="s">
-        <v>676</v>
+        <v>697</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>698</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16290,13 +16583,13 @@
         <v>382</v>
       </c>
       <c r="E21" s="38" t="s">
-        <v>675</v>
+        <v>690</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G21" s="38" t="s">
-        <v>676</v>
+        <v>691</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16313,13 +16606,13 @@
         <v>382</v>
       </c>
       <c r="E22" s="38" t="s">
-        <v>680</v>
+        <v>699</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G22" s="38" t="s">
-        <v>667</v>
+        <v>682</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16335,14 +16628,14 @@
       <c r="D23" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E23" s="38" t="s">
-        <v>679</v>
+      <c r="E23" s="3" t="s">
+        <v>693</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>670</v>
-      </c>
-      <c r="G23" s="38" t="s">
-        <v>667</v>
+        <v>685</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>694</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16359,13 +16652,13 @@
         <v>387</v>
       </c>
       <c r="E24" s="38" t="s">
-        <v>681</v>
+        <v>700</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>670</v>
+        <v>685</v>
       </c>
       <c r="G24" s="38" t="s">
-        <v>682</v>
+        <v>701</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16382,13 +16675,13 @@
         <v>387</v>
       </c>
       <c r="E25" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G25" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16405,13 +16698,13 @@
         <v>387</v>
       </c>
       <c r="E26" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G26" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16428,13 +16721,13 @@
         <v>387</v>
       </c>
       <c r="E27" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G27" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16451,13 +16744,13 @@
         <v>387</v>
       </c>
       <c r="E28" s="38" t="s">
-        <v>681</v>
+        <v>700</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>670</v>
+        <v>685</v>
       </c>
       <c r="G28" s="38" t="s">
-        <v>682</v>
+        <v>701</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16474,13 +16767,13 @@
         <v>387</v>
       </c>
       <c r="E29" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G29" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16497,13 +16790,13 @@
         <v>387</v>
       </c>
       <c r="E30" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G30" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16520,13 +16813,13 @@
         <v>387</v>
       </c>
       <c r="E31" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G31" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16543,13 +16836,13 @@
         <v>387</v>
       </c>
       <c r="E32" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G32" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16566,13 +16859,13 @@
         <v>382</v>
       </c>
       <c r="E33" s="38" t="s">
-        <v>675</v>
+        <v>690</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G33" s="38" t="s">
-        <v>676</v>
+        <v>691</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16589,13 +16882,13 @@
         <v>387</v>
       </c>
       <c r="E34" s="38" t="s">
-        <v>681</v>
+        <v>700</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>670</v>
+        <v>685</v>
       </c>
       <c r="G34" s="38" t="s">
-        <v>682</v>
+        <v>701</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16612,13 +16905,13 @@
         <v>387</v>
       </c>
       <c r="E35" s="38" t="s">
-        <v>675</v>
+        <v>690</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G35" s="38" t="s">
-        <v>676</v>
+        <v>691</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16635,13 +16928,13 @@
         <v>387</v>
       </c>
       <c r="E36" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G36" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16658,13 +16951,13 @@
         <v>387</v>
       </c>
       <c r="E37" s="38" t="s">
-        <v>681</v>
+        <v>700</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>670</v>
+        <v>685</v>
       </c>
       <c r="G37" s="38" t="s">
-        <v>682</v>
+        <v>701</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16681,13 +16974,13 @@
         <v>387</v>
       </c>
       <c r="E38" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G38" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16703,14 +16996,14 @@
       <c r="D39" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E39" s="38" t="s">
-        <v>675</v>
+      <c r="E39" s="3" t="s">
+        <v>690</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>666</v>
-      </c>
-      <c r="G39" s="38" t="s">
-        <v>676</v>
+        <v>681</v>
+      </c>
+      <c r="G39" s="3" t="s">
+        <v>702</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16727,13 +17020,13 @@
         <v>387</v>
       </c>
       <c r="E40" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G40" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16741,7 +17034,7 @@
         <v>491</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>683</v>
+        <v>703</v>
       </c>
       <c r="C41" s="12" t="n">
         <v>440300</v>
@@ -16749,14 +17042,14 @@
       <c r="D41" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="E41" s="38" t="s">
-        <v>675</v>
+      <c r="E41" s="3" t="s">
+        <v>696</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>666</v>
-      </c>
-      <c r="G41" s="38" t="s">
-        <v>676</v>
+        <v>697</v>
+      </c>
+      <c r="G41" s="3" t="s">
+        <v>704</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16773,13 +17066,13 @@
         <v>387</v>
       </c>
       <c r="E42" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G42" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16787,7 +17080,7 @@
         <v>491</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>684</v>
+        <v>705</v>
       </c>
       <c r="C43" s="12" t="n">
         <v>-88073</v>
@@ -16795,14 +17088,14 @@
       <c r="D43" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E43" s="38" t="s">
-        <v>675</v>
+      <c r="E43" s="3" t="s">
+        <v>693</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>666</v>
-      </c>
-      <c r="G43" s="38" t="s">
-        <v>676</v>
+        <v>685</v>
+      </c>
+      <c r="G43" s="3" t="s">
+        <v>694</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16818,14 +17111,14 @@
       <c r="D44" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E44" s="38" t="s">
-        <v>679</v>
+      <c r="E44" s="3" t="s">
+        <v>693</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>670</v>
-      </c>
-      <c r="G44" s="38" t="s">
-        <v>667</v>
+        <v>685</v>
+      </c>
+      <c r="G44" s="3" t="s">
+        <v>694</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16833,7 +17126,7 @@
         <v>491</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>685</v>
+        <v>706</v>
       </c>
       <c r="C45" s="12" t="n">
         <v>-36259</v>
@@ -16841,14 +17134,14 @@
       <c r="D45" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E45" s="38" t="s">
-        <v>675</v>
+      <c r="E45" s="3" t="s">
+        <v>693</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>666</v>
-      </c>
-      <c r="G45" s="38" t="s">
-        <v>676</v>
+        <v>685</v>
+      </c>
+      <c r="G45" s="3" t="s">
+        <v>694</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16864,14 +17157,14 @@
       <c r="D46" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E46" s="38" t="s">
-        <v>675</v>
+      <c r="E46" s="3" t="s">
+        <v>707</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>666</v>
-      </c>
-      <c r="G46" s="38" t="s">
-        <v>676</v>
+        <v>681</v>
+      </c>
+      <c r="G46" s="3" t="s">
+        <v>708</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16879,7 +17172,7 @@
         <v>498</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>678</v>
+        <v>695</v>
       </c>
       <c r="C47" s="12" t="n">
         <v>-77990</v>
@@ -16887,14 +17180,14 @@
       <c r="D47" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E47" s="38" t="s">
-        <v>679</v>
+      <c r="E47" s="3" t="s">
+        <v>693</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>670</v>
-      </c>
-      <c r="G47" s="38" t="s">
-        <v>667</v>
+        <v>685</v>
+      </c>
+      <c r="G47" s="3" t="s">
+        <v>694</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16911,13 +17204,13 @@
         <v>387</v>
       </c>
       <c r="E48" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G48" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16934,13 +17227,13 @@
         <v>387</v>
       </c>
       <c r="E49" s="38" t="s">
-        <v>681</v>
+        <v>700</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>670</v>
+        <v>685</v>
       </c>
       <c r="G49" s="38" t="s">
-        <v>682</v>
+        <v>701</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16957,13 +17250,13 @@
         <v>387</v>
       </c>
       <c r="E50" s="38" t="s">
-        <v>675</v>
+        <v>690</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G50" s="38" t="s">
-        <v>676</v>
+        <v>691</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16980,13 +17273,13 @@
         <v>387</v>
       </c>
       <c r="E51" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G51" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17003,13 +17296,13 @@
         <v>387</v>
       </c>
       <c r="E52" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G52" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17026,13 +17319,13 @@
         <v>387</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>669</v>
+        <v>684</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>670</v>
+        <v>685</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>671</v>
+        <v>686</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17049,13 +17342,13 @@
         <v>387</v>
       </c>
       <c r="E54" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G54" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17063,7 +17356,7 @@
         <v>505</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>668</v>
+        <v>683</v>
       </c>
       <c r="C55" s="12" t="n">
         <v>-1000000</v>
@@ -17072,13 +17365,13 @@
         <v>387</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>669</v>
+        <v>684</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>670</v>
+        <v>685</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>671</v>
+        <v>686</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17095,13 +17388,13 @@
         <v>382</v>
       </c>
       <c r="E56" s="38" t="s">
-        <v>680</v>
+        <v>699</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G56" s="38" t="s">
-        <v>667</v>
+        <v>682</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17118,13 +17411,13 @@
         <v>382</v>
       </c>
       <c r="E57" s="38" t="s">
-        <v>665</v>
+        <v>680</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G57" s="38" t="s">
-        <v>667</v>
+        <v>682</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17132,7 +17425,7 @@
         <v>505</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>686</v>
+        <v>709</v>
       </c>
       <c r="C58" s="12" t="n">
         <v>-83300</v>
@@ -17140,14 +17433,14 @@
       <c r="D58" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E58" s="38" t="s">
-        <v>679</v>
+      <c r="E58" s="3" t="s">
+        <v>693</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>670</v>
-      </c>
-      <c r="G58" s="38" t="s">
-        <v>667</v>
+        <v>685</v>
+      </c>
+      <c r="G58" s="3" t="s">
+        <v>694</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17164,13 +17457,13 @@
         <v>387</v>
       </c>
       <c r="E59" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G59" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17187,13 +17480,13 @@
         <v>387</v>
       </c>
       <c r="E60" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G60" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17210,13 +17503,13 @@
         <v>387</v>
       </c>
       <c r="E61" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G61" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17233,13 +17526,13 @@
         <v>387</v>
       </c>
       <c r="E62" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G62" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17256,13 +17549,13 @@
         <v>387</v>
       </c>
       <c r="E63" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G63" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17279,13 +17572,13 @@
         <v>387</v>
       </c>
       <c r="E64" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G64" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17302,13 +17595,13 @@
         <v>387</v>
       </c>
       <c r="E65" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G65" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17325,13 +17618,13 @@
         <v>387</v>
       </c>
       <c r="E66" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F66" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G66" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17348,13 +17641,13 @@
         <v>382</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>687</v>
+        <v>710</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>688</v>
+        <v>711</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17371,13 +17664,13 @@
         <v>387</v>
       </c>
       <c r="E68" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G68" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17394,13 +17687,13 @@
         <v>387</v>
       </c>
       <c r="E69" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F69" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G69" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17417,13 +17710,13 @@
         <v>387</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>669</v>
+        <v>684</v>
       </c>
       <c r="F70" s="3" t="s">
-        <v>670</v>
+        <v>685</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>671</v>
+        <v>686</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17431,7 +17724,7 @@
         <v>522</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>689</v>
+        <v>712</v>
       </c>
       <c r="C71" s="12" t="n">
         <v>-25000</v>
@@ -17439,14 +17732,14 @@
       <c r="D71" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E71" s="38" t="s">
-        <v>675</v>
+      <c r="E71" s="3" t="s">
+        <v>693</v>
       </c>
       <c r="F71" s="3" t="s">
-        <v>666</v>
-      </c>
-      <c r="G71" s="38" t="s">
-        <v>676</v>
+        <v>685</v>
+      </c>
+      <c r="G71" s="3" t="s">
+        <v>694</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17463,13 +17756,13 @@
         <v>387</v>
       </c>
       <c r="E72" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F72" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G72" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17486,13 +17779,13 @@
         <v>387</v>
       </c>
       <c r="E73" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F73" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G73" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17509,13 +17802,13 @@
         <v>387</v>
       </c>
       <c r="E74" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F74" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G74" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17532,13 +17825,13 @@
         <v>387</v>
       </c>
       <c r="E75" s="38" t="s">
-        <v>681</v>
+        <v>700</v>
       </c>
       <c r="F75" s="3" t="s">
-        <v>670</v>
+        <v>685</v>
       </c>
       <c r="G75" s="38" t="s">
-        <v>682</v>
+        <v>701</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17555,13 +17848,13 @@
         <v>387</v>
       </c>
       <c r="E76" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F76" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G76" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17578,13 +17871,13 @@
         <v>387</v>
       </c>
       <c r="E77" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F77" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G77" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17601,13 +17894,13 @@
         <v>387</v>
       </c>
       <c r="E78" s="38" t="s">
-        <v>681</v>
+        <v>700</v>
       </c>
       <c r="F78" s="3" t="s">
-        <v>670</v>
+        <v>685</v>
       </c>
       <c r="G78" s="38" t="s">
-        <v>682</v>
+        <v>701</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17615,7 +17908,7 @@
         <v>522</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>668</v>
+        <v>683</v>
       </c>
       <c r="C79" s="12" t="n">
         <v>-1000000</v>
@@ -17624,13 +17917,13 @@
         <v>387</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>669</v>
+        <v>684</v>
       </c>
       <c r="F79" s="3" t="s">
-        <v>670</v>
+        <v>685</v>
       </c>
       <c r="G79" s="3" t="s">
-        <v>671</v>
+        <v>686</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17647,13 +17940,13 @@
         <v>382</v>
       </c>
       <c r="E80" s="38" t="s">
-        <v>675</v>
+        <v>690</v>
       </c>
       <c r="F80" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G80" s="38" t="s">
-        <v>676</v>
+        <v>691</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17670,13 +17963,13 @@
         <v>387</v>
       </c>
       <c r="E81" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F81" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G81" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17693,13 +17986,13 @@
         <v>387</v>
       </c>
       <c r="E82" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F82" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G82" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17716,13 +18009,13 @@
         <v>387</v>
       </c>
       <c r="E83" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F83" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G83" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17739,13 +18032,13 @@
         <v>387</v>
       </c>
       <c r="E84" s="3" t="s">
-        <v>690</v>
+        <v>713</v>
       </c>
       <c r="F84" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G84" s="3" t="s">
-        <v>671</v>
+        <v>686</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17762,13 +18055,13 @@
         <v>387</v>
       </c>
       <c r="E85" s="38" t="s">
-        <v>681</v>
+        <v>700</v>
       </c>
       <c r="F85" s="3" t="s">
-        <v>670</v>
+        <v>685</v>
       </c>
       <c r="G85" s="38" t="s">
-        <v>682</v>
+        <v>701</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17785,13 +18078,13 @@
         <v>387</v>
       </c>
       <c r="E86" s="38" t="s">
-        <v>681</v>
+        <v>700</v>
       </c>
       <c r="F86" s="3" t="s">
-        <v>670</v>
+        <v>685</v>
       </c>
       <c r="G86" s="38" t="s">
-        <v>682</v>
+        <v>701</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17808,13 +18101,13 @@
         <v>387</v>
       </c>
       <c r="E87" s="38" t="s">
-        <v>675</v>
+        <v>690</v>
       </c>
       <c r="F87" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G87" s="38" t="s">
-        <v>676</v>
+        <v>691</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17831,13 +18124,13 @@
         <v>382</v>
       </c>
       <c r="E88" s="3" t="s">
-        <v>687</v>
+        <v>710</v>
       </c>
       <c r="F88" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>688</v>
+        <v>711</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17845,7 +18138,7 @@
         <v>532</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>668</v>
+        <v>683</v>
       </c>
       <c r="C89" s="12" t="n">
         <v>-160000</v>
@@ -17854,13 +18147,13 @@
         <v>387</v>
       </c>
       <c r="E89" s="3" t="s">
-        <v>669</v>
+        <v>684</v>
       </c>
       <c r="F89" s="3" t="s">
-        <v>670</v>
+        <v>685</v>
       </c>
       <c r="G89" s="3" t="s">
-        <v>671</v>
+        <v>686</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17877,13 +18170,13 @@
         <v>382</v>
       </c>
       <c r="E90" s="38" t="s">
-        <v>665</v>
+        <v>680</v>
       </c>
       <c r="F90" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G90" s="38" t="s">
-        <v>667</v>
+        <v>682</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17891,7 +18184,7 @@
         <v>532</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>668</v>
+        <v>683</v>
       </c>
       <c r="C91" s="12" t="n">
         <v>-150000</v>
@@ -17900,13 +18193,13 @@
         <v>387</v>
       </c>
       <c r="E91" s="3" t="s">
-        <v>669</v>
+        <v>684</v>
       </c>
       <c r="F91" s="3" t="s">
-        <v>670</v>
+        <v>685</v>
       </c>
       <c r="G91" s="3" t="s">
-        <v>671</v>
+        <v>686</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17923,13 +18216,13 @@
         <v>387</v>
       </c>
       <c r="E92" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F92" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G92" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17945,14 +18238,14 @@
       <c r="D93" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E93" s="38" t="s">
-        <v>675</v>
+      <c r="E93" s="3" t="s">
+        <v>693</v>
       </c>
       <c r="F93" s="3" t="s">
-        <v>666</v>
-      </c>
-      <c r="G93" s="38" t="s">
-        <v>676</v>
+        <v>685</v>
+      </c>
+      <c r="G93" s="3" t="s">
+        <v>694</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17969,13 +18262,13 @@
         <v>387</v>
       </c>
       <c r="E94" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F94" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G94" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17992,13 +18285,13 @@
         <v>387</v>
       </c>
       <c r="E95" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F95" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G95" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18015,13 +18308,13 @@
         <v>387</v>
       </c>
       <c r="E96" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F96" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G96" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18038,13 +18331,13 @@
         <v>387</v>
       </c>
       <c r="E97" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F97" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G97" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18052,7 +18345,7 @@
         <v>542</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>691</v>
+        <v>714</v>
       </c>
       <c r="C98" s="12" t="n">
         <v>-405600</v>
@@ -18060,14 +18353,14 @@
       <c r="D98" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E98" s="38" t="s">
-        <v>675</v>
+      <c r="E98" s="3" t="s">
+        <v>715</v>
       </c>
       <c r="F98" s="3" t="s">
-        <v>666</v>
-      </c>
-      <c r="G98" s="38" t="s">
-        <v>676</v>
+        <v>685</v>
+      </c>
+      <c r="G98" s="3" t="s">
+        <v>716</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18075,7 +18368,7 @@
         <v>542</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>668</v>
+        <v>683</v>
       </c>
       <c r="C99" s="12" t="n">
         <v>-1000000</v>
@@ -18084,13 +18377,13 @@
         <v>387</v>
       </c>
       <c r="E99" s="3" t="s">
-        <v>669</v>
+        <v>684</v>
       </c>
       <c r="F99" s="3" t="s">
-        <v>670</v>
+        <v>685</v>
       </c>
       <c r="G99" s="3" t="s">
-        <v>671</v>
+        <v>686</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18106,14 +18399,14 @@
       <c r="D100" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E100" s="38" t="s">
-        <v>679</v>
+      <c r="E100" s="3" t="s">
+        <v>693</v>
       </c>
       <c r="F100" s="3" t="s">
-        <v>670</v>
-      </c>
-      <c r="G100" s="38" t="s">
-        <v>667</v>
+        <v>685</v>
+      </c>
+      <c r="G100" s="3" t="s">
+        <v>694</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18130,13 +18423,13 @@
         <v>387</v>
       </c>
       <c r="E101" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F101" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G101" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18153,13 +18446,13 @@
         <v>387</v>
       </c>
       <c r="E102" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F102" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G102" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18175,14 +18468,14 @@
       <c r="D103" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E103" s="38" t="s">
-        <v>679</v>
+      <c r="E103" s="3" t="s">
+        <v>693</v>
       </c>
       <c r="F103" s="3" t="s">
-        <v>670</v>
-      </c>
-      <c r="G103" s="38" t="s">
-        <v>667</v>
+        <v>685</v>
+      </c>
+      <c r="G103" s="3" t="s">
+        <v>694</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18199,13 +18492,13 @@
         <v>387</v>
       </c>
       <c r="E104" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F104" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G104" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18222,13 +18515,13 @@
         <v>382</v>
       </c>
       <c r="E105" s="38" t="s">
-        <v>675</v>
+        <v>690</v>
       </c>
       <c r="F105" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G105" s="38" t="s">
-        <v>676</v>
+        <v>691</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18245,13 +18538,13 @@
         <v>387</v>
       </c>
       <c r="E106" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F106" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G106" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18268,13 +18561,13 @@
         <v>387</v>
       </c>
       <c r="E107" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F107" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G107" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18290,14 +18583,14 @@
       <c r="D108" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E108" s="38" t="s">
-        <v>675</v>
+      <c r="E108" s="3" t="s">
+        <v>693</v>
       </c>
       <c r="F108" s="3" t="s">
-        <v>666</v>
-      </c>
-      <c r="G108" s="38" t="s">
-        <v>676</v>
+        <v>685</v>
+      </c>
+      <c r="G108" s="3" t="s">
+        <v>694</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18313,14 +18606,14 @@
       <c r="D109" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E109" s="38" t="s">
-        <v>675</v>
+      <c r="E109" s="3" t="s">
+        <v>693</v>
       </c>
       <c r="F109" s="3" t="s">
-        <v>666</v>
-      </c>
-      <c r="G109" s="38" t="s">
-        <v>676</v>
+        <v>685</v>
+      </c>
+      <c r="G109" s="3" t="s">
+        <v>694</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18328,7 +18621,7 @@
         <v>559</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>692</v>
+        <v>717</v>
       </c>
       <c r="C110" s="12" t="n">
         <v>-6950</v>
@@ -18337,13 +18630,13 @@
         <v>387</v>
       </c>
       <c r="E110" s="38" t="s">
-        <v>675</v>
+        <v>690</v>
       </c>
       <c r="F110" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G110" s="38" t="s">
-        <v>676</v>
+        <v>691</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18360,13 +18653,13 @@
         <v>387</v>
       </c>
       <c r="E111" s="38" t="s">
-        <v>681</v>
+        <v>700</v>
       </c>
       <c r="F111" s="3" t="s">
-        <v>670</v>
+        <v>685</v>
       </c>
       <c r="G111" s="38" t="s">
-        <v>682</v>
+        <v>701</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18383,13 +18676,13 @@
         <v>387</v>
       </c>
       <c r="E112" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F112" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G112" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18405,14 +18698,14 @@
       <c r="D113" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E113" s="38" t="s">
-        <v>675</v>
+      <c r="E113" s="3" t="s">
+        <v>693</v>
       </c>
       <c r="F113" s="3" t="s">
-        <v>666</v>
-      </c>
-      <c r="G113" s="38" t="s">
-        <v>676</v>
+        <v>685</v>
+      </c>
+      <c r="G113" s="3" t="s">
+        <v>694</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18429,13 +18722,13 @@
         <v>387</v>
       </c>
       <c r="E114" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F114" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G114" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18452,13 +18745,13 @@
         <v>387</v>
       </c>
       <c r="E115" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F115" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G115" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18466,7 +18759,7 @@
         <v>559</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>693</v>
+        <v>718</v>
       </c>
       <c r="C116" s="12" t="n">
         <v>-38000</v>
@@ -18474,14 +18767,14 @@
       <c r="D116" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E116" s="38" t="s">
-        <v>675</v>
+      <c r="E116" s="3" t="s">
+        <v>693</v>
       </c>
       <c r="F116" s="3" t="s">
-        <v>666</v>
-      </c>
-      <c r="G116" s="38" t="s">
-        <v>676</v>
+        <v>685</v>
+      </c>
+      <c r="G116" s="3" t="s">
+        <v>694</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18498,13 +18791,13 @@
         <v>387</v>
       </c>
       <c r="E117" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F117" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G117" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18521,13 +18814,13 @@
         <v>387</v>
       </c>
       <c r="E118" s="38" t="s">
-        <v>681</v>
+        <v>700</v>
       </c>
       <c r="F118" s="3" t="s">
-        <v>670</v>
+        <v>685</v>
       </c>
       <c r="G118" s="38" t="s">
-        <v>682</v>
+        <v>701</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18535,7 +18828,7 @@
         <v>559</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>694</v>
+        <v>719</v>
       </c>
       <c r="C119" s="12" t="n">
         <v>-66878</v>
@@ -18544,13 +18837,13 @@
         <v>387</v>
       </c>
       <c r="E119" s="38" t="s">
-        <v>675</v>
+        <v>690</v>
       </c>
       <c r="F119" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G119" s="38" t="s">
-        <v>676</v>
+        <v>691</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18567,13 +18860,13 @@
         <v>387</v>
       </c>
       <c r="E120" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F120" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G120" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18590,13 +18883,13 @@
         <v>387</v>
       </c>
       <c r="E121" s="38" t="s">
-        <v>681</v>
+        <v>700</v>
       </c>
       <c r="F121" s="3" t="s">
-        <v>670</v>
+        <v>685</v>
       </c>
       <c r="G121" s="38" t="s">
-        <v>682</v>
+        <v>701</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18604,7 +18897,7 @@
         <v>559</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>695</v>
+        <v>720</v>
       </c>
       <c r="C122" s="12" t="n">
         <v>-296037</v>
@@ -18612,14 +18905,14 @@
       <c r="D122" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E122" s="38" t="s">
-        <v>675</v>
+      <c r="E122" s="3" t="s">
+        <v>693</v>
       </c>
       <c r="F122" s="3" t="s">
-        <v>666</v>
-      </c>
-      <c r="G122" s="38" t="s">
-        <v>676</v>
+        <v>685</v>
+      </c>
+      <c r="G122" s="3" t="s">
+        <v>694</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18636,13 +18929,13 @@
         <v>382</v>
       </c>
       <c r="E123" s="38" t="s">
-        <v>675</v>
+        <v>690</v>
       </c>
       <c r="F123" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G123" s="38" t="s">
-        <v>676</v>
+        <v>691</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18659,13 +18952,13 @@
         <v>382</v>
       </c>
       <c r="E124" s="38" t="s">
-        <v>675</v>
+        <v>690</v>
       </c>
       <c r="F124" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G124" s="38" t="s">
-        <v>676</v>
+        <v>691</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18682,13 +18975,13 @@
         <v>382</v>
       </c>
       <c r="E125" s="38" t="s">
-        <v>680</v>
+        <v>699</v>
       </c>
       <c r="F125" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G125" s="38" t="s">
-        <v>667</v>
+        <v>682</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18696,7 +18989,7 @@
         <v>559</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>696</v>
+        <v>721</v>
       </c>
       <c r="C126" s="12" t="n">
         <v>-58001</v>
@@ -18705,13 +18998,13 @@
         <v>387</v>
       </c>
       <c r="E126" s="38" t="s">
-        <v>675</v>
+        <v>690</v>
       </c>
       <c r="F126" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G126" s="38" t="s">
-        <v>676</v>
+        <v>691</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18728,13 +19021,13 @@
         <v>387</v>
       </c>
       <c r="E127" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F127" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G127" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18751,13 +19044,13 @@
         <v>387</v>
       </c>
       <c r="E128" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F128" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G128" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18765,7 +19058,7 @@
         <v>572</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>697</v>
+        <v>722</v>
       </c>
       <c r="C129" s="12" t="n">
         <v>-97000</v>
@@ -18774,13 +19067,13 @@
         <v>387</v>
       </c>
       <c r="E129" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F129" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G129" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18788,7 +19081,7 @@
         <v>572</v>
       </c>
       <c r="B130" s="3" t="s">
-        <v>668</v>
+        <v>683</v>
       </c>
       <c r="C130" s="12" t="n">
         <v>-800000</v>
@@ -18797,13 +19090,13 @@
         <v>387</v>
       </c>
       <c r="E130" s="3" t="s">
-        <v>669</v>
+        <v>684</v>
       </c>
       <c r="F130" s="3" t="s">
-        <v>670</v>
+        <v>685</v>
       </c>
       <c r="G130" s="3" t="s">
-        <v>671</v>
+        <v>686</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18820,13 +19113,13 @@
         <v>387</v>
       </c>
       <c r="E131" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F131" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G131" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18843,13 +19136,13 @@
         <v>387</v>
       </c>
       <c r="E132" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F132" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G132" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18866,13 +19159,13 @@
         <v>387</v>
       </c>
       <c r="E133" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F133" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G133" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18889,13 +19182,13 @@
         <v>387</v>
       </c>
       <c r="E134" s="38" t="s">
-        <v>681</v>
+        <v>700</v>
       </c>
       <c r="F134" s="3" t="s">
-        <v>670</v>
+        <v>685</v>
       </c>
       <c r="G134" s="38" t="s">
-        <v>682</v>
+        <v>701</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18912,13 +19205,13 @@
         <v>387</v>
       </c>
       <c r="E135" s="38" t="s">
-        <v>681</v>
+        <v>700</v>
       </c>
       <c r="F135" s="3" t="s">
-        <v>670</v>
+        <v>685</v>
       </c>
       <c r="G135" s="38" t="s">
-        <v>682</v>
+        <v>701</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18935,13 +19228,13 @@
         <v>387</v>
       </c>
       <c r="E136" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F136" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G136" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18958,13 +19251,13 @@
         <v>387</v>
       </c>
       <c r="E137" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F137" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G137" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18981,13 +19274,13 @@
         <v>382</v>
       </c>
       <c r="E138" s="38" t="s">
-        <v>665</v>
+        <v>680</v>
       </c>
       <c r="F138" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G138" s="38" t="s">
-        <v>667</v>
+        <v>682</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19004,13 +19297,13 @@
         <v>387</v>
       </c>
       <c r="E139" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F139" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G139" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19018,7 +19311,7 @@
         <v>445</v>
       </c>
       <c r="B140" s="3" t="s">
-        <v>668</v>
+        <v>683</v>
       </c>
       <c r="C140" s="12" t="n">
         <v>-700000</v>
@@ -19027,13 +19320,13 @@
         <v>387</v>
       </c>
       <c r="E140" s="3" t="s">
-        <v>669</v>
+        <v>684</v>
       </c>
       <c r="F140" s="3" t="s">
-        <v>670</v>
+        <v>685</v>
       </c>
       <c r="G140" s="3" t="s">
-        <v>671</v>
+        <v>686</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19050,13 +19343,13 @@
         <v>382</v>
       </c>
       <c r="E141" s="38" t="s">
-        <v>680</v>
+        <v>699</v>
       </c>
       <c r="F141" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G141" s="38" t="s">
-        <v>667</v>
+        <v>682</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19072,14 +19365,14 @@
       <c r="D142" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E142" s="38" t="s">
-        <v>679</v>
+      <c r="E142" s="3" t="s">
+        <v>693</v>
       </c>
       <c r="F142" s="3" t="s">
-        <v>670</v>
-      </c>
-      <c r="G142" s="38" t="s">
-        <v>667</v>
+        <v>685</v>
+      </c>
+      <c r="G142" s="3" t="s">
+        <v>694</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19096,13 +19389,13 @@
         <v>387</v>
       </c>
       <c r="E143" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F143" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G143" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19119,13 +19412,13 @@
         <v>387</v>
       </c>
       <c r="E144" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F144" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G144" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19142,13 +19435,13 @@
         <v>387</v>
       </c>
       <c r="E145" s="38" t="s">
-        <v>681</v>
+        <v>700</v>
       </c>
       <c r="F145" s="3" t="s">
-        <v>670</v>
+        <v>685</v>
       </c>
       <c r="G145" s="38" t="s">
-        <v>682</v>
+        <v>701</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19165,13 +19458,13 @@
         <v>382</v>
       </c>
       <c r="E146" s="3" t="s">
-        <v>687</v>
+        <v>710</v>
       </c>
       <c r="F146" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G146" s="3" t="s">
-        <v>688</v>
+        <v>711</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19188,13 +19481,13 @@
         <v>387</v>
       </c>
       <c r="E147" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F147" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G147" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19210,14 +19503,14 @@
       <c r="D148" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E148" s="38" t="s">
-        <v>679</v>
+      <c r="E148" s="3" t="s">
+        <v>693</v>
       </c>
       <c r="F148" s="3" t="s">
-        <v>670</v>
-      </c>
-      <c r="G148" s="38" t="s">
-        <v>667</v>
+        <v>685</v>
+      </c>
+      <c r="G148" s="3" t="s">
+        <v>694</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19225,7 +19518,7 @@
         <v>450</v>
       </c>
       <c r="B149" s="3" t="s">
-        <v>698</v>
+        <v>723</v>
       </c>
       <c r="C149" s="12" t="n">
         <v>-46550</v>
@@ -19233,14 +19526,14 @@
       <c r="D149" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E149" s="38" t="s">
-        <v>675</v>
+      <c r="E149" s="3" t="s">
+        <v>693</v>
       </c>
       <c r="F149" s="3" t="s">
-        <v>666</v>
-      </c>
-      <c r="G149" s="38" t="s">
-        <v>676</v>
+        <v>685</v>
+      </c>
+      <c r="G149" s="3" t="s">
+        <v>694</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19257,13 +19550,13 @@
         <v>387</v>
       </c>
       <c r="E150" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F150" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G150" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19280,18 +19573,18 @@
         <v>387</v>
       </c>
       <c r="E151" s="38" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="F151" s="3" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="G151" s="38" t="s">
-        <v>673</v>
+        <v>688</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="2" t="s">
-        <v>699</v>
+        <v>724</v>
       </c>
       <c r="B153" s="2"/>
       <c r="C153" s="2"/>
@@ -19302,18 +19595,18 @@
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="9" t="s">
-        <v>700</v>
+        <v>725</v>
       </c>
       <c r="B154" s="9" t="s">
-        <v>701</v>
+        <v>726</v>
       </c>
       <c r="C154" s="9" t="s">
-        <v>702</v>
+        <v>727</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="3" t="s">
-        <v>672</v>
+        <v>687</v>
       </c>
       <c r="B155" s="3" t="n">
         <v>72</v>
@@ -19324,7 +19617,7 @@
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="3" t="s">
-        <v>669</v>
+        <v>684</v>
       </c>
       <c r="B156" s="3" t="n">
         <v>10</v>
@@ -19335,78 +19628,111 @@
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="3" t="s">
-        <v>681</v>
+        <v>693</v>
       </c>
       <c r="B157" s="3" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C157" s="12" t="n">
-        <v>-1200000</v>
+        <v>-1385644</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="3" t="s">
-        <v>679</v>
+        <v>700</v>
       </c>
       <c r="B158" s="3" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C158" s="12" t="n">
-        <v>-730211</v>
+        <v>-1200000</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="3" t="s">
-        <v>690</v>
+        <v>715</v>
       </c>
       <c r="B159" s="3" t="n">
         <v>1</v>
       </c>
       <c r="C159" s="12" t="n">
-        <v>-9471</v>
+        <v>-405600</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="3" t="s">
-        <v>675</v>
+        <v>707</v>
       </c>
       <c r="B160" s="3" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="C160" s="12" t="n">
-        <v>1620714</v>
+        <v>-31955</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="3" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="B161" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C161" s="12" t="n">
-        <v>2900000</v>
+        <v>-9471</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="3" t="s">
-        <v>665</v>
+        <v>696</v>
       </c>
       <c r="B162" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C162" s="12" t="n">
-        <v>4674721</v>
+        <v>523400</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="3" t="s">
-        <v>687</v>
+        <v>690</v>
       </c>
       <c r="B163" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="C163" s="12" t="n">
+        <v>2190302</v>
+      </c>
+    </row>
+    <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A164" s="3" t="s">
+        <v>699</v>
+      </c>
+      <c r="B164" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C164" s="12" t="n">
+        <v>2900000</v>
+      </c>
+    </row>
+    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A165" s="3" t="s">
+        <v>680</v>
+      </c>
+      <c r="B165" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C165" s="12" t="n">
+        <v>4674721</v>
+      </c>
+    </row>
+    <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A166" s="3" t="s">
+        <v>710</v>
+      </c>
+      <c r="B166" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C163" s="12" t="n">
+      <c r="C166" s="12" t="n">
         <v>9673787</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Corrige Informe Julio: usa Ingreso Devengado (servicios_piloto) con desglose Facturado/Pendiente
</commit_message>
<xml_diff>
--- a/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
+++ b/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3025" uniqueCount="739">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3029" uniqueCount="746">
   <si>
     <t xml:space="preserve">SUPUESTOS DEL PRESUPUESTO — SOLLEM + TRAST</t>
   </si>
@@ -1978,13 +1978,22 @@
     <t xml:space="preserve">Este informe usa valores NETOS (sin IVA) — es la utilidad real, distinta del Saldo de caja semanal (que incluye IVA cobrado, aún no pagado al Fisco). Ver hoja Consolidado para el detalle completo.</t>
   </si>
   <si>
-    <t xml:space="preserve">INFORME DE RESULTADOS FINANCIEROS — JULIO 2026 (REAL, mes cerrado)</t>
+    <t xml:space="preserve">INFORME DE RESULTADOS FINANCIEROS — JULIO 2026 (REAL — Ingreso Devengado, mes cerrado)</t>
   </si>
   <si>
     <t xml:space="preserve">Julio 2026 (Real)</t>
   </si>
   <si>
-    <t xml:space="preserve">Ingreso Neto (ventas, RCV 8 facturas)</t>
+    <t xml:space="preserve">Ingreso Neto Devengado (servicios_piloto, 35 servicios reales)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  · de lo cual Facturado (en RCV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  · de lo cual Pendiente de Facturar (kaptura_cuentas_por_facturar)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IVA Débito Fiscal (informativo, sobre lo facturado)</t>
   </si>
   <si>
     <t xml:space="preserve">Combustible (real, Aramco+Copec vía cartola)</t>
@@ -2008,19 +2017,31 @@
     <t xml:space="preserve">Factoring (costo real: 3 comprobantes reales)</t>
   </si>
   <si>
+    <t xml:space="preserve">% Utilidad / Ingreso Devengado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CORREGIDO 31-07-2026: la primera versión de este informe usaba solo el RCV Venta ($12.340.900) como ingreso — subestimaba julio en $3.082.400 porque 3 clientes completos (Presmita, Citrus Agro, Trans Luciano) y parte de Sollem/Danilo Núñez tenían servicios reales ejecutados sin factura emitida. Ahora usa servicios_piloto (ingreso devengado real), con el detalle Facturado/Pendiente separado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Los $7.587.600 pendientes de facturar quedaron cargados en la tabla nueva kaptura_cuentas_por_facturar (21 servicios, creada 31-07-2026) — tabla que no existía en el sistema hasta ahora.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IVA Débito recalculado solo sobre lo YA facturado ($7.835.700 × 19%), no sobre el devengado total — el IVA solo se genera al emitir la factura.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Julio NO tiene presupuesto formal (el sistema de presupuesto formal parte en Agosto) — por eso esta tabla no tiene columna de comparación, solo el real.</t>
   </si>
   <si>
     <t xml:space="preserve">Costos en base CASH (lo que efectivamente salió del banco en julio), cruzados 1 a 1 contra RCV Compra/Venta y comprobantes reales donde existen (Vulko, Construmart, Cardánica, factoring) — no son supuestos.</t>
   </si>
   <si>
-    <t xml:space="preserve">'Remuneración Administrativa' ($6.656.800) es el bloque menos confiable: son 72 transferencias a personas sin desglose exacto de si son sueldo, viático o anticipo — la heurística solo separó Viático cuando el monto era múltiplo exacto de $12.000. Es probable que parte de este monto sea realmente Sueldo Conductor mal clasificado, lo que subestimaría el margen real un poco menos negativo de lo mostrado.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Costo de Factoring ($459.420) = suma de los 3 comprobantes reales de julio: folio 20+bundle $158.549, folio 22 $152.894 (dato previo de Kaptura, sin comprobante propio revisado esta sesión), folio 28 $147.977 (LATAM Trade Capital, comprobante real).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La Utilidad negativa es consistente con el subregistro ya documentado: el Ingreso Neto usado (RCV, $12.340.900) probablemente no refleja todos los servicios reales ejecutados en julio — cargar los servicios de julio en Kaptura sigue siendo el pendiente que más cambiaría este número.</t>
+    <t xml:space="preserve">'Remuneración Administrativa' ($6.656.800) sigue siendo el bloque menos confiable: 72 transferencias sin desglose exacto de sueldo/viático/anticipo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo de Factoring ($459.420) = folio 20+bundle $158.549, folio 22 $152.894 (dato previo Kaptura), folio 28 $147.977 (comprobante real LATAM Trade Capital).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S-85 (Presmita, 24-07) quedó registrado con tarifa $0 en servicios_piloto — posible error de carga, no se incluyó valor en Pendiente de Facturar por esa fila.</t>
   </si>
   <si>
     <t xml:space="preserve">PLAN vs. REAL vs. REPROYECCIÓN (flujo de caja semanal)</t>
@@ -3321,7 +3342,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>728</v>
+        <v>735</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3331,7 +3352,7 @@
     </row>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="24" t="s">
-        <v>729</v>
+        <v>736</v>
       </c>
       <c r="B2" s="24"/>
       <c r="C2" s="24"/>
@@ -3344,16 +3365,16 @@
         <v>376</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>730</v>
+        <v>737</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>731</v>
+        <v>738</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>732</v>
+        <v>739</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>733</v>
+        <v>740</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>188</v>
@@ -3367,23 +3388,23 @@
         <v>63371</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>734</v>
+        <v>741</v>
       </c>
       <c r="D5" s="37"/>
       <c r="E5" s="37"/>
       <c r="F5" s="3" t="s">
-        <v>735</v>
+        <v>742</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>736</v>
+        <v>743</v>
       </c>
       <c r="B6" s="12" t="n">
         <v>1275801</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>737</v>
+        <v>744</v>
       </c>
       <c r="D6" s="34"/>
       <c r="E6" s="12" t="str">
@@ -3391,7 +3412,7 @@
         <v/>
       </c>
       <c r="F6" s="3" t="s">
-        <v>738</v>
+        <v>745</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15459,7 +15480,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G59"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -15666,145 +15687,143 @@
       <c r="C21" s="9"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="15" t="s">
         <v>647</v>
       </c>
-      <c r="B22" s="12" t="n">
-        <v>12340900</v>
-      </c>
-      <c r="C22" s="12"/>
+      <c r="B22" s="17" t="n">
+        <v>15423300</v>
+      </c>
+      <c r="C22" s="17"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>642</v>
+        <v>648</v>
       </c>
       <c r="B23" s="12" t="n">
-        <v>2344771</v>
+        <v>7835700</v>
       </c>
       <c r="C23" s="12"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="15" t="s">
-        <v>106</v>
-      </c>
-      <c r="B24" s="17" t="n">
-        <v>14685671</v>
-      </c>
-      <c r="C24" s="17"/>
+      <c r="A24" s="3" t="s">
+        <v>649</v>
+      </c>
+      <c r="B24" s="12" t="n">
+        <v>7587600</v>
+      </c>
+      <c r="C24" s="12"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="B25" s="12" t="n">
-        <v>-6159145</v>
+        <v>1488783</v>
       </c>
       <c r="C25" s="12"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="B26" s="12" t="n">
-        <v>-405600</v>
+        <v>-6159145</v>
       </c>
       <c r="C26" s="12"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
       <c r="B27" s="12" t="n">
-        <v>-1385644</v>
+        <v>-405600</v>
       </c>
       <c r="C27" s="12"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="B28" s="12" t="n">
-        <v>-1200000</v>
+        <v>-1385644</v>
       </c>
       <c r="C28" s="12"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="B29" s="12" t="n">
+        <v>-1200000</v>
+      </c>
+      <c r="C29" s="12"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="3" t="s">
+        <v>655</v>
+      </c>
+      <c r="B30" s="12" t="n">
         <v>-31955</v>
       </c>
-      <c r="C29" s="12"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="B30" s="17" t="n">
-        <v>-9182344</v>
-      </c>
-      <c r="C30" s="17"/>
+      <c r="C30" s="12"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="B31" s="17" t="n">
+        <v>-9182344</v>
+      </c>
+      <c r="C31" s="17"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="15" t="s">
         <v>643</v>
       </c>
-      <c r="B31" s="17" t="n">
-        <v>3158556</v>
-      </c>
-      <c r="C31" s="17"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="s">
-        <v>653</v>
-      </c>
-      <c r="B32" s="12" t="n">
-        <v>-6656800</v>
-      </c>
-      <c r="C32" s="12"/>
+      <c r="B32" s="17" t="n">
+        <v>6240956</v>
+      </c>
+      <c r="C32" s="17"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
       <c r="B33" s="12" t="n">
+        <v>-6656800</v>
+      </c>
+      <c r="C33" s="12"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="3" t="s">
+        <v>657</v>
+      </c>
+      <c r="B34" s="12" t="n">
         <v>-459420</v>
       </c>
-      <c r="C33" s="12"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="15" t="s">
+      <c r="C34" s="12"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="15" t="s">
         <v>149</v>
       </c>
-      <c r="B34" s="17" t="n">
-        <v>-3957664</v>
-      </c>
-      <c r="C34" s="17"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="18" t="s">
-        <v>150</v>
-      </c>
-      <c r="B35" s="27" t="n">
-        <v>-0.269491533618042</v>
-      </c>
-      <c r="C35" s="27"/>
-    </row>
-    <row r="37" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="24" t="s">
-        <v>655</v>
-      </c>
-      <c r="B37" s="24"/>
-      <c r="C37" s="24"/>
-      <c r="D37" s="24"/>
-      <c r="E37" s="24"/>
-      <c r="F37" s="24"/>
-      <c r="G37" s="24"/>
+      <c r="B35" s="17" t="n">
+        <v>-875264</v>
+      </c>
+      <c r="C35" s="17"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="18" t="s">
+        <v>658</v>
+      </c>
+      <c r="B36" s="27" t="n">
+        <v>-0.0567494634740944</v>
+      </c>
+      <c r="C36" s="27"/>
     </row>
     <row r="38" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="24" t="s">
-        <v>656</v>
+        <v>659</v>
       </c>
       <c r="B38" s="24"/>
       <c r="C38" s="24"/>
@@ -15815,7 +15834,7 @@
     </row>
     <row r="39" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="24" t="s">
-        <v>657</v>
+        <v>660</v>
       </c>
       <c r="B39" s="24"/>
       <c r="C39" s="24"/>
@@ -15826,7 +15845,7 @@
     </row>
     <row r="40" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="24" t="s">
-        <v>658</v>
+        <v>661</v>
       </c>
       <c r="B40" s="24"/>
       <c r="C40" s="24"/>
@@ -15837,7 +15856,7 @@
     </row>
     <row r="41" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="24" t="s">
-        <v>659</v>
+        <v>662</v>
       </c>
       <c r="B41" s="24"/>
       <c r="C41" s="24"/>
@@ -15846,260 +15865,304 @@
       <c r="F41" s="24"/>
       <c r="G41" s="24"/>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="2" t="s">
-        <v>660</v>
-      </c>
-      <c r="B43" s="2"/>
-      <c r="C43" s="2"/>
-      <c r="D43" s="2"/>
-      <c r="E43" s="2"/>
-      <c r="F43" s="2"/>
-      <c r="G43" s="2"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="28" t="s">
-        <v>661</v>
-      </c>
-      <c r="B44" s="28"/>
-      <c r="C44" s="28"/>
-      <c r="D44" s="28"/>
-      <c r="E44" s="28"/>
-      <c r="F44" s="28"/>
-      <c r="G44" s="28"/>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="2" t="s">
-        <v>662</v>
-      </c>
-      <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
-      <c r="E45" s="2"/>
-      <c r="F45" s="2"/>
-      <c r="G45" s="2"/>
-    </row>
-    <row r="46" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="9" t="s">
+    <row r="42" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="24" t="s">
+        <v>663</v>
+      </c>
+      <c r="B42" s="24"/>
+      <c r="C42" s="24"/>
+      <c r="D42" s="24"/>
+      <c r="E42" s="24"/>
+      <c r="F42" s="24"/>
+      <c r="G42" s="24"/>
+    </row>
+    <row r="43" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="24" t="s">
+        <v>664</v>
+      </c>
+      <c r="B43" s="24"/>
+      <c r="C43" s="24"/>
+      <c r="D43" s="24"/>
+      <c r="E43" s="24"/>
+      <c r="F43" s="24"/>
+      <c r="G43" s="24"/>
+    </row>
+    <row r="44" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="24" t="s">
+        <v>665</v>
+      </c>
+      <c r="B44" s="24"/>
+      <c r="C44" s="24"/>
+      <c r="D44" s="24"/>
+      <c r="E44" s="24"/>
+      <c r="F44" s="24"/>
+      <c r="G44" s="24"/>
+    </row>
+    <row r="45" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="24" t="s">
+        <v>666</v>
+      </c>
+      <c r="B45" s="24"/>
+      <c r="C45" s="24"/>
+      <c r="D45" s="24"/>
+      <c r="E45" s="24"/>
+      <c r="F45" s="24"/>
+      <c r="G45" s="24"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="2" t="s">
+        <v>667</v>
+      </c>
+      <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
+      <c r="E47" s="2"/>
+      <c r="F47" s="2"/>
+      <c r="G47" s="2"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="28" t="s">
+        <v>668</v>
+      </c>
+      <c r="B48" s="28"/>
+      <c r="C48" s="28"/>
+      <c r="D48" s="28"/>
+      <c r="E48" s="28"/>
+      <c r="F48" s="28"/>
+      <c r="G48" s="28"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="2" t="s">
+        <v>669</v>
+      </c>
+      <c r="B49" s="2"/>
+      <c r="C49" s="2"/>
+      <c r="D49" s="2"/>
+      <c r="E49" s="2"/>
+      <c r="F49" s="2"/>
+      <c r="G49" s="2"/>
+    </row>
+    <row r="50" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="B46" s="9" t="s">
-        <v>663</v>
-      </c>
-      <c r="C46" s="9" t="s">
-        <v>664</v>
-      </c>
-      <c r="D46" s="9" t="s">
-        <v>665</v>
-      </c>
-      <c r="E46" s="9" t="s">
-        <v>666</v>
-      </c>
-      <c r="F46" s="9" t="s">
-        <v>667</v>
-      </c>
-      <c r="G46" s="9" t="s">
-        <v>668</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="3" t="s">
-        <v>669</v>
-      </c>
-      <c r="B47" s="33" t="n">
+      <c r="B50" s="9" t="s">
+        <v>670</v>
+      </c>
+      <c r="C50" s="9" t="s">
+        <v>671</v>
+      </c>
+      <c r="D50" s="9" t="s">
+        <v>672</v>
+      </c>
+      <c r="E50" s="9" t="s">
+        <v>673</v>
+      </c>
+      <c r="F50" s="9" t="s">
+        <v>674</v>
+      </c>
+      <c r="G50" s="9" t="s">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="3" t="s">
+        <v>676</v>
+      </c>
+      <c r="B51" s="33" t="n">
         <f aca="false">Consolidado!B32</f>
         <v>29402660.3612933</v>
       </c>
-      <c r="C47" s="12" t="n">
+      <c r="C51" s="12" t="n">
         <f aca="false">SUM(Real_vs_Presupuesto!C6:C11)</f>
         <v>0</v>
       </c>
-      <c r="D47" s="35" t="str">
+      <c r="D51" s="35" t="str">
         <f aca="false">COUNT(Real_vs_Presupuesto!C6:C11)&amp;" de 6"</f>
         <v>0 de 6</v>
       </c>
-      <c r="E47" s="12" t="n">
+      <c r="E51" s="12" t="n">
         <f aca="false">SUMIF(Real_vs_Presupuesto!C6:C11,"",Real_vs_Presupuesto!B6:B11)</f>
         <v>29402660.3612933</v>
       </c>
-      <c r="F47" s="14" t="n">
-        <f aca="false">C47+E47</f>
+      <c r="F51" s="14" t="n">
+        <f aca="false">C51+E51</f>
         <v>29402660.3612933</v>
       </c>
-      <c r="G47" s="27" t="n">
-        <f aca="false">F47/B47</f>
+      <c r="G51" s="27" t="n">
+        <f aca="false">F51/B51</f>
         <v>1</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="3" t="s">
-        <v>670</v>
-      </c>
-      <c r="B48" s="33" t="n">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="3" t="s">
+        <v>677</v>
+      </c>
+      <c r="B52" s="33" t="n">
         <f aca="false">Consolidado!C32</f>
         <v>26434798.4092921</v>
       </c>
-      <c r="C48" s="12" t="n">
+      <c r="C52" s="12" t="n">
         <f aca="false">SUM(Real_vs_Presupuesto!F6:F11)</f>
         <v>0</v>
       </c>
-      <c r="D48" s="35" t="str">
+      <c r="D52" s="35" t="str">
         <f aca="false">COUNT(Real_vs_Presupuesto!F6:F11)&amp;" de 6"</f>
         <v>0 de 6</v>
       </c>
-      <c r="E48" s="12" t="n">
+      <c r="E52" s="12" t="n">
         <f aca="false">SUMIF(Real_vs_Presupuesto!F6:F11,"",Real_vs_Presupuesto!E6:E11)</f>
         <v>26434798.4092921</v>
       </c>
-      <c r="F48" s="14" t="n">
-        <f aca="false">C48+E48</f>
+      <c r="F52" s="14" t="n">
+        <f aca="false">C52+E52</f>
         <v>26434798.4092921</v>
       </c>
-      <c r="G48" s="27" t="n">
-        <f aca="false">F48/B48</f>
+      <c r="G52" s="27" t="n">
+        <f aca="false">F52/B52</f>
         <v>1</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="18" t="s">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="18" t="s">
+        <v>678</v>
+      </c>
+      <c r="B53" s="14" t="n">
+        <f aca="false">B51-B52</f>
+        <v>2967861.9520012</v>
+      </c>
+      <c r="C53" s="14" t="n">
+        <f aca="false">C51-C52</f>
+        <v>0</v>
+      </c>
+      <c r="D53" s="37"/>
+      <c r="E53" s="14" t="n">
+        <f aca="false">E51-E52</f>
+        <v>2967861.9520012</v>
+      </c>
+      <c r="F53" s="14" t="n">
+        <f aca="false">F51-F52</f>
+        <v>2967861.9520012</v>
+      </c>
+      <c r="G53" s="37"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="2" t="s">
+        <v>679</v>
+      </c>
+      <c r="B55" s="2"/>
+      <c r="C55" s="2"/>
+      <c r="D55" s="2"/>
+      <c r="E55" s="2"/>
+      <c r="F55" s="2"/>
+      <c r="G55" s="2"/>
+    </row>
+    <row r="56" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B56" s="9" t="s">
+        <v>670</v>
+      </c>
+      <c r="C56" s="9" t="s">
         <v>671</v>
       </c>
-      <c r="B49" s="14" t="n">
-        <f aca="false">B47-B48</f>
-        <v>2967861.9520012</v>
-      </c>
-      <c r="C49" s="14" t="n">
-        <f aca="false">C47-C48</f>
-        <v>0</v>
-      </c>
-      <c r="D49" s="37"/>
-      <c r="E49" s="14" t="n">
-        <f aca="false">E47-E48</f>
-        <v>2967861.9520012</v>
-      </c>
-      <c r="F49" s="14" t="n">
-        <f aca="false">F47-F48</f>
-        <v>2967861.9520012</v>
-      </c>
-      <c r="G49" s="37"/>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="2" t="s">
+      <c r="D56" s="9" t="s">
         <v>672</v>
       </c>
-      <c r="B51" s="2"/>
-      <c r="C51" s="2"/>
-      <c r="D51" s="2"/>
-      <c r="E51" s="2"/>
-      <c r="F51" s="2"/>
-      <c r="G51" s="2"/>
-    </row>
-    <row r="52" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="B52" s="9" t="s">
-        <v>663</v>
-      </c>
-      <c r="C52" s="9" t="s">
-        <v>664</v>
-      </c>
-      <c r="D52" s="9" t="s">
-        <v>665</v>
-      </c>
-      <c r="E52" s="9" t="s">
-        <v>666</v>
-      </c>
-      <c r="F52" s="9" t="s">
-        <v>667</v>
-      </c>
-      <c r="G52" s="9" t="s">
-        <v>668</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="3" t="s">
-        <v>669</v>
-      </c>
-      <c r="B53" s="33" t="n">
+      <c r="E56" s="9" t="s">
+        <v>673</v>
+      </c>
+      <c r="F56" s="9" t="s">
+        <v>674</v>
+      </c>
+      <c r="G56" s="9" t="s">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="3" t="s">
+        <v>676</v>
+      </c>
+      <c r="B57" s="33" t="n">
         <f aca="false">Consolidado!B41</f>
         <v>38030368.58194</v>
       </c>
-      <c r="C53" s="12" t="n">
+      <c r="C57" s="12" t="n">
         <f aca="false">SUM(Real_vs_Presupuesto!C15:C19)</f>
         <v>0</v>
       </c>
-      <c r="D53" s="35" t="str">
+      <c r="D57" s="35" t="str">
         <f aca="false">COUNT(Real_vs_Presupuesto!C15:C19)&amp;" de 5"</f>
         <v>0 de 5</v>
       </c>
-      <c r="E53" s="12" t="n">
+      <c r="E57" s="12" t="n">
         <f aca="false">SUMIF(Real_vs_Presupuesto!C15:C19,"",Real_vs_Presupuesto!B15:B19)</f>
         <v>38030368.58194</v>
       </c>
-      <c r="F53" s="14" t="n">
-        <f aca="false">C53+E53</f>
+      <c r="F57" s="14" t="n">
+        <f aca="false">C57+E57</f>
         <v>38030368.58194</v>
       </c>
-      <c r="G53" s="27" t="n">
-        <f aca="false">F53/B53</f>
+      <c r="G57" s="27" t="n">
+        <f aca="false">F57/B57</f>
         <v>1</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="3" t="s">
-        <v>670</v>
-      </c>
-      <c r="B54" s="33" t="n">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="3" t="s">
+        <v>677</v>
+      </c>
+      <c r="B58" s="33" t="n">
         <f aca="false">Consolidado!C41</f>
         <v>33067690.8539382</v>
       </c>
-      <c r="C54" s="12" t="n">
+      <c r="C58" s="12" t="n">
         <f aca="false">SUM(Real_vs_Presupuesto!F15:F19)</f>
         <v>0</v>
       </c>
-      <c r="D54" s="35" t="str">
+      <c r="D58" s="35" t="str">
         <f aca="false">COUNT(Real_vs_Presupuesto!F15:F19)&amp;" de 5"</f>
         <v>0 de 5</v>
       </c>
-      <c r="E54" s="12" t="n">
+      <c r="E58" s="12" t="n">
         <f aca="false">SUMIF(Real_vs_Presupuesto!F15:F19,"",Real_vs_Presupuesto!E15:E19)</f>
         <v>33067690.8539382</v>
       </c>
-      <c r="F54" s="14" t="n">
-        <f aca="false">C54+E54</f>
+      <c r="F58" s="14" t="n">
+        <f aca="false">C58+E58</f>
         <v>33067690.8539382</v>
       </c>
-      <c r="G54" s="27" t="n">
-        <f aca="false">F54/B54</f>
+      <c r="G58" s="27" t="n">
+        <f aca="false">F58/B58</f>
         <v>1</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="18" t="s">
-        <v>671</v>
-      </c>
-      <c r="B55" s="14" t="n">
-        <f aca="false">B53-B54</f>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="18" t="s">
+        <v>678</v>
+      </c>
+      <c r="B59" s="14" t="n">
+        <f aca="false">B57-B58</f>
         <v>4962677.7280018</v>
       </c>
-      <c r="C55" s="14" t="n">
-        <f aca="false">C53-C54</f>
+      <c r="C59" s="14" t="n">
+        <f aca="false">C57-C58</f>
         <v>0</v>
       </c>
-      <c r="D55" s="37"/>
-      <c r="E55" s="14" t="n">
-        <f aca="false">E53-E54</f>
+      <c r="D59" s="37"/>
+      <c r="E59" s="14" t="n">
+        <f aca="false">E57-E58</f>
         <v>4962677.7280018</v>
       </c>
-      <c r="F55" s="14" t="n">
-        <f aca="false">F53-F54</f>
+      <c r="F59" s="14" t="n">
+        <f aca="false">F57-F58</f>
         <v>4962677.7280018</v>
       </c>
-      <c r="G55" s="37"/>
+      <c r="G59" s="37"/>
     </row>
   </sheetData>
-  <mergeCells count="28">
+  <mergeCells count="32">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A17:G17"/>
@@ -16119,15 +16182,19 @@
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="B35:C35"/>
-    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="B36:C36"/>
     <mergeCell ref="A38:G38"/>
     <mergeCell ref="A39:G39"/>
     <mergeCell ref="A40:G40"/>
     <mergeCell ref="A41:G41"/>
+    <mergeCell ref="A42:G42"/>
     <mergeCell ref="A43:G43"/>
     <mergeCell ref="A44:G44"/>
     <mergeCell ref="A45:G45"/>
-    <mergeCell ref="A51:G51"/>
+    <mergeCell ref="A47:G47"/>
+    <mergeCell ref="A48:G48"/>
+    <mergeCell ref="A49:G49"/>
+    <mergeCell ref="A55:G55"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -16158,7 +16225,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>673</v>
+        <v>680</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -16169,7 +16236,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="24" t="s">
-        <v>674</v>
+        <v>681</v>
       </c>
       <c r="B2" s="24"/>
       <c r="C2" s="24"/>
@@ -16183,22 +16250,22 @@
         <v>376</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>675</v>
+        <v>682</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>378</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>676</v>
+        <v>683</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>677</v>
+        <v>684</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>678</v>
+        <v>685</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>679</v>
+        <v>686</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16215,13 +16282,13 @@
         <v>382</v>
       </c>
       <c r="E5" s="38" t="s">
-        <v>680</v>
+        <v>687</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G5" s="38" t="s">
-        <v>682</v>
+        <v>689</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16229,7 +16296,7 @@
         <v>435</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>683</v>
+        <v>690</v>
       </c>
       <c r="C6" s="12" t="n">
         <v>-1300000</v>
@@ -16238,13 +16305,13 @@
         <v>387</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>684</v>
+        <v>691</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>686</v>
+        <v>693</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16261,13 +16328,13 @@
         <v>387</v>
       </c>
       <c r="E7" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G7" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16284,13 +16351,13 @@
         <v>387</v>
       </c>
       <c r="E8" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G8" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16307,13 +16374,13 @@
         <v>387</v>
       </c>
       <c r="E9" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G9" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16330,13 +16397,13 @@
         <v>387</v>
       </c>
       <c r="E10" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G10" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16353,13 +16420,13 @@
         <v>387</v>
       </c>
       <c r="E11" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G11" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16376,13 +16443,13 @@
         <v>387</v>
       </c>
       <c r="E12" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G12" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16390,7 +16457,7 @@
         <v>459</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>689</v>
+        <v>696</v>
       </c>
       <c r="C13" s="12" t="n">
         <v>-30000</v>
@@ -16399,13 +16466,13 @@
         <v>387</v>
       </c>
       <c r="E13" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G13" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16422,13 +16489,13 @@
         <v>387</v>
       </c>
       <c r="E14" s="38" t="s">
-        <v>690</v>
+        <v>697</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G14" s="38" t="s">
-        <v>691</v>
+        <v>698</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16445,13 +16512,13 @@
         <v>387</v>
       </c>
       <c r="E15" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G15" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16468,13 +16535,13 @@
         <v>387</v>
       </c>
       <c r="E16" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G16" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16482,7 +16549,7 @@
         <v>473</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>692</v>
+        <v>699</v>
       </c>
       <c r="C17" s="12" t="n">
         <v>-92344</v>
@@ -16491,13 +16558,13 @@
         <v>387</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16514,13 +16581,13 @@
         <v>387</v>
       </c>
       <c r="E18" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G18" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16528,7 +16595,7 @@
         <v>473</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>695</v>
+        <v>702</v>
       </c>
       <c r="C19" s="12" t="n">
         <v>-17980</v>
@@ -16537,13 +16604,13 @@
         <v>387</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16560,13 +16627,13 @@
         <v>382</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>696</v>
+        <v>703</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>697</v>
+        <v>704</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>698</v>
+        <v>705</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16583,13 +16650,13 @@
         <v>382</v>
       </c>
       <c r="E21" s="38" t="s">
-        <v>690</v>
+        <v>697</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G21" s="38" t="s">
-        <v>691</v>
+        <v>698</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16606,13 +16673,13 @@
         <v>382</v>
       </c>
       <c r="E22" s="38" t="s">
-        <v>699</v>
+        <v>706</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G22" s="38" t="s">
-        <v>682</v>
+        <v>689</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16629,13 +16696,13 @@
         <v>387</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16652,13 +16719,13 @@
         <v>387</v>
       </c>
       <c r="E24" s="38" t="s">
-        <v>700</v>
+        <v>707</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G24" s="38" t="s">
-        <v>701</v>
+        <v>708</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16675,13 +16742,13 @@
         <v>387</v>
       </c>
       <c r="E25" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G25" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16698,13 +16765,13 @@
         <v>387</v>
       </c>
       <c r="E26" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G26" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16721,13 +16788,13 @@
         <v>387</v>
       </c>
       <c r="E27" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G27" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16744,13 +16811,13 @@
         <v>387</v>
       </c>
       <c r="E28" s="38" t="s">
-        <v>700</v>
+        <v>707</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G28" s="38" t="s">
-        <v>701</v>
+        <v>708</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16767,13 +16834,13 @@
         <v>387</v>
       </c>
       <c r="E29" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G29" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16790,13 +16857,13 @@
         <v>387</v>
       </c>
       <c r="E30" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G30" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16813,13 +16880,13 @@
         <v>387</v>
       </c>
       <c r="E31" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G31" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16836,13 +16903,13 @@
         <v>387</v>
       </c>
       <c r="E32" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G32" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16859,13 +16926,13 @@
         <v>382</v>
       </c>
       <c r="E33" s="38" t="s">
-        <v>690</v>
+        <v>697</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G33" s="38" t="s">
-        <v>691</v>
+        <v>698</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16882,13 +16949,13 @@
         <v>387</v>
       </c>
       <c r="E34" s="38" t="s">
-        <v>700</v>
+        <v>707</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G34" s="38" t="s">
-        <v>701</v>
+        <v>708</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16905,13 +16972,13 @@
         <v>387</v>
       </c>
       <c r="E35" s="38" t="s">
-        <v>690</v>
+        <v>697</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G35" s="38" t="s">
-        <v>691</v>
+        <v>698</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16928,13 +16995,13 @@
         <v>387</v>
       </c>
       <c r="E36" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G36" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16951,13 +17018,13 @@
         <v>387</v>
       </c>
       <c r="E37" s="38" t="s">
-        <v>700</v>
+        <v>707</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G37" s="38" t="s">
-        <v>701</v>
+        <v>708</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16974,13 +17041,13 @@
         <v>387</v>
       </c>
       <c r="E38" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G38" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16997,13 +17064,13 @@
         <v>387</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>690</v>
+        <v>697</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>702</v>
+        <v>709</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17020,13 +17087,13 @@
         <v>387</v>
       </c>
       <c r="E40" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G40" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17034,7 +17101,7 @@
         <v>491</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>703</v>
+        <v>710</v>
       </c>
       <c r="C41" s="12" t="n">
         <v>440300</v>
@@ -17043,13 +17110,13 @@
         <v>382</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>696</v>
+        <v>703</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>697</v>
+        <v>704</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>704</v>
+        <v>711</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17066,13 +17133,13 @@
         <v>387</v>
       </c>
       <c r="E42" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G42" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17080,7 +17147,7 @@
         <v>491</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>705</v>
+        <v>712</v>
       </c>
       <c r="C43" s="12" t="n">
         <v>-88073</v>
@@ -17089,13 +17156,13 @@
         <v>387</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17112,13 +17179,13 @@
         <v>387</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17126,7 +17193,7 @@
         <v>491</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>706</v>
+        <v>713</v>
       </c>
       <c r="C45" s="12" t="n">
         <v>-36259</v>
@@ -17135,13 +17202,13 @@
         <v>387</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17158,13 +17225,13 @@
         <v>387</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>707</v>
+        <v>714</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G46" s="3" t="s">
-        <v>708</v>
+        <v>715</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17172,7 +17239,7 @@
         <v>498</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>695</v>
+        <v>702</v>
       </c>
       <c r="C47" s="12" t="n">
         <v>-77990</v>
@@ -17181,13 +17248,13 @@
         <v>387</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17204,13 +17271,13 @@
         <v>387</v>
       </c>
       <c r="E48" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G48" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17227,13 +17294,13 @@
         <v>387</v>
       </c>
       <c r="E49" s="38" t="s">
-        <v>700</v>
+        <v>707</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G49" s="38" t="s">
-        <v>701</v>
+        <v>708</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17250,13 +17317,13 @@
         <v>387</v>
       </c>
       <c r="E50" s="38" t="s">
-        <v>690</v>
+        <v>697</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G50" s="38" t="s">
-        <v>691</v>
+        <v>698</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17273,13 +17340,13 @@
         <v>387</v>
       </c>
       <c r="E51" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G51" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17296,13 +17363,13 @@
         <v>387</v>
       </c>
       <c r="E52" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G52" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17319,13 +17386,13 @@
         <v>387</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>684</v>
+        <v>691</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>686</v>
+        <v>693</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17342,13 +17409,13 @@
         <v>387</v>
       </c>
       <c r="E54" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G54" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17356,7 +17423,7 @@
         <v>505</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>683</v>
+        <v>690</v>
       </c>
       <c r="C55" s="12" t="n">
         <v>-1000000</v>
@@ -17365,13 +17432,13 @@
         <v>387</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>684</v>
+        <v>691</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>686</v>
+        <v>693</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17388,13 +17455,13 @@
         <v>382</v>
       </c>
       <c r="E56" s="38" t="s">
-        <v>699</v>
+        <v>706</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G56" s="38" t="s">
-        <v>682</v>
+        <v>689</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17411,13 +17478,13 @@
         <v>382</v>
       </c>
       <c r="E57" s="38" t="s">
-        <v>680</v>
+        <v>687</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G57" s="38" t="s">
-        <v>682</v>
+        <v>689</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17425,7 +17492,7 @@
         <v>505</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>709</v>
+        <v>716</v>
       </c>
       <c r="C58" s="12" t="n">
         <v>-83300</v>
@@ -17434,13 +17501,13 @@
         <v>387</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17457,13 +17524,13 @@
         <v>387</v>
       </c>
       <c r="E59" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G59" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17480,13 +17547,13 @@
         <v>387</v>
       </c>
       <c r="E60" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G60" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17503,13 +17570,13 @@
         <v>387</v>
       </c>
       <c r="E61" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G61" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17526,13 +17593,13 @@
         <v>387</v>
       </c>
       <c r="E62" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G62" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17549,13 +17616,13 @@
         <v>387</v>
       </c>
       <c r="E63" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G63" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17572,13 +17639,13 @@
         <v>387</v>
       </c>
       <c r="E64" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G64" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17595,13 +17662,13 @@
         <v>387</v>
       </c>
       <c r="E65" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G65" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17618,13 +17685,13 @@
         <v>387</v>
       </c>
       <c r="E66" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F66" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G66" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17641,13 +17708,13 @@
         <v>382</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>710</v>
+        <v>717</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>711</v>
+        <v>718</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17664,13 +17731,13 @@
         <v>387</v>
       </c>
       <c r="E68" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G68" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17687,13 +17754,13 @@
         <v>387</v>
       </c>
       <c r="E69" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F69" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G69" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17710,13 +17777,13 @@
         <v>387</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>684</v>
+        <v>691</v>
       </c>
       <c r="F70" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>686</v>
+        <v>693</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17724,7 +17791,7 @@
         <v>522</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>712</v>
+        <v>719</v>
       </c>
       <c r="C71" s="12" t="n">
         <v>-25000</v>
@@ -17733,13 +17800,13 @@
         <v>387</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="F71" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G71" s="3" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17756,13 +17823,13 @@
         <v>387</v>
       </c>
       <c r="E72" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F72" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G72" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17779,13 +17846,13 @@
         <v>387</v>
       </c>
       <c r="E73" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F73" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G73" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17802,13 +17869,13 @@
         <v>387</v>
       </c>
       <c r="E74" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F74" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G74" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17825,13 +17892,13 @@
         <v>387</v>
       </c>
       <c r="E75" s="38" t="s">
-        <v>700</v>
+        <v>707</v>
       </c>
       <c r="F75" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G75" s="38" t="s">
-        <v>701</v>
+        <v>708</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17848,13 +17915,13 @@
         <v>387</v>
       </c>
       <c r="E76" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F76" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G76" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17871,13 +17938,13 @@
         <v>387</v>
       </c>
       <c r="E77" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F77" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G77" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17894,13 +17961,13 @@
         <v>387</v>
       </c>
       <c r="E78" s="38" t="s">
-        <v>700</v>
+        <v>707</v>
       </c>
       <c r="F78" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G78" s="38" t="s">
-        <v>701</v>
+        <v>708</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17908,7 +17975,7 @@
         <v>522</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>683</v>
+        <v>690</v>
       </c>
       <c r="C79" s="12" t="n">
         <v>-1000000</v>
@@ -17917,13 +17984,13 @@
         <v>387</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>684</v>
+        <v>691</v>
       </c>
       <c r="F79" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G79" s="3" t="s">
-        <v>686</v>
+        <v>693</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17940,13 +18007,13 @@
         <v>382</v>
       </c>
       <c r="E80" s="38" t="s">
-        <v>690</v>
+        <v>697</v>
       </c>
       <c r="F80" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G80" s="38" t="s">
-        <v>691</v>
+        <v>698</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17963,13 +18030,13 @@
         <v>387</v>
       </c>
       <c r="E81" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F81" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G81" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17986,13 +18053,13 @@
         <v>387</v>
       </c>
       <c r="E82" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F82" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G82" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18009,13 +18076,13 @@
         <v>387</v>
       </c>
       <c r="E83" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F83" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G83" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18032,13 +18099,13 @@
         <v>387</v>
       </c>
       <c r="E84" s="3" t="s">
-        <v>713</v>
+        <v>720</v>
       </c>
       <c r="F84" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G84" s="3" t="s">
-        <v>686</v>
+        <v>693</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18055,13 +18122,13 @@
         <v>387</v>
       </c>
       <c r="E85" s="38" t="s">
-        <v>700</v>
+        <v>707</v>
       </c>
       <c r="F85" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G85" s="38" t="s">
-        <v>701</v>
+        <v>708</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18078,13 +18145,13 @@
         <v>387</v>
       </c>
       <c r="E86" s="38" t="s">
-        <v>700</v>
+        <v>707</v>
       </c>
       <c r="F86" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G86" s="38" t="s">
-        <v>701</v>
+        <v>708</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18101,13 +18168,13 @@
         <v>387</v>
       </c>
       <c r="E87" s="38" t="s">
-        <v>690</v>
+        <v>697</v>
       </c>
       <c r="F87" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G87" s="38" t="s">
-        <v>691</v>
+        <v>698</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18124,13 +18191,13 @@
         <v>382</v>
       </c>
       <c r="E88" s="3" t="s">
-        <v>710</v>
+        <v>717</v>
       </c>
       <c r="F88" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>711</v>
+        <v>718</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18138,7 +18205,7 @@
         <v>532</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>683</v>
+        <v>690</v>
       </c>
       <c r="C89" s="12" t="n">
         <v>-160000</v>
@@ -18147,13 +18214,13 @@
         <v>387</v>
       </c>
       <c r="E89" s="3" t="s">
-        <v>684</v>
+        <v>691</v>
       </c>
       <c r="F89" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G89" s="3" t="s">
-        <v>686</v>
+        <v>693</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18170,13 +18237,13 @@
         <v>382</v>
       </c>
       <c r="E90" s="38" t="s">
-        <v>680</v>
+        <v>687</v>
       </c>
       <c r="F90" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G90" s="38" t="s">
-        <v>682</v>
+        <v>689</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18184,7 +18251,7 @@
         <v>532</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>683</v>
+        <v>690</v>
       </c>
       <c r="C91" s="12" t="n">
         <v>-150000</v>
@@ -18193,13 +18260,13 @@
         <v>387</v>
       </c>
       <c r="E91" s="3" t="s">
-        <v>684</v>
+        <v>691</v>
       </c>
       <c r="F91" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G91" s="3" t="s">
-        <v>686</v>
+        <v>693</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18216,13 +18283,13 @@
         <v>387</v>
       </c>
       <c r="E92" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F92" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G92" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18239,13 +18306,13 @@
         <v>387</v>
       </c>
       <c r="E93" s="3" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="F93" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G93" s="3" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18262,13 +18329,13 @@
         <v>387</v>
       </c>
       <c r="E94" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F94" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G94" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18285,13 +18352,13 @@
         <v>387</v>
       </c>
       <c r="E95" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F95" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G95" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18308,13 +18375,13 @@
         <v>387</v>
       </c>
       <c r="E96" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F96" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G96" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18331,13 +18398,13 @@
         <v>387</v>
       </c>
       <c r="E97" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F97" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G97" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18345,7 +18412,7 @@
         <v>542</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>714</v>
+        <v>721</v>
       </c>
       <c r="C98" s="12" t="n">
         <v>-405600</v>
@@ -18354,13 +18421,13 @@
         <v>387</v>
       </c>
       <c r="E98" s="3" t="s">
-        <v>715</v>
+        <v>722</v>
       </c>
       <c r="F98" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G98" s="3" t="s">
-        <v>716</v>
+        <v>723</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18368,7 +18435,7 @@
         <v>542</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>683</v>
+        <v>690</v>
       </c>
       <c r="C99" s="12" t="n">
         <v>-1000000</v>
@@ -18377,13 +18444,13 @@
         <v>387</v>
       </c>
       <c r="E99" s="3" t="s">
-        <v>684</v>
+        <v>691</v>
       </c>
       <c r="F99" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G99" s="3" t="s">
-        <v>686</v>
+        <v>693</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18400,13 +18467,13 @@
         <v>387</v>
       </c>
       <c r="E100" s="3" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="F100" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G100" s="3" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18423,13 +18490,13 @@
         <v>387</v>
       </c>
       <c r="E101" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F101" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G101" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18446,13 +18513,13 @@
         <v>387</v>
       </c>
       <c r="E102" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F102" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G102" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18469,13 +18536,13 @@
         <v>387</v>
       </c>
       <c r="E103" s="3" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="F103" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G103" s="3" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18492,13 +18559,13 @@
         <v>387</v>
       </c>
       <c r="E104" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F104" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G104" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18515,13 +18582,13 @@
         <v>382</v>
       </c>
       <c r="E105" s="38" t="s">
-        <v>690</v>
+        <v>697</v>
       </c>
       <c r="F105" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G105" s="38" t="s">
-        <v>691</v>
+        <v>698</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18538,13 +18605,13 @@
         <v>387</v>
       </c>
       <c r="E106" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F106" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G106" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18561,13 +18628,13 @@
         <v>387</v>
       </c>
       <c r="E107" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F107" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G107" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18584,13 +18651,13 @@
         <v>387</v>
       </c>
       <c r="E108" s="3" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="F108" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G108" s="3" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18607,13 +18674,13 @@
         <v>387</v>
       </c>
       <c r="E109" s="3" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="F109" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G109" s="3" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18621,7 +18688,7 @@
         <v>559</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>717</v>
+        <v>724</v>
       </c>
       <c r="C110" s="12" t="n">
         <v>-6950</v>
@@ -18630,13 +18697,13 @@
         <v>387</v>
       </c>
       <c r="E110" s="38" t="s">
-        <v>690</v>
+        <v>697</v>
       </c>
       <c r="F110" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G110" s="38" t="s">
-        <v>691</v>
+        <v>698</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18653,13 +18720,13 @@
         <v>387</v>
       </c>
       <c r="E111" s="38" t="s">
-        <v>700</v>
+        <v>707</v>
       </c>
       <c r="F111" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G111" s="38" t="s">
-        <v>701</v>
+        <v>708</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18676,13 +18743,13 @@
         <v>387</v>
       </c>
       <c r="E112" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F112" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G112" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18699,13 +18766,13 @@
         <v>387</v>
       </c>
       <c r="E113" s="3" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="F113" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G113" s="3" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18722,13 +18789,13 @@
         <v>387</v>
       </c>
       <c r="E114" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F114" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G114" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18745,13 +18812,13 @@
         <v>387</v>
       </c>
       <c r="E115" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F115" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G115" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18759,7 +18826,7 @@
         <v>559</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>718</v>
+        <v>725</v>
       </c>
       <c r="C116" s="12" t="n">
         <v>-38000</v>
@@ -18768,13 +18835,13 @@
         <v>387</v>
       </c>
       <c r="E116" s="3" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="F116" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G116" s="3" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18791,13 +18858,13 @@
         <v>387</v>
       </c>
       <c r="E117" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F117" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G117" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18814,13 +18881,13 @@
         <v>387</v>
       </c>
       <c r="E118" s="38" t="s">
-        <v>700</v>
+        <v>707</v>
       </c>
       <c r="F118" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G118" s="38" t="s">
-        <v>701</v>
+        <v>708</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18828,7 +18895,7 @@
         <v>559</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>719</v>
+        <v>726</v>
       </c>
       <c r="C119" s="12" t="n">
         <v>-66878</v>
@@ -18837,13 +18904,13 @@
         <v>387</v>
       </c>
       <c r="E119" s="38" t="s">
-        <v>690</v>
+        <v>697</v>
       </c>
       <c r="F119" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G119" s="38" t="s">
-        <v>691</v>
+        <v>698</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18860,13 +18927,13 @@
         <v>387</v>
       </c>
       <c r="E120" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F120" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G120" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18883,13 +18950,13 @@
         <v>387</v>
       </c>
       <c r="E121" s="38" t="s">
-        <v>700</v>
+        <v>707</v>
       </c>
       <c r="F121" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G121" s="38" t="s">
-        <v>701</v>
+        <v>708</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18897,7 +18964,7 @@
         <v>559</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>720</v>
+        <v>727</v>
       </c>
       <c r="C122" s="12" t="n">
         <v>-296037</v>
@@ -18906,13 +18973,13 @@
         <v>387</v>
       </c>
       <c r="E122" s="3" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="F122" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G122" s="3" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18929,13 +18996,13 @@
         <v>382</v>
       </c>
       <c r="E123" s="38" t="s">
-        <v>690</v>
+        <v>697</v>
       </c>
       <c r="F123" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G123" s="38" t="s">
-        <v>691</v>
+        <v>698</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18952,13 +19019,13 @@
         <v>382</v>
       </c>
       <c r="E124" s="38" t="s">
-        <v>690</v>
+        <v>697</v>
       </c>
       <c r="F124" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G124" s="38" t="s">
-        <v>691</v>
+        <v>698</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18975,13 +19042,13 @@
         <v>382</v>
       </c>
       <c r="E125" s="38" t="s">
-        <v>699</v>
+        <v>706</v>
       </c>
       <c r="F125" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G125" s="38" t="s">
-        <v>682</v>
+        <v>689</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18989,7 +19056,7 @@
         <v>559</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>721</v>
+        <v>728</v>
       </c>
       <c r="C126" s="12" t="n">
         <v>-58001</v>
@@ -18998,13 +19065,13 @@
         <v>387</v>
       </c>
       <c r="E126" s="38" t="s">
-        <v>690</v>
+        <v>697</v>
       </c>
       <c r="F126" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G126" s="38" t="s">
-        <v>691</v>
+        <v>698</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19021,13 +19088,13 @@
         <v>387</v>
       </c>
       <c r="E127" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F127" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G127" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19044,13 +19111,13 @@
         <v>387</v>
       </c>
       <c r="E128" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F128" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G128" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19058,7 +19125,7 @@
         <v>572</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>722</v>
+        <v>729</v>
       </c>
       <c r="C129" s="12" t="n">
         <v>-97000</v>
@@ -19067,13 +19134,13 @@
         <v>387</v>
       </c>
       <c r="E129" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F129" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G129" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19081,7 +19148,7 @@
         <v>572</v>
       </c>
       <c r="B130" s="3" t="s">
-        <v>683</v>
+        <v>690</v>
       </c>
       <c r="C130" s="12" t="n">
         <v>-800000</v>
@@ -19090,13 +19157,13 @@
         <v>387</v>
       </c>
       <c r="E130" s="3" t="s">
-        <v>684</v>
+        <v>691</v>
       </c>
       <c r="F130" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G130" s="3" t="s">
-        <v>686</v>
+        <v>693</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19113,13 +19180,13 @@
         <v>387</v>
       </c>
       <c r="E131" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F131" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G131" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19136,13 +19203,13 @@
         <v>387</v>
       </c>
       <c r="E132" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F132" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G132" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19159,13 +19226,13 @@
         <v>387</v>
       </c>
       <c r="E133" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F133" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G133" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19182,13 +19249,13 @@
         <v>387</v>
       </c>
       <c r="E134" s="38" t="s">
-        <v>700</v>
+        <v>707</v>
       </c>
       <c r="F134" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G134" s="38" t="s">
-        <v>701</v>
+        <v>708</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19205,13 +19272,13 @@
         <v>387</v>
       </c>
       <c r="E135" s="38" t="s">
-        <v>700</v>
+        <v>707</v>
       </c>
       <c r="F135" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G135" s="38" t="s">
-        <v>701</v>
+        <v>708</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19228,13 +19295,13 @@
         <v>387</v>
       </c>
       <c r="E136" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F136" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G136" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19251,13 +19318,13 @@
         <v>387</v>
       </c>
       <c r="E137" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F137" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G137" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19274,13 +19341,13 @@
         <v>382</v>
       </c>
       <c r="E138" s="38" t="s">
-        <v>680</v>
+        <v>687</v>
       </c>
       <c r="F138" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G138" s="38" t="s">
-        <v>682</v>
+        <v>689</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19297,13 +19364,13 @@
         <v>387</v>
       </c>
       <c r="E139" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F139" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G139" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19311,7 +19378,7 @@
         <v>445</v>
       </c>
       <c r="B140" s="3" t="s">
-        <v>683</v>
+        <v>690</v>
       </c>
       <c r="C140" s="12" t="n">
         <v>-700000</v>
@@ -19320,13 +19387,13 @@
         <v>387</v>
       </c>
       <c r="E140" s="3" t="s">
-        <v>684</v>
+        <v>691</v>
       </c>
       <c r="F140" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G140" s="3" t="s">
-        <v>686</v>
+        <v>693</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19343,13 +19410,13 @@
         <v>382</v>
       </c>
       <c r="E141" s="38" t="s">
-        <v>699</v>
+        <v>706</v>
       </c>
       <c r="F141" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G141" s="38" t="s">
-        <v>682</v>
+        <v>689</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19366,13 +19433,13 @@
         <v>387</v>
       </c>
       <c r="E142" s="3" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="F142" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G142" s="3" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19389,13 +19456,13 @@
         <v>387</v>
       </c>
       <c r="E143" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F143" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G143" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19412,13 +19479,13 @@
         <v>387</v>
       </c>
       <c r="E144" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F144" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G144" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19435,13 +19502,13 @@
         <v>387</v>
       </c>
       <c r="E145" s="38" t="s">
-        <v>700</v>
+        <v>707</v>
       </c>
       <c r="F145" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G145" s="38" t="s">
-        <v>701</v>
+        <v>708</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19458,13 +19525,13 @@
         <v>382</v>
       </c>
       <c r="E146" s="3" t="s">
-        <v>710</v>
+        <v>717</v>
       </c>
       <c r="F146" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G146" s="3" t="s">
-        <v>711</v>
+        <v>718</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19481,13 +19548,13 @@
         <v>387</v>
       </c>
       <c r="E147" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F147" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G147" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19504,13 +19571,13 @@
         <v>387</v>
       </c>
       <c r="E148" s="3" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="F148" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G148" s="3" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19518,7 +19585,7 @@
         <v>450</v>
       </c>
       <c r="B149" s="3" t="s">
-        <v>723</v>
+        <v>730</v>
       </c>
       <c r="C149" s="12" t="n">
         <v>-46550</v>
@@ -19527,13 +19594,13 @@
         <v>387</v>
       </c>
       <c r="E149" s="3" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="F149" s="3" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="G149" s="3" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19550,13 +19617,13 @@
         <v>387</v>
       </c>
       <c r="E150" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F150" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G150" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19573,18 +19640,18 @@
         <v>387</v>
       </c>
       <c r="E151" s="38" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F151" s="3" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="G151" s="38" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="2" t="s">
-        <v>724</v>
+        <v>731</v>
       </c>
       <c r="B153" s="2"/>
       <c r="C153" s="2"/>
@@ -19595,18 +19662,18 @@
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="9" t="s">
-        <v>725</v>
+        <v>732</v>
       </c>
       <c r="B154" s="9" t="s">
-        <v>726</v>
+        <v>733</v>
       </c>
       <c r="C154" s="9" t="s">
-        <v>727</v>
+        <v>734</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="3" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="B155" s="3" t="n">
         <v>72</v>
@@ -19617,7 +19684,7 @@
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="3" t="s">
-        <v>684</v>
+        <v>691</v>
       </c>
       <c r="B156" s="3" t="n">
         <v>10</v>
@@ -19628,7 +19695,7 @@
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="3" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="B157" s="3" t="n">
         <v>20</v>
@@ -19639,7 +19706,7 @@
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="3" t="s">
-        <v>700</v>
+        <v>707</v>
       </c>
       <c r="B158" s="3" t="n">
         <v>15</v>
@@ -19650,7 +19717,7 @@
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="3" t="s">
-        <v>715</v>
+        <v>722</v>
       </c>
       <c r="B159" s="3" t="n">
         <v>1</v>
@@ -19661,7 +19728,7 @@
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="3" t="s">
-        <v>707</v>
+        <v>714</v>
       </c>
       <c r="B160" s="3" t="n">
         <v>1</v>
@@ -19672,7 +19739,7 @@
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="3" t="s">
-        <v>713</v>
+        <v>720</v>
       </c>
       <c r="B161" s="3" t="n">
         <v>1</v>
@@ -19683,7 +19750,7 @@
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="3" t="s">
-        <v>696</v>
+        <v>703</v>
       </c>
       <c r="B162" s="3" t="n">
         <v>2</v>
@@ -19694,7 +19761,7 @@
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="3" t="s">
-        <v>690</v>
+        <v>697</v>
       </c>
       <c r="B163" s="3" t="n">
         <v>14</v>
@@ -19705,7 +19772,7 @@
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="3" t="s">
-        <v>699</v>
+        <v>706</v>
       </c>
       <c r="B164" s="3" t="n">
         <v>4</v>
@@ -19716,7 +19783,7 @@
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="3" t="s">
-        <v>680</v>
+        <v>687</v>
       </c>
       <c r="B165" s="3" t="n">
         <v>4</v>
@@ -19727,7 +19794,7 @@
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="3" t="s">
-        <v>710</v>
+        <v>717</v>
       </c>
       <c r="B166" s="3" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Agrega detalle Remuneraciones por Beneficiario y tabla CxC/CxF Pendientes al Informe de Julio
</commit_message>
<xml_diff>
--- a/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
+++ b/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3029" uniqueCount="746">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3077" uniqueCount="782">
   <si>
     <t xml:space="preserve">SUPUESTOS DEL PRESUPUESTO — SOLLEM + TRAST</t>
   </si>
@@ -2042,6 +2042,114 @@
   </si>
   <si>
     <t xml:space="preserve">S-85 (Presmita, 24-07) quedó registrado con tarifa $0 en servicios_piloto — posible error de carga, no se incluyó valor en Pendiente de Facturar por esa fila.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DETALLE — REMUNERACIONES POR BENEFICIARIO, JULIO (nombres truncados por el banco a 35 caracteres)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beneficiario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N° Transferencias</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Felipe Madaria[ga]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sebastián Zúñi[ga]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Francisco Manc[...]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multiaceros SA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Felipe Vidal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Riquelme Olea (Pablo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manuel Madrid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Felipe Tapia D[...]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marcelo Lira</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nicolás Carval[lo]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valdés Cornejo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">José Acevedo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Servicios Inte[grales]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL (13 beneficiarios reales, excluye traspaso interno Global Solutions)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CxC / CxF PENDIENTES AL CIERRE DE JULIO (kaptura_cuentas_por_cobrar + kaptura_cuentas_por_facturar)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estado / Fecha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CxC — facturado, sin cobrar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Servicios Logísticos Integrales SPA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Factoring programado 03-08-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Presmita (factura 27)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pendiente, sin fecha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Danilo Núñez (factura 24, junio)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CxF — ejecutado, sin facturar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Presmita</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 servicios julio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Citrus Agro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Danilo Núñez</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 servicios julio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sollem SpA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 servicios julio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trans Luciano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL PENDIENTE (CxC + CxF)</t>
   </si>
   <si>
     <t xml:space="preserve">PLAN vs. REAL vs. REPROYECCIÓN (flujo de caja semanal)</t>
@@ -2482,7 +2590,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2629,6 +2737,10 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
@@ -3342,7 +3454,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>735</v>
+        <v>771</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3352,7 +3464,7 @@
     </row>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="24" t="s">
-        <v>736</v>
+        <v>772</v>
       </c>
       <c r="B2" s="24"/>
       <c r="C2" s="24"/>
@@ -3365,16 +3477,16 @@
         <v>376</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>737</v>
+        <v>773</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>738</v>
+        <v>774</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>739</v>
+        <v>775</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>740</v>
+        <v>776</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>188</v>
@@ -3388,23 +3500,23 @@
         <v>63371</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>741</v>
-      </c>
-      <c r="D5" s="37"/>
-      <c r="E5" s="37"/>
+        <v>777</v>
+      </c>
+      <c r="D5" s="38"/>
+      <c r="E5" s="38"/>
       <c r="F5" s="3" t="s">
-        <v>742</v>
+        <v>778</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>743</v>
+        <v>779</v>
       </c>
       <c r="B6" s="12" t="n">
         <v>1275801</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>744</v>
+        <v>780</v>
       </c>
       <c r="D6" s="34"/>
       <c r="E6" s="12" t="str">
@@ -3412,283 +3524,283 @@
         <v/>
       </c>
       <c r="F6" s="3" t="s">
-        <v>745</v>
+        <v>781</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="39"/>
+      <c r="A7" s="40"/>
       <c r="B7" s="34"/>
-      <c r="C7" s="39"/>
+      <c r="C7" s="40"/>
       <c r="D7" s="34"/>
       <c r="E7" s="12" t="str">
         <f aca="false">IF(OR(B7="",D7=""),"",B7-D7)</f>
         <v/>
       </c>
-      <c r="F7" s="39"/>
+      <c r="F7" s="40"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="39"/>
+      <c r="A8" s="40"/>
       <c r="B8" s="34"/>
-      <c r="C8" s="39"/>
+      <c r="C8" s="40"/>
       <c r="D8" s="34"/>
       <c r="E8" s="12" t="str">
         <f aca="false">IF(OR(B8="",D8=""),"",B8-D8)</f>
         <v/>
       </c>
-      <c r="F8" s="39"/>
+      <c r="F8" s="40"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="39"/>
+      <c r="A9" s="40"/>
       <c r="B9" s="34"/>
-      <c r="C9" s="39"/>
+      <c r="C9" s="40"/>
       <c r="D9" s="34"/>
       <c r="E9" s="12" t="str">
         <f aca="false">IF(OR(B9="",D9=""),"",B9-D9)</f>
         <v/>
       </c>
-      <c r="F9" s="39"/>
+      <c r="F9" s="40"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="39"/>
+      <c r="A10" s="40"/>
       <c r="B10" s="34"/>
-      <c r="C10" s="39"/>
+      <c r="C10" s="40"/>
       <c r="D10" s="34"/>
       <c r="E10" s="12" t="str">
         <f aca="false">IF(OR(B10="",D10=""),"",B10-D10)</f>
         <v/>
       </c>
-      <c r="F10" s="39"/>
+      <c r="F10" s="40"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="39"/>
+      <c r="A11" s="40"/>
       <c r="B11" s="34"/>
-      <c r="C11" s="39"/>
+      <c r="C11" s="40"/>
       <c r="D11" s="34"/>
       <c r="E11" s="12" t="str">
         <f aca="false">IF(OR(B11="",D11=""),"",B11-D11)</f>
         <v/>
       </c>
-      <c r="F11" s="39"/>
+      <c r="F11" s="40"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="39"/>
+      <c r="A12" s="40"/>
       <c r="B12" s="34"/>
-      <c r="C12" s="39"/>
+      <c r="C12" s="40"/>
       <c r="D12" s="34"/>
       <c r="E12" s="12" t="str">
         <f aca="false">IF(OR(B12="",D12=""),"",B12-D12)</f>
         <v/>
       </c>
-      <c r="F12" s="39"/>
+      <c r="F12" s="40"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="39"/>
+      <c r="A13" s="40"/>
       <c r="B13" s="34"/>
-      <c r="C13" s="39"/>
+      <c r="C13" s="40"/>
       <c r="D13" s="34"/>
       <c r="E13" s="12" t="str">
         <f aca="false">IF(OR(B13="",D13=""),"",B13-D13)</f>
         <v/>
       </c>
-      <c r="F13" s="39"/>
+      <c r="F13" s="40"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="39"/>
+      <c r="A14" s="40"/>
       <c r="B14" s="34"/>
-      <c r="C14" s="39"/>
+      <c r="C14" s="40"/>
       <c r="D14" s="34"/>
       <c r="E14" s="12" t="str">
         <f aca="false">IF(OR(B14="",D14=""),"",B14-D14)</f>
         <v/>
       </c>
-      <c r="F14" s="39"/>
+      <c r="F14" s="40"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="39"/>
+      <c r="A15" s="40"/>
       <c r="B15" s="34"/>
-      <c r="C15" s="39"/>
+      <c r="C15" s="40"/>
       <c r="D15" s="34"/>
       <c r="E15" s="12" t="str">
         <f aca="false">IF(OR(B15="",D15=""),"",B15-D15)</f>
         <v/>
       </c>
-      <c r="F15" s="39"/>
+      <c r="F15" s="40"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="39"/>
+      <c r="A16" s="40"/>
       <c r="B16" s="34"/>
-      <c r="C16" s="39"/>
+      <c r="C16" s="40"/>
       <c r="D16" s="34"/>
       <c r="E16" s="12" t="str">
         <f aca="false">IF(OR(B16="",D16=""),"",B16-D16)</f>
         <v/>
       </c>
-      <c r="F16" s="39"/>
+      <c r="F16" s="40"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="39"/>
+      <c r="A17" s="40"/>
       <c r="B17" s="34"/>
-      <c r="C17" s="39"/>
+      <c r="C17" s="40"/>
       <c r="D17" s="34"/>
       <c r="E17" s="12" t="str">
         <f aca="false">IF(OR(B17="",D17=""),"",B17-D17)</f>
         <v/>
       </c>
-      <c r="F17" s="39"/>
+      <c r="F17" s="40"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="39"/>
+      <c r="A18" s="40"/>
       <c r="B18" s="34"/>
-      <c r="C18" s="39"/>
+      <c r="C18" s="40"/>
       <c r="D18" s="34"/>
       <c r="E18" s="12" t="str">
         <f aca="false">IF(OR(B18="",D18=""),"",B18-D18)</f>
         <v/>
       </c>
-      <c r="F18" s="39"/>
+      <c r="F18" s="40"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="39"/>
+      <c r="A19" s="40"/>
       <c r="B19" s="34"/>
-      <c r="C19" s="39"/>
+      <c r="C19" s="40"/>
       <c r="D19" s="34"/>
       <c r="E19" s="12" t="str">
         <f aca="false">IF(OR(B19="",D19=""),"",B19-D19)</f>
         <v/>
       </c>
-      <c r="F19" s="39"/>
+      <c r="F19" s="40"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="39"/>
+      <c r="A20" s="40"/>
       <c r="B20" s="34"/>
-      <c r="C20" s="39"/>
+      <c r="C20" s="40"/>
       <c r="D20" s="34"/>
       <c r="E20" s="12" t="str">
         <f aca="false">IF(OR(B20="",D20=""),"",B20-D20)</f>
         <v/>
       </c>
-      <c r="F20" s="39"/>
+      <c r="F20" s="40"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="39"/>
+      <c r="A21" s="40"/>
       <c r="B21" s="34"/>
-      <c r="C21" s="39"/>
+      <c r="C21" s="40"/>
       <c r="D21" s="34"/>
       <c r="E21" s="12" t="str">
         <f aca="false">IF(OR(B21="",D21=""),"",B21-D21)</f>
         <v/>
       </c>
-      <c r="F21" s="39"/>
+      <c r="F21" s="40"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="39"/>
+      <c r="A22" s="40"/>
       <c r="B22" s="34"/>
-      <c r="C22" s="39"/>
+      <c r="C22" s="40"/>
       <c r="D22" s="34"/>
       <c r="E22" s="12" t="str">
         <f aca="false">IF(OR(B22="",D22=""),"",B22-D22)</f>
         <v/>
       </c>
-      <c r="F22" s="39"/>
+      <c r="F22" s="40"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="39"/>
+      <c r="A23" s="40"/>
       <c r="B23" s="34"/>
-      <c r="C23" s="39"/>
+      <c r="C23" s="40"/>
       <c r="D23" s="34"/>
       <c r="E23" s="12" t="str">
         <f aca="false">IF(OR(B23="",D23=""),"",B23-D23)</f>
         <v/>
       </c>
-      <c r="F23" s="39"/>
+      <c r="F23" s="40"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="39"/>
+      <c r="A24" s="40"/>
       <c r="B24" s="34"/>
-      <c r="C24" s="39"/>
+      <c r="C24" s="40"/>
       <c r="D24" s="34"/>
       <c r="E24" s="12" t="str">
         <f aca="false">IF(OR(B24="",D24=""),"",B24-D24)</f>
         <v/>
       </c>
-      <c r="F24" s="39"/>
+      <c r="F24" s="40"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="39"/>
+      <c r="A25" s="40"/>
       <c r="B25" s="34"/>
-      <c r="C25" s="39"/>
+      <c r="C25" s="40"/>
       <c r="D25" s="34"/>
       <c r="E25" s="12" t="str">
         <f aca="false">IF(OR(B25="",D25=""),"",B25-D25)</f>
         <v/>
       </c>
-      <c r="F25" s="39"/>
+      <c r="F25" s="40"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="39"/>
+      <c r="A26" s="40"/>
       <c r="B26" s="34"/>
-      <c r="C26" s="39"/>
+      <c r="C26" s="40"/>
       <c r="D26" s="34"/>
       <c r="E26" s="12" t="str">
         <f aca="false">IF(OR(B26="",D26=""),"",B26-D26)</f>
         <v/>
       </c>
-      <c r="F26" s="39"/>
+      <c r="F26" s="40"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="39"/>
+      <c r="A27" s="40"/>
       <c r="B27" s="34"/>
-      <c r="C27" s="39"/>
+      <c r="C27" s="40"/>
       <c r="D27" s="34"/>
       <c r="E27" s="12" t="str">
         <f aca="false">IF(OR(B27="",D27=""),"",B27-D27)</f>
         <v/>
       </c>
-      <c r="F27" s="39"/>
+      <c r="F27" s="40"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="39"/>
+      <c r="A28" s="40"/>
       <c r="B28" s="34"/>
-      <c r="C28" s="39"/>
+      <c r="C28" s="40"/>
       <c r="D28" s="34"/>
       <c r="E28" s="12" t="str">
         <f aca="false">IF(OR(B28="",D28=""),"",B28-D28)</f>
         <v/>
       </c>
-      <c r="F28" s="39"/>
+      <c r="F28" s="40"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="39"/>
+      <c r="A29" s="40"/>
       <c r="B29" s="34"/>
-      <c r="C29" s="39"/>
+      <c r="C29" s="40"/>
       <c r="D29" s="34"/>
       <c r="E29" s="12" t="str">
         <f aca="false">IF(OR(B29="",D29=""),"",B29-D29)</f>
         <v/>
       </c>
-      <c r="F29" s="39"/>
+      <c r="F29" s="40"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="39"/>
+      <c r="A30" s="40"/>
       <c r="B30" s="34"/>
-      <c r="C30" s="39"/>
+      <c r="C30" s="40"/>
       <c r="D30" s="34"/>
       <c r="E30" s="12" t="str">
         <f aca="false">IF(OR(B30="",D30=""),"",B30-D30)</f>
         <v/>
       </c>
-      <c r="F30" s="39"/>
+      <c r="F30" s="40"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="39"/>
+      <c r="A31" s="40"/>
       <c r="B31" s="34"/>
-      <c r="C31" s="39"/>
+      <c r="C31" s="40"/>
       <c r="D31" s="34"/>
       <c r="E31" s="12" t="str">
         <f aca="false">IF(OR(B31="",D31=""),"",B31-D31)</f>
         <v/>
       </c>
-      <c r="F31" s="39"/>
+      <c r="F31" s="40"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -15480,7 +15592,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G88"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -15916,253 +16028,570 @@
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
-      <c r="E47" s="2"/>
-      <c r="F47" s="2"/>
-      <c r="G47" s="2"/>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="28" t="s">
+    </row>
+    <row r="48" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="9" t="s">
         <v>668</v>
       </c>
-      <c r="B48" s="28"/>
-      <c r="C48" s="28"/>
-      <c r="D48" s="28"/>
-      <c r="E48" s="28"/>
-      <c r="F48" s="28"/>
-      <c r="G48" s="28"/>
+      <c r="B48" s="9" t="s">
+        <v>669</v>
+      </c>
+      <c r="C48" s="9" t="s">
+        <v>186</v>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="2" t="s">
-        <v>669</v>
-      </c>
-      <c r="B49" s="2"/>
-      <c r="C49" s="2"/>
-      <c r="D49" s="2"/>
-      <c r="E49" s="2"/>
-      <c r="F49" s="2"/>
-      <c r="G49" s="2"/>
-    </row>
-    <row r="50" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="B50" s="9" t="s">
+      <c r="A49" s="3" t="s">
         <v>670</v>
       </c>
-      <c r="C50" s="9" t="s">
+      <c r="B49" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="C49" s="12" t="n">
+        <v>1301800</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="3" t="s">
         <v>671</v>
       </c>
-      <c r="D50" s="9" t="s">
-        <v>672</v>
-      </c>
-      <c r="E50" s="9" t="s">
-        <v>673</v>
-      </c>
-      <c r="F50" s="9" t="s">
-        <v>674</v>
-      </c>
-      <c r="G50" s="9" t="s">
-        <v>675</v>
+      <c r="B50" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="C50" s="12" t="n">
+        <v>1122000</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
+        <v>672</v>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="C51" s="12" t="n">
+        <v>1005000</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="3" t="s">
+        <v>673</v>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" s="12" t="n">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="3" t="s">
+        <v>674</v>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C53" s="12" t="n">
+        <v>900000</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="3" t="s">
+        <v>675</v>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C54" s="12" t="n">
+        <v>855000</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="3" t="s">
         <v>676</v>
       </c>
-      <c r="B51" s="33" t="n">
+      <c r="B55" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C55" s="12" t="n">
+        <v>432000</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="3" t="s">
+        <v>677</v>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C56" s="12" t="n">
+        <v>280000</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="3" t="s">
+        <v>678</v>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C57" s="12" t="n">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="3" t="s">
+        <v>679</v>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C58" s="12" t="n">
+        <v>190000</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="3" t="s">
+        <v>680</v>
+      </c>
+      <c r="B59" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C59" s="12" t="n">
+        <v>97000</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="3" t="s">
+        <v>681</v>
+      </c>
+      <c r="B60" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C60" s="12" t="n">
+        <v>54000</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="3" t="s">
+        <v>682</v>
+      </c>
+      <c r="B61" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C61" s="12" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="15" t="s">
+        <v>683</v>
+      </c>
+      <c r="B62" s="15" t="n">
+        <v>82</v>
+      </c>
+      <c r="C62" s="17" t="n">
+        <v>7516800</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="2" t="s">
+        <v>684</v>
+      </c>
+      <c r="B64" s="2"/>
+      <c r="C64" s="2"/>
+      <c r="D64" s="2"/>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="9" t="s">
+        <v>685</v>
+      </c>
+      <c r="B65" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="C65" s="9" t="s">
+        <v>378</v>
+      </c>
+      <c r="D65" s="9" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="3" t="s">
+        <v>687</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>688</v>
+      </c>
+      <c r="C66" s="12" t="n">
+        <v>3053216</v>
+      </c>
+      <c r="D66" s="3" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="3" t="s">
+        <v>687</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>690</v>
+      </c>
+      <c r="C67" s="12" t="n">
+        <v>1428000</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="3" t="s">
+        <v>687</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>692</v>
+      </c>
+      <c r="C68" s="12" t="n">
+        <v>690200</v>
+      </c>
+      <c r="D68" s="3" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="3" t="s">
+        <v>693</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>694</v>
+      </c>
+      <c r="C69" s="12" t="n">
+        <v>2700000</v>
+      </c>
+      <c r="D69" s="3" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="3" t="s">
+        <v>693</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>696</v>
+      </c>
+      <c r="C70" s="12" t="n">
+        <v>2602400</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="3" t="s">
+        <v>693</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>697</v>
+      </c>
+      <c r="C71" s="12" t="n">
+        <v>1130000</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="3" t="s">
+        <v>693</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>699</v>
+      </c>
+      <c r="C72" s="12" t="n">
+        <v>1100800</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="3" t="s">
+        <v>693</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>701</v>
+      </c>
+      <c r="C73" s="12" t="n">
+        <v>630000</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="15" t="s">
+        <v>702</v>
+      </c>
+      <c r="B74" s="37"/>
+      <c r="C74" s="17" t="n">
+        <v>13334616</v>
+      </c>
+      <c r="D74" s="37"/>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="2" t="s">
+        <v>703</v>
+      </c>
+      <c r="B76" s="2"/>
+      <c r="C76" s="2"/>
+      <c r="D76" s="2"/>
+      <c r="E76" s="2"/>
+      <c r="F76" s="2"/>
+      <c r="G76" s="2"/>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="28" t="s">
+        <v>704</v>
+      </c>
+      <c r="B77" s="28"/>
+      <c r="C77" s="28"/>
+      <c r="D77" s="28"/>
+      <c r="E77" s="28"/>
+      <c r="F77" s="28"/>
+      <c r="G77" s="28"/>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="B78" s="2"/>
+      <c r="C78" s="2"/>
+      <c r="D78" s="2"/>
+      <c r="E78" s="2"/>
+      <c r="F78" s="2"/>
+      <c r="G78" s="2"/>
+    </row>
+    <row r="79" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B79" s="9" t="s">
+        <v>706</v>
+      </c>
+      <c r="C79" s="9" t="s">
+        <v>707</v>
+      </c>
+      <c r="D79" s="9" t="s">
+        <v>708</v>
+      </c>
+      <c r="E79" s="9" t="s">
+        <v>709</v>
+      </c>
+      <c r="F79" s="9" t="s">
+        <v>710</v>
+      </c>
+      <c r="G79" s="9" t="s">
+        <v>711</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="3" t="s">
+        <v>712</v>
+      </c>
+      <c r="B80" s="33" t="n">
         <f aca="false">Consolidado!B32</f>
         <v>29402660.3612933</v>
       </c>
-      <c r="C51" s="12" t="n">
+      <c r="C80" s="12" t="n">
         <f aca="false">SUM(Real_vs_Presupuesto!C6:C11)</f>
         <v>0</v>
       </c>
-      <c r="D51" s="35" t="str">
+      <c r="D80" s="35" t="str">
         <f aca="false">COUNT(Real_vs_Presupuesto!C6:C11)&amp;" de 6"</f>
         <v>0 de 6</v>
       </c>
-      <c r="E51" s="12" t="n">
+      <c r="E80" s="12" t="n">
         <f aca="false">SUMIF(Real_vs_Presupuesto!C6:C11,"",Real_vs_Presupuesto!B6:B11)</f>
         <v>29402660.3612933</v>
       </c>
-      <c r="F51" s="14" t="n">
-        <f aca="false">C51+E51</f>
+      <c r="F80" s="14" t="n">
+        <f aca="false">C80+E80</f>
         <v>29402660.3612933</v>
       </c>
-      <c r="G51" s="27" t="n">
-        <f aca="false">F51/B51</f>
+      <c r="G80" s="27" t="n">
+        <f aca="false">F80/B80</f>
         <v>1</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="3" t="s">
-        <v>677</v>
-      </c>
-      <c r="B52" s="33" t="n">
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="3" t="s">
+        <v>713</v>
+      </c>
+      <c r="B81" s="33" t="n">
         <f aca="false">Consolidado!C32</f>
         <v>26434798.4092921</v>
       </c>
-      <c r="C52" s="12" t="n">
+      <c r="C81" s="12" t="n">
         <f aca="false">SUM(Real_vs_Presupuesto!F6:F11)</f>
         <v>0</v>
       </c>
-      <c r="D52" s="35" t="str">
+      <c r="D81" s="35" t="str">
         <f aca="false">COUNT(Real_vs_Presupuesto!F6:F11)&amp;" de 6"</f>
         <v>0 de 6</v>
       </c>
-      <c r="E52" s="12" t="n">
+      <c r="E81" s="12" t="n">
         <f aca="false">SUMIF(Real_vs_Presupuesto!F6:F11,"",Real_vs_Presupuesto!E6:E11)</f>
         <v>26434798.4092921</v>
       </c>
-      <c r="F52" s="14" t="n">
-        <f aca="false">C52+E52</f>
+      <c r="F81" s="14" t="n">
+        <f aca="false">C81+E81</f>
         <v>26434798.4092921</v>
       </c>
-      <c r="G52" s="27" t="n">
-        <f aca="false">F52/B52</f>
+      <c r="G81" s="27" t="n">
+        <f aca="false">F81/B81</f>
         <v>1</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="18" t="s">
-        <v>678</v>
-      </c>
-      <c r="B53" s="14" t="n">
-        <f aca="false">B51-B52</f>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="18" t="s">
+        <v>714</v>
+      </c>
+      <c r="B82" s="14" t="n">
+        <f aca="false">B80-B81</f>
         <v>2967861.9520012</v>
       </c>
-      <c r="C53" s="14" t="n">
-        <f aca="false">C51-C52</f>
+      <c r="C82" s="14" t="n">
+        <f aca="false">C80-C81</f>
         <v>0</v>
       </c>
-      <c r="D53" s="37"/>
-      <c r="E53" s="14" t="n">
-        <f aca="false">E51-E52</f>
+      <c r="D82" s="38"/>
+      <c r="E82" s="14" t="n">
+        <f aca="false">E80-E81</f>
         <v>2967861.9520012</v>
       </c>
-      <c r="F53" s="14" t="n">
-        <f aca="false">F51-F52</f>
+      <c r="F82" s="14" t="n">
+        <f aca="false">F80-F81</f>
         <v>2967861.9520012</v>
       </c>
-      <c r="G53" s="37"/>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="2" t="s">
-        <v>679</v>
-      </c>
-      <c r="B55" s="2"/>
-      <c r="C55" s="2"/>
-      <c r="D55" s="2"/>
-      <c r="E55" s="2"/>
-      <c r="F55" s="2"/>
-      <c r="G55" s="2"/>
-    </row>
-    <row r="56" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="9" t="s">
+      <c r="G82" s="38"/>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="2" t="s">
+        <v>715</v>
+      </c>
+      <c r="B84" s="2"/>
+      <c r="C84" s="2"/>
+      <c r="D84" s="2"/>
+      <c r="E84" s="2"/>
+      <c r="F84" s="2"/>
+      <c r="G84" s="2"/>
+    </row>
+    <row r="85" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="B56" s="9" t="s">
-        <v>670</v>
-      </c>
-      <c r="C56" s="9" t="s">
-        <v>671</v>
-      </c>
-      <c r="D56" s="9" t="s">
-        <v>672</v>
-      </c>
-      <c r="E56" s="9" t="s">
-        <v>673</v>
-      </c>
-      <c r="F56" s="9" t="s">
-        <v>674</v>
-      </c>
-      <c r="G56" s="9" t="s">
-        <v>675</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="3" t="s">
-        <v>676</v>
-      </c>
-      <c r="B57" s="33" t="n">
+      <c r="B85" s="9" t="s">
+        <v>706</v>
+      </c>
+      <c r="C85" s="9" t="s">
+        <v>707</v>
+      </c>
+      <c r="D85" s="9" t="s">
+        <v>708</v>
+      </c>
+      <c r="E85" s="9" t="s">
+        <v>709</v>
+      </c>
+      <c r="F85" s="9" t="s">
+        <v>710</v>
+      </c>
+      <c r="G85" s="9" t="s">
+        <v>711</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="3" t="s">
+        <v>712</v>
+      </c>
+      <c r="B86" s="33" t="n">
         <f aca="false">Consolidado!B41</f>
         <v>38030368.58194</v>
       </c>
-      <c r="C57" s="12" t="n">
+      <c r="C86" s="12" t="n">
         <f aca="false">SUM(Real_vs_Presupuesto!C15:C19)</f>
         <v>0</v>
       </c>
-      <c r="D57" s="35" t="str">
+      <c r="D86" s="35" t="str">
         <f aca="false">COUNT(Real_vs_Presupuesto!C15:C19)&amp;" de 5"</f>
         <v>0 de 5</v>
       </c>
-      <c r="E57" s="12" t="n">
+      <c r="E86" s="12" t="n">
         <f aca="false">SUMIF(Real_vs_Presupuesto!C15:C19,"",Real_vs_Presupuesto!B15:B19)</f>
         <v>38030368.58194</v>
       </c>
-      <c r="F57" s="14" t="n">
-        <f aca="false">C57+E57</f>
+      <c r="F86" s="14" t="n">
+        <f aca="false">C86+E86</f>
         <v>38030368.58194</v>
       </c>
-      <c r="G57" s="27" t="n">
-        <f aca="false">F57/B57</f>
+      <c r="G86" s="27" t="n">
+        <f aca="false">F86/B86</f>
         <v>1</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="3" t="s">
-        <v>677</v>
-      </c>
-      <c r="B58" s="33" t="n">
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="3" t="s">
+        <v>713</v>
+      </c>
+      <c r="B87" s="33" t="n">
         <f aca="false">Consolidado!C41</f>
         <v>33067690.8539382</v>
       </c>
-      <c r="C58" s="12" t="n">
+      <c r="C87" s="12" t="n">
         <f aca="false">SUM(Real_vs_Presupuesto!F15:F19)</f>
         <v>0</v>
       </c>
-      <c r="D58" s="35" t="str">
+      <c r="D87" s="35" t="str">
         <f aca="false">COUNT(Real_vs_Presupuesto!F15:F19)&amp;" de 5"</f>
         <v>0 de 5</v>
       </c>
-      <c r="E58" s="12" t="n">
+      <c r="E87" s="12" t="n">
         <f aca="false">SUMIF(Real_vs_Presupuesto!F15:F19,"",Real_vs_Presupuesto!E15:E19)</f>
         <v>33067690.8539382</v>
       </c>
-      <c r="F58" s="14" t="n">
-        <f aca="false">C58+E58</f>
+      <c r="F87" s="14" t="n">
+        <f aca="false">C87+E87</f>
         <v>33067690.8539382</v>
       </c>
-      <c r="G58" s="27" t="n">
-        <f aca="false">F58/B58</f>
+      <c r="G87" s="27" t="n">
+        <f aca="false">F87/B87</f>
         <v>1</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="18" t="s">
-        <v>678</v>
-      </c>
-      <c r="B59" s="14" t="n">
-        <f aca="false">B57-B58</f>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="18" t="s">
+        <v>714</v>
+      </c>
+      <c r="B88" s="14" t="n">
+        <f aca="false">B86-B87</f>
         <v>4962677.7280018</v>
       </c>
-      <c r="C59" s="14" t="n">
-        <f aca="false">C57-C58</f>
+      <c r="C88" s="14" t="n">
+        <f aca="false">C86-C87</f>
         <v>0</v>
       </c>
-      <c r="D59" s="37"/>
-      <c r="E59" s="14" t="n">
-        <f aca="false">E57-E58</f>
+      <c r="D88" s="38"/>
+      <c r="E88" s="14" t="n">
+        <f aca="false">E86-E87</f>
         <v>4962677.7280018</v>
       </c>
-      <c r="F59" s="14" t="n">
-        <f aca="false">F57-F58</f>
+      <c r="F88" s="14" t="n">
+        <f aca="false">F86-F87</f>
         <v>4962677.7280018</v>
       </c>
-      <c r="G59" s="37"/>
+      <c r="G88" s="38"/>
     </row>
   </sheetData>
-  <mergeCells count="32">
+  <mergeCells count="34">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A17:G17"/>
@@ -16191,10 +16620,12 @@
     <mergeCell ref="A43:G43"/>
     <mergeCell ref="A44:G44"/>
     <mergeCell ref="A45:G45"/>
-    <mergeCell ref="A47:G47"/>
-    <mergeCell ref="A48:G48"/>
-    <mergeCell ref="A49:G49"/>
-    <mergeCell ref="A55:G55"/>
+    <mergeCell ref="A47:D47"/>
+    <mergeCell ref="A64:D64"/>
+    <mergeCell ref="A76:G76"/>
+    <mergeCell ref="A77:G77"/>
+    <mergeCell ref="A78:G78"/>
+    <mergeCell ref="A84:G84"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -16225,7 +16656,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>680</v>
+        <v>716</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -16236,7 +16667,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="24" t="s">
-        <v>681</v>
+        <v>717</v>
       </c>
       <c r="B2" s="24"/>
       <c r="C2" s="24"/>
@@ -16250,22 +16681,22 @@
         <v>376</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>378</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>683</v>
+        <v>719</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>684</v>
+        <v>720</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>685</v>
+        <v>721</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>686</v>
+        <v>722</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16281,14 +16712,14 @@
       <c r="D5" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="E5" s="38" t="s">
-        <v>687</v>
+      <c r="E5" s="39" t="s">
+        <v>723</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G5" s="38" t="s">
-        <v>689</v>
+        <v>724</v>
+      </c>
+      <c r="G5" s="39" t="s">
+        <v>725</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16296,7 +16727,7 @@
         <v>435</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>690</v>
+        <v>726</v>
       </c>
       <c r="C6" s="12" t="n">
         <v>-1300000</v>
@@ -16305,13 +16736,13 @@
         <v>387</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>691</v>
+        <v>727</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>693</v>
+        <v>729</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16327,14 +16758,14 @@
       <c r="D7" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E7" s="38" t="s">
-        <v>694</v>
+      <c r="E7" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G7" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G7" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16350,14 +16781,14 @@
       <c r="D8" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E8" s="38" t="s">
-        <v>694</v>
+      <c r="E8" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G8" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G8" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16373,14 +16804,14 @@
       <c r="D9" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E9" s="38" t="s">
-        <v>694</v>
+      <c r="E9" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G9" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G9" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16396,14 +16827,14 @@
       <c r="D10" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E10" s="38" t="s">
-        <v>694</v>
+      <c r="E10" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G10" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G10" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16419,14 +16850,14 @@
       <c r="D11" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E11" s="38" t="s">
-        <v>694</v>
+      <c r="E11" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G11" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G11" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16442,14 +16873,14 @@
       <c r="D12" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E12" s="38" t="s">
-        <v>694</v>
+      <c r="E12" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G12" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G12" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16457,7 +16888,7 @@
         <v>459</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>696</v>
+        <v>732</v>
       </c>
       <c r="C13" s="12" t="n">
         <v>-30000</v>
@@ -16465,14 +16896,14 @@
       <c r="D13" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E13" s="38" t="s">
-        <v>694</v>
+      <c r="E13" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G13" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G13" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16488,14 +16919,14 @@
       <c r="D14" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E14" s="38" t="s">
-        <v>697</v>
+      <c r="E14" s="39" t="s">
+        <v>733</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G14" s="38" t="s">
-        <v>698</v>
+        <v>724</v>
+      </c>
+      <c r="G14" s="39" t="s">
+        <v>734</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16511,14 +16942,14 @@
       <c r="D15" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E15" s="38" t="s">
-        <v>694</v>
+      <c r="E15" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G15" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G15" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16534,14 +16965,14 @@
       <c r="D16" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E16" s="38" t="s">
-        <v>694</v>
+      <c r="E16" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G16" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G16" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16549,7 +16980,7 @@
         <v>473</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>699</v>
+        <v>735</v>
       </c>
       <c r="C17" s="12" t="n">
         <v>-92344</v>
@@ -16558,13 +16989,13 @@
         <v>387</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>700</v>
+        <v>736</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>701</v>
+        <v>737</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16580,14 +17011,14 @@
       <c r="D18" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E18" s="38" t="s">
-        <v>694</v>
+      <c r="E18" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G18" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G18" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16595,7 +17026,7 @@
         <v>473</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>702</v>
+        <v>738</v>
       </c>
       <c r="C19" s="12" t="n">
         <v>-17980</v>
@@ -16604,13 +17035,13 @@
         <v>387</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>700</v>
+        <v>736</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>701</v>
+        <v>737</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16627,13 +17058,13 @@
         <v>382</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>703</v>
+        <v>739</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>704</v>
+        <v>740</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>705</v>
+        <v>741</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16649,14 +17080,14 @@
       <c r="D21" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="E21" s="38" t="s">
-        <v>697</v>
+      <c r="E21" s="39" t="s">
+        <v>733</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G21" s="38" t="s">
-        <v>698</v>
+        <v>724</v>
+      </c>
+      <c r="G21" s="39" t="s">
+        <v>734</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16672,14 +17103,14 @@
       <c r="D22" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="E22" s="38" t="s">
-        <v>706</v>
+      <c r="E22" s="39" t="s">
+        <v>742</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G22" s="38" t="s">
-        <v>689</v>
+        <v>724</v>
+      </c>
+      <c r="G22" s="39" t="s">
+        <v>725</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16696,13 +17127,13 @@
         <v>387</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>700</v>
+        <v>736</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>701</v>
+        <v>737</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16718,14 +17149,14 @@
       <c r="D24" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E24" s="38" t="s">
-        <v>707</v>
+      <c r="E24" s="39" t="s">
+        <v>743</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>692</v>
-      </c>
-      <c r="G24" s="38" t="s">
-        <v>708</v>
+        <v>728</v>
+      </c>
+      <c r="G24" s="39" t="s">
+        <v>744</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16741,14 +17172,14 @@
       <c r="D25" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E25" s="38" t="s">
-        <v>694</v>
+      <c r="E25" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G25" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G25" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16764,14 +17195,14 @@
       <c r="D26" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E26" s="38" t="s">
-        <v>694</v>
+      <c r="E26" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G26" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G26" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16787,14 +17218,14 @@
       <c r="D27" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E27" s="38" t="s">
-        <v>694</v>
+      <c r="E27" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G27" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G27" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16810,14 +17241,14 @@
       <c r="D28" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E28" s="38" t="s">
-        <v>707</v>
+      <c r="E28" s="39" t="s">
+        <v>743</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>692</v>
-      </c>
-      <c r="G28" s="38" t="s">
-        <v>708</v>
+        <v>728</v>
+      </c>
+      <c r="G28" s="39" t="s">
+        <v>744</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16833,14 +17264,14 @@
       <c r="D29" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E29" s="38" t="s">
-        <v>694</v>
+      <c r="E29" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G29" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G29" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16856,14 +17287,14 @@
       <c r="D30" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E30" s="38" t="s">
-        <v>694</v>
+      <c r="E30" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G30" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G30" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16879,14 +17310,14 @@
       <c r="D31" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E31" s="38" t="s">
-        <v>694</v>
+      <c r="E31" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G31" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G31" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16902,14 +17333,14 @@
       <c r="D32" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E32" s="38" t="s">
-        <v>694</v>
+      <c r="E32" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G32" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G32" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16925,14 +17356,14 @@
       <c r="D33" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="E33" s="38" t="s">
-        <v>697</v>
+      <c r="E33" s="39" t="s">
+        <v>733</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G33" s="38" t="s">
-        <v>698</v>
+        <v>724</v>
+      </c>
+      <c r="G33" s="39" t="s">
+        <v>734</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16948,14 +17379,14 @@
       <c r="D34" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E34" s="38" t="s">
-        <v>707</v>
+      <c r="E34" s="39" t="s">
+        <v>743</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>692</v>
-      </c>
-      <c r="G34" s="38" t="s">
-        <v>708</v>
+        <v>728</v>
+      </c>
+      <c r="G34" s="39" t="s">
+        <v>744</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16971,14 +17402,14 @@
       <c r="D35" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E35" s="38" t="s">
-        <v>697</v>
+      <c r="E35" s="39" t="s">
+        <v>733</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G35" s="38" t="s">
-        <v>698</v>
+        <v>724</v>
+      </c>
+      <c r="G35" s="39" t="s">
+        <v>734</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16994,14 +17425,14 @@
       <c r="D36" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E36" s="38" t="s">
-        <v>694</v>
+      <c r="E36" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G36" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G36" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17017,14 +17448,14 @@
       <c r="D37" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E37" s="38" t="s">
-        <v>707</v>
+      <c r="E37" s="39" t="s">
+        <v>743</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>692</v>
-      </c>
-      <c r="G37" s="38" t="s">
-        <v>708</v>
+        <v>728</v>
+      </c>
+      <c r="G37" s="39" t="s">
+        <v>744</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17040,14 +17471,14 @@
       <c r="D38" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E38" s="38" t="s">
-        <v>694</v>
+      <c r="E38" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G38" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G38" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17064,13 +17495,13 @@
         <v>387</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>697</v>
+        <v>733</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>688</v>
+        <v>724</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>709</v>
+        <v>745</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17086,14 +17517,14 @@
       <c r="D40" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E40" s="38" t="s">
-        <v>694</v>
+      <c r="E40" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G40" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G40" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17101,7 +17532,7 @@
         <v>491</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>710</v>
+        <v>746</v>
       </c>
       <c r="C41" s="12" t="n">
         <v>440300</v>
@@ -17110,13 +17541,13 @@
         <v>382</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>703</v>
+        <v>739</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>704</v>
+        <v>740</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>711</v>
+        <v>747</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17132,14 +17563,14 @@
       <c r="D42" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E42" s="38" t="s">
-        <v>694</v>
+      <c r="E42" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G42" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G42" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17147,7 +17578,7 @@
         <v>491</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>712</v>
+        <v>748</v>
       </c>
       <c r="C43" s="12" t="n">
         <v>-88073</v>
@@ -17156,13 +17587,13 @@
         <v>387</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>700</v>
+        <v>736</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>701</v>
+        <v>737</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17179,13 +17610,13 @@
         <v>387</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>700</v>
+        <v>736</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>701</v>
+        <v>737</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17193,7 +17624,7 @@
         <v>491</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>713</v>
+        <v>749</v>
       </c>
       <c r="C45" s="12" t="n">
         <v>-36259</v>
@@ -17202,13 +17633,13 @@
         <v>387</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>700</v>
+        <v>736</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>701</v>
+        <v>737</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17225,13 +17656,13 @@
         <v>387</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>714</v>
+        <v>750</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>688</v>
+        <v>724</v>
       </c>
       <c r="G46" s="3" t="s">
-        <v>715</v>
+        <v>751</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17239,7 +17670,7 @@
         <v>498</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>702</v>
+        <v>738</v>
       </c>
       <c r="C47" s="12" t="n">
         <v>-77990</v>
@@ -17248,13 +17679,13 @@
         <v>387</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>700</v>
+        <v>736</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>701</v>
+        <v>737</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17270,14 +17701,14 @@
       <c r="D48" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E48" s="38" t="s">
-        <v>694</v>
+      <c r="E48" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G48" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G48" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17293,14 +17724,14 @@
       <c r="D49" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E49" s="38" t="s">
-        <v>707</v>
+      <c r="E49" s="39" t="s">
+        <v>743</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>692</v>
-      </c>
-      <c r="G49" s="38" t="s">
-        <v>708</v>
+        <v>728</v>
+      </c>
+      <c r="G49" s="39" t="s">
+        <v>744</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17316,14 +17747,14 @@
       <c r="D50" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E50" s="38" t="s">
-        <v>697</v>
+      <c r="E50" s="39" t="s">
+        <v>733</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G50" s="38" t="s">
-        <v>698</v>
+        <v>724</v>
+      </c>
+      <c r="G50" s="39" t="s">
+        <v>734</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17339,14 +17770,14 @@
       <c r="D51" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E51" s="38" t="s">
-        <v>694</v>
+      <c r="E51" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G51" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G51" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17362,14 +17793,14 @@
       <c r="D52" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E52" s="38" t="s">
-        <v>694</v>
+      <c r="E52" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G52" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G52" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17386,13 +17817,13 @@
         <v>387</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>691</v>
+        <v>727</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>693</v>
+        <v>729</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17408,14 +17839,14 @@
       <c r="D54" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E54" s="38" t="s">
-        <v>694</v>
+      <c r="E54" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G54" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G54" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17423,7 +17854,7 @@
         <v>505</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>690</v>
+        <v>726</v>
       </c>
       <c r="C55" s="12" t="n">
         <v>-1000000</v>
@@ -17432,13 +17863,13 @@
         <v>387</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>691</v>
+        <v>727</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>693</v>
+        <v>729</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17454,14 +17885,14 @@
       <c r="D56" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="E56" s="38" t="s">
-        <v>706</v>
+      <c r="E56" s="39" t="s">
+        <v>742</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G56" s="38" t="s">
-        <v>689</v>
+        <v>724</v>
+      </c>
+      <c r="G56" s="39" t="s">
+        <v>725</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17477,14 +17908,14 @@
       <c r="D57" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="E57" s="38" t="s">
-        <v>687</v>
+      <c r="E57" s="39" t="s">
+        <v>723</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G57" s="38" t="s">
-        <v>689</v>
+        <v>724</v>
+      </c>
+      <c r="G57" s="39" t="s">
+        <v>725</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17492,7 +17923,7 @@
         <v>505</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>716</v>
+        <v>752</v>
       </c>
       <c r="C58" s="12" t="n">
         <v>-83300</v>
@@ -17501,13 +17932,13 @@
         <v>387</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>700</v>
+        <v>736</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>701</v>
+        <v>737</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17523,14 +17954,14 @@
       <c r="D59" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E59" s="38" t="s">
-        <v>694</v>
+      <c r="E59" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G59" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G59" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17546,14 +17977,14 @@
       <c r="D60" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E60" s="38" t="s">
-        <v>694</v>
+      <c r="E60" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G60" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G60" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17569,14 +18000,14 @@
       <c r="D61" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E61" s="38" t="s">
-        <v>694</v>
+      <c r="E61" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G61" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G61" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17592,14 +18023,14 @@
       <c r="D62" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E62" s="38" t="s">
-        <v>694</v>
+      <c r="E62" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G62" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G62" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17615,14 +18046,14 @@
       <c r="D63" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E63" s="38" t="s">
-        <v>694</v>
+      <c r="E63" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G63" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G63" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17638,14 +18069,14 @@
       <c r="D64" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E64" s="38" t="s">
-        <v>694</v>
+      <c r="E64" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G64" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G64" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17661,14 +18092,14 @@
       <c r="D65" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E65" s="38" t="s">
-        <v>694</v>
+      <c r="E65" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G65" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G65" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17684,14 +18115,14 @@
       <c r="D66" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E66" s="38" t="s">
-        <v>694</v>
+      <c r="E66" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F66" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G66" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G66" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17708,13 +18139,13 @@
         <v>382</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>717</v>
+        <v>753</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>688</v>
+        <v>724</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>718</v>
+        <v>754</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17730,14 +18161,14 @@
       <c r="D68" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E68" s="38" t="s">
-        <v>694</v>
+      <c r="E68" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G68" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G68" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17753,14 +18184,14 @@
       <c r="D69" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E69" s="38" t="s">
-        <v>694</v>
+      <c r="E69" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F69" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G69" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G69" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17777,13 +18208,13 @@
         <v>387</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>691</v>
+        <v>727</v>
       </c>
       <c r="F70" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>693</v>
+        <v>729</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17791,7 +18222,7 @@
         <v>522</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>719</v>
+        <v>755</v>
       </c>
       <c r="C71" s="12" t="n">
         <v>-25000</v>
@@ -17800,13 +18231,13 @@
         <v>387</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>700</v>
+        <v>736</v>
       </c>
       <c r="F71" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G71" s="3" t="s">
-        <v>701</v>
+        <v>737</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17822,14 +18253,14 @@
       <c r="D72" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E72" s="38" t="s">
-        <v>694</v>
+      <c r="E72" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F72" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G72" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G72" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17845,14 +18276,14 @@
       <c r="D73" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E73" s="38" t="s">
-        <v>694</v>
+      <c r="E73" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F73" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G73" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G73" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17868,14 +18299,14 @@
       <c r="D74" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E74" s="38" t="s">
-        <v>694</v>
+      <c r="E74" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F74" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G74" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G74" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17891,14 +18322,14 @@
       <c r="D75" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E75" s="38" t="s">
-        <v>707</v>
+      <c r="E75" s="39" t="s">
+        <v>743</v>
       </c>
       <c r="F75" s="3" t="s">
-        <v>692</v>
-      </c>
-      <c r="G75" s="38" t="s">
-        <v>708</v>
+        <v>728</v>
+      </c>
+      <c r="G75" s="39" t="s">
+        <v>744</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17914,14 +18345,14 @@
       <c r="D76" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E76" s="38" t="s">
-        <v>694</v>
+      <c r="E76" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F76" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G76" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G76" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17937,14 +18368,14 @@
       <c r="D77" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E77" s="38" t="s">
-        <v>694</v>
+      <c r="E77" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F77" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G77" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G77" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17960,14 +18391,14 @@
       <c r="D78" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E78" s="38" t="s">
-        <v>707</v>
+      <c r="E78" s="39" t="s">
+        <v>743</v>
       </c>
       <c r="F78" s="3" t="s">
-        <v>692</v>
-      </c>
-      <c r="G78" s="38" t="s">
-        <v>708</v>
+        <v>728</v>
+      </c>
+      <c r="G78" s="39" t="s">
+        <v>744</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17975,7 +18406,7 @@
         <v>522</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>690</v>
+        <v>726</v>
       </c>
       <c r="C79" s="12" t="n">
         <v>-1000000</v>
@@ -17984,13 +18415,13 @@
         <v>387</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>691</v>
+        <v>727</v>
       </c>
       <c r="F79" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G79" s="3" t="s">
-        <v>693</v>
+        <v>729</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18006,14 +18437,14 @@
       <c r="D80" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="E80" s="38" t="s">
-        <v>697</v>
+      <c r="E80" s="39" t="s">
+        <v>733</v>
       </c>
       <c r="F80" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G80" s="38" t="s">
-        <v>698</v>
+        <v>724</v>
+      </c>
+      <c r="G80" s="39" t="s">
+        <v>734</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18029,14 +18460,14 @@
       <c r="D81" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E81" s="38" t="s">
-        <v>694</v>
+      <c r="E81" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F81" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G81" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G81" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18052,14 +18483,14 @@
       <c r="D82" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E82" s="38" t="s">
-        <v>694</v>
+      <c r="E82" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F82" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G82" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G82" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18075,14 +18506,14 @@
       <c r="D83" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E83" s="38" t="s">
-        <v>694</v>
+      <c r="E83" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F83" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G83" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G83" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18099,13 +18530,13 @@
         <v>387</v>
       </c>
       <c r="E84" s="3" t="s">
-        <v>720</v>
+        <v>756</v>
       </c>
       <c r="F84" s="3" t="s">
-        <v>688</v>
+        <v>724</v>
       </c>
       <c r="G84" s="3" t="s">
-        <v>693</v>
+        <v>729</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18121,14 +18552,14 @@
       <c r="D85" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E85" s="38" t="s">
-        <v>707</v>
+      <c r="E85" s="39" t="s">
+        <v>743</v>
       </c>
       <c r="F85" s="3" t="s">
-        <v>692</v>
-      </c>
-      <c r="G85" s="38" t="s">
-        <v>708</v>
+        <v>728</v>
+      </c>
+      <c r="G85" s="39" t="s">
+        <v>744</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18144,14 +18575,14 @@
       <c r="D86" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E86" s="38" t="s">
-        <v>707</v>
+      <c r="E86" s="39" t="s">
+        <v>743</v>
       </c>
       <c r="F86" s="3" t="s">
-        <v>692</v>
-      </c>
-      <c r="G86" s="38" t="s">
-        <v>708</v>
+        <v>728</v>
+      </c>
+      <c r="G86" s="39" t="s">
+        <v>744</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18167,14 +18598,14 @@
       <c r="D87" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E87" s="38" t="s">
-        <v>697</v>
+      <c r="E87" s="39" t="s">
+        <v>733</v>
       </c>
       <c r="F87" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G87" s="38" t="s">
-        <v>698</v>
+        <v>724</v>
+      </c>
+      <c r="G87" s="39" t="s">
+        <v>734</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18191,13 +18622,13 @@
         <v>382</v>
       </c>
       <c r="E88" s="3" t="s">
-        <v>717</v>
+        <v>753</v>
       </c>
       <c r="F88" s="3" t="s">
-        <v>688</v>
+        <v>724</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>718</v>
+        <v>754</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18205,7 +18636,7 @@
         <v>532</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>690</v>
+        <v>726</v>
       </c>
       <c r="C89" s="12" t="n">
         <v>-160000</v>
@@ -18214,13 +18645,13 @@
         <v>387</v>
       </c>
       <c r="E89" s="3" t="s">
-        <v>691</v>
+        <v>727</v>
       </c>
       <c r="F89" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G89" s="3" t="s">
-        <v>693</v>
+        <v>729</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18236,14 +18667,14 @@
       <c r="D90" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="E90" s="38" t="s">
-        <v>687</v>
+      <c r="E90" s="39" t="s">
+        <v>723</v>
       </c>
       <c r="F90" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G90" s="38" t="s">
-        <v>689</v>
+        <v>724</v>
+      </c>
+      <c r="G90" s="39" t="s">
+        <v>725</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18251,7 +18682,7 @@
         <v>532</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>690</v>
+        <v>726</v>
       </c>
       <c r="C91" s="12" t="n">
         <v>-150000</v>
@@ -18260,13 +18691,13 @@
         <v>387</v>
       </c>
       <c r="E91" s="3" t="s">
-        <v>691</v>
+        <v>727</v>
       </c>
       <c r="F91" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G91" s="3" t="s">
-        <v>693</v>
+        <v>729</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18282,14 +18713,14 @@
       <c r="D92" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E92" s="38" t="s">
-        <v>694</v>
+      <c r="E92" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F92" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G92" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G92" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18306,13 +18737,13 @@
         <v>387</v>
       </c>
       <c r="E93" s="3" t="s">
-        <v>700</v>
+        <v>736</v>
       </c>
       <c r="F93" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G93" s="3" t="s">
-        <v>701</v>
+        <v>737</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18328,14 +18759,14 @@
       <c r="D94" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E94" s="38" t="s">
-        <v>694</v>
+      <c r="E94" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F94" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G94" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G94" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18351,14 +18782,14 @@
       <c r="D95" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E95" s="38" t="s">
-        <v>694</v>
+      <c r="E95" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F95" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G95" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G95" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18374,14 +18805,14 @@
       <c r="D96" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E96" s="38" t="s">
-        <v>694</v>
+      <c r="E96" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F96" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G96" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G96" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18397,14 +18828,14 @@
       <c r="D97" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E97" s="38" t="s">
-        <v>694</v>
+      <c r="E97" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F97" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G97" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G97" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18412,7 +18843,7 @@
         <v>542</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>721</v>
+        <v>757</v>
       </c>
       <c r="C98" s="12" t="n">
         <v>-405600</v>
@@ -18421,13 +18852,13 @@
         <v>387</v>
       </c>
       <c r="E98" s="3" t="s">
-        <v>722</v>
+        <v>758</v>
       </c>
       <c r="F98" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G98" s="3" t="s">
-        <v>723</v>
+        <v>759</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18435,7 +18866,7 @@
         <v>542</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>690</v>
+        <v>726</v>
       </c>
       <c r="C99" s="12" t="n">
         <v>-1000000</v>
@@ -18444,13 +18875,13 @@
         <v>387</v>
       </c>
       <c r="E99" s="3" t="s">
-        <v>691</v>
+        <v>727</v>
       </c>
       <c r="F99" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G99" s="3" t="s">
-        <v>693</v>
+        <v>729</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18467,13 +18898,13 @@
         <v>387</v>
       </c>
       <c r="E100" s="3" t="s">
-        <v>700</v>
+        <v>736</v>
       </c>
       <c r="F100" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G100" s="3" t="s">
-        <v>701</v>
+        <v>737</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18489,14 +18920,14 @@
       <c r="D101" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E101" s="38" t="s">
-        <v>694</v>
+      <c r="E101" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F101" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G101" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G101" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18512,14 +18943,14 @@
       <c r="D102" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E102" s="38" t="s">
-        <v>694</v>
+      <c r="E102" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F102" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G102" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G102" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18536,13 +18967,13 @@
         <v>387</v>
       </c>
       <c r="E103" s="3" t="s">
-        <v>700</v>
+        <v>736</v>
       </c>
       <c r="F103" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G103" s="3" t="s">
-        <v>701</v>
+        <v>737</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18558,14 +18989,14 @@
       <c r="D104" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E104" s="38" t="s">
-        <v>694</v>
+      <c r="E104" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F104" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G104" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G104" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18581,14 +19012,14 @@
       <c r="D105" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="E105" s="38" t="s">
-        <v>697</v>
+      <c r="E105" s="39" t="s">
+        <v>733</v>
       </c>
       <c r="F105" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G105" s="38" t="s">
-        <v>698</v>
+        <v>724</v>
+      </c>
+      <c r="G105" s="39" t="s">
+        <v>734</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18604,14 +19035,14 @@
       <c r="D106" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E106" s="38" t="s">
-        <v>694</v>
+      <c r="E106" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F106" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G106" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G106" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18627,14 +19058,14 @@
       <c r="D107" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E107" s="38" t="s">
-        <v>694</v>
+      <c r="E107" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F107" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G107" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G107" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18651,13 +19082,13 @@
         <v>387</v>
       </c>
       <c r="E108" s="3" t="s">
-        <v>700</v>
+        <v>736</v>
       </c>
       <c r="F108" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G108" s="3" t="s">
-        <v>701</v>
+        <v>737</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18674,13 +19105,13 @@
         <v>387</v>
       </c>
       <c r="E109" s="3" t="s">
-        <v>700</v>
+        <v>736</v>
       </c>
       <c r="F109" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G109" s="3" t="s">
-        <v>701</v>
+        <v>737</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18688,7 +19119,7 @@
         <v>559</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>724</v>
+        <v>760</v>
       </c>
       <c r="C110" s="12" t="n">
         <v>-6950</v>
@@ -18696,14 +19127,14 @@
       <c r="D110" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E110" s="38" t="s">
-        <v>697</v>
+      <c r="E110" s="39" t="s">
+        <v>733</v>
       </c>
       <c r="F110" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G110" s="38" t="s">
-        <v>698</v>
+        <v>724</v>
+      </c>
+      <c r="G110" s="39" t="s">
+        <v>734</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18719,14 +19150,14 @@
       <c r="D111" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E111" s="38" t="s">
-        <v>707</v>
+      <c r="E111" s="39" t="s">
+        <v>743</v>
       </c>
       <c r="F111" s="3" t="s">
-        <v>692</v>
-      </c>
-      <c r="G111" s="38" t="s">
-        <v>708</v>
+        <v>728</v>
+      </c>
+      <c r="G111" s="39" t="s">
+        <v>744</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18742,14 +19173,14 @@
       <c r="D112" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E112" s="38" t="s">
-        <v>694</v>
+      <c r="E112" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F112" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G112" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G112" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18766,13 +19197,13 @@
         <v>387</v>
       </c>
       <c r="E113" s="3" t="s">
-        <v>700</v>
+        <v>736</v>
       </c>
       <c r="F113" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G113" s="3" t="s">
-        <v>701</v>
+        <v>737</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18788,14 +19219,14 @@
       <c r="D114" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E114" s="38" t="s">
-        <v>694</v>
+      <c r="E114" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F114" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G114" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G114" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18811,14 +19242,14 @@
       <c r="D115" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E115" s="38" t="s">
-        <v>694</v>
+      <c r="E115" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F115" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G115" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G115" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18826,7 +19257,7 @@
         <v>559</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>725</v>
+        <v>761</v>
       </c>
       <c r="C116" s="12" t="n">
         <v>-38000</v>
@@ -18835,13 +19266,13 @@
         <v>387</v>
       </c>
       <c r="E116" s="3" t="s">
-        <v>700</v>
+        <v>736</v>
       </c>
       <c r="F116" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G116" s="3" t="s">
-        <v>701</v>
+        <v>737</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18857,14 +19288,14 @@
       <c r="D117" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E117" s="38" t="s">
-        <v>694</v>
+      <c r="E117" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F117" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G117" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G117" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18880,14 +19311,14 @@
       <c r="D118" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E118" s="38" t="s">
-        <v>707</v>
+      <c r="E118" s="39" t="s">
+        <v>743</v>
       </c>
       <c r="F118" s="3" t="s">
-        <v>692</v>
-      </c>
-      <c r="G118" s="38" t="s">
-        <v>708</v>
+        <v>728</v>
+      </c>
+      <c r="G118" s="39" t="s">
+        <v>744</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18895,7 +19326,7 @@
         <v>559</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>726</v>
+        <v>762</v>
       </c>
       <c r="C119" s="12" t="n">
         <v>-66878</v>
@@ -18903,14 +19334,14 @@
       <c r="D119" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E119" s="38" t="s">
-        <v>697</v>
+      <c r="E119" s="39" t="s">
+        <v>733</v>
       </c>
       <c r="F119" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G119" s="38" t="s">
-        <v>698</v>
+        <v>724</v>
+      </c>
+      <c r="G119" s="39" t="s">
+        <v>734</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18926,14 +19357,14 @@
       <c r="D120" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E120" s="38" t="s">
-        <v>694</v>
+      <c r="E120" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F120" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G120" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G120" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18949,14 +19380,14 @@
       <c r="D121" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E121" s="38" t="s">
-        <v>707</v>
+      <c r="E121" s="39" t="s">
+        <v>743</v>
       </c>
       <c r="F121" s="3" t="s">
-        <v>692</v>
-      </c>
-      <c r="G121" s="38" t="s">
-        <v>708</v>
+        <v>728</v>
+      </c>
+      <c r="G121" s="39" t="s">
+        <v>744</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18964,7 +19395,7 @@
         <v>559</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>727</v>
+        <v>763</v>
       </c>
       <c r="C122" s="12" t="n">
         <v>-296037</v>
@@ -18973,13 +19404,13 @@
         <v>387</v>
       </c>
       <c r="E122" s="3" t="s">
-        <v>700</v>
+        <v>736</v>
       </c>
       <c r="F122" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G122" s="3" t="s">
-        <v>701</v>
+        <v>737</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18995,14 +19426,14 @@
       <c r="D123" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="E123" s="38" t="s">
-        <v>697</v>
+      <c r="E123" s="39" t="s">
+        <v>733</v>
       </c>
       <c r="F123" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G123" s="38" t="s">
-        <v>698</v>
+        <v>724</v>
+      </c>
+      <c r="G123" s="39" t="s">
+        <v>734</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19018,14 +19449,14 @@
       <c r="D124" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="E124" s="38" t="s">
-        <v>697</v>
+      <c r="E124" s="39" t="s">
+        <v>733</v>
       </c>
       <c r="F124" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G124" s="38" t="s">
-        <v>698</v>
+        <v>724</v>
+      </c>
+      <c r="G124" s="39" t="s">
+        <v>734</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19041,14 +19472,14 @@
       <c r="D125" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="E125" s="38" t="s">
-        <v>706</v>
+      <c r="E125" s="39" t="s">
+        <v>742</v>
       </c>
       <c r="F125" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G125" s="38" t="s">
-        <v>689</v>
+        <v>724</v>
+      </c>
+      <c r="G125" s="39" t="s">
+        <v>725</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19056,7 +19487,7 @@
         <v>559</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>728</v>
+        <v>764</v>
       </c>
       <c r="C126" s="12" t="n">
         <v>-58001</v>
@@ -19064,14 +19495,14 @@
       <c r="D126" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E126" s="38" t="s">
-        <v>697</v>
+      <c r="E126" s="39" t="s">
+        <v>733</v>
       </c>
       <c r="F126" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G126" s="38" t="s">
-        <v>698</v>
+        <v>724</v>
+      </c>
+      <c r="G126" s="39" t="s">
+        <v>734</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19087,14 +19518,14 @@
       <c r="D127" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E127" s="38" t="s">
-        <v>694</v>
+      <c r="E127" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F127" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G127" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G127" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19110,14 +19541,14 @@
       <c r="D128" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E128" s="38" t="s">
-        <v>694</v>
+      <c r="E128" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F128" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G128" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G128" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19125,7 +19556,7 @@
         <v>572</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>729</v>
+        <v>765</v>
       </c>
       <c r="C129" s="12" t="n">
         <v>-97000</v>
@@ -19133,14 +19564,14 @@
       <c r="D129" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E129" s="38" t="s">
-        <v>694</v>
+      <c r="E129" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F129" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G129" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G129" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19148,7 +19579,7 @@
         <v>572</v>
       </c>
       <c r="B130" s="3" t="s">
-        <v>690</v>
+        <v>726</v>
       </c>
       <c r="C130" s="12" t="n">
         <v>-800000</v>
@@ -19157,13 +19588,13 @@
         <v>387</v>
       </c>
       <c r="E130" s="3" t="s">
-        <v>691</v>
+        <v>727</v>
       </c>
       <c r="F130" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G130" s="3" t="s">
-        <v>693</v>
+        <v>729</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19179,14 +19610,14 @@
       <c r="D131" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E131" s="38" t="s">
-        <v>694</v>
+      <c r="E131" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F131" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G131" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G131" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19202,14 +19633,14 @@
       <c r="D132" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E132" s="38" t="s">
-        <v>694</v>
+      <c r="E132" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F132" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G132" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G132" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19225,14 +19656,14 @@
       <c r="D133" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E133" s="38" t="s">
-        <v>694</v>
+      <c r="E133" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F133" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G133" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G133" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19248,14 +19679,14 @@
       <c r="D134" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E134" s="38" t="s">
-        <v>707</v>
+      <c r="E134" s="39" t="s">
+        <v>743</v>
       </c>
       <c r="F134" s="3" t="s">
-        <v>692</v>
-      </c>
-      <c r="G134" s="38" t="s">
-        <v>708</v>
+        <v>728</v>
+      </c>
+      <c r="G134" s="39" t="s">
+        <v>744</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19271,14 +19702,14 @@
       <c r="D135" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E135" s="38" t="s">
-        <v>707</v>
+      <c r="E135" s="39" t="s">
+        <v>743</v>
       </c>
       <c r="F135" s="3" t="s">
-        <v>692</v>
-      </c>
-      <c r="G135" s="38" t="s">
-        <v>708</v>
+        <v>728</v>
+      </c>
+      <c r="G135" s="39" t="s">
+        <v>744</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19294,14 +19725,14 @@
       <c r="D136" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E136" s="38" t="s">
-        <v>694</v>
+      <c r="E136" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F136" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G136" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G136" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19317,14 +19748,14 @@
       <c r="D137" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E137" s="38" t="s">
-        <v>694</v>
+      <c r="E137" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F137" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G137" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G137" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19340,14 +19771,14 @@
       <c r="D138" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="E138" s="38" t="s">
-        <v>687</v>
+      <c r="E138" s="39" t="s">
+        <v>723</v>
       </c>
       <c r="F138" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G138" s="38" t="s">
-        <v>689</v>
+        <v>724</v>
+      </c>
+      <c r="G138" s="39" t="s">
+        <v>725</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19363,14 +19794,14 @@
       <c r="D139" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E139" s="38" t="s">
-        <v>694</v>
+      <c r="E139" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F139" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G139" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G139" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19378,7 +19809,7 @@
         <v>445</v>
       </c>
       <c r="B140" s="3" t="s">
-        <v>690</v>
+        <v>726</v>
       </c>
       <c r="C140" s="12" t="n">
         <v>-700000</v>
@@ -19387,13 +19818,13 @@
         <v>387</v>
       </c>
       <c r="E140" s="3" t="s">
-        <v>691</v>
+        <v>727</v>
       </c>
       <c r="F140" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G140" s="3" t="s">
-        <v>693</v>
+        <v>729</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19409,14 +19840,14 @@
       <c r="D141" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="E141" s="38" t="s">
-        <v>706</v>
+      <c r="E141" s="39" t="s">
+        <v>742</v>
       </c>
       <c r="F141" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G141" s="38" t="s">
-        <v>689</v>
+        <v>724</v>
+      </c>
+      <c r="G141" s="39" t="s">
+        <v>725</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19433,13 +19864,13 @@
         <v>387</v>
       </c>
       <c r="E142" s="3" t="s">
-        <v>700</v>
+        <v>736</v>
       </c>
       <c r="F142" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G142" s="3" t="s">
-        <v>701</v>
+        <v>737</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19455,14 +19886,14 @@
       <c r="D143" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E143" s="38" t="s">
-        <v>694</v>
+      <c r="E143" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F143" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G143" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G143" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19478,14 +19909,14 @@
       <c r="D144" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E144" s="38" t="s">
-        <v>694</v>
+      <c r="E144" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F144" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G144" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G144" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19501,14 +19932,14 @@
       <c r="D145" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E145" s="38" t="s">
-        <v>707</v>
+      <c r="E145" s="39" t="s">
+        <v>743</v>
       </c>
       <c r="F145" s="3" t="s">
-        <v>692</v>
-      </c>
-      <c r="G145" s="38" t="s">
-        <v>708</v>
+        <v>728</v>
+      </c>
+      <c r="G145" s="39" t="s">
+        <v>744</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19525,13 +19956,13 @@
         <v>382</v>
       </c>
       <c r="E146" s="3" t="s">
-        <v>717</v>
+        <v>753</v>
       </c>
       <c r="F146" s="3" t="s">
-        <v>688</v>
+        <v>724</v>
       </c>
       <c r="G146" s="3" t="s">
-        <v>718</v>
+        <v>754</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19547,14 +19978,14 @@
       <c r="D147" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E147" s="38" t="s">
-        <v>694</v>
+      <c r="E147" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F147" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G147" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G147" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19571,13 +20002,13 @@
         <v>387</v>
       </c>
       <c r="E148" s="3" t="s">
-        <v>700</v>
+        <v>736</v>
       </c>
       <c r="F148" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G148" s="3" t="s">
-        <v>701</v>
+        <v>737</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19585,7 +20016,7 @@
         <v>450</v>
       </c>
       <c r="B149" s="3" t="s">
-        <v>730</v>
+        <v>766</v>
       </c>
       <c r="C149" s="12" t="n">
         <v>-46550</v>
@@ -19594,13 +20025,13 @@
         <v>387</v>
       </c>
       <c r="E149" s="3" t="s">
-        <v>700</v>
+        <v>736</v>
       </c>
       <c r="F149" s="3" t="s">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="G149" s="3" t="s">
-        <v>701</v>
+        <v>737</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19616,14 +20047,14 @@
       <c r="D150" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E150" s="38" t="s">
-        <v>694</v>
+      <c r="E150" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F150" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G150" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G150" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19639,19 +20070,19 @@
       <c r="D151" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E151" s="38" t="s">
-        <v>694</v>
+      <c r="E151" s="39" t="s">
+        <v>730</v>
       </c>
       <c r="F151" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="G151" s="38" t="s">
-        <v>695</v>
+        <v>724</v>
+      </c>
+      <c r="G151" s="39" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="2" t="s">
-        <v>731</v>
+        <v>767</v>
       </c>
       <c r="B153" s="2"/>
       <c r="C153" s="2"/>
@@ -19662,18 +20093,18 @@
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="9" t="s">
-        <v>732</v>
+        <v>768</v>
       </c>
       <c r="B154" s="9" t="s">
-        <v>733</v>
+        <v>769</v>
       </c>
       <c r="C154" s="9" t="s">
-        <v>734</v>
+        <v>770</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="3" t="s">
-        <v>694</v>
+        <v>730</v>
       </c>
       <c r="B155" s="3" t="n">
         <v>72</v>
@@ -19684,7 +20115,7 @@
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="3" t="s">
-        <v>691</v>
+        <v>727</v>
       </c>
       <c r="B156" s="3" t="n">
         <v>10</v>
@@ -19695,7 +20126,7 @@
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="3" t="s">
-        <v>700</v>
+        <v>736</v>
       </c>
       <c r="B157" s="3" t="n">
         <v>20</v>
@@ -19706,7 +20137,7 @@
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="3" t="s">
-        <v>707</v>
+        <v>743</v>
       </c>
       <c r="B158" s="3" t="n">
         <v>15</v>
@@ -19717,7 +20148,7 @@
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="3" t="s">
-        <v>722</v>
+        <v>758</v>
       </c>
       <c r="B159" s="3" t="n">
         <v>1</v>
@@ -19728,7 +20159,7 @@
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="3" t="s">
-        <v>714</v>
+        <v>750</v>
       </c>
       <c r="B160" s="3" t="n">
         <v>1</v>
@@ -19739,7 +20170,7 @@
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="3" t="s">
-        <v>720</v>
+        <v>756</v>
       </c>
       <c r="B161" s="3" t="n">
         <v>1</v>
@@ -19750,7 +20181,7 @@
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="3" t="s">
-        <v>703</v>
+        <v>739</v>
       </c>
       <c r="B162" s="3" t="n">
         <v>2</v>
@@ -19761,7 +20192,7 @@
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="3" t="s">
-        <v>697</v>
+        <v>733</v>
       </c>
       <c r="B163" s="3" t="n">
         <v>14</v>
@@ -19772,7 +20203,7 @@
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="3" t="s">
-        <v>706</v>
+        <v>742</v>
       </c>
       <c r="B164" s="3" t="n">
         <v>4</v>
@@ -19783,7 +20214,7 @@
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="3" t="s">
-        <v>687</v>
+        <v>723</v>
       </c>
       <c r="B165" s="3" t="n">
         <v>4</v>
@@ -19794,7 +20225,7 @@
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="3" t="s">
-        <v>717</v>
+        <v>753</v>
       </c>
       <c r="B166" s="3" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Agrega hoja Seguimiento_Factoring (plantilla correo + logica Centinela 3 fuentes)
</commit_message>
<xml_diff>
--- a/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
+++ b/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
@@ -17,7 +17,8 @@
     <sheet name="Real_vs_Presupuesto" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="Resumen_Ejecutivo" sheetId="8" state="visible" r:id="rId10"/>
     <sheet name="Categorizacion_Cartola_Julio" sheetId="9" state="visible" r:id="rId11"/>
-    <sheet name="Bitácora_Saldo_Diario" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="Seguimiento_Factoring" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="Bitácora_Saldo_Diario" sheetId="11" state="visible" r:id="rId13"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3077" uniqueCount="782">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3118" uniqueCount="815">
   <si>
     <t xml:space="preserve">SUPUESTOS DEL PRESUPUESTO — SOLLEM + TRAST</t>
   </si>
@@ -2360,6 +2361,105 @@
   </si>
   <si>
     <t xml:space="preserve">Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SEGUIMIENTO DE OPERACIONES CON FACTORING — plantilla para enviar por correo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copiar la tabla de abajo (filas 5 en adelante) y enviarla a cada entidad de factoring para que complete las columnas H, I, J (Estado actual / Días de Mora / Monto en Mora). Las columnas A-G ya las llenamos nosotros con lo que tenemos registrado. Al recibir la respuesta, actualizar acá y avisar para correr el Centinela (3 fuentes: nuestro registro + respuesta del factoring + cartola real — ver notas abajo).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entidad Factoring</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N° Operación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cliente (deudor)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N° Factura(s)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monto Financiado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha Compromiso Pago</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nuestro Estado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estado (factoring)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Días Mora (factoring)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monto Mora (factoring)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Observaciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LATAM Trade Capital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">103103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-07-31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pagado — confirmado cartola 31-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Financia Capital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20 + 1 doc adicional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-07-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pagado — confirmado cartola 17-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-07-22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pagado — confirmado cartola 22-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45910523</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26 + 29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Programado — aún no vence, sin confirmar en cartola</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CÓMO TRABAJA EL CENTINELA (3 fuentes cruzadas, no solo días transcurridos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Factoring reporta 'Pagado' pero NO hay abono en la cartola → ALERTA INMEDIATA (posible pago a cuenta equivocada).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Factoring reporta 'En mora' → ALERTA INMEDIATA, sin esperar ningún umbral de días — su información manda sobre nuestro conteo interno.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Monto en mora reportado por el factoring NO calza con nuestro Monto Financiado esperado → ALERTA de discrepancia, investigar antes de aceptar cualquiera de los 2 números.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Factoring no responde el correo dentro de 5 días hábiles → ALERTA 'sin respuesta', reenviar y escalar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Fecha Compromiso de Pago ya pasó y el factoring no ha dicho nada (ni pagado ni mora) → respaldo del umbral de 75 días de PROC-FIN-14 — se usa solo cuando no hay respuesta directa de ellos, es el último recurso, no la primera línea.</t>
   </si>
   <si>
     <t xml:space="preserve">BITÁCORA DE SALDO DIARIO — Banco Santander 0-000-3776731-0</t>
@@ -3444,6 +3544,303 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:K15"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="30"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>771</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="24" t="s">
+        <v>772</v>
+      </c>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
+      <c r="I2" s="24"/>
+      <c r="J2" s="24"/>
+      <c r="K2" s="24"/>
+    </row>
+    <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
+        <v>773</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>774</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>775</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>776</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>777</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>778</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>779</v>
+      </c>
+      <c r="H4" s="9" t="s">
+        <v>780</v>
+      </c>
+      <c r="I4" s="9" t="s">
+        <v>781</v>
+      </c>
+      <c r="J4" s="9" t="s">
+        <v>782</v>
+      </c>
+      <c r="K4" s="9" t="s">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>784</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>785</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>699</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="E5" s="12" t="n">
+        <v>4773447</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>786</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>787</v>
+      </c>
+      <c r="H5" s="40"/>
+      <c r="I5" s="40"/>
+      <c r="J5" s="40"/>
+      <c r="K5" s="40"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>788</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3" t="s">
+        <v>699</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>789</v>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>2972144</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>790</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>791</v>
+      </c>
+      <c r="H6" s="40"/>
+      <c r="I6" s="40"/>
+      <c r="J6" s="40"/>
+      <c r="K6" s="40"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>788</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3" t="s">
+        <v>699</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>439</v>
+      </c>
+      <c r="E7" s="12" t="n">
+        <v>2387616</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>792</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>793</v>
+      </c>
+      <c r="H7" s="40"/>
+      <c r="I7" s="40"/>
+      <c r="J7" s="40"/>
+      <c r="K7" s="40"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>794</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>688</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>795</v>
+      </c>
+      <c r="E8" s="12" t="n">
+        <v>3099712</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>796</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>797</v>
+      </c>
+      <c r="H8" s="40"/>
+      <c r="I8" s="40"/>
+      <c r="J8" s="40"/>
+      <c r="K8" s="40"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>798</v>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
+    </row>
+    <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="24" t="s">
+        <v>799</v>
+      </c>
+      <c r="B11" s="24"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="24"/>
+      <c r="E11" s="24"/>
+      <c r="F11" s="24"/>
+      <c r="G11" s="24"/>
+      <c r="H11" s="24"/>
+      <c r="I11" s="24"/>
+      <c r="J11" s="24"/>
+      <c r="K11" s="24"/>
+    </row>
+    <row r="12" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="24" t="s">
+        <v>800</v>
+      </c>
+      <c r="B12" s="24"/>
+      <c r="C12" s="24"/>
+      <c r="D12" s="24"/>
+      <c r="E12" s="24"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="24"/>
+      <c r="H12" s="24"/>
+      <c r="I12" s="24"/>
+      <c r="J12" s="24"/>
+      <c r="K12" s="24"/>
+    </row>
+    <row r="13" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="24" t="s">
+        <v>801</v>
+      </c>
+      <c r="B13" s="24"/>
+      <c r="C13" s="24"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="24"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="24"/>
+      <c r="H13" s="24"/>
+      <c r="I13" s="24"/>
+      <c r="J13" s="24"/>
+      <c r="K13" s="24"/>
+    </row>
+    <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="24" t="s">
+        <v>802</v>
+      </c>
+      <c r="B14" s="24"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="24"/>
+      <c r="H14" s="24"/>
+      <c r="I14" s="24"/>
+      <c r="J14" s="24"/>
+      <c r="K14" s="24"/>
+    </row>
+    <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="24" t="s">
+        <v>803</v>
+      </c>
+      <c r="B15" s="24"/>
+      <c r="C15" s="24"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="24"/>
+      <c r="F15" s="24"/>
+      <c r="G15" s="24"/>
+      <c r="H15" s="24"/>
+      <c r="I15" s="24"/>
+      <c r="J15" s="24"/>
+      <c r="K15" s="24"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A10:K10"/>
+    <mergeCell ref="A11:K11"/>
+    <mergeCell ref="A12:K12"/>
+    <mergeCell ref="A13:K13"/>
+    <mergeCell ref="A14:K14"/>
+    <mergeCell ref="A15:K15"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:F31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -3454,7 +3851,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>771</v>
+        <v>804</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3464,7 +3861,7 @@
     </row>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="24" t="s">
-        <v>772</v>
+        <v>805</v>
       </c>
       <c r="B2" s="24"/>
       <c r="C2" s="24"/>
@@ -3477,16 +3874,16 @@
         <v>376</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>773</v>
+        <v>806</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>774</v>
+        <v>807</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>775</v>
+        <v>808</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>776</v>
+        <v>809</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>188</v>
@@ -3500,23 +3897,23 @@
         <v>63371</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>777</v>
+        <v>810</v>
       </c>
       <c r="D5" s="38"/>
       <c r="E5" s="38"/>
       <c r="F5" s="3" t="s">
-        <v>778</v>
+        <v>811</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>779</v>
+        <v>812</v>
       </c>
       <c r="B6" s="12" t="n">
         <v>1275801</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>780</v>
+        <v>813</v>
       </c>
       <c r="D6" s="34"/>
       <c r="E6" s="12" t="str">
@@ -3524,7 +3921,7 @@
         <v/>
       </c>
       <c r="F6" s="3" t="s">
-        <v>781</v>
+        <v>814</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Agrega hoja Seguimiento_Pago_Clientes con mora real Sollem (LATAM 04-08-2026)
</commit_message>
<xml_diff>
--- a/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
+++ b/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
@@ -18,7 +18,8 @@
     <sheet name="Resumen_Ejecutivo" sheetId="8" state="visible" r:id="rId10"/>
     <sheet name="Categorizacion_Cartola_Julio" sheetId="9" state="visible" r:id="rId11"/>
     <sheet name="Seguimiento_Factoring" sheetId="10" state="visible" r:id="rId12"/>
-    <sheet name="Bitácora_Saldo_Diario" sheetId="11" state="visible" r:id="rId13"/>
+    <sheet name="Seguimiento_Pago_Clientes" sheetId="11" state="visible" r:id="rId13"/>
+    <sheet name="Bitácora_Saldo_Diario" sheetId="12" state="visible" r:id="rId14"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3118" uniqueCount="815">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3160" uniqueCount="837">
   <si>
     <t xml:space="preserve">SUPUESTOS DEL PRESUPUESTO — SOLLEM + TRAST</t>
   </si>
@@ -2460,6 +2461,72 @@
   </si>
   <si>
     <t xml:space="preserve">5. Fecha Compromiso de Pago ya pasó y el factoring no ha dicho nada (ni pagado ni mora) → respaldo del umbral de 75 días de PROC-FIN-14 — se usa solo cuando no hay respuesta directa de ellos, es el último recurso, no la primera línea.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SEGUIMIENTO DE PAGO — CLIENTES (envío semanal informativo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copiar la tabla de abajo y enviarla semanalmente a cada cliente — objetivo: que tengan clara la fecha de vencimiento ANTES de que llegue, para presionar el pago a tiempo y evitar mora con el factoring. Fuente: kaptura_cuentas_por_cobrar + comunicaciones reales de las entidades de factoring (ej. correo LATAM Trade Capital 04-08-2026).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha Vencimiento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Días para Vencer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monto en Mora</t>
+  </si>
+  <si>
+    <t xml:space="preserve">761,776,754,741,747,763,775,74,745,794,807,832,830,827</t>
+  </si>
+  <si>
+    <t xml:space="preserve">—</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MORA YA LIQUIDADA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmado por LATAM Trade Capital 04-08-2026, incluye pago 08-07 de $315.876</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1-Global-841-836-832</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Por confirmar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PENDIENTE DE LIQUIDAR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmado por LATAM Trade Capital 04-08-2026 — sin fecha de vencimiento aún informada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vence hoy/mañana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Programado (factoring)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Financiamiento en trámite, aún no confirmado en cartola</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Facturado, sin fecha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pendiente definir fecha de vencimiento con el cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Danilo Enrique Núñez Osorio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24 (junio)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOTA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filas rojas = mora confirmada. Filas amarillas = operación en trámite, sin confirmar todavía. Actualizar cada semana con la Fecha de Vencimiento real de cada factura antes de enviar — hoy varias figuran "Por confirmar" porque no tenemos ese dato todavía.</t>
   </si>
   <si>
     <t xml:space="preserve">BITÁCORA DE SALDO DIARIO — Banco Santander 0-000-3776731-0</t>
@@ -2609,7 +2676,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2638,6 +2705,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor rgb="FFD9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -2690,7 +2769,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="44">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2855,6 +2934,18 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2901,11 +2992,11 @@
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FFFFEB9C"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFFFC7CE"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -3841,6 +3932,244 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:H12"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="30"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>804</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="24" t="s">
+        <v>805</v>
+      </c>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
+    </row>
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>776</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>378</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>806</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>807</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>808</v>
+      </c>
+      <c r="H4" s="9" t="s">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>699</v>
+      </c>
+      <c r="B5" s="41" t="s">
+        <v>809</v>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>1991728</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>810</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>810</v>
+      </c>
+      <c r="F5" s="42" t="s">
+        <v>811</v>
+      </c>
+      <c r="G5" s="12" t="n">
+        <v>1991728</v>
+      </c>
+      <c r="H5" s="41" t="s">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>699</v>
+      </c>
+      <c r="B6" s="41" t="s">
+        <v>813</v>
+      </c>
+      <c r="C6" s="12" t="n">
+        <v>508969</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>814</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>810</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>815</v>
+      </c>
+      <c r="G6" s="12" t="n">
+        <v>508969</v>
+      </c>
+      <c r="H6" s="41" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>688</v>
+      </c>
+      <c r="B7" s="41" t="s">
+        <v>795</v>
+      </c>
+      <c r="C7" s="12" t="n">
+        <v>3053216</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>796</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>817</v>
+      </c>
+      <c r="F7" s="43" t="s">
+        <v>818</v>
+      </c>
+      <c r="G7" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="41" t="s">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>694</v>
+      </c>
+      <c r="B8" s="41" t="s">
+        <v>447</v>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>1428000</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>814</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>810</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>820</v>
+      </c>
+      <c r="G8" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="41" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>822</v>
+      </c>
+      <c r="B9" s="41" t="s">
+        <v>823</v>
+      </c>
+      <c r="C9" s="12" t="n">
+        <v>690200</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>814</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>810</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>820</v>
+      </c>
+      <c r="G9" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="41" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>824</v>
+      </c>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+    </row>
+    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="s">
+        <v>825</v>
+      </c>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="10"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A12:H12"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:F31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -3851,7 +4180,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>804</v>
+        <v>826</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3861,7 +4190,7 @@
     </row>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="24" t="s">
-        <v>805</v>
+        <v>827</v>
       </c>
       <c r="B2" s="24"/>
       <c r="C2" s="24"/>
@@ -3874,16 +4203,16 @@
         <v>376</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>806</v>
+        <v>828</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>807</v>
+        <v>829</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>808</v>
+        <v>830</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>809</v>
+        <v>831</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>188</v>
@@ -3897,23 +4226,23 @@
         <v>63371</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>810</v>
+        <v>832</v>
       </c>
       <c r="D5" s="38"/>
       <c r="E5" s="38"/>
       <c r="F5" s="3" t="s">
-        <v>811</v>
+        <v>833</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>812</v>
+        <v>834</v>
       </c>
       <c r="B6" s="12" t="n">
         <v>1275801</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>813</v>
+        <v>835</v>
       </c>
       <c r="D6" s="34"/>
       <c r="E6" s="12" t="str">
@@ -3921,7 +4250,7 @@
         <v/>
       </c>
       <c r="F6" s="3" t="s">
-        <v>814</v>
+        <v>836</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Agrega hoja Control_Caja_7_Dias (3 bloques separados); cierra gap kaptura_caja 24jul-02ago; responde instrucciones del Director
</commit_message>
<xml_diff>
--- a/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
+++ b/finanzas/conciliacion_bancaria/Presupuesto_Flujo_Caja_Conciliacion_Ago_Sep_2026.xlsx
@@ -19,7 +19,8 @@
     <sheet name="Categorizacion_Cartola_Julio" sheetId="9" state="visible" r:id="rId11"/>
     <sheet name="Seguimiento_Factoring" sheetId="10" state="visible" r:id="rId12"/>
     <sheet name="Seguimiento_Pago_Clientes" sheetId="11" state="visible" r:id="rId13"/>
-    <sheet name="Bitácora_Saldo_Diario" sheetId="12" state="visible" r:id="rId14"/>
+    <sheet name="Control_Caja_7_Dias" sheetId="12" state="visible" r:id="rId14"/>
+    <sheet name="Bitácora_Saldo_Diario" sheetId="13" state="visible" r:id="rId15"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3160" uniqueCount="837">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3197" uniqueCount="858">
   <si>
     <t xml:space="preserve">SUPUESTOS DEL PRESUPUESTO — SOLLEM + TRAST</t>
   </si>
@@ -2527,6 +2528,69 @@
   </si>
   <si>
     <t xml:space="preserve">Filas rojas = mora confirmada. Filas amarillas = operación en trámite, sin confirmar todavía. Actualizar cada semana con la Fecha de Vencimiento real de cada factura antes de enviar — hoy varias figuran "Por confirmar" porque no tenemos ese dato todavía.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONTROL DE CAJA — PRÓXIMOS 7 DÍAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Global Solutions SPA — al 06-08-2026. 3 bloques separados: REAL (lo que ya está en el banco) / PRESUPUESTO-PROVISIÓN (÷20 días hábiles, regla fija) / SERVICIOS REALES (kaptura, no facturados aún).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BLOQUE 1 — SALDO REAL HOY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Banco Santander</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aramco (estimado: topups−consumo real)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copec (reembolso directo, sin saldo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL SALDO REAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BLOQUE 2 — PRESUPUESTO / PROVISIÓN (7 días = Consolidado Agosto ÷ 20 días hábiles × 7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ventas presupuestadas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viáticos (regla: $12.000×3 equipos×7d)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peajes (regla: $50.000/servicio×servicios/semana)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remuneraciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BLOQUE 3 — SERVICIOS REALES (kaptura_cuentas_por_facturar / por_cobrar, no presupuesto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pendiente de facturar (10 de 11 servicios agosto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pendiente de facturar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pendiente de facturar (agosto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sin servicios en agosto — confirmado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Presmita (jul)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Danilo Núñez (jun)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sollem — mora LATAM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CxC — mora a cobrar</t>
   </si>
   <si>
     <t xml:space="preserve">BITÁCORA DE SALDO DIARIO — Banco Santander 0-000-3776731-0</t>
@@ -4170,6 +4234,259 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:C28"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>826</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="24" t="s">
+        <v>827</v>
+      </c>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>828</v>
+      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>829</v>
+      </c>
+      <c r="B6" s="12" t="n">
+        <v>339213</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>830</v>
+      </c>
+      <c r="B7" s="12" t="n">
+        <v>4556521</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>831</v>
+      </c>
+      <c r="B8" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="15" t="s">
+        <v>832</v>
+      </c>
+      <c r="B9" s="17" t="n">
+        <v>4895734</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>833</v>
+      </c>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
+        <v>834</v>
+      </c>
+      <c r="B13" s="12" t="n">
+        <v>10290931</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B14" s="12" t="n">
+        <v>2010000</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
+        <v>835</v>
+      </c>
+      <c r="B15" s="12" t="n">
+        <v>252000</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
+        <v>836</v>
+      </c>
+      <c r="B16" s="12" t="n">
+        <v>303333</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>837</v>
+      </c>
+      <c r="B17" s="12" t="n">
+        <v>2174087</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>838</v>
+      </c>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>378</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>699</v>
+      </c>
+      <c r="B21" s="12" t="n">
+        <v>3596789</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
+        <v>696</v>
+      </c>
+      <c r="B22" s="12" t="n">
+        <v>576037</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
+        <v>694</v>
+      </c>
+      <c r="B23" s="12" t="n">
+        <v>450000</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
+        <v>701</v>
+      </c>
+      <c r="B24" s="12" t="n">
+        <v>420000</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="s">
+        <v>697</v>
+      </c>
+      <c r="B25" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="s">
+        <v>843</v>
+      </c>
+      <c r="B26" s="12" t="n">
+        <v>1699320</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="3" t="s">
+        <v>844</v>
+      </c>
+      <c r="B27" s="12" t="n">
+        <v>821338</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="3" t="s">
+        <v>845</v>
+      </c>
+      <c r="B28" s="12" t="n">
+        <v>508969</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>846</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A19:C19"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:F31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -4180,7 +4497,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>826</v>
+        <v>847</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4190,7 +4507,7 @@
     </row>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="24" t="s">
-        <v>827</v>
+        <v>848</v>
       </c>
       <c r="B2" s="24"/>
       <c r="C2" s="24"/>
@@ -4203,16 +4520,16 @@
         <v>376</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>828</v>
+        <v>849</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>829</v>
+        <v>850</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>830</v>
+        <v>851</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>831</v>
+        <v>852</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>188</v>
@@ -4226,23 +4543,23 @@
         <v>63371</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>832</v>
+        <v>853</v>
       </c>
       <c r="D5" s="38"/>
       <c r="E5" s="38"/>
       <c r="F5" s="3" t="s">
-        <v>833</v>
+        <v>854</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>834</v>
+        <v>855</v>
       </c>
       <c r="B6" s="12" t="n">
         <v>1275801</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>835</v>
+        <v>856</v>
       </c>
       <c r="D6" s="34"/>
       <c r="E6" s="12" t="str">
@@ -4250,7 +4567,7 @@
         <v/>
       </c>
       <c r="F6" s="3" t="s">
-        <v>836</v>
+        <v>857</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>